<commit_message>
Auto pipeline update 2026-02-24 16:07:51
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0832189-B742-47A0-863E-F1D3733FAA7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7960855B-C925-4E83-AB01-57F09A0DD5FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="787" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="787" activeTab="1" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet Names Check" sheetId="1" r:id="rId1"/>
-    <sheet name="TB 408 Stringing Template Check" sheetId="2" r:id="rId2"/>
-    <sheet name="TA 509 Erection Template Check" sheetId="3" r:id="rId3"/>
+    <sheet name="TB 401 Stringing Template Check" sheetId="6" r:id="rId2"/>
+    <sheet name="TB 408 Stringing Template Check" sheetId="2" r:id="rId3"/>
+    <sheet name="TA 509 Erection Template Check" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="78">
   <si>
     <t>Project Code</t>
   </si>
@@ -254,13 +255,34 @@
   </si>
   <si>
     <t>Stringing Template Check</t>
+  </si>
+  <si>
+    <t>Stringing - PKG-G</t>
+  </si>
+  <si>
+    <t>S. No</t>
+  </si>
+  <si>
+    <t>Paying Out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of Gang </t>
+  </si>
+  <si>
+    <t>Finish Date</t>
+  </si>
+  <si>
+    <t>Month</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -307,8 +329,27 @@
       <family val="1"/>
       <scheme val="major"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -339,8 +380,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD8D8D8"/>
+        <bgColor rgb="FFD8D8D8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -444,13 +491,136 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -497,13 +667,68 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="8">
+    <cellStyle name="Comma 2" xfId="5" xr:uid="{1517F127-7F55-42AF-952C-D923BD4ECBE3}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 15" xfId="1" xr:uid="{34FE60CE-A1DA-4616-AA23-0BBDDF9DD7D6}"/>
+    <cellStyle name="Normal 2" xfId="4" xr:uid="{E561867F-C8CF-4869-A143-7DB56F2EE69B}"/>
+    <cellStyle name="Normal 3" xfId="6" xr:uid="{02E4DB69-C37B-458C-97B6-3E554FA1E55A}"/>
+    <cellStyle name="Normal 4" xfId="7" xr:uid="{91588BA5-8ED7-4728-AC43-559C5A5DAACB}"/>
+    <cellStyle name="Normal 5" xfId="3" xr:uid="{72642DE1-8DD2-444D-8A81-E2A5D7BD22B8}"/>
     <cellStyle name="Normal 8 2" xfId="2" xr:uid="{E356B690-246D-43B2-86AF-A6FE97B16461}"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -871,7 +1096,11 @@
   <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="4" width="10.453125" customWidth="1"/>
+    <col min="1" max="1" width="10.453125" customWidth="1"/>
+    <col min="2" max="2" width="28.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -1039,7 +1268,7 @@
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>9</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -1053,7 +1282,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>27</v>
       </c>
@@ -1064,15 +1293,24 @@
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>28</v>
       </c>
       <c r="B18" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>29</v>
       </c>
@@ -1080,12 +1318,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -1102,6 +1340,142 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0CAA689-52FE-4282-BFA7-7FA3F37BB8D4}">
+  <dimension ref="A2:W7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="22"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F3" s="22"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" s="22"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="L3" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="M3" s="16"/>
+      <c r="N3" s="17"/>
+    </row>
+    <row r="4" spans="1:23" ht="31" x14ac:dyDescent="0.35">
+      <c r="A4" s="25"/>
+      <c r="B4" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="F4" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="G4" s="26" t="s">
+        <v>77</v>
+      </c>
+      <c r="H4" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="I4" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="J4" s="26" t="s">
+        <v>77</v>
+      </c>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="19"/>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="H7" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="L7" s="4"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="4"/>
+      <c r="R7" s="3"/>
+      <c r="T7" s="3"/>
+      <c r="U7" s="3"/>
+      <c r="V7" s="3"/>
+      <c r="W7" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="A3:A4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B7">
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C7">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B225AA6-68BC-47EB-9948-84B6B216E727}">
   <dimension ref="A2:W7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1245,7 +1619,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBFB976A-1B92-4632-9799-0237B459A61D}">
   <dimension ref="A1:P5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Auto pipeline update 2026-03-03 12:13:27
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7960855B-C925-4E83-AB01-57F09A0DD5FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AFEDFCD-5AC2-4451-83C2-3D962A2B4680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="787" activeTab="1" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet Names Check" sheetId="1" r:id="rId1"/>
     <sheet name="TB 401 Stringing Template Check" sheetId="6" r:id="rId2"/>
     <sheet name="TB 408 Stringing Template Check" sheetId="2" r:id="rId3"/>
     <sheet name="TA 509 Erection Template Check" sheetId="3" r:id="rId4"/>
+    <sheet name="TA 601 Erection Template Check" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="85">
   <si>
     <t>Project Code</t>
   </si>
@@ -273,6 +274,27 @@
   </si>
   <si>
     <t>Month</t>
+  </si>
+  <si>
+    <t>Tower Type</t>
+  </si>
+  <si>
+    <t>Classification</t>
+  </si>
+  <si>
+    <t>MT</t>
+  </si>
+  <si>
+    <t>Gang Strength</t>
+  </si>
+  <si>
+    <t>Tower Weight</t>
+  </si>
+  <si>
+    <t>Erection Line Names</t>
+  </si>
+  <si>
+    <t>TA 605 - Jammu; TA 605 - Punjab</t>
   </si>
 </sst>
 </file>
@@ -282,7 +304,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -348,8 +370,14 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -386,8 +414,14 @@
         <bgColor rgb="FFD8D8D8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor rgb="FF00B0F0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="19">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -609,6 +643,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color theme="8" tint="0.39997558519241921"/>
+      </left>
+      <right style="medium">
+        <color theme="8" tint="0.39997558519241921"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -620,7 +665,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -643,30 +688,6 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -679,9 +700,25 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -690,12 +727,29 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -763,14 +817,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DBDF0E1F-C881-4514-9437-5BEB0B253989}" name="Table1" displayName="Table1" ref="A1:E21" totalsRowShown="0">
-  <autoFilter ref="A1:E21" xr:uid="{DBDF0E1F-C881-4514-9437-5BEB0B253989}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DBDF0E1F-C881-4514-9437-5BEB0B253989}" name="Table1" displayName="Table1" ref="A1:F21" totalsRowShown="0">
+  <autoFilter ref="A1:F21" xr:uid="{DBDF0E1F-C881-4514-9437-5BEB0B253989}"/>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1C0814EE-AA83-4802-806C-8F58A35BCB7F}" name="Project Code"/>
     <tableColumn id="2" xr3:uid="{648AD748-C4AF-4406-94C1-AD47F69D9A33}" name="Erection Sheet Names"/>
     <tableColumn id="3" xr3:uid="{21E38DD6-7CC4-48AB-83F3-B20FE2132DBD}" name="Stringing Sheet Names"/>
     <tableColumn id="4" xr3:uid="{5D52F2DE-F5A4-4050-A631-7A7FCEDEEF0F}" name="Erection Template Check"/>
     <tableColumn id="5" xr3:uid="{9023B235-6439-4C22-8371-541AC872F757}" name="Stringing Template Check"/>
+    <tableColumn id="6" xr3:uid="{626EFD59-910E-4A23-B6DD-324D4B001C75}" name="Erection Line Names"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1093,7 +1148,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEA00114-109C-4365-898D-B35AA94B9EEF}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" customWidth="1"/>
@@ -1103,7 +1158,7 @@
     <col min="5" max="5" width="24.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1119,16 +1174,22 @@
       <c r="E1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1139,7 +1200,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1150,7 +1211,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1161,7 +1222,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -1172,7 +1233,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1180,7 +1241,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -1191,7 +1252,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1202,7 +1263,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -1213,7 +1274,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -1224,7 +1285,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1235,7 +1296,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1246,7 +1307,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1260,7 +1321,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -1271,7 +1332,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1350,66 +1411,66 @@
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="21" t="s">
+      <c r="C3" s="20"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="22"/>
-      <c r="G3" s="23"/>
-      <c r="H3" s="21" t="s">
+      <c r="F3" s="20"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="I3" s="22"/>
-      <c r="J3" s="23"/>
-      <c r="K3" s="20" t="s">
+      <c r="I3" s="20"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="L3" s="24" t="s">
+      <c r="L3" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="M3" s="16"/>
-      <c r="N3" s="17"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="31" x14ac:dyDescent="0.35">
-      <c r="A4" s="25"/>
-      <c r="B4" s="26" t="s">
+      <c r="A4" s="18"/>
+      <c r="B4" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="E4" s="26" t="s">
+      <c r="E4" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="G4" s="26" t="s">
+      <c r="G4" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="H4" s="26" t="s">
+      <c r="H4" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="I4" s="26" t="s">
+      <c r="I4" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="J4" s="26" t="s">
+      <c r="J4" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="K4" s="25"/>
-      <c r="L4" s="25"/>
-      <c r="M4" s="18"/>
-      <c r="N4" s="19"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="11"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -1458,12 +1519,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="E3:G3"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="K3:K4"/>
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="A3:A4"/>
   </mergeCells>
   <conditionalFormatting sqref="B7">
     <cfRule type="duplicateValues" dxfId="3" priority="2"/>
@@ -1486,46 +1547,46 @@
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11" t="s">
+      <c r="C3" s="26"/>
+      <c r="D3" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="G3" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="8" t="s">
+      <c r="H3" s="27"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="10"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="24"/>
+      <c r="M3" s="24"/>
+      <c r="N3" s="25"/>
     </row>
     <row r="4" spans="1:23" ht="26" x14ac:dyDescent="0.35">
-      <c r="A4" s="11"/>
+      <c r="A4" s="26"/>
       <c r="B4" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
       <c r="G4" s="1" t="s">
         <v>36</v>
       </c>
@@ -1656,14 +1717,14 @@
       <c r="C3" s="7"/>
       <c r="D3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="15"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="30"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="13"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="15"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="29"/>
+      <c r="P3" s="30"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -1687,6 +1748,101 @@
         <v>66</v>
       </c>
       <c r="F5" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="N3:P3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46CC22E7-0431-4564-825A-DCAC81041178}">
+  <dimension ref="A1:P5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="26" x14ac:dyDescent="0.35">
+      <c r="A2" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="G2" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C3" s="7"/>
+      <c r="D3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="30"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="29"/>
+      <c r="P3" s="30"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="I5" s="6" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto pipeline update 2026-03-10 12:09:27
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -8,17 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AFEDFCD-5AC2-4451-83C2-3D962A2B4680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B076A407-5D36-4761-9F9E-6F389CDF3CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" activeTab="4" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet Names Check" sheetId="1" r:id="rId1"/>
-    <sheet name="TB 401 Stringing Template Check" sheetId="6" r:id="rId2"/>
-    <sheet name="TB 408 Stringing Template Check" sheetId="2" r:id="rId3"/>
-    <sheet name="TA 509 Erection Template Check" sheetId="3" r:id="rId4"/>
-    <sheet name="TA 601 Erection Template Check" sheetId="7" r:id="rId5"/>
+    <sheet name="Test 000 Stringing 132kV" sheetId="11" r:id="rId2"/>
+    <sheet name="Test 000 Stringing 220kV" sheetId="10" r:id="rId3"/>
+    <sheet name="Test 000 Erection 220kV" sheetId="9" r:id="rId4"/>
+    <sheet name="Test 000 Erection 132kV" sheetId="8" r:id="rId5"/>
+    <sheet name="TB 401 Stringing" sheetId="6" r:id="rId6"/>
+    <sheet name="TB 408 Stringing" sheetId="2" r:id="rId7"/>
+    <sheet name="TA 509 Erection" sheetId="3" r:id="rId8"/>
+    <sheet name="TA 601 Erection" sheetId="7" r:id="rId9"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId10"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="151">
   <si>
     <t>Project Code</t>
   </si>
@@ -295,16 +302,220 @@
   </si>
   <si>
     <t>TA 605 - Jammu; TA 605 - Punjab</t>
+  </si>
+  <si>
+    <t>Test 000</t>
+  </si>
+  <si>
+    <t>Progress-132kV, Progress-220kV</t>
+  </si>
+  <si>
+    <t>Stringing Line Names</t>
+  </si>
+  <si>
+    <t>Erection 132kV; Erection 220 kV</t>
+  </si>
+  <si>
+    <t>Stringing 132kV; Stringing 220kV</t>
+  </si>
+  <si>
+    <t>Stringing-132KV; Stringing-220kV</t>
+  </si>
+  <si>
+    <t>Stringing Progress (Conductor &amp; Earthwire)</t>
+  </si>
+  <si>
+    <t>OPGW Progress</t>
+  </si>
+  <si>
+    <t>Stringing Section</t>
+  </si>
+  <si>
+    <t>Sl. No.</t>
+  </si>
+  <si>
+    <t>Section Length (m)</t>
+  </si>
+  <si>
+    <t>Stretch Readiness</t>
+  </si>
+  <si>
+    <t>Insulator Hoisting</t>
+  </si>
+  <si>
+    <t>Conductor Paying Out</t>
+  </si>
+  <si>
+    <t>Clipping</t>
+  </si>
+  <si>
+    <t>Spacer</t>
+  </si>
+  <si>
+    <t>Jumper</t>
+  </si>
+  <si>
+    <t>Sub-Contractor Name</t>
+  </si>
+  <si>
+    <t>MP</t>
+  </si>
+  <si>
+    <t>OPGW Paying Out</t>
+  </si>
+  <si>
+    <t>OPGW Final Sag</t>
+  </si>
+  <si>
+    <t>DOS</t>
+  </si>
+  <si>
+    <t>DOC</t>
+  </si>
+  <si>
+    <t>Sec</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Section Readiness</t>
+  </si>
+  <si>
+    <t>Jumpering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spacering </t>
+  </si>
+  <si>
+    <t>Number of Fitters</t>
+  </si>
+  <si>
+    <t>Hindrance</t>
+  </si>
+  <si>
+    <t>220 KV D/C Neemuch - TS</t>
+  </si>
+  <si>
+    <t>Foundation</t>
+  </si>
+  <si>
+    <t>Earthing</t>
+  </si>
+  <si>
+    <t>Tower Checking-1</t>
+  </si>
+  <si>
+    <t>Tack-Welding</t>
+  </si>
+  <si>
+    <t>Tower Checking-2</t>
+  </si>
+  <si>
+    <t>LOC NO</t>
+  </si>
+  <si>
+    <t>Stub Weight</t>
+  </si>
+  <si>
+    <t>Chimney Extension</t>
+  </si>
+  <si>
+    <t>Span Length(m)</t>
+  </si>
+  <si>
+    <t>Excavation Volume (m3)</t>
+  </si>
+  <si>
+    <t>Concreting Volume</t>
+  </si>
+  <si>
+    <t>8mm Steel</t>
+  </si>
+  <si>
+    <t>10mm Steel</t>
+  </si>
+  <si>
+    <t>12mm Steel</t>
+  </si>
+  <si>
+    <t>16mm Steel</t>
+  </si>
+  <si>
+    <t>20mm Steel</t>
+  </si>
+  <si>
+    <t>25mmSteel</t>
+  </si>
+  <si>
+    <t>Total Steel (MT)</t>
+  </si>
+  <si>
+    <t>Status
+(C/WIP)</t>
+  </si>
+  <si>
+    <t>Excavation</t>
+  </si>
+  <si>
+    <t>Concreting</t>
+  </si>
+  <si>
+    <t>Status
+C/WIP</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Painting</t>
+  </si>
+  <si>
+    <t>HT</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>BnA</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>M10
+(1:3:6) (m3)</t>
+  </si>
+  <si>
+    <t>M20 (1:1.5:3) (m3)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="166" formatCode="[$-4009]0.00"/>
+    <numFmt numFmtId="167" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -376,8 +587,22 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -420,8 +645,26 @@
         <bgColor rgb="FF00B0F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFAEABAB"/>
+        <bgColor rgb="FFAEABAB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="20">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -654,6 +897,210 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="double">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="double">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="double">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="double">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -665,7 +1112,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -715,18 +1162,21 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -750,6 +1200,168 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="9" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="10" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -762,7 +1374,47 @@
     <cellStyle name="Normal 5" xfId="3" xr:uid="{72642DE1-8DD2-444D-8A81-E2A5D7BD22B8}"/>
     <cellStyle name="Normal 8 2" xfId="2" xr:uid="{E356B690-246D-43B2-86AF-A6FE97B16461}"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -816,16 +1468,75 @@
 </styleSheet>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Detail Survey-220kV"/>
+      <sheetName val="Check Survey-220kV"/>
+      <sheetName val="Detail Survey-132kV"/>
+      <sheetName val="Check Survey-132kV"/>
+      <sheetName val="Summary"/>
+      <sheetName val="Statutory"/>
+      <sheetName val="Progress-132kV"/>
+      <sheetName val="Progress-220kV"/>
+      <sheetName val="Stringing-220kV"/>
+      <sheetName val="Stringing-132KV"/>
+      <sheetName val="VC-220kV"/>
+      <sheetName val="VC-132kV"/>
+      <sheetName val="Supply"/>
+      <sheetName val="Mail Body"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4">
+        <row r="2">
+          <cell r="A2" t="str">
+            <v>Name of the Line: 220KV DC AL59 line from Neemuch - Chanderiya + 132KV DC ACSS Line from Chanderiya to Hindustan Zinc</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="A4" t="str">
+            <v>Office:  Neemuch</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="A5" t="str">
+            <v>Progress of 220kV Line</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DBDF0E1F-C881-4514-9437-5BEB0B253989}" name="Table1" displayName="Table1" ref="A1:F21" totalsRowShown="0">
-  <autoFilter ref="A1:F21" xr:uid="{DBDF0E1F-C881-4514-9437-5BEB0B253989}"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DBDF0E1F-C881-4514-9437-5BEB0B253989}" name="Table1" displayName="Table1" ref="A1:G22" totalsRowShown="0">
+  <autoFilter ref="A1:G22" xr:uid="{DBDF0E1F-C881-4514-9437-5BEB0B253989}"/>
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{1C0814EE-AA83-4802-806C-8F58A35BCB7F}" name="Project Code"/>
     <tableColumn id="2" xr3:uid="{648AD748-C4AF-4406-94C1-AD47F69D9A33}" name="Erection Sheet Names"/>
     <tableColumn id="3" xr3:uid="{21E38DD6-7CC4-48AB-83F3-B20FE2132DBD}" name="Stringing Sheet Names"/>
     <tableColumn id="4" xr3:uid="{5D52F2DE-F5A4-4050-A631-7A7FCEDEEF0F}" name="Erection Template Check"/>
     <tableColumn id="5" xr3:uid="{9023B235-6439-4C22-8371-541AC872F757}" name="Stringing Template Check"/>
     <tableColumn id="6" xr3:uid="{626EFD59-910E-4A23-B6DD-324D4B001C75}" name="Erection Line Names"/>
+    <tableColumn id="7" xr3:uid="{6BB72CD2-5BEC-461E-851B-37A24191EC2F}" name="Stringing Line Names"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1148,7 +1859,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEA00114-109C-4365-898D-B35AA94B9EEF}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" customWidth="1"/>
@@ -1158,7 +1869,7 @@
     <col min="5" max="5" width="24.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1177,8 +1888,11 @@
       <c r="F1" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1189,7 +1903,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1200,7 +1914,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1211,7 +1925,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1222,7 +1936,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -1233,7 +1947,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1241,7 +1955,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -1252,7 +1966,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1263,7 +1977,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -1274,7 +1988,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -1285,7 +1999,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1296,7 +2010,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1307,7 +2021,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1321,7 +2035,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -1332,7 +2046,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1343,7 +2057,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>27</v>
       </c>
@@ -1354,7 +2068,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -1371,7 +2085,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>29</v>
       </c>
@@ -1379,17 +2093,40 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>31</v>
       </c>
       <c r="B21" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>85</v>
+      </c>
+      <c r="B22" t="s">
+        <v>86</v>
+      </c>
+      <c r="C22" t="s">
+        <v>90</v>
+      </c>
+      <c r="D22" t="s">
+        <v>67</v>
+      </c>
+      <c r="E22" t="s">
+        <v>67</v>
+      </c>
+      <c r="F22" t="s">
+        <v>88</v>
+      </c>
+      <c r="G22" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1401,6 +2138,1588 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAEF05BD-52B1-49ED-A017-76486C00039F}">
+  <dimension ref="A2:Z16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A3" s="32" t="str">
+        <f>+[1]Summary!A4</f>
+        <v>Office:  Neemuch</v>
+      </c>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="22"/>
+      <c r="R3" s="22"/>
+      <c r="S3" s="22"/>
+      <c r="T3" s="22"/>
+      <c r="U3" s="22"/>
+      <c r="V3" s="22"/>
+      <c r="W3" s="22"/>
+      <c r="X3" s="22"/>
+      <c r="Y3" s="22"/>
+      <c r="Z3" s="23"/>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A4" s="32">
+        <f>+[1]Summary!A7</f>
+        <v>0</v>
+      </c>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="34"/>
+      <c r="T4" s="32" t="s">
+        <v>92</v>
+      </c>
+      <c r="U4" s="22"/>
+      <c r="V4" s="22"/>
+      <c r="W4" s="22"/>
+      <c r="X4" s="22"/>
+      <c r="Y4" s="22"/>
+      <c r="Z4" s="23"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A5" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" s="22"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="35">
+        <f>[1]Summary!R7</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="36">
+        <f>SUMIF(E8:E215,"C",$D$6:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38">
+        <f>SUMIF(G9:G215,"WIP",$D$7:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="I5" s="36">
+        <f>SUMIF(G8:G215,"C",$D$6:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="37"/>
+      <c r="K5" s="38">
+        <f>SUMIF(J9:J215,"WIP",$D$7:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="36">
+        <f>SUMIF(J8:J215,"C",$D$6:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="37"/>
+      <c r="N5" s="37"/>
+      <c r="O5" s="37"/>
+      <c r="P5" s="37"/>
+      <c r="Q5" s="37"/>
+      <c r="R5" s="37"/>
+      <c r="S5" s="39"/>
+      <c r="T5" s="37"/>
+      <c r="U5" s="38">
+        <f>SUMIF(T9:T215,"WIP",$D$7:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="V5" s="38">
+        <f>SUMIF(T9:T215,"C",$D$7:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="W5" s="38"/>
+      <c r="X5" s="38">
+        <f>SUMIF(W9:W215,"WIP",$D$7:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="38">
+        <f>SUMIF(W9:W215,"C",$D$7:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="37"/>
+    </row>
+    <row r="6" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="40" t="s">
+        <v>94</v>
+      </c>
+      <c r="B6" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="23"/>
+      <c r="D6" s="40" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" s="42" t="s">
+        <v>96</v>
+      </c>
+      <c r="F6" s="43" t="s">
+        <v>97</v>
+      </c>
+      <c r="G6" s="44" t="s">
+        <v>98</v>
+      </c>
+      <c r="H6" s="22"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="22"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="45" t="s">
+        <v>99</v>
+      </c>
+      <c r="N6" s="46" t="s">
+        <v>100</v>
+      </c>
+      <c r="O6" s="47" t="s">
+        <v>101</v>
+      </c>
+      <c r="P6" s="48" t="s">
+        <v>102</v>
+      </c>
+      <c r="Q6" s="49" t="s">
+        <v>103</v>
+      </c>
+      <c r="R6" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="S6" s="50"/>
+      <c r="T6" s="51" t="s">
+        <v>104</v>
+      </c>
+      <c r="U6" s="22"/>
+      <c r="V6" s="23"/>
+      <c r="W6" s="51" t="s">
+        <v>105</v>
+      </c>
+      <c r="X6" s="22"/>
+      <c r="Y6" s="23"/>
+      <c r="Z6" s="48" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A7" s="40"/>
+      <c r="B7" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="52" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="40"/>
+      <c r="E7" s="53"/>
+      <c r="F7" s="54"/>
+      <c r="G7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="H7" s="55" t="s">
+        <v>106</v>
+      </c>
+      <c r="I7" s="47" t="s">
+        <v>107</v>
+      </c>
+      <c r="J7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="K7" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="L7" s="47" t="s">
+        <v>107</v>
+      </c>
+      <c r="M7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="N7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="O7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="P7" s="48"/>
+      <c r="Q7" s="56"/>
+      <c r="R7" s="54"/>
+      <c r="S7" s="57"/>
+      <c r="T7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="U7" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="V7" s="47" t="s">
+        <v>107</v>
+      </c>
+      <c r="W7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="X7" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="Y7" s="47" t="s">
+        <v>107</v>
+      </c>
+      <c r="Z7" s="48"/>
+    </row>
+    <row r="10" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="58" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="59" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="59" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="59" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="61" t="s">
+        <v>110</v>
+      </c>
+      <c r="F11" s="62" t="s">
+        <v>97</v>
+      </c>
+      <c r="H11" s="63" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" s="60" t="s">
+        <v>50</v>
+      </c>
+      <c r="K11" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="L11" s="64" t="s">
+        <v>53</v>
+      </c>
+      <c r="M11" s="66" t="s">
+        <v>99</v>
+      </c>
+      <c r="N11" s="65" t="s">
+        <v>112</v>
+      </c>
+      <c r="O11" s="58" t="s">
+        <v>111</v>
+      </c>
+      <c r="P11" s="59" t="s">
+        <v>35</v>
+      </c>
+      <c r="R11" s="66" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="16" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B16" s="59" t="s">
+        <v>108</v>
+      </c>
+      <c r="F16" s="60" t="s">
+        <v>109</v>
+      </c>
+      <c r="K16" s="59" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q16" s="67" t="s">
+        <v>54</v>
+      </c>
+      <c r="R16" s="59" t="s">
+        <v>55</v>
+      </c>
+      <c r="T16" s="59" t="s">
+        <v>81</v>
+      </c>
+      <c r="U16" s="59" t="s">
+        <v>113</v>
+      </c>
+      <c r="V16" s="59" t="s">
+        <v>114</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A3:Z3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="F4:R4"/>
+    <mergeCell ref="T4:Z4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="W6:Y6"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B11">
+    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C11">
+    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9301C2D9-B641-4509-82EB-A6381EB78A1E}">
+  <dimension ref="A2:Z11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A3" s="32" t="str">
+        <f>+[1]Summary!A4</f>
+        <v>Office:  Neemuch</v>
+      </c>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="22"/>
+      <c r="R3" s="22"/>
+      <c r="S3" s="22"/>
+      <c r="T3" s="22"/>
+      <c r="U3" s="22"/>
+      <c r="V3" s="22"/>
+      <c r="W3" s="22"/>
+      <c r="X3" s="22"/>
+      <c r="Y3" s="22"/>
+      <c r="Z3" s="23"/>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A4" s="32">
+        <f>+[1]Summary!A7</f>
+        <v>0</v>
+      </c>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="34"/>
+      <c r="T4" s="32" t="s">
+        <v>92</v>
+      </c>
+      <c r="U4" s="22"/>
+      <c r="V4" s="22"/>
+      <c r="W4" s="22"/>
+      <c r="X4" s="22"/>
+      <c r="Y4" s="22"/>
+      <c r="Z4" s="23"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A5" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" s="22"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="35">
+        <f>[1]Summary!R7</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="36">
+        <f>SUMIF(E8:E215,"C",$D$6:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38">
+        <f>SUMIF(G9:G215,"WIP",$D$7:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="I5" s="36">
+        <f>SUMIF(G8:G215,"C",$D$6:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="37"/>
+      <c r="K5" s="38">
+        <f>SUMIF(J9:J215,"WIP",$D$7:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="36">
+        <f>SUMIF(J8:J215,"C",$D$6:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="37"/>
+      <c r="N5" s="37"/>
+      <c r="O5" s="37"/>
+      <c r="P5" s="37"/>
+      <c r="Q5" s="37"/>
+      <c r="R5" s="37"/>
+      <c r="S5" s="39"/>
+      <c r="T5" s="37"/>
+      <c r="U5" s="38">
+        <f>SUMIF(T9:T215,"WIP",$D$7:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="V5" s="38">
+        <f>SUMIF(T9:T215,"C",$D$7:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="W5" s="38"/>
+      <c r="X5" s="38">
+        <f>SUMIF(W9:W215,"WIP",$D$7:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="38">
+        <f>SUMIF(W9:W215,"C",$D$7:$D$213)/1000</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="37"/>
+    </row>
+    <row r="6" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="40" t="s">
+        <v>94</v>
+      </c>
+      <c r="B6" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="23"/>
+      <c r="D6" s="40" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" s="42" t="s">
+        <v>96</v>
+      </c>
+      <c r="F6" s="43" t="s">
+        <v>97</v>
+      </c>
+      <c r="G6" s="44" t="s">
+        <v>98</v>
+      </c>
+      <c r="H6" s="22"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="22"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="45" t="s">
+        <v>99</v>
+      </c>
+      <c r="N6" s="46" t="s">
+        <v>100</v>
+      </c>
+      <c r="O6" s="47" t="s">
+        <v>101</v>
+      </c>
+      <c r="P6" s="48" t="s">
+        <v>102</v>
+      </c>
+      <c r="Q6" s="49" t="s">
+        <v>103</v>
+      </c>
+      <c r="R6" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="S6" s="50"/>
+      <c r="T6" s="51" t="s">
+        <v>104</v>
+      </c>
+      <c r="U6" s="22"/>
+      <c r="V6" s="23"/>
+      <c r="W6" s="51" t="s">
+        <v>105</v>
+      </c>
+      <c r="X6" s="22"/>
+      <c r="Y6" s="23"/>
+      <c r="Z6" s="48" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A7" s="40"/>
+      <c r="B7" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="52" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="40"/>
+      <c r="E7" s="53"/>
+      <c r="F7" s="54"/>
+      <c r="G7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="H7" s="55" t="s">
+        <v>106</v>
+      </c>
+      <c r="I7" s="47" t="s">
+        <v>107</v>
+      </c>
+      <c r="J7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="K7" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="L7" s="47" t="s">
+        <v>107</v>
+      </c>
+      <c r="M7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="N7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="O7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="P7" s="48"/>
+      <c r="Q7" s="56"/>
+      <c r="R7" s="54"/>
+      <c r="S7" s="57"/>
+      <c r="T7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="U7" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="V7" s="47" t="s">
+        <v>107</v>
+      </c>
+      <c r="W7" s="47" t="s">
+        <v>55</v>
+      </c>
+      <c r="X7" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="Y7" s="47" t="s">
+        <v>107</v>
+      </c>
+      <c r="Z7" s="48"/>
+    </row>
+    <row r="10" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="58" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="59" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="59" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="59" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="61" t="s">
+        <v>110</v>
+      </c>
+      <c r="F11" s="62" t="s">
+        <v>97</v>
+      </c>
+      <c r="H11" s="63" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" s="60" t="s">
+        <v>50</v>
+      </c>
+      <c r="K11" s="60" t="s">
+        <v>52</v>
+      </c>
+      <c r="L11" s="64" t="s">
+        <v>53</v>
+      </c>
+      <c r="M11" s="66" t="s">
+        <v>99</v>
+      </c>
+      <c r="N11" s="65" t="s">
+        <v>112</v>
+      </c>
+      <c r="O11" s="58" t="s">
+        <v>111</v>
+      </c>
+      <c r="P11" s="59" t="s">
+        <v>35</v>
+      </c>
+      <c r="R11" s="66" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A3:Z3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="F4:R4"/>
+    <mergeCell ref="T4:Z4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="W6:Y6"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B11">
+    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C11">
+    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B501B5B8-47AF-4D49-A01B-A8E1BEE40158}">
+  <dimension ref="A1:BA10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:53" x14ac:dyDescent="0.35">
+      <c r="A1" s="51" t="str">
+        <f>+[1]Summary!A2</f>
+        <v>Name of the Line: 220KV DC AL59 line from Neemuch - Chanderiya + 132KV DC ACSS Line from Chanderiya to Hindustan Zinc</v>
+      </c>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="N1" s="68"/>
+      <c r="O1" s="68"/>
+      <c r="P1" s="68"/>
+      <c r="Q1" s="68"/>
+      <c r="R1" s="68"/>
+      <c r="S1" s="68"/>
+      <c r="T1" s="68"/>
+      <c r="U1" s="68"/>
+      <c r="V1" s="68"/>
+      <c r="W1" s="68"/>
+      <c r="X1" s="68"/>
+      <c r="Y1" s="68"/>
+      <c r="Z1" s="68"/>
+      <c r="AA1" s="68"/>
+      <c r="AB1" s="68"/>
+      <c r="AC1" s="68"/>
+      <c r="AD1" s="68"/>
+      <c r="AE1" s="68"/>
+      <c r="AF1" s="68"/>
+      <c r="AG1" s="68"/>
+      <c r="AH1" s="68"/>
+      <c r="AI1" s="68"/>
+      <c r="AJ1" s="68"/>
+      <c r="AK1" s="68"/>
+      <c r="AL1" s="22"/>
+      <c r="AM1" s="22"/>
+      <c r="AN1" s="22"/>
+      <c r="AO1" s="22"/>
+      <c r="AP1" s="22"/>
+      <c r="AQ1" s="68"/>
+      <c r="AR1" s="68"/>
+      <c r="AS1" s="68"/>
+      <c r="AT1" s="68"/>
+      <c r="AU1" s="68"/>
+      <c r="AV1" s="68"/>
+      <c r="AW1" s="68"/>
+      <c r="AX1" s="68"/>
+      <c r="AY1" s="68"/>
+      <c r="AZ1" s="68"/>
+      <c r="BA1" s="69"/>
+    </row>
+    <row r="2" spans="1:53" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:53" x14ac:dyDescent="0.35">
+      <c r="A3" s="51" t="str">
+        <f>+[1]Summary!A5</f>
+        <v>Progress of 220kV Line</v>
+      </c>
+      <c r="B3" s="68"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
+      <c r="I3" s="68"/>
+      <c r="J3" s="68"/>
+      <c r="K3" s="68"/>
+      <c r="L3" s="68"/>
+      <c r="M3" s="68"/>
+      <c r="N3" s="68"/>
+      <c r="O3" s="68"/>
+      <c r="P3" s="68"/>
+      <c r="Q3" s="68"/>
+      <c r="R3" s="68"/>
+      <c r="S3" s="68"/>
+      <c r="T3" s="68"/>
+      <c r="U3" s="68"/>
+      <c r="V3" s="68"/>
+      <c r="W3" s="68"/>
+      <c r="X3" s="68"/>
+      <c r="Y3" s="68"/>
+      <c r="Z3" s="68"/>
+      <c r="AA3" s="68"/>
+      <c r="AB3" s="68"/>
+      <c r="AC3" s="68"/>
+      <c r="AD3" s="68"/>
+      <c r="AE3" s="68"/>
+      <c r="AF3" s="68"/>
+      <c r="AG3" s="68"/>
+      <c r="AH3" s="68"/>
+      <c r="AI3" s="68"/>
+      <c r="AJ3" s="68"/>
+      <c r="AK3" s="68"/>
+      <c r="AL3" s="22"/>
+      <c r="AM3" s="22"/>
+      <c r="AN3" s="22"/>
+      <c r="AO3" s="22"/>
+      <c r="AP3" s="22"/>
+      <c r="AQ3" s="68"/>
+      <c r="AR3" s="68"/>
+      <c r="AS3" s="68"/>
+      <c r="AT3" s="68"/>
+      <c r="AU3" s="68"/>
+      <c r="AV3" s="68"/>
+      <c r="AW3" s="68"/>
+      <c r="AX3" s="68"/>
+      <c r="AY3" s="68"/>
+      <c r="AZ3" s="68"/>
+      <c r="BA3" s="69"/>
+    </row>
+    <row r="4" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="51" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" s="68"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="68"/>
+      <c r="E4" s="68"/>
+      <c r="F4" s="68"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="68"/>
+      <c r="I4" s="68"/>
+      <c r="J4" s="68"/>
+      <c r="K4" s="68"/>
+      <c r="L4" s="68"/>
+      <c r="M4" s="68"/>
+      <c r="N4" s="68"/>
+      <c r="O4" s="68"/>
+      <c r="P4" s="68"/>
+      <c r="Q4" s="68"/>
+      <c r="R4" s="68"/>
+      <c r="S4" s="69"/>
+      <c r="T4" s="51" t="s">
+        <v>116</v>
+      </c>
+      <c r="U4" s="68"/>
+      <c r="V4" s="68"/>
+      <c r="W4" s="68"/>
+      <c r="X4" s="68"/>
+      <c r="Y4" s="68"/>
+      <c r="Z4" s="68"/>
+      <c r="AA4" s="68"/>
+      <c r="AB4" s="68"/>
+      <c r="AC4" s="68"/>
+      <c r="AD4" s="68"/>
+      <c r="AE4" s="68"/>
+      <c r="AF4" s="68"/>
+      <c r="AG4" s="68"/>
+      <c r="AH4" s="68"/>
+      <c r="AI4" s="68"/>
+      <c r="AJ4" s="68"/>
+      <c r="AK4" s="69"/>
+      <c r="AL4" s="51" t="s">
+        <v>117</v>
+      </c>
+      <c r="AM4" s="22"/>
+      <c r="AN4" s="22"/>
+      <c r="AO4" s="22"/>
+      <c r="AP4" s="23"/>
+      <c r="AQ4" s="51" t="s">
+        <v>2</v>
+      </c>
+      <c r="AR4" s="68"/>
+      <c r="AS4" s="68"/>
+      <c r="AT4" s="69"/>
+      <c r="AU4" s="43" t="s">
+        <v>118</v>
+      </c>
+      <c r="AV4" s="51" t="s">
+        <v>119</v>
+      </c>
+      <c r="AW4" s="68"/>
+      <c r="AX4" s="68"/>
+      <c r="AY4" s="68"/>
+      <c r="AZ4" s="69"/>
+      <c r="BA4" s="43" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:53" ht="58.5" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="48" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" s="48" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5" s="48" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="70"/>
+      <c r="E5" s="70"/>
+      <c r="F5" s="70"/>
+      <c r="G5" s="71" t="s">
+        <v>82</v>
+      </c>
+      <c r="H5" s="72"/>
+      <c r="I5" s="72"/>
+      <c r="J5" s="73"/>
+      <c r="K5" s="71" t="s">
+        <v>122</v>
+      </c>
+      <c r="L5" s="72"/>
+      <c r="M5" s="72"/>
+      <c r="N5" s="73"/>
+      <c r="O5" s="74" t="s">
+        <v>123</v>
+      </c>
+      <c r="P5" s="68"/>
+      <c r="Q5" s="68"/>
+      <c r="R5" s="69"/>
+      <c r="S5" s="75" t="s">
+        <v>124</v>
+      </c>
+      <c r="T5" s="43" t="s">
+        <v>79</v>
+      </c>
+      <c r="U5" s="48" t="s">
+        <v>125</v>
+      </c>
+      <c r="V5" s="51" t="s">
+        <v>126</v>
+      </c>
+      <c r="W5" s="68"/>
+      <c r="X5" s="69"/>
+      <c r="Y5" s="76" t="s">
+        <v>127</v>
+      </c>
+      <c r="Z5" s="76" t="s">
+        <v>128</v>
+      </c>
+      <c r="AA5" s="76" t="s">
+        <v>129</v>
+      </c>
+      <c r="AB5" s="76" t="s">
+        <v>130</v>
+      </c>
+      <c r="AC5" s="76" t="s">
+        <v>131</v>
+      </c>
+      <c r="AD5" s="76" t="s">
+        <v>132</v>
+      </c>
+      <c r="AE5" s="77" t="s">
+        <v>133</v>
+      </c>
+      <c r="AF5" s="43" t="s">
+        <v>134</v>
+      </c>
+      <c r="AG5" s="78" t="s">
+        <v>135</v>
+      </c>
+      <c r="AH5" s="69"/>
+      <c r="AI5" s="51" t="s">
+        <v>136</v>
+      </c>
+      <c r="AJ5" s="69"/>
+      <c r="AK5" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="AL5" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="AM5" s="43" t="s">
+        <v>138</v>
+      </c>
+      <c r="AN5" s="79" t="s">
+        <v>106</v>
+      </c>
+      <c r="AO5" s="79" t="s">
+        <v>107</v>
+      </c>
+      <c r="AP5" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="AQ5" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="AR5" s="79" t="s">
+        <v>106</v>
+      </c>
+      <c r="AS5" s="79" t="s">
+        <v>107</v>
+      </c>
+      <c r="AT5" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="AU5" s="77"/>
+      <c r="AV5" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="AW5" s="79" t="s">
+        <v>106</v>
+      </c>
+      <c r="AX5" s="79" t="s">
+        <v>107</v>
+      </c>
+      <c r="AY5" s="80" t="s">
+        <v>139</v>
+      </c>
+      <c r="AZ5" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="BA5" s="77"/>
+    </row>
+    <row r="6" spans="1:53" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="48"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="81" t="s">
+        <v>140</v>
+      </c>
+      <c r="H6" s="48" t="s">
+        <v>141</v>
+      </c>
+      <c r="I6" s="48" t="s">
+        <v>142</v>
+      </c>
+      <c r="J6" s="82" t="s">
+        <v>143</v>
+      </c>
+      <c r="K6" s="81" t="s">
+        <v>140</v>
+      </c>
+      <c r="L6" s="46" t="s">
+        <v>141</v>
+      </c>
+      <c r="M6" s="48" t="s">
+        <v>142</v>
+      </c>
+      <c r="N6" s="82" t="s">
+        <v>143</v>
+      </c>
+      <c r="O6" s="79" t="s">
+        <v>144</v>
+      </c>
+      <c r="P6" s="79" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q6" s="79" t="s">
+        <v>146</v>
+      </c>
+      <c r="R6" s="79" t="s">
+        <v>147</v>
+      </c>
+      <c r="S6" s="83" t="s">
+        <v>148</v>
+      </c>
+      <c r="T6" s="54"/>
+      <c r="U6" s="43"/>
+      <c r="V6" s="43" t="s">
+        <v>149</v>
+      </c>
+      <c r="W6" s="43" t="s">
+        <v>150</v>
+      </c>
+      <c r="X6" s="43" t="s">
+        <v>143</v>
+      </c>
+      <c r="Y6" s="77"/>
+      <c r="Z6" s="77"/>
+      <c r="AA6" s="77"/>
+      <c r="AB6" s="77"/>
+      <c r="AC6" s="77"/>
+      <c r="AD6" s="77"/>
+      <c r="AE6" s="54"/>
+      <c r="AF6" s="54"/>
+      <c r="AG6" s="79" t="s">
+        <v>106</v>
+      </c>
+      <c r="AH6" s="79" t="s">
+        <v>107</v>
+      </c>
+      <c r="AI6" s="79" t="s">
+        <v>106</v>
+      </c>
+      <c r="AJ6" s="79" t="s">
+        <v>107</v>
+      </c>
+      <c r="AK6" s="54"/>
+      <c r="AL6" s="54"/>
+      <c r="AM6" s="54"/>
+      <c r="AN6" s="79"/>
+      <c r="AO6" s="79"/>
+      <c r="AP6" s="54"/>
+      <c r="AQ6" s="54"/>
+      <c r="AR6" s="79"/>
+      <c r="AS6" s="79"/>
+      <c r="AT6" s="54"/>
+      <c r="AU6" s="54"/>
+      <c r="AV6" s="54"/>
+      <c r="AW6" s="79"/>
+      <c r="AX6" s="79"/>
+      <c r="AY6" s="84"/>
+      <c r="AZ6" s="54"/>
+      <c r="BA6" s="54"/>
+    </row>
+    <row r="9" spans="1:53" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:53" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="6"/>
+      <c r="H10" s="86"/>
+      <c r="I10" s="86"/>
+      <c r="J10" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="M10" s="6"/>
+      <c r="N10" s="17"/>
+      <c r="O10" s="85"/>
+      <c r="P10" s="86"/>
+      <c r="Q10" s="87"/>
+      <c r="AQ10" s="85" t="s">
+        <v>55</v>
+      </c>
+      <c r="AR10" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="AS10" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="AT10" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="O5:R5"/>
+    <mergeCell ref="V5:X5"/>
+    <mergeCell ref="AG5:AH5"/>
+    <mergeCell ref="AI5:AJ5"/>
+    <mergeCell ref="A1:BA1"/>
+    <mergeCell ref="A3:BA3"/>
+    <mergeCell ref="A4:S4"/>
+    <mergeCell ref="T4:AK4"/>
+    <mergeCell ref="AL4:AP4"/>
+    <mergeCell ref="AQ4:AT4"/>
+    <mergeCell ref="AV4:AZ4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECB08AFA-BF49-47F5-B095-34C6A355FE30}">
+  <dimension ref="A2:BA10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="2" spans="1:53" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:53" x14ac:dyDescent="0.35">
+      <c r="A3" s="51" t="str">
+        <f>+[1]Summary!A5</f>
+        <v>Progress of 220kV Line</v>
+      </c>
+      <c r="B3" s="68"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
+      <c r="I3" s="68"/>
+      <c r="J3" s="68"/>
+      <c r="K3" s="68"/>
+      <c r="L3" s="68"/>
+      <c r="M3" s="68"/>
+      <c r="N3" s="68"/>
+      <c r="O3" s="68"/>
+      <c r="P3" s="68"/>
+      <c r="Q3" s="68"/>
+      <c r="R3" s="68"/>
+      <c r="S3" s="68"/>
+      <c r="T3" s="68"/>
+      <c r="U3" s="68"/>
+      <c r="V3" s="68"/>
+      <c r="W3" s="68"/>
+      <c r="X3" s="68"/>
+      <c r="Y3" s="68"/>
+      <c r="Z3" s="68"/>
+      <c r="AA3" s="68"/>
+      <c r="AB3" s="68"/>
+      <c r="AC3" s="68"/>
+      <c r="AD3" s="68"/>
+      <c r="AE3" s="68"/>
+      <c r="AF3" s="68"/>
+      <c r="AG3" s="68"/>
+      <c r="AH3" s="68"/>
+      <c r="AI3" s="68"/>
+      <c r="AJ3" s="68"/>
+      <c r="AK3" s="68"/>
+      <c r="AL3" s="22"/>
+      <c r="AM3" s="22"/>
+      <c r="AN3" s="22"/>
+      <c r="AO3" s="22"/>
+      <c r="AP3" s="22"/>
+      <c r="AQ3" s="68"/>
+      <c r="AR3" s="68"/>
+      <c r="AS3" s="68"/>
+      <c r="AT3" s="68"/>
+      <c r="AU3" s="68"/>
+      <c r="AV3" s="68"/>
+      <c r="AW3" s="68"/>
+      <c r="AX3" s="68"/>
+      <c r="AY3" s="68"/>
+      <c r="AZ3" s="68"/>
+      <c r="BA3" s="69"/>
+    </row>
+    <row r="4" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="51" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" s="68"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="68"/>
+      <c r="E4" s="68"/>
+      <c r="F4" s="68"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="68"/>
+      <c r="I4" s="68"/>
+      <c r="J4" s="68"/>
+      <c r="K4" s="68"/>
+      <c r="L4" s="68"/>
+      <c r="M4" s="68"/>
+      <c r="N4" s="68"/>
+      <c r="O4" s="68"/>
+      <c r="P4" s="68"/>
+      <c r="Q4" s="68"/>
+      <c r="R4" s="68"/>
+      <c r="S4" s="69"/>
+      <c r="T4" s="51" t="s">
+        <v>116</v>
+      </c>
+      <c r="U4" s="68"/>
+      <c r="V4" s="68"/>
+      <c r="W4" s="68"/>
+      <c r="X4" s="68"/>
+      <c r="Y4" s="68"/>
+      <c r="Z4" s="68"/>
+      <c r="AA4" s="68"/>
+      <c r="AB4" s="68"/>
+      <c r="AC4" s="68"/>
+      <c r="AD4" s="68"/>
+      <c r="AE4" s="68"/>
+      <c r="AF4" s="68"/>
+      <c r="AG4" s="68"/>
+      <c r="AH4" s="68"/>
+      <c r="AI4" s="68"/>
+      <c r="AJ4" s="68"/>
+      <c r="AK4" s="69"/>
+      <c r="AL4" s="51" t="s">
+        <v>117</v>
+      </c>
+      <c r="AM4" s="22"/>
+      <c r="AN4" s="22"/>
+      <c r="AO4" s="22"/>
+      <c r="AP4" s="23"/>
+      <c r="AQ4" s="51" t="s">
+        <v>2</v>
+      </c>
+      <c r="AR4" s="68"/>
+      <c r="AS4" s="68"/>
+      <c r="AT4" s="69"/>
+      <c r="AU4" s="43" t="s">
+        <v>118</v>
+      </c>
+      <c r="AV4" s="51" t="s">
+        <v>119</v>
+      </c>
+      <c r="AW4" s="68"/>
+      <c r="AX4" s="68"/>
+      <c r="AY4" s="68"/>
+      <c r="AZ4" s="69"/>
+      <c r="BA4" s="43" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:53" ht="58.5" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="48" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" s="48" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5" s="48" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="70"/>
+      <c r="E5" s="70"/>
+      <c r="F5" s="70"/>
+      <c r="G5" s="71" t="s">
+        <v>82</v>
+      </c>
+      <c r="H5" s="72"/>
+      <c r="I5" s="72"/>
+      <c r="J5" s="73"/>
+      <c r="K5" s="71" t="s">
+        <v>122</v>
+      </c>
+      <c r="L5" s="72"/>
+      <c r="M5" s="72"/>
+      <c r="N5" s="73"/>
+      <c r="O5" s="74" t="s">
+        <v>123</v>
+      </c>
+      <c r="P5" s="68"/>
+      <c r="Q5" s="68"/>
+      <c r="R5" s="69"/>
+      <c r="S5" s="75" t="s">
+        <v>124</v>
+      </c>
+      <c r="T5" s="43" t="s">
+        <v>79</v>
+      </c>
+      <c r="U5" s="48" t="s">
+        <v>125</v>
+      </c>
+      <c r="V5" s="51" t="s">
+        <v>126</v>
+      </c>
+      <c r="W5" s="68"/>
+      <c r="X5" s="69"/>
+      <c r="Y5" s="76" t="s">
+        <v>127</v>
+      </c>
+      <c r="Z5" s="76" t="s">
+        <v>128</v>
+      </c>
+      <c r="AA5" s="76" t="s">
+        <v>129</v>
+      </c>
+      <c r="AB5" s="76" t="s">
+        <v>130</v>
+      </c>
+      <c r="AC5" s="76" t="s">
+        <v>131</v>
+      </c>
+      <c r="AD5" s="76" t="s">
+        <v>132</v>
+      </c>
+      <c r="AE5" s="77" t="s">
+        <v>133</v>
+      </c>
+      <c r="AF5" s="43" t="s">
+        <v>134</v>
+      </c>
+      <c r="AG5" s="78" t="s">
+        <v>135</v>
+      </c>
+      <c r="AH5" s="69"/>
+      <c r="AI5" s="51" t="s">
+        <v>136</v>
+      </c>
+      <c r="AJ5" s="69"/>
+      <c r="AK5" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="AL5" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="AM5" s="43" t="s">
+        <v>138</v>
+      </c>
+      <c r="AN5" s="79" t="s">
+        <v>106</v>
+      </c>
+      <c r="AO5" s="79" t="s">
+        <v>107</v>
+      </c>
+      <c r="AP5" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="AQ5" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="AR5" s="79" t="s">
+        <v>106</v>
+      </c>
+      <c r="AS5" s="79" t="s">
+        <v>107</v>
+      </c>
+      <c r="AT5" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="AU5" s="77"/>
+      <c r="AV5" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="AW5" s="79" t="s">
+        <v>106</v>
+      </c>
+      <c r="AX5" s="79" t="s">
+        <v>107</v>
+      </c>
+      <c r="AY5" s="80" t="s">
+        <v>139</v>
+      </c>
+      <c r="AZ5" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="BA5" s="77"/>
+    </row>
+    <row r="6" spans="1:53" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="48"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="81" t="s">
+        <v>140</v>
+      </c>
+      <c r="H6" s="48" t="s">
+        <v>141</v>
+      </c>
+      <c r="I6" s="48" t="s">
+        <v>142</v>
+      </c>
+      <c r="J6" s="82" t="s">
+        <v>143</v>
+      </c>
+      <c r="K6" s="81" t="s">
+        <v>140</v>
+      </c>
+      <c r="L6" s="46" t="s">
+        <v>141</v>
+      </c>
+      <c r="M6" s="48" t="s">
+        <v>142</v>
+      </c>
+      <c r="N6" s="82" t="s">
+        <v>143</v>
+      </c>
+      <c r="O6" s="79" t="s">
+        <v>144</v>
+      </c>
+      <c r="P6" s="79" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q6" s="79" t="s">
+        <v>146</v>
+      </c>
+      <c r="R6" s="79" t="s">
+        <v>147</v>
+      </c>
+      <c r="S6" s="83" t="s">
+        <v>148</v>
+      </c>
+      <c r="T6" s="54"/>
+      <c r="U6" s="43"/>
+      <c r="V6" s="43" t="s">
+        <v>149</v>
+      </c>
+      <c r="W6" s="43" t="s">
+        <v>150</v>
+      </c>
+      <c r="X6" s="43" t="s">
+        <v>143</v>
+      </c>
+      <c r="Y6" s="77"/>
+      <c r="Z6" s="77"/>
+      <c r="AA6" s="77"/>
+      <c r="AB6" s="77"/>
+      <c r="AC6" s="77"/>
+      <c r="AD6" s="77"/>
+      <c r="AE6" s="54"/>
+      <c r="AF6" s="54"/>
+      <c r="AG6" s="79" t="s">
+        <v>106</v>
+      </c>
+      <c r="AH6" s="79" t="s">
+        <v>107</v>
+      </c>
+      <c r="AI6" s="79" t="s">
+        <v>106</v>
+      </c>
+      <c r="AJ6" s="79" t="s">
+        <v>107</v>
+      </c>
+      <c r="AK6" s="54"/>
+      <c r="AL6" s="54"/>
+      <c r="AM6" s="54"/>
+      <c r="AN6" s="79"/>
+      <c r="AO6" s="79"/>
+      <c r="AP6" s="54"/>
+      <c r="AQ6" s="54"/>
+      <c r="AR6" s="79"/>
+      <c r="AS6" s="79"/>
+      <c r="AT6" s="54"/>
+      <c r="AU6" s="54"/>
+      <c r="AV6" s="54"/>
+      <c r="AW6" s="79"/>
+      <c r="AX6" s="79"/>
+      <c r="AY6" s="84"/>
+      <c r="AZ6" s="54"/>
+      <c r="BA6" s="54"/>
+    </row>
+    <row r="9" spans="1:53" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:53" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="6"/>
+      <c r="H10" s="86"/>
+      <c r="I10" s="86"/>
+      <c r="J10" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="M10" s="6"/>
+      <c r="N10" s="17"/>
+      <c r="O10" s="85"/>
+      <c r="P10" s="86"/>
+      <c r="Q10" s="87"/>
+      <c r="AQ10" s="85" t="s">
+        <v>55</v>
+      </c>
+      <c r="AR10" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="AS10" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="AT10" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="O5:R5"/>
+    <mergeCell ref="V5:X5"/>
+    <mergeCell ref="AG5:AH5"/>
+    <mergeCell ref="AI5:AJ5"/>
+    <mergeCell ref="A3:BA3"/>
+    <mergeCell ref="A4:S4"/>
+    <mergeCell ref="T4:AK4"/>
+    <mergeCell ref="AL4:AP4"/>
+    <mergeCell ref="AQ4:AT4"/>
+    <mergeCell ref="AV4:AZ4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0CAA689-52FE-4282-BFA7-7FA3F37BB8D4}">
   <dimension ref="A2:W7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1411,35 +3730,35 @@
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="19" t="s">
+      <c r="C3" s="22"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="20"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="19" t="s">
+      <c r="F3" s="22"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="I3" s="20"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="17" t="s">
+      <c r="I3" s="22"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="L3" s="22" t="s">
+      <c r="L3" s="18" t="s">
         <v>43</v>
       </c>
       <c r="M3" s="8"/>
       <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="31" x14ac:dyDescent="0.35">
-      <c r="A4" s="18"/>
+      <c r="A4" s="19"/>
       <c r="B4" s="12" t="s">
         <v>39</v>
       </c>
@@ -1467,8 +3786,8 @@
       <c r="J4" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
       <c r="M4" s="10"/>
       <c r="N4" s="11"/>
     </row>
@@ -1536,7 +3855,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B225AA6-68BC-47EB-9948-84B6B216E727}">
   <dimension ref="A2:W7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1547,46 +3866,46 @@
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26" t="s">
+      <c r="C3" s="27"/>
+      <c r="D3" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="26" t="s">
+      <c r="E3" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="27" t="s">
+      <c r="G3" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
-      <c r="J3" s="23" t="s">
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
-      <c r="N3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="25"/>
+      <c r="N3" s="26"/>
     </row>
     <row r="4" spans="1:23" ht="26" x14ac:dyDescent="0.35">
-      <c r="A4" s="26"/>
+      <c r="A4" s="27"/>
       <c r="B4" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
       <c r="G4" s="1" t="s">
         <v>36</v>
       </c>
@@ -1680,7 +3999,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBFB976A-1B92-4632-9799-0237B459A61D}">
   <dimension ref="A1:P5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1717,14 +4036,14 @@
       <c r="C3" s="7"/>
       <c r="D3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="30"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="31"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="28"/>
-      <c r="O3" s="29"/>
-      <c r="P3" s="30"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="30"/>
+      <c r="P3" s="31"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -1760,7 +4079,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46CC22E7-0431-4564-825A-DCAC81041178}">
   <dimension ref="A1:P5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1806,14 +4125,14 @@
       <c r="C3" s="7"/>
       <c r="D3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="30"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="31"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="28"/>
-      <c r="O3" s="29"/>
-      <c r="P3" s="30"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="30"/>
+      <c r="P3" s="31"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">

</xml_diff>

<commit_message>
Auto pipeline update 2026-03-10 16:07:50
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B076A407-5D36-4761-9F9E-6F389CDF3CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE42CA59-227D-4A30-BF0E-6B703D25797D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" activeTab="4" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet Names Check" sheetId="1" r:id="rId1"/>
-    <sheet name="Test 000 Stringing 132kV" sheetId="11" r:id="rId2"/>
-    <sheet name="Test 000 Stringing 220kV" sheetId="10" r:id="rId3"/>
-    <sheet name="Test 000 Erection 220kV" sheetId="9" r:id="rId4"/>
-    <sheet name="Test 000 Erection 132kV" sheetId="8" r:id="rId5"/>
+    <sheet name="Test 000 132kV Stringing" sheetId="11" r:id="rId2"/>
+    <sheet name="Test 000 220kV Stringing" sheetId="10" r:id="rId3"/>
+    <sheet name="Test 000 220kV Erection" sheetId="9" r:id="rId4"/>
+    <sheet name="Test 000 132kV Erection" sheetId="8" r:id="rId5"/>
     <sheet name="TB 401 Stringing" sheetId="6" r:id="rId6"/>
     <sheet name="TB 408 Stringing" sheetId="2" r:id="rId7"/>
     <sheet name="TA 509 Erection" sheetId="3" r:id="rId8"/>
@@ -1165,45 +1165,6 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1222,86 +1183,142 @@
     <xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1309,59 +1326,42 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -1491,10 +1491,10 @@
       <sheetName val="Mail Body"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
       <sheetData sheetId="4">
         <row r="2">
           <cell r="A2" t="str">
@@ -1512,15 +1512,15 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2148,252 +2148,252 @@
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="32" t="str">
+      <c r="A3" s="63" t="str">
         <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
-      <c r="Y3" s="22"/>
-      <c r="Z3" s="23"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
+      <c r="L3" s="64"/>
+      <c r="M3" s="64"/>
+      <c r="N3" s="64"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="64"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="64"/>
+      <c r="V3" s="64"/>
+      <c r="W3" s="64"/>
+      <c r="X3" s="64"/>
+      <c r="Y3" s="64"/>
+      <c r="Z3" s="65"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="32">
+      <c r="A4" s="63">
         <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="32" t="s">
+      <c r="B4" s="64"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="63" t="s">
         <v>91</v>
       </c>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="22"/>
-      <c r="O4" s="22"/>
-      <c r="P4" s="22"/>
-      <c r="Q4" s="22"/>
-      <c r="R4" s="23"/>
-      <c r="S4" s="34"/>
-      <c r="T4" s="32" t="s">
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
+      <c r="I4" s="64"/>
+      <c r="J4" s="64"/>
+      <c r="K4" s="64"/>
+      <c r="L4" s="64"/>
+      <c r="M4" s="64"/>
+      <c r="N4" s="64"/>
+      <c r="O4" s="64"/>
+      <c r="P4" s="64"/>
+      <c r="Q4" s="64"/>
+      <c r="R4" s="65"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="63" t="s">
         <v>92</v>
       </c>
-      <c r="U4" s="22"/>
-      <c r="V4" s="22"/>
-      <c r="W4" s="22"/>
-      <c r="X4" s="22"/>
-      <c r="Y4" s="22"/>
-      <c r="Z4" s="23"/>
+      <c r="U4" s="64"/>
+      <c r="V4" s="64"/>
+      <c r="W4" s="64"/>
+      <c r="X4" s="64"/>
+      <c r="Y4" s="64"/>
+      <c r="Z4" s="65"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="63" t="s">
         <v>93</v>
       </c>
-      <c r="B5" s="22"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="35">
+      <c r="B5" s="64"/>
+      <c r="C5" s="65"/>
+      <c r="D5" s="20">
         <f>[1]Summary!R7</f>
         <v>0</v>
       </c>
-      <c r="E5" s="36">
+      <c r="E5" s="21">
         <f>SUMIF(E8:E215,"C",$D$6:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="38">
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="23">
         <f>SUMIF(G9:G215,"WIP",$D$7:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="I5" s="36">
+      <c r="I5" s="21">
         <f>SUMIF(G8:G215,"C",$D$6:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="J5" s="37"/>
-      <c r="K5" s="38">
+      <c r="J5" s="22"/>
+      <c r="K5" s="23">
         <f>SUMIF(J9:J215,"WIP",$D$7:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="L5" s="36">
+      <c r="L5" s="21">
         <f>SUMIF(J8:J215,"C",$D$6:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="M5" s="37"/>
-      <c r="N5" s="37"/>
-      <c r="O5" s="37"/>
-      <c r="P5" s="37"/>
-      <c r="Q5" s="37"/>
-      <c r="R5" s="37"/>
-      <c r="S5" s="39"/>
-      <c r="T5" s="37"/>
-      <c r="U5" s="38">
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="22"/>
+      <c r="R5" s="22"/>
+      <c r="S5" s="24"/>
+      <c r="T5" s="22"/>
+      <c r="U5" s="23">
         <f>SUMIF(T9:T215,"WIP",$D$7:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="V5" s="38">
+      <c r="V5" s="23">
         <f>SUMIF(T9:T215,"C",$D$7:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="W5" s="38"/>
-      <c r="X5" s="38">
+      <c r="W5" s="23"/>
+      <c r="X5" s="23">
         <f>SUMIF(W9:W215,"WIP",$D$7:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="Y5" s="38">
+      <c r="Y5" s="23">
         <f>SUMIF(W9:W215,"C",$D$7:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="Z5" s="37"/>
+      <c r="Z5" s="22"/>
     </row>
     <row r="6" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="23"/>
-      <c r="D6" s="40" t="s">
+      <c r="C6" s="65"/>
+      <c r="D6" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="F6" s="43" t="s">
+      <c r="F6" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G6" s="44" t="s">
+      <c r="G6" s="67" t="s">
         <v>98</v>
       </c>
-      <c r="H6" s="22"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="44" t="s">
+      <c r="H6" s="64"/>
+      <c r="I6" s="65"/>
+      <c r="J6" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="K6" s="22"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="45" t="s">
+      <c r="K6" s="64"/>
+      <c r="L6" s="65"/>
+      <c r="M6" s="28" t="s">
         <v>99</v>
       </c>
-      <c r="N6" s="46" t="s">
+      <c r="N6" s="29" t="s">
         <v>100</v>
       </c>
-      <c r="O6" s="47" t="s">
+      <c r="O6" s="30" t="s">
         <v>101</v>
       </c>
-      <c r="P6" s="48" t="s">
+      <c r="P6" s="31" t="s">
         <v>102</v>
       </c>
-      <c r="Q6" s="49" t="s">
+      <c r="Q6" s="32" t="s">
         <v>103</v>
       </c>
-      <c r="R6" s="43" t="s">
+      <c r="R6" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="S6" s="50"/>
-      <c r="T6" s="51" t="s">
+      <c r="S6" s="33"/>
+      <c r="T6" s="68" t="s">
         <v>104</v>
       </c>
-      <c r="U6" s="22"/>
-      <c r="V6" s="23"/>
-      <c r="W6" s="51" t="s">
+      <c r="U6" s="64"/>
+      <c r="V6" s="65"/>
+      <c r="W6" s="68" t="s">
         <v>105</v>
       </c>
-      <c r="X6" s="22"/>
-      <c r="Y6" s="23"/>
-      <c r="Z6" s="48" t="s">
+      <c r="X6" s="64"/>
+      <c r="Y6" s="65"/>
+      <c r="Z6" s="31" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A7" s="40"/>
-      <c r="B7" s="52" t="s">
+      <c r="A7" s="25"/>
+      <c r="B7" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="52" t="s">
+      <c r="C7" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="40"/>
-      <c r="E7" s="53"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="47" t="s">
+      <c r="D7" s="25"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="H7" s="55" t="s">
+      <c r="H7" s="37" t="s">
         <v>106</v>
       </c>
-      <c r="I7" s="47" t="s">
+      <c r="I7" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="J7" s="47" t="s">
+      <c r="J7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="K7" s="47" t="s">
+      <c r="K7" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="L7" s="47" t="s">
+      <c r="L7" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="M7" s="47" t="s">
+      <c r="M7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="N7" s="47" t="s">
+      <c r="N7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="O7" s="47" t="s">
+      <c r="O7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="P7" s="48"/>
-      <c r="Q7" s="56"/>
-      <c r="R7" s="54"/>
-      <c r="S7" s="57"/>
-      <c r="T7" s="47" t="s">
+      <c r="P7" s="31"/>
+      <c r="Q7" s="38"/>
+      <c r="R7" s="36"/>
+      <c r="S7" s="39"/>
+      <c r="T7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="U7" s="47" t="s">
+      <c r="U7" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="V7" s="47" t="s">
+      <c r="V7" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="W7" s="47" t="s">
+      <c r="W7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="X7" s="47" t="s">
+      <c r="X7" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="Y7" s="47" t="s">
+      <c r="Y7" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="Z7" s="48"/>
+      <c r="Z7" s="31"/>
     </row>
     <row r="10" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
@@ -2401,91 +2401,91 @@
       </c>
     </row>
     <row r="11" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="58" t="s">
+      <c r="A11" s="40" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="59" t="s">
+      <c r="B11" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="59" t="s">
+      <c r="C11" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="59" t="s">
+      <c r="D11" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="61" t="s">
+      <c r="E11" s="43" t="s">
         <v>110</v>
       </c>
-      <c r="F11" s="62" t="s">
+      <c r="F11" s="44" t="s">
         <v>97</v>
       </c>
-      <c r="H11" s="63" t="s">
+      <c r="H11" s="45" t="s">
         <v>49</v>
       </c>
-      <c r="I11" s="60" t="s">
+      <c r="I11" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="K11" s="60" t="s">
+      <c r="K11" s="42" t="s">
         <v>52</v>
       </c>
-      <c r="L11" s="64" t="s">
+      <c r="L11" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="M11" s="66" t="s">
+      <c r="M11" s="48" t="s">
         <v>99</v>
       </c>
-      <c r="N11" s="65" t="s">
+      <c r="N11" s="47" t="s">
         <v>112</v>
       </c>
-      <c r="O11" s="58" t="s">
+      <c r="O11" s="40" t="s">
         <v>111</v>
       </c>
-      <c r="P11" s="59" t="s">
+      <c r="P11" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="R11" s="66" t="s">
+      <c r="R11" s="48" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="16" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="59" t="s">
+      <c r="B16" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="F16" s="60" t="s">
+      <c r="F16" s="42" t="s">
         <v>109</v>
       </c>
-      <c r="K16" s="59" t="s">
+      <c r="K16" s="41" t="s">
         <v>51</v>
       </c>
-      <c r="Q16" s="67" t="s">
+      <c r="Q16" s="49" t="s">
         <v>54</v>
       </c>
-      <c r="R16" s="59" t="s">
+      <c r="R16" s="41" t="s">
         <v>55</v>
       </c>
-      <c r="T16" s="59" t="s">
+      <c r="T16" s="41" t="s">
         <v>81</v>
       </c>
-      <c r="U16" s="59" t="s">
+      <c r="U16" s="41" t="s">
         <v>113</v>
       </c>
-      <c r="V16" s="59" t="s">
+      <c r="V16" s="41" t="s">
         <v>114</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="W6:Y6"/>
     <mergeCell ref="A3:Z3"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:R4"/>
     <mergeCell ref="T4:Z4"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="W6:Y6"/>
   </mergeCells>
   <conditionalFormatting sqref="B11">
     <cfRule type="duplicateValues" dxfId="7" priority="2"/>
@@ -2508,252 +2508,252 @@
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="32" t="str">
+      <c r="A3" s="63" t="str">
         <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
-      <c r="Y3" s="22"/>
-      <c r="Z3" s="23"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
+      <c r="L3" s="64"/>
+      <c r="M3" s="64"/>
+      <c r="N3" s="64"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="64"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="64"/>
+      <c r="V3" s="64"/>
+      <c r="W3" s="64"/>
+      <c r="X3" s="64"/>
+      <c r="Y3" s="64"/>
+      <c r="Z3" s="65"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="32">
+      <c r="A4" s="63">
         <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="32" t="s">
+      <c r="B4" s="64"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="63" t="s">
         <v>91</v>
       </c>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="22"/>
-      <c r="O4" s="22"/>
-      <c r="P4" s="22"/>
-      <c r="Q4" s="22"/>
-      <c r="R4" s="23"/>
-      <c r="S4" s="34"/>
-      <c r="T4" s="32" t="s">
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
+      <c r="I4" s="64"/>
+      <c r="J4" s="64"/>
+      <c r="K4" s="64"/>
+      <c r="L4" s="64"/>
+      <c r="M4" s="64"/>
+      <c r="N4" s="64"/>
+      <c r="O4" s="64"/>
+      <c r="P4" s="64"/>
+      <c r="Q4" s="64"/>
+      <c r="R4" s="65"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="63" t="s">
         <v>92</v>
       </c>
-      <c r="U4" s="22"/>
-      <c r="V4" s="22"/>
-      <c r="W4" s="22"/>
-      <c r="X4" s="22"/>
-      <c r="Y4" s="22"/>
-      <c r="Z4" s="23"/>
+      <c r="U4" s="64"/>
+      <c r="V4" s="64"/>
+      <c r="W4" s="64"/>
+      <c r="X4" s="64"/>
+      <c r="Y4" s="64"/>
+      <c r="Z4" s="65"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="63" t="s">
         <v>93</v>
       </c>
-      <c r="B5" s="22"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="35">
+      <c r="B5" s="64"/>
+      <c r="C5" s="65"/>
+      <c r="D5" s="20">
         <f>[1]Summary!R7</f>
         <v>0</v>
       </c>
-      <c r="E5" s="36">
+      <c r="E5" s="21">
         <f>SUMIF(E8:E215,"C",$D$6:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="38">
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="23">
         <f>SUMIF(G9:G215,"WIP",$D$7:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="I5" s="36">
+      <c r="I5" s="21">
         <f>SUMIF(G8:G215,"C",$D$6:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="J5" s="37"/>
-      <c r="K5" s="38">
+      <c r="J5" s="22"/>
+      <c r="K5" s="23">
         <f>SUMIF(J9:J215,"WIP",$D$7:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="L5" s="36">
+      <c r="L5" s="21">
         <f>SUMIF(J8:J215,"C",$D$6:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="M5" s="37"/>
-      <c r="N5" s="37"/>
-      <c r="O5" s="37"/>
-      <c r="P5" s="37"/>
-      <c r="Q5" s="37"/>
-      <c r="R5" s="37"/>
-      <c r="S5" s="39"/>
-      <c r="T5" s="37"/>
-      <c r="U5" s="38">
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="22"/>
+      <c r="R5" s="22"/>
+      <c r="S5" s="24"/>
+      <c r="T5" s="22"/>
+      <c r="U5" s="23">
         <f>SUMIF(T9:T215,"WIP",$D$7:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="V5" s="38">
+      <c r="V5" s="23">
         <f>SUMIF(T9:T215,"C",$D$7:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="W5" s="38"/>
-      <c r="X5" s="38">
+      <c r="W5" s="23"/>
+      <c r="X5" s="23">
         <f>SUMIF(W9:W215,"WIP",$D$7:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="Y5" s="38">
+      <c r="Y5" s="23">
         <f>SUMIF(W9:W215,"C",$D$7:$D$213)/1000</f>
         <v>0</v>
       </c>
-      <c r="Z5" s="37"/>
+      <c r="Z5" s="22"/>
     </row>
     <row r="6" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="23"/>
-      <c r="D6" s="40" t="s">
+      <c r="C6" s="65"/>
+      <c r="D6" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="F6" s="43" t="s">
+      <c r="F6" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="G6" s="44" t="s">
+      <c r="G6" s="67" t="s">
         <v>98</v>
       </c>
-      <c r="H6" s="22"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="44" t="s">
+      <c r="H6" s="64"/>
+      <c r="I6" s="65"/>
+      <c r="J6" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="K6" s="22"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="45" t="s">
+      <c r="K6" s="64"/>
+      <c r="L6" s="65"/>
+      <c r="M6" s="28" t="s">
         <v>99</v>
       </c>
-      <c r="N6" s="46" t="s">
+      <c r="N6" s="29" t="s">
         <v>100</v>
       </c>
-      <c r="O6" s="47" t="s">
+      <c r="O6" s="30" t="s">
         <v>101</v>
       </c>
-      <c r="P6" s="48" t="s">
+      <c r="P6" s="31" t="s">
         <v>102</v>
       </c>
-      <c r="Q6" s="49" t="s">
+      <c r="Q6" s="32" t="s">
         <v>103</v>
       </c>
-      <c r="R6" s="43" t="s">
+      <c r="R6" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="S6" s="50"/>
-      <c r="T6" s="51" t="s">
+      <c r="S6" s="33"/>
+      <c r="T6" s="68" t="s">
         <v>104</v>
       </c>
-      <c r="U6" s="22"/>
-      <c r="V6" s="23"/>
-      <c r="W6" s="51" t="s">
+      <c r="U6" s="64"/>
+      <c r="V6" s="65"/>
+      <c r="W6" s="68" t="s">
         <v>105</v>
       </c>
-      <c r="X6" s="22"/>
-      <c r="Y6" s="23"/>
-      <c r="Z6" s="48" t="s">
+      <c r="X6" s="64"/>
+      <c r="Y6" s="65"/>
+      <c r="Z6" s="31" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A7" s="40"/>
-      <c r="B7" s="52" t="s">
+      <c r="A7" s="25"/>
+      <c r="B7" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="52" t="s">
+      <c r="C7" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="40"/>
-      <c r="E7" s="53"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="47" t="s">
+      <c r="D7" s="25"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="H7" s="55" t="s">
+      <c r="H7" s="37" t="s">
         <v>106</v>
       </c>
-      <c r="I7" s="47" t="s">
+      <c r="I7" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="J7" s="47" t="s">
+      <c r="J7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="K7" s="47" t="s">
+      <c r="K7" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="L7" s="47" t="s">
+      <c r="L7" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="M7" s="47" t="s">
+      <c r="M7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="N7" s="47" t="s">
+      <c r="N7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="O7" s="47" t="s">
+      <c r="O7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="P7" s="48"/>
-      <c r="Q7" s="56"/>
-      <c r="R7" s="54"/>
-      <c r="S7" s="57"/>
-      <c r="T7" s="47" t="s">
+      <c r="P7" s="31"/>
+      <c r="Q7" s="38"/>
+      <c r="R7" s="36"/>
+      <c r="S7" s="39"/>
+      <c r="T7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="U7" s="47" t="s">
+      <c r="U7" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="V7" s="47" t="s">
+      <c r="V7" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="W7" s="47" t="s">
+      <c r="W7" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="X7" s="47" t="s">
+      <c r="X7" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="Y7" s="47" t="s">
+      <c r="Y7" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="Z7" s="48"/>
+      <c r="Z7" s="31"/>
     </row>
     <row r="10" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
@@ -2761,64 +2761,64 @@
       </c>
     </row>
     <row r="11" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="58" t="s">
+      <c r="A11" s="40" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="59" t="s">
+      <c r="B11" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="59" t="s">
+      <c r="C11" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="59" t="s">
+      <c r="D11" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="61" t="s">
+      <c r="E11" s="43" t="s">
         <v>110</v>
       </c>
-      <c r="F11" s="62" t="s">
+      <c r="F11" s="44" t="s">
         <v>97</v>
       </c>
-      <c r="H11" s="63" t="s">
+      <c r="H11" s="45" t="s">
         <v>49</v>
       </c>
-      <c r="I11" s="60" t="s">
+      <c r="I11" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="K11" s="60" t="s">
+      <c r="K11" s="42" t="s">
         <v>52</v>
       </c>
-      <c r="L11" s="64" t="s">
+      <c r="L11" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="M11" s="66" t="s">
+      <c r="M11" s="48" t="s">
         <v>99</v>
       </c>
-      <c r="N11" s="65" t="s">
+      <c r="N11" s="47" t="s">
         <v>112</v>
       </c>
-      <c r="O11" s="58" t="s">
+      <c r="O11" s="40" t="s">
         <v>111</v>
       </c>
-      <c r="P11" s="59" t="s">
+      <c r="P11" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="R11" s="66" t="s">
+      <c r="R11" s="48" t="s">
         <v>43</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="W6:Y6"/>
     <mergeCell ref="A3:Z3"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:R4"/>
     <mergeCell ref="T4:Z4"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="W6:Y6"/>
   </mergeCells>
   <conditionalFormatting sqref="B11">
     <cfRule type="duplicateValues" dxfId="5" priority="2"/>
@@ -2836,62 +2836,62 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A1" s="51" t="str">
+      <c r="A1" s="68" t="str">
         <f>+[1]Summary!A2</f>
         <v>Name of the Line: 220KV DC AL59 line from Neemuch - Chanderiya + 132KV DC ACSS Line from Chanderiya to Hindustan Zinc</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-      <c r="O1" s="68"/>
-      <c r="P1" s="68"/>
-      <c r="Q1" s="68"/>
-      <c r="R1" s="68"/>
-      <c r="S1" s="68"/>
-      <c r="T1" s="68"/>
-      <c r="U1" s="68"/>
-      <c r="V1" s="68"/>
-      <c r="W1" s="68"/>
-      <c r="X1" s="68"/>
-      <c r="Y1" s="68"/>
-      <c r="Z1" s="68"/>
-      <c r="AA1" s="68"/>
-      <c r="AB1" s="68"/>
-      <c r="AC1" s="68"/>
-      <c r="AD1" s="68"/>
-      <c r="AE1" s="68"/>
-      <c r="AF1" s="68"/>
-      <c r="AG1" s="68"/>
-      <c r="AH1" s="68"/>
-      <c r="AI1" s="68"/>
-      <c r="AJ1" s="68"/>
-      <c r="AK1" s="68"/>
-      <c r="AL1" s="22"/>
-      <c r="AM1" s="22"/>
-      <c r="AN1" s="22"/>
-      <c r="AO1" s="22"/>
-      <c r="AP1" s="22"/>
-      <c r="AQ1" s="68"/>
-      <c r="AR1" s="68"/>
-      <c r="AS1" s="68"/>
-      <c r="AT1" s="68"/>
-      <c r="AU1" s="68"/>
-      <c r="AV1" s="68"/>
-      <c r="AW1" s="68"/>
-      <c r="AX1" s="68"/>
-      <c r="AY1" s="68"/>
-      <c r="AZ1" s="68"/>
-      <c r="BA1" s="69"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+      <c r="O1" s="73"/>
+      <c r="P1" s="73"/>
+      <c r="Q1" s="73"/>
+      <c r="R1" s="73"/>
+      <c r="S1" s="73"/>
+      <c r="T1" s="73"/>
+      <c r="U1" s="73"/>
+      <c r="V1" s="73"/>
+      <c r="W1" s="73"/>
+      <c r="X1" s="73"/>
+      <c r="Y1" s="73"/>
+      <c r="Z1" s="73"/>
+      <c r="AA1" s="73"/>
+      <c r="AB1" s="73"/>
+      <c r="AC1" s="73"/>
+      <c r="AD1" s="73"/>
+      <c r="AE1" s="73"/>
+      <c r="AF1" s="73"/>
+      <c r="AG1" s="73"/>
+      <c r="AH1" s="73"/>
+      <c r="AI1" s="73"/>
+      <c r="AJ1" s="73"/>
+      <c r="AK1" s="73"/>
+      <c r="AL1" s="64"/>
+      <c r="AM1" s="64"/>
+      <c r="AN1" s="64"/>
+      <c r="AO1" s="64"/>
+      <c r="AP1" s="64"/>
+      <c r="AQ1" s="73"/>
+      <c r="AR1" s="73"/>
+      <c r="AS1" s="73"/>
+      <c r="AT1" s="73"/>
+      <c r="AU1" s="73"/>
+      <c r="AV1" s="73"/>
+      <c r="AW1" s="73"/>
+      <c r="AX1" s="73"/>
+      <c r="AY1" s="73"/>
+      <c r="AZ1" s="73"/>
+      <c r="BA1" s="74"/>
     </row>
     <row r="2" spans="1:53" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -2899,351 +2899,351 @@
       </c>
     </row>
     <row r="3" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A3" s="51" t="str">
+      <c r="A3" s="68" t="str">
         <f>+[1]Summary!A5</f>
         <v>Progress of 220kV Line</v>
       </c>
-      <c r="B3" s="68"/>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="68"/>
-      <c r="K3" s="68"/>
-      <c r="L3" s="68"/>
-      <c r="M3" s="68"/>
-      <c r="N3" s="68"/>
-      <c r="O3" s="68"/>
-      <c r="P3" s="68"/>
-      <c r="Q3" s="68"/>
-      <c r="R3" s="68"/>
-      <c r="S3" s="68"/>
-      <c r="T3" s="68"/>
-      <c r="U3" s="68"/>
-      <c r="V3" s="68"/>
-      <c r="W3" s="68"/>
-      <c r="X3" s="68"/>
-      <c r="Y3" s="68"/>
-      <c r="Z3" s="68"/>
-      <c r="AA3" s="68"/>
-      <c r="AB3" s="68"/>
-      <c r="AC3" s="68"/>
-      <c r="AD3" s="68"/>
-      <c r="AE3" s="68"/>
-      <c r="AF3" s="68"/>
-      <c r="AG3" s="68"/>
-      <c r="AH3" s="68"/>
-      <c r="AI3" s="68"/>
-      <c r="AJ3" s="68"/>
-      <c r="AK3" s="68"/>
-      <c r="AL3" s="22"/>
-      <c r="AM3" s="22"/>
-      <c r="AN3" s="22"/>
-      <c r="AO3" s="22"/>
-      <c r="AP3" s="22"/>
-      <c r="AQ3" s="68"/>
-      <c r="AR3" s="68"/>
-      <c r="AS3" s="68"/>
-      <c r="AT3" s="68"/>
-      <c r="AU3" s="68"/>
-      <c r="AV3" s="68"/>
-      <c r="AW3" s="68"/>
-      <c r="AX3" s="68"/>
-      <c r="AY3" s="68"/>
-      <c r="AZ3" s="68"/>
-      <c r="BA3" s="69"/>
+      <c r="B3" s="73"/>
+      <c r="C3" s="73"/>
+      <c r="D3" s="73"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="73"/>
+      <c r="G3" s="73"/>
+      <c r="H3" s="73"/>
+      <c r="I3" s="73"/>
+      <c r="J3" s="73"/>
+      <c r="K3" s="73"/>
+      <c r="L3" s="73"/>
+      <c r="M3" s="73"/>
+      <c r="N3" s="73"/>
+      <c r="O3" s="73"/>
+      <c r="P3" s="73"/>
+      <c r="Q3" s="73"/>
+      <c r="R3" s="73"/>
+      <c r="S3" s="73"/>
+      <c r="T3" s="73"/>
+      <c r="U3" s="73"/>
+      <c r="V3" s="73"/>
+      <c r="W3" s="73"/>
+      <c r="X3" s="73"/>
+      <c r="Y3" s="73"/>
+      <c r="Z3" s="73"/>
+      <c r="AA3" s="73"/>
+      <c r="AB3" s="73"/>
+      <c r="AC3" s="73"/>
+      <c r="AD3" s="73"/>
+      <c r="AE3" s="73"/>
+      <c r="AF3" s="73"/>
+      <c r="AG3" s="73"/>
+      <c r="AH3" s="73"/>
+      <c r="AI3" s="73"/>
+      <c r="AJ3" s="73"/>
+      <c r="AK3" s="73"/>
+      <c r="AL3" s="64"/>
+      <c r="AM3" s="64"/>
+      <c r="AN3" s="64"/>
+      <c r="AO3" s="64"/>
+      <c r="AP3" s="64"/>
+      <c r="AQ3" s="73"/>
+      <c r="AR3" s="73"/>
+      <c r="AS3" s="73"/>
+      <c r="AT3" s="73"/>
+      <c r="AU3" s="73"/>
+      <c r="AV3" s="73"/>
+      <c r="AW3" s="73"/>
+      <c r="AX3" s="73"/>
+      <c r="AY3" s="73"/>
+      <c r="AZ3" s="73"/>
+      <c r="BA3" s="74"/>
     </row>
     <row r="4" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="68" t="s">
         <v>115</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="68"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
-      <c r="N4" s="68"/>
-      <c r="O4" s="68"/>
-      <c r="P4" s="68"/>
-      <c r="Q4" s="68"/>
-      <c r="R4" s="68"/>
-      <c r="S4" s="69"/>
-      <c r="T4" s="51" t="s">
+      <c r="B4" s="73"/>
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
+      <c r="I4" s="73"/>
+      <c r="J4" s="73"/>
+      <c r="K4" s="73"/>
+      <c r="L4" s="73"/>
+      <c r="M4" s="73"/>
+      <c r="N4" s="73"/>
+      <c r="O4" s="73"/>
+      <c r="P4" s="73"/>
+      <c r="Q4" s="73"/>
+      <c r="R4" s="73"/>
+      <c r="S4" s="74"/>
+      <c r="T4" s="68" t="s">
         <v>116</v>
       </c>
-      <c r="U4" s="68"/>
-      <c r="V4" s="68"/>
-      <c r="W4" s="68"/>
-      <c r="X4" s="68"/>
-      <c r="Y4" s="68"/>
-      <c r="Z4" s="68"/>
-      <c r="AA4" s="68"/>
-      <c r="AB4" s="68"/>
-      <c r="AC4" s="68"/>
-      <c r="AD4" s="68"/>
-      <c r="AE4" s="68"/>
-      <c r="AF4" s="68"/>
-      <c r="AG4" s="68"/>
-      <c r="AH4" s="68"/>
-      <c r="AI4" s="68"/>
-      <c r="AJ4" s="68"/>
-      <c r="AK4" s="69"/>
-      <c r="AL4" s="51" t="s">
+      <c r="U4" s="73"/>
+      <c r="V4" s="73"/>
+      <c r="W4" s="73"/>
+      <c r="X4" s="73"/>
+      <c r="Y4" s="73"/>
+      <c r="Z4" s="73"/>
+      <c r="AA4" s="73"/>
+      <c r="AB4" s="73"/>
+      <c r="AC4" s="73"/>
+      <c r="AD4" s="73"/>
+      <c r="AE4" s="73"/>
+      <c r="AF4" s="73"/>
+      <c r="AG4" s="73"/>
+      <c r="AH4" s="73"/>
+      <c r="AI4" s="73"/>
+      <c r="AJ4" s="73"/>
+      <c r="AK4" s="74"/>
+      <c r="AL4" s="68" t="s">
         <v>117</v>
       </c>
-      <c r="AM4" s="22"/>
-      <c r="AN4" s="22"/>
-      <c r="AO4" s="22"/>
-      <c r="AP4" s="23"/>
-      <c r="AQ4" s="51" t="s">
+      <c r="AM4" s="64"/>
+      <c r="AN4" s="64"/>
+      <c r="AO4" s="64"/>
+      <c r="AP4" s="65"/>
+      <c r="AQ4" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="AR4" s="68"/>
-      <c r="AS4" s="68"/>
-      <c r="AT4" s="69"/>
-      <c r="AU4" s="43" t="s">
+      <c r="AR4" s="73"/>
+      <c r="AS4" s="73"/>
+      <c r="AT4" s="74"/>
+      <c r="AU4" s="27" t="s">
         <v>118</v>
       </c>
-      <c r="AV4" s="51" t="s">
+      <c r="AV4" s="68" t="s">
         <v>119</v>
       </c>
-      <c r="AW4" s="68"/>
-      <c r="AX4" s="68"/>
-      <c r="AY4" s="68"/>
-      <c r="AZ4" s="69"/>
-      <c r="BA4" s="43" t="s">
+      <c r="AW4" s="73"/>
+      <c r="AX4" s="73"/>
+      <c r="AY4" s="73"/>
+      <c r="AZ4" s="74"/>
+      <c r="BA4" s="27" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:53" ht="58.5" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="48" t="s">
+      <c r="A5" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="31" t="s">
         <v>121</v>
       </c>
-      <c r="C5" s="48" t="s">
+      <c r="C5" s="31" t="s">
         <v>78</v>
       </c>
-      <c r="D5" s="70"/>
-      <c r="E5" s="70"/>
-      <c r="F5" s="70"/>
-      <c r="G5" s="71" t="s">
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="50"/>
+      <c r="G5" s="69" t="s">
         <v>82</v>
       </c>
-      <c r="H5" s="72"/>
-      <c r="I5" s="72"/>
-      <c r="J5" s="73"/>
-      <c r="K5" s="71" t="s">
+      <c r="H5" s="70"/>
+      <c r="I5" s="70"/>
+      <c r="J5" s="71"/>
+      <c r="K5" s="69" t="s">
         <v>122</v>
       </c>
-      <c r="L5" s="72"/>
-      <c r="M5" s="72"/>
-      <c r="N5" s="73"/>
-      <c r="O5" s="74" t="s">
+      <c r="L5" s="70"/>
+      <c r="M5" s="70"/>
+      <c r="N5" s="71"/>
+      <c r="O5" s="72" t="s">
         <v>123</v>
       </c>
-      <c r="P5" s="68"/>
-      <c r="Q5" s="68"/>
-      <c r="R5" s="69"/>
-      <c r="S5" s="75" t="s">
+      <c r="P5" s="73"/>
+      <c r="Q5" s="73"/>
+      <c r="R5" s="74"/>
+      <c r="S5" s="51" t="s">
         <v>124</v>
       </c>
-      <c r="T5" s="43" t="s">
+      <c r="T5" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="U5" s="48" t="s">
+      <c r="U5" s="31" t="s">
         <v>125</v>
       </c>
-      <c r="V5" s="51" t="s">
+      <c r="V5" s="68" t="s">
         <v>126</v>
       </c>
-      <c r="W5" s="68"/>
-      <c r="X5" s="69"/>
-      <c r="Y5" s="76" t="s">
+      <c r="W5" s="73"/>
+      <c r="X5" s="74"/>
+      <c r="Y5" s="52" t="s">
         <v>127</v>
       </c>
-      <c r="Z5" s="76" t="s">
+      <c r="Z5" s="52" t="s">
         <v>128</v>
       </c>
-      <c r="AA5" s="76" t="s">
+      <c r="AA5" s="52" t="s">
         <v>129</v>
       </c>
-      <c r="AB5" s="76" t="s">
+      <c r="AB5" s="52" t="s">
         <v>130</v>
       </c>
-      <c r="AC5" s="76" t="s">
+      <c r="AC5" s="52" t="s">
         <v>131</v>
       </c>
-      <c r="AD5" s="76" t="s">
+      <c r="AD5" s="52" t="s">
         <v>132</v>
       </c>
-      <c r="AE5" s="77" t="s">
+      <c r="AE5" s="53" t="s">
         <v>133</v>
       </c>
-      <c r="AF5" s="43" t="s">
+      <c r="AF5" s="27" t="s">
         <v>134</v>
       </c>
-      <c r="AG5" s="78" t="s">
+      <c r="AG5" s="75" t="s">
         <v>135</v>
       </c>
-      <c r="AH5" s="69"/>
-      <c r="AI5" s="51" t="s">
+      <c r="AH5" s="74"/>
+      <c r="AI5" s="68" t="s">
         <v>136</v>
       </c>
-      <c r="AJ5" s="69"/>
-      <c r="AK5" s="43" t="s">
+      <c r="AJ5" s="74"/>
+      <c r="AK5" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="AL5" s="43" t="s">
+      <c r="AL5" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AM5" s="43" t="s">
+      <c r="AM5" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="AN5" s="79" t="s">
+      <c r="AN5" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AO5" s="79" t="s">
+      <c r="AO5" s="54" t="s">
         <v>107</v>
       </c>
-      <c r="AP5" s="43" t="s">
+      <c r="AP5" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="AQ5" s="43" t="s">
+      <c r="AQ5" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AR5" s="79" t="s">
+      <c r="AR5" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AS5" s="79" t="s">
+      <c r="AS5" s="54" t="s">
         <v>107</v>
       </c>
-      <c r="AT5" s="43" t="s">
+      <c r="AT5" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="AU5" s="77"/>
-      <c r="AV5" s="43" t="s">
+      <c r="AU5" s="53"/>
+      <c r="AV5" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AW5" s="79" t="s">
+      <c r="AW5" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AX5" s="79" t="s">
+      <c r="AX5" s="54" t="s">
         <v>107</v>
       </c>
-      <c r="AY5" s="80" t="s">
+      <c r="AY5" s="55" t="s">
         <v>139</v>
       </c>
-      <c r="AZ5" s="43" t="s">
+      <c r="AZ5" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="BA5" s="77"/>
+      <c r="BA5" s="53"/>
     </row>
     <row r="6" spans="1:53" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="48"/>
-      <c r="B6" s="48"/>
-      <c r="C6" s="48"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-      <c r="G6" s="81" t="s">
+      <c r="A6" s="31"/>
+      <c r="B6" s="31"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="56" t="s">
         <v>140</v>
       </c>
-      <c r="H6" s="48" t="s">
+      <c r="H6" s="31" t="s">
         <v>141</v>
       </c>
-      <c r="I6" s="48" t="s">
+      <c r="I6" s="31" t="s">
         <v>142</v>
       </c>
-      <c r="J6" s="82" t="s">
+      <c r="J6" s="57" t="s">
         <v>143</v>
       </c>
-      <c r="K6" s="81" t="s">
+      <c r="K6" s="56" t="s">
         <v>140</v>
       </c>
-      <c r="L6" s="46" t="s">
+      <c r="L6" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="M6" s="48" t="s">
+      <c r="M6" s="31" t="s">
         <v>142</v>
       </c>
-      <c r="N6" s="82" t="s">
+      <c r="N6" s="57" t="s">
         <v>143</v>
       </c>
-      <c r="O6" s="79" t="s">
+      <c r="O6" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="P6" s="79" t="s">
+      <c r="P6" s="54" t="s">
         <v>145</v>
       </c>
-      <c r="Q6" s="79" t="s">
+      <c r="Q6" s="54" t="s">
         <v>146</v>
       </c>
-      <c r="R6" s="79" t="s">
+      <c r="R6" s="54" t="s">
         <v>147</v>
       </c>
-      <c r="S6" s="83" t="s">
+      <c r="S6" s="58" t="s">
         <v>148</v>
       </c>
-      <c r="T6" s="54"/>
-      <c r="U6" s="43"/>
-      <c r="V6" s="43" t="s">
+      <c r="T6" s="36"/>
+      <c r="U6" s="27"/>
+      <c r="V6" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="W6" s="43" t="s">
+      <c r="W6" s="27" t="s">
         <v>150</v>
       </c>
-      <c r="X6" s="43" t="s">
+      <c r="X6" s="27" t="s">
         <v>143</v>
       </c>
-      <c r="Y6" s="77"/>
-      <c r="Z6" s="77"/>
-      <c r="AA6" s="77"/>
-      <c r="AB6" s="77"/>
-      <c r="AC6" s="77"/>
-      <c r="AD6" s="77"/>
-      <c r="AE6" s="54"/>
-      <c r="AF6" s="54"/>
-      <c r="AG6" s="79" t="s">
+      <c r="Y6" s="53"/>
+      <c r="Z6" s="53"/>
+      <c r="AA6" s="53"/>
+      <c r="AB6" s="53"/>
+      <c r="AC6" s="53"/>
+      <c r="AD6" s="53"/>
+      <c r="AE6" s="36"/>
+      <c r="AF6" s="36"/>
+      <c r="AG6" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AH6" s="79" t="s">
+      <c r="AH6" s="54" t="s">
         <v>107</v>
       </c>
-      <c r="AI6" s="79" t="s">
+      <c r="AI6" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AJ6" s="79" t="s">
+      <c r="AJ6" s="54" t="s">
         <v>107</v>
       </c>
-      <c r="AK6" s="54"/>
-      <c r="AL6" s="54"/>
-      <c r="AM6" s="54"/>
-      <c r="AN6" s="79"/>
-      <c r="AO6" s="79"/>
-      <c r="AP6" s="54"/>
-      <c r="AQ6" s="54"/>
-      <c r="AR6" s="79"/>
-      <c r="AS6" s="79"/>
-      <c r="AT6" s="54"/>
-      <c r="AU6" s="54"/>
-      <c r="AV6" s="54"/>
-      <c r="AW6" s="79"/>
-      <c r="AX6" s="79"/>
-      <c r="AY6" s="84"/>
-      <c r="AZ6" s="54"/>
-      <c r="BA6" s="54"/>
+      <c r="AK6" s="36"/>
+      <c r="AL6" s="36"/>
+      <c r="AM6" s="36"/>
+      <c r="AN6" s="54"/>
+      <c r="AO6" s="54"/>
+      <c r="AP6" s="36"/>
+      <c r="AQ6" s="36"/>
+      <c r="AR6" s="54"/>
+      <c r="AS6" s="54"/>
+      <c r="AT6" s="36"/>
+      <c r="AU6" s="36"/>
+      <c r="AV6" s="36"/>
+      <c r="AW6" s="54"/>
+      <c r="AX6" s="54"/>
+      <c r="AY6" s="59"/>
+      <c r="AZ6" s="36"/>
+      <c r="BA6" s="36"/>
     </row>
     <row r="9" spans="1:53" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -3261,17 +3261,17 @@
         <v>78</v>
       </c>
       <c r="D10" s="6"/>
-      <c r="H10" s="86"/>
-      <c r="I10" s="86"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="61"/>
       <c r="J10" s="6" t="s">
         <v>82</v>
       </c>
       <c r="M10" s="6"/>
       <c r="N10" s="17"/>
-      <c r="O10" s="85"/>
-      <c r="P10" s="86"/>
-      <c r="Q10" s="87"/>
-      <c r="AQ10" s="85" t="s">
+      <c r="O10" s="60"/>
+      <c r="P10" s="61"/>
+      <c r="Q10" s="62"/>
+      <c r="AQ10" s="60" t="s">
         <v>55</v>
       </c>
       <c r="AR10" s="6" t="s">
@@ -3286,11 +3286,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="O5:R5"/>
-    <mergeCell ref="V5:X5"/>
-    <mergeCell ref="AG5:AH5"/>
     <mergeCell ref="AI5:AJ5"/>
     <mergeCell ref="A1:BA1"/>
     <mergeCell ref="A3:BA3"/>
@@ -3299,6 +3294,11 @@
     <mergeCell ref="AL4:AP4"/>
     <mergeCell ref="AQ4:AT4"/>
     <mergeCell ref="AV4:AZ4"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="O5:R5"/>
+    <mergeCell ref="V5:X5"/>
+    <mergeCell ref="AG5:AH5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3308,6 +3308,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECB08AFA-BF49-47F5-B095-34C6A355FE30}">
   <dimension ref="A2:BA10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="6" max="6" width="11.6328125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="2" spans="1:53" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -3315,351 +3318,351 @@
       </c>
     </row>
     <row r="3" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A3" s="51" t="str">
+      <c r="A3" s="68" t="str">
         <f>+[1]Summary!A5</f>
         <v>Progress of 220kV Line</v>
       </c>
-      <c r="B3" s="68"/>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="68"/>
-      <c r="K3" s="68"/>
-      <c r="L3" s="68"/>
-      <c r="M3" s="68"/>
-      <c r="N3" s="68"/>
-      <c r="O3" s="68"/>
-      <c r="P3" s="68"/>
-      <c r="Q3" s="68"/>
-      <c r="R3" s="68"/>
-      <c r="S3" s="68"/>
-      <c r="T3" s="68"/>
-      <c r="U3" s="68"/>
-      <c r="V3" s="68"/>
-      <c r="W3" s="68"/>
-      <c r="X3" s="68"/>
-      <c r="Y3" s="68"/>
-      <c r="Z3" s="68"/>
-      <c r="AA3" s="68"/>
-      <c r="AB3" s="68"/>
-      <c r="AC3" s="68"/>
-      <c r="AD3" s="68"/>
-      <c r="AE3" s="68"/>
-      <c r="AF3" s="68"/>
-      <c r="AG3" s="68"/>
-      <c r="AH3" s="68"/>
-      <c r="AI3" s="68"/>
-      <c r="AJ3" s="68"/>
-      <c r="AK3" s="68"/>
-      <c r="AL3" s="22"/>
-      <c r="AM3" s="22"/>
-      <c r="AN3" s="22"/>
-      <c r="AO3" s="22"/>
-      <c r="AP3" s="22"/>
-      <c r="AQ3" s="68"/>
-      <c r="AR3" s="68"/>
-      <c r="AS3" s="68"/>
-      <c r="AT3" s="68"/>
-      <c r="AU3" s="68"/>
-      <c r="AV3" s="68"/>
-      <c r="AW3" s="68"/>
-      <c r="AX3" s="68"/>
-      <c r="AY3" s="68"/>
-      <c r="AZ3" s="68"/>
-      <c r="BA3" s="69"/>
+      <c r="B3" s="73"/>
+      <c r="C3" s="73"/>
+      <c r="D3" s="73"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="73"/>
+      <c r="G3" s="73"/>
+      <c r="H3" s="73"/>
+      <c r="I3" s="73"/>
+      <c r="J3" s="73"/>
+      <c r="K3" s="73"/>
+      <c r="L3" s="73"/>
+      <c r="M3" s="73"/>
+      <c r="N3" s="73"/>
+      <c r="O3" s="73"/>
+      <c r="P3" s="73"/>
+      <c r="Q3" s="73"/>
+      <c r="R3" s="73"/>
+      <c r="S3" s="73"/>
+      <c r="T3" s="73"/>
+      <c r="U3" s="73"/>
+      <c r="V3" s="73"/>
+      <c r="W3" s="73"/>
+      <c r="X3" s="73"/>
+      <c r="Y3" s="73"/>
+      <c r="Z3" s="73"/>
+      <c r="AA3" s="73"/>
+      <c r="AB3" s="73"/>
+      <c r="AC3" s="73"/>
+      <c r="AD3" s="73"/>
+      <c r="AE3" s="73"/>
+      <c r="AF3" s="73"/>
+      <c r="AG3" s="73"/>
+      <c r="AH3" s="73"/>
+      <c r="AI3" s="73"/>
+      <c r="AJ3" s="73"/>
+      <c r="AK3" s="73"/>
+      <c r="AL3" s="64"/>
+      <c r="AM3" s="64"/>
+      <c r="AN3" s="64"/>
+      <c r="AO3" s="64"/>
+      <c r="AP3" s="64"/>
+      <c r="AQ3" s="73"/>
+      <c r="AR3" s="73"/>
+      <c r="AS3" s="73"/>
+      <c r="AT3" s="73"/>
+      <c r="AU3" s="73"/>
+      <c r="AV3" s="73"/>
+      <c r="AW3" s="73"/>
+      <c r="AX3" s="73"/>
+      <c r="AY3" s="73"/>
+      <c r="AZ3" s="73"/>
+      <c r="BA3" s="74"/>
     </row>
     <row r="4" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="68" t="s">
         <v>115</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="68"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
-      <c r="N4" s="68"/>
-      <c r="O4" s="68"/>
-      <c r="P4" s="68"/>
-      <c r="Q4" s="68"/>
-      <c r="R4" s="68"/>
-      <c r="S4" s="69"/>
-      <c r="T4" s="51" t="s">
+      <c r="B4" s="73"/>
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
+      <c r="I4" s="73"/>
+      <c r="J4" s="73"/>
+      <c r="K4" s="73"/>
+      <c r="L4" s="73"/>
+      <c r="M4" s="73"/>
+      <c r="N4" s="73"/>
+      <c r="O4" s="73"/>
+      <c r="P4" s="73"/>
+      <c r="Q4" s="73"/>
+      <c r="R4" s="73"/>
+      <c r="S4" s="74"/>
+      <c r="T4" s="68" t="s">
         <v>116</v>
       </c>
-      <c r="U4" s="68"/>
-      <c r="V4" s="68"/>
-      <c r="W4" s="68"/>
-      <c r="X4" s="68"/>
-      <c r="Y4" s="68"/>
-      <c r="Z4" s="68"/>
-      <c r="AA4" s="68"/>
-      <c r="AB4" s="68"/>
-      <c r="AC4" s="68"/>
-      <c r="AD4" s="68"/>
-      <c r="AE4" s="68"/>
-      <c r="AF4" s="68"/>
-      <c r="AG4" s="68"/>
-      <c r="AH4" s="68"/>
-      <c r="AI4" s="68"/>
-      <c r="AJ4" s="68"/>
-      <c r="AK4" s="69"/>
-      <c r="AL4" s="51" t="s">
+      <c r="U4" s="73"/>
+      <c r="V4" s="73"/>
+      <c r="W4" s="73"/>
+      <c r="X4" s="73"/>
+      <c r="Y4" s="73"/>
+      <c r="Z4" s="73"/>
+      <c r="AA4" s="73"/>
+      <c r="AB4" s="73"/>
+      <c r="AC4" s="73"/>
+      <c r="AD4" s="73"/>
+      <c r="AE4" s="73"/>
+      <c r="AF4" s="73"/>
+      <c r="AG4" s="73"/>
+      <c r="AH4" s="73"/>
+      <c r="AI4" s="73"/>
+      <c r="AJ4" s="73"/>
+      <c r="AK4" s="74"/>
+      <c r="AL4" s="68" t="s">
         <v>117</v>
       </c>
-      <c r="AM4" s="22"/>
-      <c r="AN4" s="22"/>
-      <c r="AO4" s="22"/>
-      <c r="AP4" s="23"/>
-      <c r="AQ4" s="51" t="s">
+      <c r="AM4" s="64"/>
+      <c r="AN4" s="64"/>
+      <c r="AO4" s="64"/>
+      <c r="AP4" s="65"/>
+      <c r="AQ4" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="AR4" s="68"/>
-      <c r="AS4" s="68"/>
-      <c r="AT4" s="69"/>
-      <c r="AU4" s="43" t="s">
+      <c r="AR4" s="73"/>
+      <c r="AS4" s="73"/>
+      <c r="AT4" s="74"/>
+      <c r="AU4" s="27" t="s">
         <v>118</v>
       </c>
-      <c r="AV4" s="51" t="s">
+      <c r="AV4" s="68" t="s">
         <v>119</v>
       </c>
-      <c r="AW4" s="68"/>
-      <c r="AX4" s="68"/>
-      <c r="AY4" s="68"/>
-      <c r="AZ4" s="69"/>
-      <c r="BA4" s="43" t="s">
+      <c r="AW4" s="73"/>
+      <c r="AX4" s="73"/>
+      <c r="AY4" s="73"/>
+      <c r="AZ4" s="74"/>
+      <c r="BA4" s="27" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:53" ht="58.5" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="48" t="s">
+      <c r="A5" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="31" t="s">
         <v>121</v>
       </c>
-      <c r="C5" s="48" t="s">
+      <c r="C5" s="31" t="s">
         <v>78</v>
       </c>
-      <c r="D5" s="70"/>
-      <c r="E5" s="70"/>
-      <c r="F5" s="70"/>
-      <c r="G5" s="71" t="s">
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="50"/>
+      <c r="G5" s="69" t="s">
         <v>82</v>
       </c>
-      <c r="H5" s="72"/>
-      <c r="I5" s="72"/>
-      <c r="J5" s="73"/>
-      <c r="K5" s="71" t="s">
+      <c r="H5" s="70"/>
+      <c r="I5" s="70"/>
+      <c r="J5" s="71"/>
+      <c r="K5" s="69" t="s">
         <v>122</v>
       </c>
-      <c r="L5" s="72"/>
-      <c r="M5" s="72"/>
-      <c r="N5" s="73"/>
-      <c r="O5" s="74" t="s">
+      <c r="L5" s="70"/>
+      <c r="M5" s="70"/>
+      <c r="N5" s="71"/>
+      <c r="O5" s="72" t="s">
         <v>123</v>
       </c>
-      <c r="P5" s="68"/>
-      <c r="Q5" s="68"/>
-      <c r="R5" s="69"/>
-      <c r="S5" s="75" t="s">
+      <c r="P5" s="73"/>
+      <c r="Q5" s="73"/>
+      <c r="R5" s="74"/>
+      <c r="S5" s="51" t="s">
         <v>124</v>
       </c>
-      <c r="T5" s="43" t="s">
+      <c r="T5" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="U5" s="48" t="s">
+      <c r="U5" s="31" t="s">
         <v>125</v>
       </c>
-      <c r="V5" s="51" t="s">
+      <c r="V5" s="68" t="s">
         <v>126</v>
       </c>
-      <c r="W5" s="68"/>
-      <c r="X5" s="69"/>
-      <c r="Y5" s="76" t="s">
+      <c r="W5" s="73"/>
+      <c r="X5" s="74"/>
+      <c r="Y5" s="52" t="s">
         <v>127</v>
       </c>
-      <c r="Z5" s="76" t="s">
+      <c r="Z5" s="52" t="s">
         <v>128</v>
       </c>
-      <c r="AA5" s="76" t="s">
+      <c r="AA5" s="52" t="s">
         <v>129</v>
       </c>
-      <c r="AB5" s="76" t="s">
+      <c r="AB5" s="52" t="s">
         <v>130</v>
       </c>
-      <c r="AC5" s="76" t="s">
+      <c r="AC5" s="52" t="s">
         <v>131</v>
       </c>
-      <c r="AD5" s="76" t="s">
+      <c r="AD5" s="52" t="s">
         <v>132</v>
       </c>
-      <c r="AE5" s="77" t="s">
+      <c r="AE5" s="53" t="s">
         <v>133</v>
       </c>
-      <c r="AF5" s="43" t="s">
+      <c r="AF5" s="27" t="s">
         <v>134</v>
       </c>
-      <c r="AG5" s="78" t="s">
+      <c r="AG5" s="75" t="s">
         <v>135</v>
       </c>
-      <c r="AH5" s="69"/>
-      <c r="AI5" s="51" t="s">
+      <c r="AH5" s="74"/>
+      <c r="AI5" s="68" t="s">
         <v>136</v>
       </c>
-      <c r="AJ5" s="69"/>
-      <c r="AK5" s="43" t="s">
+      <c r="AJ5" s="74"/>
+      <c r="AK5" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="AL5" s="43" t="s">
+      <c r="AL5" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AM5" s="43" t="s">
+      <c r="AM5" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="AN5" s="79" t="s">
+      <c r="AN5" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AO5" s="79" t="s">
+      <c r="AO5" s="54" t="s">
         <v>107</v>
       </c>
-      <c r="AP5" s="43" t="s">
+      <c r="AP5" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="AQ5" s="43" t="s">
+      <c r="AQ5" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AR5" s="79" t="s">
+      <c r="AR5" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AS5" s="79" t="s">
+      <c r="AS5" s="54" t="s">
         <v>107</v>
       </c>
-      <c r="AT5" s="43" t="s">
+      <c r="AT5" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="AU5" s="77"/>
-      <c r="AV5" s="43" t="s">
+      <c r="AU5" s="53"/>
+      <c r="AV5" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AW5" s="79" t="s">
+      <c r="AW5" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AX5" s="79" t="s">
+      <c r="AX5" s="54" t="s">
         <v>107</v>
       </c>
-      <c r="AY5" s="80" t="s">
+      <c r="AY5" s="55" t="s">
         <v>139</v>
       </c>
-      <c r="AZ5" s="43" t="s">
+      <c r="AZ5" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="BA5" s="77"/>
+      <c r="BA5" s="53"/>
     </row>
     <row r="6" spans="1:53" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="48"/>
-      <c r="B6" s="48"/>
-      <c r="C6" s="48"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-      <c r="G6" s="81" t="s">
+      <c r="A6" s="31"/>
+      <c r="B6" s="31"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="56" t="s">
         <v>140</v>
       </c>
-      <c r="H6" s="48" t="s">
+      <c r="H6" s="31" t="s">
         <v>141</v>
       </c>
-      <c r="I6" s="48" t="s">
+      <c r="I6" s="31" t="s">
         <v>142</v>
       </c>
-      <c r="J6" s="82" t="s">
+      <c r="J6" s="57" t="s">
         <v>143</v>
       </c>
-      <c r="K6" s="81" t="s">
+      <c r="K6" s="56" t="s">
         <v>140</v>
       </c>
-      <c r="L6" s="46" t="s">
+      <c r="L6" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="M6" s="48" t="s">
+      <c r="M6" s="31" t="s">
         <v>142</v>
       </c>
-      <c r="N6" s="82" t="s">
+      <c r="N6" s="57" t="s">
         <v>143</v>
       </c>
-      <c r="O6" s="79" t="s">
+      <c r="O6" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="P6" s="79" t="s">
+      <c r="P6" s="54" t="s">
         <v>145</v>
       </c>
-      <c r="Q6" s="79" t="s">
+      <c r="Q6" s="54" t="s">
         <v>146</v>
       </c>
-      <c r="R6" s="79" t="s">
+      <c r="R6" s="54" t="s">
         <v>147</v>
       </c>
-      <c r="S6" s="83" t="s">
+      <c r="S6" s="58" t="s">
         <v>148</v>
       </c>
-      <c r="T6" s="54"/>
-      <c r="U6" s="43"/>
-      <c r="V6" s="43" t="s">
+      <c r="T6" s="36"/>
+      <c r="U6" s="27"/>
+      <c r="V6" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="W6" s="43" t="s">
+      <c r="W6" s="27" t="s">
         <v>150</v>
       </c>
-      <c r="X6" s="43" t="s">
+      <c r="X6" s="27" t="s">
         <v>143</v>
       </c>
-      <c r="Y6" s="77"/>
-      <c r="Z6" s="77"/>
-      <c r="AA6" s="77"/>
-      <c r="AB6" s="77"/>
-      <c r="AC6" s="77"/>
-      <c r="AD6" s="77"/>
-      <c r="AE6" s="54"/>
-      <c r="AF6" s="54"/>
-      <c r="AG6" s="79" t="s">
+      <c r="Y6" s="53"/>
+      <c r="Z6" s="53"/>
+      <c r="AA6" s="53"/>
+      <c r="AB6" s="53"/>
+      <c r="AC6" s="53"/>
+      <c r="AD6" s="53"/>
+      <c r="AE6" s="36"/>
+      <c r="AF6" s="36"/>
+      <c r="AG6" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AH6" s="79" t="s">
+      <c r="AH6" s="54" t="s">
         <v>107</v>
       </c>
-      <c r="AI6" s="79" t="s">
+      <c r="AI6" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AJ6" s="79" t="s">
+      <c r="AJ6" s="54" t="s">
         <v>107</v>
       </c>
-      <c r="AK6" s="54"/>
-      <c r="AL6" s="54"/>
-      <c r="AM6" s="54"/>
-      <c r="AN6" s="79"/>
-      <c r="AO6" s="79"/>
-      <c r="AP6" s="54"/>
-      <c r="AQ6" s="54"/>
-      <c r="AR6" s="79"/>
-      <c r="AS6" s="79"/>
-      <c r="AT6" s="54"/>
-      <c r="AU6" s="54"/>
-      <c r="AV6" s="54"/>
-      <c r="AW6" s="79"/>
-      <c r="AX6" s="79"/>
-      <c r="AY6" s="84"/>
-      <c r="AZ6" s="54"/>
-      <c r="BA6" s="54"/>
+      <c r="AK6" s="36"/>
+      <c r="AL6" s="36"/>
+      <c r="AM6" s="36"/>
+      <c r="AN6" s="54"/>
+      <c r="AO6" s="54"/>
+      <c r="AP6" s="36"/>
+      <c r="AQ6" s="36"/>
+      <c r="AR6" s="54"/>
+      <c r="AS6" s="54"/>
+      <c r="AT6" s="36"/>
+      <c r="AU6" s="36"/>
+      <c r="AV6" s="36"/>
+      <c r="AW6" s="54"/>
+      <c r="AX6" s="54"/>
+      <c r="AY6" s="59"/>
+      <c r="AZ6" s="36"/>
+      <c r="BA6" s="36"/>
     </row>
     <row r="9" spans="1:53" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -3677,17 +3680,17 @@
         <v>78</v>
       </c>
       <c r="D10" s="6"/>
-      <c r="H10" s="86"/>
-      <c r="I10" s="86"/>
+      <c r="H10" s="61"/>
+      <c r="I10" s="61"/>
       <c r="J10" s="6" t="s">
         <v>82</v>
       </c>
       <c r="M10" s="6"/>
       <c r="N10" s="17"/>
-      <c r="O10" s="85"/>
-      <c r="P10" s="86"/>
-      <c r="Q10" s="87"/>
-      <c r="AQ10" s="85" t="s">
+      <c r="O10" s="60"/>
+      <c r="P10" s="61"/>
+      <c r="Q10" s="62"/>
+      <c r="AQ10" s="60" t="s">
         <v>55</v>
       </c>
       <c r="AR10" s="6" t="s">
@@ -3702,11 +3705,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="O5:R5"/>
-    <mergeCell ref="V5:X5"/>
-    <mergeCell ref="AG5:AH5"/>
     <mergeCell ref="AI5:AJ5"/>
     <mergeCell ref="A3:BA3"/>
     <mergeCell ref="A4:S4"/>
@@ -3714,6 +3712,11 @@
     <mergeCell ref="AL4:AP4"/>
     <mergeCell ref="AQ4:AT4"/>
     <mergeCell ref="AV4:AZ4"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="O5:R5"/>
+    <mergeCell ref="V5:X5"/>
+    <mergeCell ref="AG5:AH5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3730,35 +3733,35 @@
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="78" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="79" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="21" t="s">
+      <c r="C3" s="64"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="79" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="22"/>
-      <c r="G3" s="23"/>
-      <c r="H3" s="21" t="s">
+      <c r="F3" s="64"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="79" t="s">
         <v>38</v>
       </c>
-      <c r="I3" s="22"/>
-      <c r="J3" s="23"/>
-      <c r="K3" s="20" t="s">
+      <c r="I3" s="64"/>
+      <c r="J3" s="65"/>
+      <c r="K3" s="78" t="s">
         <v>75</v>
       </c>
-      <c r="L3" s="18" t="s">
+      <c r="L3" s="76" t="s">
         <v>43</v>
       </c>
       <c r="M3" s="8"/>
       <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="31" x14ac:dyDescent="0.35">
-      <c r="A4" s="19"/>
+      <c r="A4" s="77"/>
       <c r="B4" s="12" t="s">
         <v>39</v>
       </c>
@@ -3786,8 +3789,8 @@
       <c r="J4" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
+      <c r="K4" s="77"/>
+      <c r="L4" s="77"/>
       <c r="M4" s="10"/>
       <c r="N4" s="11"/>
     </row>
@@ -3866,46 +3869,46 @@
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="83" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27" t="s">
+      <c r="C3" s="83"/>
+      <c r="D3" s="83" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="27" t="s">
+      <c r="E3" s="83" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="27" t="s">
+      <c r="F3" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="84" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="24" t="s">
+      <c r="H3" s="84"/>
+      <c r="I3" s="84"/>
+      <c r="J3" s="80" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="25"/>
-      <c r="L3" s="25"/>
-      <c r="M3" s="25"/>
-      <c r="N3" s="26"/>
+      <c r="K3" s="81"/>
+      <c r="L3" s="81"/>
+      <c r="M3" s="81"/>
+      <c r="N3" s="82"/>
     </row>
     <row r="4" spans="1:23" ht="26" x14ac:dyDescent="0.35">
-      <c r="A4" s="27"/>
+      <c r="A4" s="83"/>
       <c r="B4" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
+      <c r="D4" s="83"/>
+      <c r="E4" s="83"/>
+      <c r="F4" s="83"/>
       <c r="G4" s="1" t="s">
         <v>36</v>
       </c>
@@ -4036,14 +4039,14 @@
       <c r="C3" s="7"/>
       <c r="D3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="31"/>
+      <c r="G3" s="85"/>
+      <c r="H3" s="86"/>
+      <c r="I3" s="86"/>
+      <c r="J3" s="87"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="29"/>
-      <c r="O3" s="30"/>
-      <c r="P3" s="31"/>
+      <c r="N3" s="85"/>
+      <c r="O3" s="86"/>
+      <c r="P3" s="87"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -4125,14 +4128,14 @@
       <c r="C3" s="7"/>
       <c r="D3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="31"/>
+      <c r="G3" s="85"/>
+      <c r="H3" s="86"/>
+      <c r="I3" s="86"/>
+      <c r="J3" s="87"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="29"/>
-      <c r="O3" s="30"/>
-      <c r="P3" s="31"/>
+      <c r="N3" s="85"/>
+      <c r="O3" s="86"/>
+      <c r="P3" s="87"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">

</xml_diff>

<commit_message>
Auto pipeline update 2026-03-11 16:07:37
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE42CA59-227D-4A30-BF0E-6B703D25797D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{107148DA-437E-400F-B495-5E88B165F41E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" activeTab="4" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" activeTab="5" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet Names Check" sheetId="1" r:id="rId1"/>
-    <sheet name="Test 000 132kV Stringing" sheetId="11" r:id="rId2"/>
-    <sheet name="Test 000 220kV Stringing" sheetId="10" r:id="rId3"/>
-    <sheet name="Test 000 220kV Erection" sheetId="9" r:id="rId4"/>
-    <sheet name="Test 000 132kV Erection" sheetId="8" r:id="rId5"/>
+    <sheet name="TB 501 132kV Stringing" sheetId="11" r:id="rId2"/>
+    <sheet name="TB 501 220kV Stringing" sheetId="10" r:id="rId3"/>
+    <sheet name="TB 501 220kV Erection" sheetId="9" r:id="rId4"/>
+    <sheet name="TB 501 132kV Erection" sheetId="8" r:id="rId5"/>
     <sheet name="TB 401 Stringing" sheetId="6" r:id="rId6"/>
     <sheet name="TB 408 Stringing" sheetId="2" r:id="rId7"/>
     <sheet name="TA 509 Erection" sheetId="3" r:id="rId8"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="150">
   <si>
     <t>Project Code</t>
   </si>
@@ -302,9 +302,6 @@
   </si>
   <si>
     <t>TA 605 - Jammu; TA 605 - Punjab</t>
-  </si>
-  <si>
-    <t>Test 000</t>
   </si>
   <si>
     <t>Progress-132kV, Progress-220kV</t>
@@ -1295,38 +1292,38 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1859,7 +1856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEA00114-109C-4365-898D-B35AA94B9EEF}">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" customWidth="1"/>
@@ -1889,7 +1886,7 @@
         <v>83</v>
       </c>
       <c r="G1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -2090,7 +2087,22 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>6</v>
+        <v>85</v>
+      </c>
+      <c r="C19" t="s">
+        <v>89</v>
+      </c>
+      <c r="D19" t="s">
+        <v>67</v>
+      </c>
+      <c r="E19" t="s">
+        <v>67</v>
+      </c>
+      <c r="F19" t="s">
+        <v>87</v>
+      </c>
+      <c r="G19" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
@@ -2104,29 +2116,6 @@
       </c>
       <c r="B21" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>85</v>
-      </c>
-      <c r="B22" t="s">
-        <v>86</v>
-      </c>
-      <c r="C22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D22" t="s">
-        <v>67</v>
-      </c>
-      <c r="E22" t="s">
-        <v>67</v>
-      </c>
-      <c r="F22" t="s">
-        <v>88</v>
-      </c>
-      <c r="G22" t="s">
-        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -2148,77 +2137,77 @@
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="63" t="str">
+      <c r="A3" s="73" t="str">
         <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="64"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
-      <c r="L3" s="64"/>
-      <c r="M3" s="64"/>
-      <c r="N3" s="64"/>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="64"/>
-      <c r="S3" s="64"/>
-      <c r="T3" s="64"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="64"/>
-      <c r="W3" s="64"/>
-      <c r="X3" s="64"/>
-      <c r="Y3" s="64"/>
-      <c r="Z3" s="65"/>
+      <c r="B3" s="66"/>
+      <c r="C3" s="66"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="66"/>
+      <c r="J3" s="66"/>
+      <c r="K3" s="66"/>
+      <c r="L3" s="66"/>
+      <c r="M3" s="66"/>
+      <c r="N3" s="66"/>
+      <c r="O3" s="66"/>
+      <c r="P3" s="66"/>
+      <c r="Q3" s="66"/>
+      <c r="R3" s="66"/>
+      <c r="S3" s="66"/>
+      <c r="T3" s="66"/>
+      <c r="U3" s="66"/>
+      <c r="V3" s="66"/>
+      <c r="W3" s="66"/>
+      <c r="X3" s="66"/>
+      <c r="Y3" s="66"/>
+      <c r="Z3" s="67"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="63">
+      <c r="A4" s="73">
         <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="64"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="65"/>
+      <c r="B4" s="66"/>
+      <c r="C4" s="66"/>
+      <c r="D4" s="67"/>
       <c r="E4" s="18"/>
-      <c r="F4" s="63" t="s">
+      <c r="F4" s="73" t="s">
+        <v>90</v>
+      </c>
+      <c r="G4" s="66"/>
+      <c r="H4" s="66"/>
+      <c r="I4" s="66"/>
+      <c r="J4" s="66"/>
+      <c r="K4" s="66"/>
+      <c r="L4" s="66"/>
+      <c r="M4" s="66"/>
+      <c r="N4" s="66"/>
+      <c r="O4" s="66"/>
+      <c r="P4" s="66"/>
+      <c r="Q4" s="66"/>
+      <c r="R4" s="67"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="73" t="s">
         <v>91</v>
       </c>
-      <c r="G4" s="64"/>
-      <c r="H4" s="64"/>
-      <c r="I4" s="64"/>
-      <c r="J4" s="64"/>
-      <c r="K4" s="64"/>
-      <c r="L4" s="64"/>
-      <c r="M4" s="64"/>
-      <c r="N4" s="64"/>
-      <c r="O4" s="64"/>
-      <c r="P4" s="64"/>
-      <c r="Q4" s="64"/>
-      <c r="R4" s="65"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="63" t="s">
+      <c r="U4" s="66"/>
+      <c r="V4" s="66"/>
+      <c r="W4" s="66"/>
+      <c r="X4" s="66"/>
+      <c r="Y4" s="66"/>
+      <c r="Z4" s="67"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A5" s="73" t="s">
         <v>92</v>
       </c>
-      <c r="U4" s="64"/>
-      <c r="V4" s="64"/>
-      <c r="W4" s="64"/>
-      <c r="X4" s="64"/>
-      <c r="Y4" s="64"/>
-      <c r="Z4" s="65"/>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="63" t="s">
-        <v>93</v>
-      </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="65"/>
+      <c r="B5" s="66"/>
+      <c r="C5" s="67"/>
       <c r="D5" s="20">
         <f>[1]Summary!R7</f>
         <v>0</v>
@@ -2275,62 +2264,62 @@
     </row>
     <row r="6" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="74" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="67"/>
+      <c r="D6" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="B6" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="65"/>
-      <c r="D6" s="25" t="s">
+      <c r="E6" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="26" t="s">
+      <c r="F6" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="G6" s="75" t="s">
         <v>97</v>
       </c>
-      <c r="G6" s="67" t="s">
+      <c r="H6" s="66"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="75" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="66"/>
+      <c r="L6" s="67"/>
+      <c r="M6" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="H6" s="64"/>
-      <c r="I6" s="65"/>
-      <c r="J6" s="67" t="s">
-        <v>38</v>
-      </c>
-      <c r="K6" s="64"/>
-      <c r="L6" s="65"/>
-      <c r="M6" s="28" t="s">
+      <c r="N6" s="29" t="s">
         <v>99</v>
       </c>
-      <c r="N6" s="29" t="s">
+      <c r="O6" s="30" t="s">
         <v>100</v>
       </c>
-      <c r="O6" s="30" t="s">
+      <c r="P6" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="P6" s="31" t="s">
+      <c r="Q6" s="32" t="s">
         <v>102</v>
-      </c>
-      <c r="Q6" s="32" t="s">
-        <v>103</v>
       </c>
       <c r="R6" s="27" t="s">
         <v>43</v>
       </c>
       <c r="S6" s="33"/>
-      <c r="T6" s="68" t="s">
+      <c r="T6" s="63" t="s">
+        <v>103</v>
+      </c>
+      <c r="U6" s="66"/>
+      <c r="V6" s="67"/>
+      <c r="W6" s="63" t="s">
         <v>104</v>
       </c>
-      <c r="U6" s="64"/>
-      <c r="V6" s="65"/>
-      <c r="W6" s="68" t="s">
-        <v>105</v>
-      </c>
-      <c r="X6" s="64"/>
-      <c r="Y6" s="65"/>
+      <c r="X6" s="66"/>
+      <c r="Y6" s="67"/>
       <c r="Z6" s="31" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.35">
@@ -2348,19 +2337,19 @@
         <v>55</v>
       </c>
       <c r="H7" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="I7" s="30" t="s">
         <v>106</v>
-      </c>
-      <c r="I7" s="30" t="s">
-        <v>107</v>
       </c>
       <c r="J7" s="30" t="s">
         <v>55</v>
       </c>
       <c r="K7" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="L7" s="30" t="s">
         <v>106</v>
-      </c>
-      <c r="L7" s="30" t="s">
-        <v>107</v>
       </c>
       <c r="M7" s="30" t="s">
         <v>55</v>
@@ -2379,19 +2368,19 @@
         <v>55</v>
       </c>
       <c r="U7" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="V7" s="30" t="s">
         <v>106</v>
-      </c>
-      <c r="V7" s="30" t="s">
-        <v>107</v>
       </c>
       <c r="W7" s="30" t="s">
         <v>55</v>
       </c>
       <c r="X7" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="Y7" s="30" t="s">
         <v>106</v>
-      </c>
-      <c r="Y7" s="30" t="s">
-        <v>107</v>
       </c>
       <c r="Z7" s="31"/>
     </row>
@@ -2414,10 +2403,10 @@
         <v>48</v>
       </c>
       <c r="E11" s="43" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F11" s="44" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H11" s="45" t="s">
         <v>49</v>
@@ -2432,13 +2421,13 @@
         <v>53</v>
       </c>
       <c r="M11" s="48" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N11" s="47" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O11" s="40" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P11" s="41" t="s">
         <v>35</v>
@@ -2450,10 +2439,10 @@
     <row r="15" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="16" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B16" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="F16" s="42" t="s">
         <v>108</v>
-      </c>
-      <c r="F16" s="42" t="s">
-        <v>109</v>
       </c>
       <c r="K16" s="41" t="s">
         <v>51</v>
@@ -2468,10 +2457,10 @@
         <v>81</v>
       </c>
       <c r="U16" s="41" t="s">
+        <v>112</v>
+      </c>
+      <c r="V16" s="41" t="s">
         <v>113</v>
-      </c>
-      <c r="V16" s="41" t="s">
-        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -2508,77 +2497,77 @@
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="63" t="str">
+      <c r="A3" s="73" t="str">
         <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="64"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
-      <c r="L3" s="64"/>
-      <c r="M3" s="64"/>
-      <c r="N3" s="64"/>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="64"/>
-      <c r="S3" s="64"/>
-      <c r="T3" s="64"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="64"/>
-      <c r="W3" s="64"/>
-      <c r="X3" s="64"/>
-      <c r="Y3" s="64"/>
-      <c r="Z3" s="65"/>
+      <c r="B3" s="66"/>
+      <c r="C3" s="66"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="66"/>
+      <c r="J3" s="66"/>
+      <c r="K3" s="66"/>
+      <c r="L3" s="66"/>
+      <c r="M3" s="66"/>
+      <c r="N3" s="66"/>
+      <c r="O3" s="66"/>
+      <c r="P3" s="66"/>
+      <c r="Q3" s="66"/>
+      <c r="R3" s="66"/>
+      <c r="S3" s="66"/>
+      <c r="T3" s="66"/>
+      <c r="U3" s="66"/>
+      <c r="V3" s="66"/>
+      <c r="W3" s="66"/>
+      <c r="X3" s="66"/>
+      <c r="Y3" s="66"/>
+      <c r="Z3" s="67"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="63">
+      <c r="A4" s="73">
         <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="64"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="65"/>
+      <c r="B4" s="66"/>
+      <c r="C4" s="66"/>
+      <c r="D4" s="67"/>
       <c r="E4" s="18"/>
-      <c r="F4" s="63" t="s">
+      <c r="F4" s="73" t="s">
+        <v>90</v>
+      </c>
+      <c r="G4" s="66"/>
+      <c r="H4" s="66"/>
+      <c r="I4" s="66"/>
+      <c r="J4" s="66"/>
+      <c r="K4" s="66"/>
+      <c r="L4" s="66"/>
+      <c r="M4" s="66"/>
+      <c r="N4" s="66"/>
+      <c r="O4" s="66"/>
+      <c r="P4" s="66"/>
+      <c r="Q4" s="66"/>
+      <c r="R4" s="67"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="73" t="s">
         <v>91</v>
       </c>
-      <c r="G4" s="64"/>
-      <c r="H4" s="64"/>
-      <c r="I4" s="64"/>
-      <c r="J4" s="64"/>
-      <c r="K4" s="64"/>
-      <c r="L4" s="64"/>
-      <c r="M4" s="64"/>
-      <c r="N4" s="64"/>
-      <c r="O4" s="64"/>
-      <c r="P4" s="64"/>
-      <c r="Q4" s="64"/>
-      <c r="R4" s="65"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="63" t="s">
+      <c r="U4" s="66"/>
+      <c r="V4" s="66"/>
+      <c r="W4" s="66"/>
+      <c r="X4" s="66"/>
+      <c r="Y4" s="66"/>
+      <c r="Z4" s="67"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A5" s="73" t="s">
         <v>92</v>
       </c>
-      <c r="U4" s="64"/>
-      <c r="V4" s="64"/>
-      <c r="W4" s="64"/>
-      <c r="X4" s="64"/>
-      <c r="Y4" s="64"/>
-      <c r="Z4" s="65"/>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="63" t="s">
-        <v>93</v>
-      </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="65"/>
+      <c r="B5" s="66"/>
+      <c r="C5" s="67"/>
       <c r="D5" s="20">
         <f>[1]Summary!R7</f>
         <v>0</v>
@@ -2635,62 +2624,62 @@
     </row>
     <row r="6" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="74" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="67"/>
+      <c r="D6" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="B6" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="65"/>
-      <c r="D6" s="25" t="s">
+      <c r="E6" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="E6" s="26" t="s">
+      <c r="F6" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="G6" s="75" t="s">
         <v>97</v>
       </c>
-      <c r="G6" s="67" t="s">
+      <c r="H6" s="66"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="75" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="66"/>
+      <c r="L6" s="67"/>
+      <c r="M6" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="H6" s="64"/>
-      <c r="I6" s="65"/>
-      <c r="J6" s="67" t="s">
-        <v>38</v>
-      </c>
-      <c r="K6" s="64"/>
-      <c r="L6" s="65"/>
-      <c r="M6" s="28" t="s">
+      <c r="N6" s="29" t="s">
         <v>99</v>
       </c>
-      <c r="N6" s="29" t="s">
+      <c r="O6" s="30" t="s">
         <v>100</v>
       </c>
-      <c r="O6" s="30" t="s">
+      <c r="P6" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="P6" s="31" t="s">
+      <c r="Q6" s="32" t="s">
         <v>102</v>
-      </c>
-      <c r="Q6" s="32" t="s">
-        <v>103</v>
       </c>
       <c r="R6" s="27" t="s">
         <v>43</v>
       </c>
       <c r="S6" s="33"/>
-      <c r="T6" s="68" t="s">
+      <c r="T6" s="63" t="s">
+        <v>103</v>
+      </c>
+      <c r="U6" s="66"/>
+      <c r="V6" s="67"/>
+      <c r="W6" s="63" t="s">
         <v>104</v>
       </c>
-      <c r="U6" s="64"/>
-      <c r="V6" s="65"/>
-      <c r="W6" s="68" t="s">
-        <v>105</v>
-      </c>
-      <c r="X6" s="64"/>
-      <c r="Y6" s="65"/>
+      <c r="X6" s="66"/>
+      <c r="Y6" s="67"/>
       <c r="Z6" s="31" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.35">
@@ -2708,19 +2697,19 @@
         <v>55</v>
       </c>
       <c r="H7" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="I7" s="30" t="s">
         <v>106</v>
-      </c>
-      <c r="I7" s="30" t="s">
-        <v>107</v>
       </c>
       <c r="J7" s="30" t="s">
         <v>55</v>
       </c>
       <c r="K7" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="L7" s="30" t="s">
         <v>106</v>
-      </c>
-      <c r="L7" s="30" t="s">
-        <v>107</v>
       </c>
       <c r="M7" s="30" t="s">
         <v>55</v>
@@ -2739,19 +2728,19 @@
         <v>55</v>
       </c>
       <c r="U7" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="V7" s="30" t="s">
         <v>106</v>
-      </c>
-      <c r="V7" s="30" t="s">
-        <v>107</v>
       </c>
       <c r="W7" s="30" t="s">
         <v>55</v>
       </c>
       <c r="X7" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="Y7" s="30" t="s">
         <v>106</v>
-      </c>
-      <c r="Y7" s="30" t="s">
-        <v>107</v>
       </c>
       <c r="Z7" s="31"/>
     </row>
@@ -2774,10 +2763,10 @@
         <v>48</v>
       </c>
       <c r="E11" s="43" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F11" s="44" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H11" s="45" t="s">
         <v>49</v>
@@ -2792,13 +2781,13 @@
         <v>53</v>
       </c>
       <c r="M11" s="48" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N11" s="47" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O11" s="40" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P11" s="41" t="s">
         <v>35</v>
@@ -2836,62 +2825,62 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A1" s="68" t="str">
+      <c r="A1" s="63" t="str">
         <f>+[1]Summary!A2</f>
         <v>Name of the Line: 220KV DC AL59 line from Neemuch - Chanderiya + 132KV DC ACSS Line from Chanderiya to Hindustan Zinc</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-      <c r="P1" s="73"/>
-      <c r="Q1" s="73"/>
-      <c r="R1" s="73"/>
-      <c r="S1" s="73"/>
-      <c r="T1" s="73"/>
-      <c r="U1" s="73"/>
-      <c r="V1" s="73"/>
-      <c r="W1" s="73"/>
-      <c r="X1" s="73"/>
-      <c r="Y1" s="73"/>
-      <c r="Z1" s="73"/>
-      <c r="AA1" s="73"/>
-      <c r="AB1" s="73"/>
-      <c r="AC1" s="73"/>
-      <c r="AD1" s="73"/>
-      <c r="AE1" s="73"/>
-      <c r="AF1" s="73"/>
-      <c r="AG1" s="73"/>
-      <c r="AH1" s="73"/>
-      <c r="AI1" s="73"/>
-      <c r="AJ1" s="73"/>
-      <c r="AK1" s="73"/>
-      <c r="AL1" s="64"/>
-      <c r="AM1" s="64"/>
-      <c r="AN1" s="64"/>
-      <c r="AO1" s="64"/>
-      <c r="AP1" s="64"/>
-      <c r="AQ1" s="73"/>
-      <c r="AR1" s="73"/>
-      <c r="AS1" s="73"/>
-      <c r="AT1" s="73"/>
-      <c r="AU1" s="73"/>
-      <c r="AV1" s="73"/>
-      <c r="AW1" s="73"/>
-      <c r="AX1" s="73"/>
-      <c r="AY1" s="73"/>
-      <c r="AZ1" s="73"/>
-      <c r="BA1" s="74"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
+      <c r="N1" s="65"/>
+      <c r="O1" s="65"/>
+      <c r="P1" s="65"/>
+      <c r="Q1" s="65"/>
+      <c r="R1" s="65"/>
+      <c r="S1" s="65"/>
+      <c r="T1" s="65"/>
+      <c r="U1" s="65"/>
+      <c r="V1" s="65"/>
+      <c r="W1" s="65"/>
+      <c r="X1" s="65"/>
+      <c r="Y1" s="65"/>
+      <c r="Z1" s="65"/>
+      <c r="AA1" s="65"/>
+      <c r="AB1" s="65"/>
+      <c r="AC1" s="65"/>
+      <c r="AD1" s="65"/>
+      <c r="AE1" s="65"/>
+      <c r="AF1" s="65"/>
+      <c r="AG1" s="65"/>
+      <c r="AH1" s="65"/>
+      <c r="AI1" s="65"/>
+      <c r="AJ1" s="65"/>
+      <c r="AK1" s="65"/>
+      <c r="AL1" s="66"/>
+      <c r="AM1" s="66"/>
+      <c r="AN1" s="66"/>
+      <c r="AO1" s="66"/>
+      <c r="AP1" s="66"/>
+      <c r="AQ1" s="65"/>
+      <c r="AR1" s="65"/>
+      <c r="AS1" s="65"/>
+      <c r="AT1" s="65"/>
+      <c r="AU1" s="65"/>
+      <c r="AV1" s="65"/>
+      <c r="AW1" s="65"/>
+      <c r="AX1" s="65"/>
+      <c r="AY1" s="65"/>
+      <c r="AZ1" s="65"/>
+      <c r="BA1" s="64"/>
     </row>
     <row r="2" spans="1:53" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -2899,138 +2888,138 @@
       </c>
     </row>
     <row r="3" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A3" s="68" t="str">
+      <c r="A3" s="63" t="str">
         <f>+[1]Summary!A5</f>
         <v>Progress of 220kV Line</v>
       </c>
-      <c r="B3" s="73"/>
-      <c r="C3" s="73"/>
-      <c r="D3" s="73"/>
-      <c r="E3" s="73"/>
-      <c r="F3" s="73"/>
-      <c r="G3" s="73"/>
-      <c r="H3" s="73"/>
-      <c r="I3" s="73"/>
-      <c r="J3" s="73"/>
-      <c r="K3" s="73"/>
-      <c r="L3" s="73"/>
-      <c r="M3" s="73"/>
-      <c r="N3" s="73"/>
-      <c r="O3" s="73"/>
-      <c r="P3" s="73"/>
-      <c r="Q3" s="73"/>
-      <c r="R3" s="73"/>
-      <c r="S3" s="73"/>
-      <c r="T3" s="73"/>
-      <c r="U3" s="73"/>
-      <c r="V3" s="73"/>
-      <c r="W3" s="73"/>
-      <c r="X3" s="73"/>
-      <c r="Y3" s="73"/>
-      <c r="Z3" s="73"/>
-      <c r="AA3" s="73"/>
-      <c r="AB3" s="73"/>
-      <c r="AC3" s="73"/>
-      <c r="AD3" s="73"/>
-      <c r="AE3" s="73"/>
-      <c r="AF3" s="73"/>
-      <c r="AG3" s="73"/>
-      <c r="AH3" s="73"/>
-      <c r="AI3" s="73"/>
-      <c r="AJ3" s="73"/>
-      <c r="AK3" s="73"/>
-      <c r="AL3" s="64"/>
-      <c r="AM3" s="64"/>
-      <c r="AN3" s="64"/>
-      <c r="AO3" s="64"/>
-      <c r="AP3" s="64"/>
-      <c r="AQ3" s="73"/>
-      <c r="AR3" s="73"/>
-      <c r="AS3" s="73"/>
-      <c r="AT3" s="73"/>
-      <c r="AU3" s="73"/>
-      <c r="AV3" s="73"/>
-      <c r="AW3" s="73"/>
-      <c r="AX3" s="73"/>
-      <c r="AY3" s="73"/>
-      <c r="AZ3" s="73"/>
-      <c r="BA3" s="74"/>
+      <c r="B3" s="65"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="65"/>
+      <c r="I3" s="65"/>
+      <c r="J3" s="65"/>
+      <c r="K3" s="65"/>
+      <c r="L3" s="65"/>
+      <c r="M3" s="65"/>
+      <c r="N3" s="65"/>
+      <c r="O3" s="65"/>
+      <c r="P3" s="65"/>
+      <c r="Q3" s="65"/>
+      <c r="R3" s="65"/>
+      <c r="S3" s="65"/>
+      <c r="T3" s="65"/>
+      <c r="U3" s="65"/>
+      <c r="V3" s="65"/>
+      <c r="W3" s="65"/>
+      <c r="X3" s="65"/>
+      <c r="Y3" s="65"/>
+      <c r="Z3" s="65"/>
+      <c r="AA3" s="65"/>
+      <c r="AB3" s="65"/>
+      <c r="AC3" s="65"/>
+      <c r="AD3" s="65"/>
+      <c r="AE3" s="65"/>
+      <c r="AF3" s="65"/>
+      <c r="AG3" s="65"/>
+      <c r="AH3" s="65"/>
+      <c r="AI3" s="65"/>
+      <c r="AJ3" s="65"/>
+      <c r="AK3" s="65"/>
+      <c r="AL3" s="66"/>
+      <c r="AM3" s="66"/>
+      <c r="AN3" s="66"/>
+      <c r="AO3" s="66"/>
+      <c r="AP3" s="66"/>
+      <c r="AQ3" s="65"/>
+      <c r="AR3" s="65"/>
+      <c r="AS3" s="65"/>
+      <c r="AT3" s="65"/>
+      <c r="AU3" s="65"/>
+      <c r="AV3" s="65"/>
+      <c r="AW3" s="65"/>
+      <c r="AX3" s="65"/>
+      <c r="AY3" s="65"/>
+      <c r="AZ3" s="65"/>
+      <c r="BA3" s="64"/>
     </row>
     <row r="4" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="63" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" s="65"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="65"/>
+      <c r="I4" s="65"/>
+      <c r="J4" s="65"/>
+      <c r="K4" s="65"/>
+      <c r="L4" s="65"/>
+      <c r="M4" s="65"/>
+      <c r="N4" s="65"/>
+      <c r="O4" s="65"/>
+      <c r="P4" s="65"/>
+      <c r="Q4" s="65"/>
+      <c r="R4" s="65"/>
+      <c r="S4" s="64"/>
+      <c r="T4" s="63" t="s">
         <v>115</v>
       </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="73"/>
-      <c r="D4" s="73"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="73"/>
-      <c r="I4" s="73"/>
-      <c r="J4" s="73"/>
-      <c r="K4" s="73"/>
-      <c r="L4" s="73"/>
-      <c r="M4" s="73"/>
-      <c r="N4" s="73"/>
-      <c r="O4" s="73"/>
-      <c r="P4" s="73"/>
-      <c r="Q4" s="73"/>
-      <c r="R4" s="73"/>
-      <c r="S4" s="74"/>
-      <c r="T4" s="68" t="s">
+      <c r="U4" s="65"/>
+      <c r="V4" s="65"/>
+      <c r="W4" s="65"/>
+      <c r="X4" s="65"/>
+      <c r="Y4" s="65"/>
+      <c r="Z4" s="65"/>
+      <c r="AA4" s="65"/>
+      <c r="AB4" s="65"/>
+      <c r="AC4" s="65"/>
+      <c r="AD4" s="65"/>
+      <c r="AE4" s="65"/>
+      <c r="AF4" s="65"/>
+      <c r="AG4" s="65"/>
+      <c r="AH4" s="65"/>
+      <c r="AI4" s="65"/>
+      <c r="AJ4" s="65"/>
+      <c r="AK4" s="64"/>
+      <c r="AL4" s="63" t="s">
         <v>116</v>
       </c>
-      <c r="U4" s="73"/>
-      <c r="V4" s="73"/>
-      <c r="W4" s="73"/>
-      <c r="X4" s="73"/>
-      <c r="Y4" s="73"/>
-      <c r="Z4" s="73"/>
-      <c r="AA4" s="73"/>
-      <c r="AB4" s="73"/>
-      <c r="AC4" s="73"/>
-      <c r="AD4" s="73"/>
-      <c r="AE4" s="73"/>
-      <c r="AF4" s="73"/>
-      <c r="AG4" s="73"/>
-      <c r="AH4" s="73"/>
-      <c r="AI4" s="73"/>
-      <c r="AJ4" s="73"/>
-      <c r="AK4" s="74"/>
-      <c r="AL4" s="68" t="s">
+      <c r="AM4" s="66"/>
+      <c r="AN4" s="66"/>
+      <c r="AO4" s="66"/>
+      <c r="AP4" s="67"/>
+      <c r="AQ4" s="63" t="s">
+        <v>2</v>
+      </c>
+      <c r="AR4" s="65"/>
+      <c r="AS4" s="65"/>
+      <c r="AT4" s="64"/>
+      <c r="AU4" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="AM4" s="64"/>
-      <c r="AN4" s="64"/>
-      <c r="AO4" s="64"/>
-      <c r="AP4" s="65"/>
-      <c r="AQ4" s="68" t="s">
-        <v>2</v>
-      </c>
-      <c r="AR4" s="73"/>
-      <c r="AS4" s="73"/>
-      <c r="AT4" s="74"/>
-      <c r="AU4" s="27" t="s">
+      <c r="AV4" s="63" t="s">
         <v>118</v>
       </c>
-      <c r="AV4" s="68" t="s">
+      <c r="AW4" s="65"/>
+      <c r="AX4" s="65"/>
+      <c r="AY4" s="65"/>
+      <c r="AZ4" s="64"/>
+      <c r="BA4" s="27" t="s">
         <v>119</v>
-      </c>
-      <c r="AW4" s="73"/>
-      <c r="AX4" s="73"/>
-      <c r="AY4" s="73"/>
-      <c r="AZ4" s="74"/>
-      <c r="BA4" s="27" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:53" ht="58.5" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A5" s="31" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B5" s="31" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C5" s="31" t="s">
         <v>78</v>
@@ -3038,115 +3027,115 @@
       <c r="D5" s="50"/>
       <c r="E5" s="50"/>
       <c r="F5" s="50"/>
-      <c r="G5" s="69" t="s">
+      <c r="G5" s="68" t="s">
         <v>82</v>
       </c>
-      <c r="H5" s="70"/>
-      <c r="I5" s="70"/>
-      <c r="J5" s="71"/>
-      <c r="K5" s="69" t="s">
+      <c r="H5" s="69"/>
+      <c r="I5" s="69"/>
+      <c r="J5" s="70"/>
+      <c r="K5" s="68" t="s">
+        <v>121</v>
+      </c>
+      <c r="L5" s="69"/>
+      <c r="M5" s="69"/>
+      <c r="N5" s="70"/>
+      <c r="O5" s="71" t="s">
         <v>122</v>
       </c>
-      <c r="L5" s="70"/>
-      <c r="M5" s="70"/>
-      <c r="N5" s="71"/>
-      <c r="O5" s="72" t="s">
+      <c r="P5" s="65"/>
+      <c r="Q5" s="65"/>
+      <c r="R5" s="64"/>
+      <c r="S5" s="51" t="s">
         <v>123</v>
-      </c>
-      <c r="P5" s="73"/>
-      <c r="Q5" s="73"/>
-      <c r="R5" s="74"/>
-      <c r="S5" s="51" t="s">
-        <v>124</v>
       </c>
       <c r="T5" s="27" t="s">
         <v>79</v>
       </c>
       <c r="U5" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="V5" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V5" s="68" t="s">
+      <c r="W5" s="65"/>
+      <c r="X5" s="64"/>
+      <c r="Y5" s="52" t="s">
         <v>126</v>
       </c>
-      <c r="W5" s="73"/>
-      <c r="X5" s="74"/>
-      <c r="Y5" s="52" t="s">
+      <c r="Z5" s="52" t="s">
         <v>127</v>
       </c>
-      <c r="Z5" s="52" t="s">
+      <c r="AA5" s="52" t="s">
         <v>128</v>
       </c>
-      <c r="AA5" s="52" t="s">
+      <c r="AB5" s="52" t="s">
         <v>129</v>
       </c>
-      <c r="AB5" s="52" t="s">
+      <c r="AC5" s="52" t="s">
         <v>130</v>
       </c>
-      <c r="AC5" s="52" t="s">
+      <c r="AD5" s="52" t="s">
         <v>131</v>
       </c>
-      <c r="AD5" s="52" t="s">
+      <c r="AE5" s="53" t="s">
         <v>132</v>
       </c>
-      <c r="AE5" s="53" t="s">
+      <c r="AF5" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="AF5" s="27" t="s">
+      <c r="AG5" s="72" t="s">
         <v>134</v>
       </c>
-      <c r="AG5" s="75" t="s">
+      <c r="AH5" s="64"/>
+      <c r="AI5" s="63" t="s">
         <v>135</v>
       </c>
-      <c r="AH5" s="74"/>
-      <c r="AI5" s="68" t="s">
+      <c r="AJ5" s="64"/>
+      <c r="AK5" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="AL5" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="AJ5" s="74"/>
-      <c r="AK5" s="27" t="s">
-        <v>102</v>
-      </c>
-      <c r="AL5" s="27" t="s">
+      <c r="AM5" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AM5" s="27" t="s">
-        <v>138</v>
-      </c>
       <c r="AN5" s="54" t="s">
+        <v>105</v>
+      </c>
+      <c r="AO5" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AO5" s="54" t="s">
-        <v>107</v>
-      </c>
       <c r="AP5" s="27" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AQ5" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AR5" s="54" t="s">
+        <v>105</v>
+      </c>
+      <c r="AS5" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AS5" s="54" t="s">
-        <v>107</v>
-      </c>
       <c r="AT5" s="27" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AU5" s="53"/>
       <c r="AV5" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AW5" s="54" t="s">
+        <v>105</v>
+      </c>
+      <c r="AX5" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AX5" s="54" t="s">
-        <v>107</v>
-      </c>
       <c r="AY5" s="55" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AZ5" s="27" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="BA5" s="53"/>
     </row>
@@ -3158,54 +3147,54 @@
       <c r="E6" s="29"/>
       <c r="F6" s="29"/>
       <c r="G6" s="56" t="s">
+        <v>139</v>
+      </c>
+      <c r="H6" s="31" t="s">
         <v>140</v>
       </c>
-      <c r="H6" s="31" t="s">
+      <c r="I6" s="31" t="s">
         <v>141</v>
       </c>
-      <c r="I6" s="31" t="s">
+      <c r="J6" s="57" t="s">
         <v>142</v>
       </c>
-      <c r="J6" s="57" t="s">
+      <c r="K6" s="56" t="s">
+        <v>139</v>
+      </c>
+      <c r="L6" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M6" s="31" t="s">
+        <v>141</v>
+      </c>
+      <c r="N6" s="57" t="s">
+        <v>142</v>
+      </c>
+      <c r="O6" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="K6" s="56" t="s">
-        <v>140</v>
-      </c>
-      <c r="L6" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="M6" s="31" t="s">
-        <v>142</v>
-      </c>
-      <c r="N6" s="57" t="s">
-        <v>143</v>
-      </c>
-      <c r="O6" s="54" t="s">
+      <c r="P6" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="P6" s="54" t="s">
+      <c r="Q6" s="54" t="s">
         <v>145</v>
       </c>
-      <c r="Q6" s="54" t="s">
+      <c r="R6" s="54" t="s">
         <v>146</v>
       </c>
-      <c r="R6" s="54" t="s">
+      <c r="S6" s="58" t="s">
         <v>147</v>
-      </c>
-      <c r="S6" s="58" t="s">
-        <v>148</v>
       </c>
       <c r="T6" s="36"/>
       <c r="U6" s="27"/>
       <c r="V6" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="W6" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="W6" s="27" t="s">
-        <v>150</v>
-      </c>
       <c r="X6" s="27" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="Y6" s="53"/>
       <c r="Z6" s="53"/>
@@ -3216,16 +3205,16 @@
       <c r="AE6" s="36"/>
       <c r="AF6" s="36"/>
       <c r="AG6" s="54" t="s">
+        <v>105</v>
+      </c>
+      <c r="AH6" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AH6" s="54" t="s">
-        <v>107</v>
-      </c>
       <c r="AI6" s="54" t="s">
+        <v>105</v>
+      </c>
+      <c r="AJ6" s="54" t="s">
         <v>106</v>
-      </c>
-      <c r="AJ6" s="54" t="s">
-        <v>107</v>
       </c>
       <c r="AK6" s="36"/>
       <c r="AL6" s="36"/>
@@ -3318,138 +3307,138 @@
       </c>
     </row>
     <row r="3" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A3" s="68" t="str">
+      <c r="A3" s="63" t="str">
         <f>+[1]Summary!A5</f>
         <v>Progress of 220kV Line</v>
       </c>
-      <c r="B3" s="73"/>
-      <c r="C3" s="73"/>
-      <c r="D3" s="73"/>
-      <c r="E3" s="73"/>
-      <c r="F3" s="73"/>
-      <c r="G3" s="73"/>
-      <c r="H3" s="73"/>
-      <c r="I3" s="73"/>
-      <c r="J3" s="73"/>
-      <c r="K3" s="73"/>
-      <c r="L3" s="73"/>
-      <c r="M3" s="73"/>
-      <c r="N3" s="73"/>
-      <c r="O3" s="73"/>
-      <c r="P3" s="73"/>
-      <c r="Q3" s="73"/>
-      <c r="R3" s="73"/>
-      <c r="S3" s="73"/>
-      <c r="T3" s="73"/>
-      <c r="U3" s="73"/>
-      <c r="V3" s="73"/>
-      <c r="W3" s="73"/>
-      <c r="X3" s="73"/>
-      <c r="Y3" s="73"/>
-      <c r="Z3" s="73"/>
-      <c r="AA3" s="73"/>
-      <c r="AB3" s="73"/>
-      <c r="AC3" s="73"/>
-      <c r="AD3" s="73"/>
-      <c r="AE3" s="73"/>
-      <c r="AF3" s="73"/>
-      <c r="AG3" s="73"/>
-      <c r="AH3" s="73"/>
-      <c r="AI3" s="73"/>
-      <c r="AJ3" s="73"/>
-      <c r="AK3" s="73"/>
-      <c r="AL3" s="64"/>
-      <c r="AM3" s="64"/>
-      <c r="AN3" s="64"/>
-      <c r="AO3" s="64"/>
-      <c r="AP3" s="64"/>
-      <c r="AQ3" s="73"/>
-      <c r="AR3" s="73"/>
-      <c r="AS3" s="73"/>
-      <c r="AT3" s="73"/>
-      <c r="AU3" s="73"/>
-      <c r="AV3" s="73"/>
-      <c r="AW3" s="73"/>
-      <c r="AX3" s="73"/>
-      <c r="AY3" s="73"/>
-      <c r="AZ3" s="73"/>
-      <c r="BA3" s="74"/>
+      <c r="B3" s="65"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="65"/>
+      <c r="I3" s="65"/>
+      <c r="J3" s="65"/>
+      <c r="K3" s="65"/>
+      <c r="L3" s="65"/>
+      <c r="M3" s="65"/>
+      <c r="N3" s="65"/>
+      <c r="O3" s="65"/>
+      <c r="P3" s="65"/>
+      <c r="Q3" s="65"/>
+      <c r="R3" s="65"/>
+      <c r="S3" s="65"/>
+      <c r="T3" s="65"/>
+      <c r="U3" s="65"/>
+      <c r="V3" s="65"/>
+      <c r="W3" s="65"/>
+      <c r="X3" s="65"/>
+      <c r="Y3" s="65"/>
+      <c r="Z3" s="65"/>
+      <c r="AA3" s="65"/>
+      <c r="AB3" s="65"/>
+      <c r="AC3" s="65"/>
+      <c r="AD3" s="65"/>
+      <c r="AE3" s="65"/>
+      <c r="AF3" s="65"/>
+      <c r="AG3" s="65"/>
+      <c r="AH3" s="65"/>
+      <c r="AI3" s="65"/>
+      <c r="AJ3" s="65"/>
+      <c r="AK3" s="65"/>
+      <c r="AL3" s="66"/>
+      <c r="AM3" s="66"/>
+      <c r="AN3" s="66"/>
+      <c r="AO3" s="66"/>
+      <c r="AP3" s="66"/>
+      <c r="AQ3" s="65"/>
+      <c r="AR3" s="65"/>
+      <c r="AS3" s="65"/>
+      <c r="AT3" s="65"/>
+      <c r="AU3" s="65"/>
+      <c r="AV3" s="65"/>
+      <c r="AW3" s="65"/>
+      <c r="AX3" s="65"/>
+      <c r="AY3" s="65"/>
+      <c r="AZ3" s="65"/>
+      <c r="BA3" s="64"/>
     </row>
     <row r="4" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="63" t="s">
+        <v>114</v>
+      </c>
+      <c r="B4" s="65"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="65"/>
+      <c r="I4" s="65"/>
+      <c r="J4" s="65"/>
+      <c r="K4" s="65"/>
+      <c r="L4" s="65"/>
+      <c r="M4" s="65"/>
+      <c r="N4" s="65"/>
+      <c r="O4" s="65"/>
+      <c r="P4" s="65"/>
+      <c r="Q4" s="65"/>
+      <c r="R4" s="65"/>
+      <c r="S4" s="64"/>
+      <c r="T4" s="63" t="s">
         <v>115</v>
       </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="73"/>
-      <c r="D4" s="73"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="73"/>
-      <c r="I4" s="73"/>
-      <c r="J4" s="73"/>
-      <c r="K4" s="73"/>
-      <c r="L4" s="73"/>
-      <c r="M4" s="73"/>
-      <c r="N4" s="73"/>
-      <c r="O4" s="73"/>
-      <c r="P4" s="73"/>
-      <c r="Q4" s="73"/>
-      <c r="R4" s="73"/>
-      <c r="S4" s="74"/>
-      <c r="T4" s="68" t="s">
+      <c r="U4" s="65"/>
+      <c r="V4" s="65"/>
+      <c r="W4" s="65"/>
+      <c r="X4" s="65"/>
+      <c r="Y4" s="65"/>
+      <c r="Z4" s="65"/>
+      <c r="AA4" s="65"/>
+      <c r="AB4" s="65"/>
+      <c r="AC4" s="65"/>
+      <c r="AD4" s="65"/>
+      <c r="AE4" s="65"/>
+      <c r="AF4" s="65"/>
+      <c r="AG4" s="65"/>
+      <c r="AH4" s="65"/>
+      <c r="AI4" s="65"/>
+      <c r="AJ4" s="65"/>
+      <c r="AK4" s="64"/>
+      <c r="AL4" s="63" t="s">
         <v>116</v>
       </c>
-      <c r="U4" s="73"/>
-      <c r="V4" s="73"/>
-      <c r="W4" s="73"/>
-      <c r="X4" s="73"/>
-      <c r="Y4" s="73"/>
-      <c r="Z4" s="73"/>
-      <c r="AA4" s="73"/>
-      <c r="AB4" s="73"/>
-      <c r="AC4" s="73"/>
-      <c r="AD4" s="73"/>
-      <c r="AE4" s="73"/>
-      <c r="AF4" s="73"/>
-      <c r="AG4" s="73"/>
-      <c r="AH4" s="73"/>
-      <c r="AI4" s="73"/>
-      <c r="AJ4" s="73"/>
-      <c r="AK4" s="74"/>
-      <c r="AL4" s="68" t="s">
+      <c r="AM4" s="66"/>
+      <c r="AN4" s="66"/>
+      <c r="AO4" s="66"/>
+      <c r="AP4" s="67"/>
+      <c r="AQ4" s="63" t="s">
+        <v>2</v>
+      </c>
+      <c r="AR4" s="65"/>
+      <c r="AS4" s="65"/>
+      <c r="AT4" s="64"/>
+      <c r="AU4" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="AM4" s="64"/>
-      <c r="AN4" s="64"/>
-      <c r="AO4" s="64"/>
-      <c r="AP4" s="65"/>
-      <c r="AQ4" s="68" t="s">
-        <v>2</v>
-      </c>
-      <c r="AR4" s="73"/>
-      <c r="AS4" s="73"/>
-      <c r="AT4" s="74"/>
-      <c r="AU4" s="27" t="s">
+      <c r="AV4" s="63" t="s">
         <v>118</v>
       </c>
-      <c r="AV4" s="68" t="s">
+      <c r="AW4" s="65"/>
+      <c r="AX4" s="65"/>
+      <c r="AY4" s="65"/>
+      <c r="AZ4" s="64"/>
+      <c r="BA4" s="27" t="s">
         <v>119</v>
-      </c>
-      <c r="AW4" s="73"/>
-      <c r="AX4" s="73"/>
-      <c r="AY4" s="73"/>
-      <c r="AZ4" s="74"/>
-      <c r="BA4" s="27" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:53" ht="58.5" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A5" s="31" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B5" s="31" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C5" s="31" t="s">
         <v>78</v>
@@ -3457,115 +3446,115 @@
       <c r="D5" s="50"/>
       <c r="E5" s="50"/>
       <c r="F5" s="50"/>
-      <c r="G5" s="69" t="s">
+      <c r="G5" s="68" t="s">
         <v>82</v>
       </c>
-      <c r="H5" s="70"/>
-      <c r="I5" s="70"/>
-      <c r="J5" s="71"/>
-      <c r="K5" s="69" t="s">
+      <c r="H5" s="69"/>
+      <c r="I5" s="69"/>
+      <c r="J5" s="70"/>
+      <c r="K5" s="68" t="s">
+        <v>121</v>
+      </c>
+      <c r="L5" s="69"/>
+      <c r="M5" s="69"/>
+      <c r="N5" s="70"/>
+      <c r="O5" s="71" t="s">
         <v>122</v>
       </c>
-      <c r="L5" s="70"/>
-      <c r="M5" s="70"/>
-      <c r="N5" s="71"/>
-      <c r="O5" s="72" t="s">
+      <c r="P5" s="65"/>
+      <c r="Q5" s="65"/>
+      <c r="R5" s="64"/>
+      <c r="S5" s="51" t="s">
         <v>123</v>
-      </c>
-      <c r="P5" s="73"/>
-      <c r="Q5" s="73"/>
-      <c r="R5" s="74"/>
-      <c r="S5" s="51" t="s">
-        <v>124</v>
       </c>
       <c r="T5" s="27" t="s">
         <v>79</v>
       </c>
       <c r="U5" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="V5" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="V5" s="68" t="s">
+      <c r="W5" s="65"/>
+      <c r="X5" s="64"/>
+      <c r="Y5" s="52" t="s">
         <v>126</v>
       </c>
-      <c r="W5" s="73"/>
-      <c r="X5" s="74"/>
-      <c r="Y5" s="52" t="s">
+      <c r="Z5" s="52" t="s">
         <v>127</v>
       </c>
-      <c r="Z5" s="52" t="s">
+      <c r="AA5" s="52" t="s">
         <v>128</v>
       </c>
-      <c r="AA5" s="52" t="s">
+      <c r="AB5" s="52" t="s">
         <v>129</v>
       </c>
-      <c r="AB5" s="52" t="s">
+      <c r="AC5" s="52" t="s">
         <v>130</v>
       </c>
-      <c r="AC5" s="52" t="s">
+      <c r="AD5" s="52" t="s">
         <v>131</v>
       </c>
-      <c r="AD5" s="52" t="s">
+      <c r="AE5" s="53" t="s">
         <v>132</v>
       </c>
-      <c r="AE5" s="53" t="s">
+      <c r="AF5" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="AF5" s="27" t="s">
+      <c r="AG5" s="72" t="s">
         <v>134</v>
       </c>
-      <c r="AG5" s="75" t="s">
+      <c r="AH5" s="64"/>
+      <c r="AI5" s="63" t="s">
         <v>135</v>
       </c>
-      <c r="AH5" s="74"/>
-      <c r="AI5" s="68" t="s">
+      <c r="AJ5" s="64"/>
+      <c r="AK5" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="AL5" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="AJ5" s="74"/>
-      <c r="AK5" s="27" t="s">
-        <v>102</v>
-      </c>
-      <c r="AL5" s="27" t="s">
+      <c r="AM5" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AM5" s="27" t="s">
-        <v>138</v>
-      </c>
       <c r="AN5" s="54" t="s">
+        <v>105</v>
+      </c>
+      <c r="AO5" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AO5" s="54" t="s">
-        <v>107</v>
-      </c>
       <c r="AP5" s="27" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AQ5" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AR5" s="54" t="s">
+        <v>105</v>
+      </c>
+      <c r="AS5" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AS5" s="54" t="s">
-        <v>107</v>
-      </c>
       <c r="AT5" s="27" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AU5" s="53"/>
       <c r="AV5" s="27" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AW5" s="54" t="s">
+        <v>105</v>
+      </c>
+      <c r="AX5" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AX5" s="54" t="s">
-        <v>107</v>
-      </c>
       <c r="AY5" s="55" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AZ5" s="27" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="BA5" s="53"/>
     </row>
@@ -3577,54 +3566,54 @@
       <c r="E6" s="29"/>
       <c r="F6" s="29"/>
       <c r="G6" s="56" t="s">
+        <v>139</v>
+      </c>
+      <c r="H6" s="31" t="s">
         <v>140</v>
       </c>
-      <c r="H6" s="31" t="s">
+      <c r="I6" s="31" t="s">
         <v>141</v>
       </c>
-      <c r="I6" s="31" t="s">
+      <c r="J6" s="57" t="s">
         <v>142</v>
       </c>
-      <c r="J6" s="57" t="s">
+      <c r="K6" s="56" t="s">
+        <v>139</v>
+      </c>
+      <c r="L6" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M6" s="31" t="s">
+        <v>141</v>
+      </c>
+      <c r="N6" s="57" t="s">
+        <v>142</v>
+      </c>
+      <c r="O6" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="K6" s="56" t="s">
-        <v>140</v>
-      </c>
-      <c r="L6" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="M6" s="31" t="s">
-        <v>142</v>
-      </c>
-      <c r="N6" s="57" t="s">
-        <v>143</v>
-      </c>
-      <c r="O6" s="54" t="s">
+      <c r="P6" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="P6" s="54" t="s">
+      <c r="Q6" s="54" t="s">
         <v>145</v>
       </c>
-      <c r="Q6" s="54" t="s">
+      <c r="R6" s="54" t="s">
         <v>146</v>
       </c>
-      <c r="R6" s="54" t="s">
+      <c r="S6" s="58" t="s">
         <v>147</v>
-      </c>
-      <c r="S6" s="58" t="s">
-        <v>148</v>
       </c>
       <c r="T6" s="36"/>
       <c r="U6" s="27"/>
       <c r="V6" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="W6" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="W6" s="27" t="s">
-        <v>150</v>
-      </c>
       <c r="X6" s="27" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="Y6" s="53"/>
       <c r="Z6" s="53"/>
@@ -3635,16 +3624,16 @@
       <c r="AE6" s="36"/>
       <c r="AF6" s="36"/>
       <c r="AG6" s="54" t="s">
+        <v>105</v>
+      </c>
+      <c r="AH6" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AH6" s="54" t="s">
-        <v>107</v>
-      </c>
       <c r="AI6" s="54" t="s">
+        <v>105</v>
+      </c>
+      <c r="AJ6" s="54" t="s">
         <v>106</v>
-      </c>
-      <c r="AJ6" s="54" t="s">
-        <v>107</v>
       </c>
       <c r="AK6" s="36"/>
       <c r="AL6" s="36"/>
@@ -3739,18 +3728,18 @@
       <c r="B3" s="79" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="65"/>
+      <c r="C3" s="66"/>
+      <c r="D3" s="67"/>
       <c r="E3" s="79" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="64"/>
-      <c r="G3" s="65"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="67"/>
       <c r="H3" s="79" t="s">
         <v>38</v>
       </c>
-      <c r="I3" s="64"/>
-      <c r="J3" s="65"/>
+      <c r="I3" s="66"/>
+      <c r="J3" s="67"/>
       <c r="K3" s="78" t="s">
         <v>75</v>
       </c>

</xml_diff>

<commit_message>
Auto pipeline update 2026-04-02 12:10:22
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{107148DA-437E-400F-B495-5E88B165F41E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3742A297-9DD6-461F-BF71-EB403A6381F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" activeTab="5" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" activeTab="4" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet Names Check" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,7 @@
   </sheets>
   <externalReferences>
     <externalReference r:id="rId10"/>
+    <externalReference r:id="rId11"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="179">
   <si>
     <t>Project Code</t>
   </si>
@@ -500,6 +501,96 @@
   </si>
   <si>
     <t>M20 (1:1.5:3) (m3)</t>
+  </si>
+  <si>
+    <t>pack Washar</t>
+  </si>
+  <si>
+    <t>Total Tower Weight</t>
+  </si>
+  <si>
+    <t>Total Stub Weight</t>
+  </si>
+  <si>
+    <t>Deviation of Angle</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>Cement Required</t>
+  </si>
+  <si>
+    <t>Total Steel (Kgs) per Tower</t>
+  </si>
+  <si>
+    <t>Fnd Status
+(C/WIP)</t>
+  </si>
+  <si>
+    <t>Manual Checklist</t>
+  </si>
+  <si>
+    <t>Earthing Status
+C/WIP</t>
+  </si>
+  <si>
+    <t>Earthing Type</t>
+  </si>
+  <si>
+    <t>S/C</t>
+  </si>
+  <si>
+    <t>Erection Status
+C/WIP</t>
+  </si>
+  <si>
+    <t>NB qty</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>B2B</t>
+  </si>
+  <si>
+    <t>B2B x 4</t>
+  </si>
+  <si>
+    <t>Barbed Wire</t>
+  </si>
+  <si>
+    <t>RC Portion</t>
+  </si>
+  <si>
+    <t>DMS</t>
+  </si>
+  <si>
+    <t>nos of bags</t>
+  </si>
+  <si>
+    <t>in kg</t>
+  </si>
+  <si>
+    <t>8mm</t>
+  </si>
+  <si>
+    <t>10mm</t>
+  </si>
+  <si>
+    <t>12mm</t>
+  </si>
+  <si>
+    <t>16mm</t>
+  </si>
+  <si>
+    <t>20mm</t>
+  </si>
+  <si>
+    <t>25mm</t>
+  </si>
+  <si>
+    <t>Total Steel (Kgs)</t>
   </si>
 </sst>
 </file>
@@ -661,7 +752,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="36">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -1098,6 +1189,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1109,7 +1209,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1291,17 +1391,35 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1315,15 +1433,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1503,11 +1612,6 @@
             <v>Office:  Neemuch</v>
           </cell>
         </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>Progress of 220kV Line</v>
-          </cell>
-        </row>
       </sheetData>
       <sheetData sheetId="5" refreshError="1"/>
       <sheetData sheetId="6" refreshError="1"/>
@@ -1518,6 +1622,54 @@
       <sheetData sheetId="11" refreshError="1"/>
       <sheetData sheetId="12" refreshError="1"/>
       <sheetData sheetId="13" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Detail Survey-220kV"/>
+      <sheetName val="Check Survey-220kV"/>
+      <sheetName val="Detail Survey-132kV"/>
+      <sheetName val="Check Survey-132kV"/>
+      <sheetName val="Summary"/>
+      <sheetName val="Statutory"/>
+      <sheetName val="Progress-132kV"/>
+      <sheetName val="Progress-220kV"/>
+      <sheetName val="Stringing-220kV"/>
+      <sheetName val="Stringing-132KV"/>
+      <sheetName val="VC-220kV"/>
+      <sheetName val="VC-132kV"/>
+      <sheetName val="Supply"/>
+      <sheetName val="Mail Body"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4">
+        <row r="4">
+          <cell r="A4" t="str">
+            <v>Office:  Neemuch</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2137,77 +2289,77 @@
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="73" t="str">
+      <c r="A3" s="70" t="str">
         <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
-      <c r="L3" s="66"/>
-      <c r="M3" s="66"/>
-      <c r="N3" s="66"/>
-      <c r="O3" s="66"/>
-      <c r="P3" s="66"/>
-      <c r="Q3" s="66"/>
-      <c r="R3" s="66"/>
-      <c r="S3" s="66"/>
-      <c r="T3" s="66"/>
-      <c r="U3" s="66"/>
-      <c r="V3" s="66"/>
-      <c r="W3" s="66"/>
-      <c r="X3" s="66"/>
-      <c r="Y3" s="66"/>
-      <c r="Z3" s="67"/>
+      <c r="B3" s="68"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
+      <c r="I3" s="68"/>
+      <c r="J3" s="68"/>
+      <c r="K3" s="68"/>
+      <c r="L3" s="68"/>
+      <c r="M3" s="68"/>
+      <c r="N3" s="68"/>
+      <c r="O3" s="68"/>
+      <c r="P3" s="68"/>
+      <c r="Q3" s="68"/>
+      <c r="R3" s="68"/>
+      <c r="S3" s="68"/>
+      <c r="T3" s="68"/>
+      <c r="U3" s="68"/>
+      <c r="V3" s="68"/>
+      <c r="W3" s="68"/>
+      <c r="X3" s="68"/>
+      <c r="Y3" s="68"/>
+      <c r="Z3" s="71"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="73">
+      <c r="A4" s="70">
         <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="66"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="67"/>
+      <c r="B4" s="68"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="71"/>
       <c r="E4" s="18"/>
-      <c r="F4" s="73" t="s">
+      <c r="F4" s="70" t="s">
         <v>90</v>
       </c>
-      <c r="G4" s="66"/>
-      <c r="H4" s="66"/>
-      <c r="I4" s="66"/>
-      <c r="J4" s="66"/>
-      <c r="K4" s="66"/>
-      <c r="L4" s="66"/>
-      <c r="M4" s="66"/>
-      <c r="N4" s="66"/>
-      <c r="O4" s="66"/>
-      <c r="P4" s="66"/>
-      <c r="Q4" s="66"/>
-      <c r="R4" s="67"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="68"/>
+      <c r="I4" s="68"/>
+      <c r="J4" s="68"/>
+      <c r="K4" s="68"/>
+      <c r="L4" s="68"/>
+      <c r="M4" s="68"/>
+      <c r="N4" s="68"/>
+      <c r="O4" s="68"/>
+      <c r="P4" s="68"/>
+      <c r="Q4" s="68"/>
+      <c r="R4" s="71"/>
       <c r="S4" s="19"/>
-      <c r="T4" s="73" t="s">
+      <c r="T4" s="70" t="s">
         <v>91</v>
       </c>
-      <c r="U4" s="66"/>
-      <c r="V4" s="66"/>
-      <c r="W4" s="66"/>
-      <c r="X4" s="66"/>
-      <c r="Y4" s="66"/>
-      <c r="Z4" s="67"/>
+      <c r="U4" s="68"/>
+      <c r="V4" s="68"/>
+      <c r="W4" s="68"/>
+      <c r="X4" s="68"/>
+      <c r="Y4" s="68"/>
+      <c r="Z4" s="71"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="73" t="s">
+      <c r="A5" s="70" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="66"/>
-      <c r="C5" s="67"/>
+      <c r="B5" s="68"/>
+      <c r="C5" s="71"/>
       <c r="D5" s="20">
         <f>[1]Summary!R7</f>
         <v>0</v>
@@ -2266,10 +2418,10 @@
       <c r="A6" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="B6" s="74" t="s">
+      <c r="B6" s="72" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="67"/>
+      <c r="C6" s="71"/>
       <c r="D6" s="25" t="s">
         <v>94</v>
       </c>
@@ -2279,16 +2431,16 @@
       <c r="F6" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="75" t="s">
+      <c r="G6" s="73" t="s">
         <v>97</v>
       </c>
-      <c r="H6" s="66"/>
-      <c r="I6" s="67"/>
-      <c r="J6" s="75" t="s">
+      <c r="H6" s="68"/>
+      <c r="I6" s="71"/>
+      <c r="J6" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="K6" s="66"/>
-      <c r="L6" s="67"/>
+      <c r="K6" s="68"/>
+      <c r="L6" s="71"/>
       <c r="M6" s="28" t="s">
         <v>98</v>
       </c>
@@ -2308,16 +2460,16 @@
         <v>43</v>
       </c>
       <c r="S6" s="33"/>
-      <c r="T6" s="63" t="s">
+      <c r="T6" s="66" t="s">
         <v>103</v>
       </c>
-      <c r="U6" s="66"/>
-      <c r="V6" s="67"/>
-      <c r="W6" s="63" t="s">
+      <c r="U6" s="68"/>
+      <c r="V6" s="71"/>
+      <c r="W6" s="66" t="s">
         <v>104</v>
       </c>
-      <c r="X6" s="66"/>
-      <c r="Y6" s="67"/>
+      <c r="X6" s="68"/>
+      <c r="Y6" s="71"/>
       <c r="Z6" s="31" t="s">
         <v>101</v>
       </c>
@@ -2497,77 +2649,77 @@
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="73" t="str">
+      <c r="A3" s="70" t="str">
         <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
-      <c r="L3" s="66"/>
-      <c r="M3" s="66"/>
-      <c r="N3" s="66"/>
-      <c r="O3" s="66"/>
-      <c r="P3" s="66"/>
-      <c r="Q3" s="66"/>
-      <c r="R3" s="66"/>
-      <c r="S3" s="66"/>
-      <c r="T3" s="66"/>
-      <c r="U3" s="66"/>
-      <c r="V3" s="66"/>
-      <c r="W3" s="66"/>
-      <c r="X3" s="66"/>
-      <c r="Y3" s="66"/>
-      <c r="Z3" s="67"/>
+      <c r="B3" s="68"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
+      <c r="I3" s="68"/>
+      <c r="J3" s="68"/>
+      <c r="K3" s="68"/>
+      <c r="L3" s="68"/>
+      <c r="M3" s="68"/>
+      <c r="N3" s="68"/>
+      <c r="O3" s="68"/>
+      <c r="P3" s="68"/>
+      <c r="Q3" s="68"/>
+      <c r="R3" s="68"/>
+      <c r="S3" s="68"/>
+      <c r="T3" s="68"/>
+      <c r="U3" s="68"/>
+      <c r="V3" s="68"/>
+      <c r="W3" s="68"/>
+      <c r="X3" s="68"/>
+      <c r="Y3" s="68"/>
+      <c r="Z3" s="71"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="73">
+      <c r="A4" s="70">
         <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="66"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="67"/>
+      <c r="B4" s="68"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="71"/>
       <c r="E4" s="18"/>
-      <c r="F4" s="73" t="s">
+      <c r="F4" s="70" t="s">
         <v>90</v>
       </c>
-      <c r="G4" s="66"/>
-      <c r="H4" s="66"/>
-      <c r="I4" s="66"/>
-      <c r="J4" s="66"/>
-      <c r="K4" s="66"/>
-      <c r="L4" s="66"/>
-      <c r="M4" s="66"/>
-      <c r="N4" s="66"/>
-      <c r="O4" s="66"/>
-      <c r="P4" s="66"/>
-      <c r="Q4" s="66"/>
-      <c r="R4" s="67"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="68"/>
+      <c r="I4" s="68"/>
+      <c r="J4" s="68"/>
+      <c r="K4" s="68"/>
+      <c r="L4" s="68"/>
+      <c r="M4" s="68"/>
+      <c r="N4" s="68"/>
+      <c r="O4" s="68"/>
+      <c r="P4" s="68"/>
+      <c r="Q4" s="68"/>
+      <c r="R4" s="71"/>
       <c r="S4" s="19"/>
-      <c r="T4" s="73" t="s">
+      <c r="T4" s="70" t="s">
         <v>91</v>
       </c>
-      <c r="U4" s="66"/>
-      <c r="V4" s="66"/>
-      <c r="W4" s="66"/>
-      <c r="X4" s="66"/>
-      <c r="Y4" s="66"/>
-      <c r="Z4" s="67"/>
+      <c r="U4" s="68"/>
+      <c r="V4" s="68"/>
+      <c r="W4" s="68"/>
+      <c r="X4" s="68"/>
+      <c r="Y4" s="68"/>
+      <c r="Z4" s="71"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="73" t="s">
+      <c r="A5" s="70" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="66"/>
-      <c r="C5" s="67"/>
+      <c r="B5" s="68"/>
+      <c r="C5" s="71"/>
       <c r="D5" s="20">
         <f>[1]Summary!R7</f>
         <v>0</v>
@@ -2626,10 +2778,10 @@
       <c r="A6" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="B6" s="74" t="s">
+      <c r="B6" s="72" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="67"/>
+      <c r="C6" s="71"/>
       <c r="D6" s="25" t="s">
         <v>94</v>
       </c>
@@ -2639,16 +2791,16 @@
       <c r="F6" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="75" t="s">
+      <c r="G6" s="73" t="s">
         <v>97</v>
       </c>
-      <c r="H6" s="66"/>
-      <c r="I6" s="67"/>
-      <c r="J6" s="75" t="s">
+      <c r="H6" s="68"/>
+      <c r="I6" s="71"/>
+      <c r="J6" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="K6" s="66"/>
-      <c r="L6" s="67"/>
+      <c r="K6" s="68"/>
+      <c r="L6" s="71"/>
       <c r="M6" s="28" t="s">
         <v>98</v>
       </c>
@@ -2668,16 +2820,16 @@
         <v>43</v>
       </c>
       <c r="S6" s="33"/>
-      <c r="T6" s="63" t="s">
+      <c r="T6" s="66" t="s">
         <v>103</v>
       </c>
-      <c r="U6" s="66"/>
-      <c r="V6" s="67"/>
-      <c r="W6" s="63" t="s">
+      <c r="U6" s="68"/>
+      <c r="V6" s="71"/>
+      <c r="W6" s="66" t="s">
         <v>104</v>
       </c>
-      <c r="X6" s="66"/>
-      <c r="Y6" s="67"/>
+      <c r="X6" s="68"/>
+      <c r="Y6" s="71"/>
       <c r="Z6" s="31" t="s">
         <v>101</v>
       </c>
@@ -2821,425 +2973,405 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B501B5B8-47AF-4D49-A01B-A8E1BEE40158}">
-  <dimension ref="A1:BA10"/>
+  <dimension ref="A1:BM10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A1" s="63" t="str">
-        <f>+[1]Summary!A2</f>
-        <v>Name of the Line: 220KV DC AL59 line from Neemuch - Chanderiya + 132KV DC ACSS Line from Chanderiya to Hindustan Zinc</v>
-      </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="65"/>
-      <c r="L1" s="65"/>
-      <c r="M1" s="65"/>
-      <c r="N1" s="65"/>
-      <c r="O1" s="65"/>
-      <c r="P1" s="65"/>
-      <c r="Q1" s="65"/>
-      <c r="R1" s="65"/>
-      <c r="S1" s="65"/>
-      <c r="T1" s="65"/>
-      <c r="U1" s="65"/>
-      <c r="V1" s="65"/>
-      <c r="W1" s="65"/>
-      <c r="X1" s="65"/>
-      <c r="Y1" s="65"/>
-      <c r="Z1" s="65"/>
-      <c r="AA1" s="65"/>
-      <c r="AB1" s="65"/>
-      <c r="AC1" s="65"/>
-      <c r="AD1" s="65"/>
-      <c r="AE1" s="65"/>
-      <c r="AF1" s="65"/>
-      <c r="AG1" s="65"/>
-      <c r="AH1" s="65"/>
-      <c r="AI1" s="65"/>
-      <c r="AJ1" s="65"/>
-      <c r="AK1" s="65"/>
-      <c r="AL1" s="66"/>
-      <c r="AM1" s="66"/>
-      <c r="AN1" s="66"/>
-      <c r="AO1" s="66"/>
-      <c r="AP1" s="66"/>
-      <c r="AQ1" s="65"/>
-      <c r="AR1" s="65"/>
-      <c r="AS1" s="65"/>
-      <c r="AT1" s="65"/>
-      <c r="AU1" s="65"/>
-      <c r="AV1" s="65"/>
-      <c r="AW1" s="65"/>
-      <c r="AX1" s="65"/>
-      <c r="AY1" s="65"/>
-      <c r="AZ1" s="65"/>
-      <c r="BA1" s="64"/>
-    </row>
-    <row r="2" spans="1:53" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:65" x14ac:dyDescent="0.35">
+      <c r="A1" s="66"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
+      <c r="AD1" s="67"/>
+      <c r="AE1" s="67"/>
+      <c r="AF1" s="67"/>
+      <c r="AG1" s="67"/>
+      <c r="AH1" s="67"/>
+      <c r="AI1" s="67"/>
+      <c r="AJ1" s="67"/>
+      <c r="AK1" s="67"/>
+      <c r="AL1" s="68"/>
+      <c r="AM1" s="68"/>
+      <c r="AN1" s="68"/>
+      <c r="AO1" s="68"/>
+      <c r="AP1" s="68"/>
+      <c r="AQ1" s="67"/>
+      <c r="AR1" s="67"/>
+      <c r="AS1" s="67"/>
+      <c r="AT1" s="67"/>
+      <c r="AU1" s="67"/>
+      <c r="AV1" s="67"/>
+      <c r="AW1" s="67"/>
+      <c r="AX1" s="67"/>
+      <c r="AY1" s="67"/>
+      <c r="AZ1" s="67"/>
+      <c r="BA1" s="69"/>
+    </row>
+    <row r="2" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A3" s="63" t="str">
-        <f>+[1]Summary!A5</f>
-        <v>Progress of 220kV Line</v>
-      </c>
-      <c r="B3" s="65"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="65"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="65"/>
-      <c r="I3" s="65"/>
-      <c r="J3" s="65"/>
-      <c r="K3" s="65"/>
-      <c r="L3" s="65"/>
-      <c r="M3" s="65"/>
-      <c r="N3" s="65"/>
-      <c r="O3" s="65"/>
-      <c r="P3" s="65"/>
-      <c r="Q3" s="65"/>
-      <c r="R3" s="65"/>
-      <c r="S3" s="65"/>
-      <c r="T3" s="65"/>
-      <c r="U3" s="65"/>
-      <c r="V3" s="65"/>
-      <c r="W3" s="65"/>
-      <c r="X3" s="65"/>
-      <c r="Y3" s="65"/>
-      <c r="Z3" s="65"/>
-      <c r="AA3" s="65"/>
-      <c r="AB3" s="65"/>
-      <c r="AC3" s="65"/>
-      <c r="AD3" s="65"/>
-      <c r="AE3" s="65"/>
-      <c r="AF3" s="65"/>
-      <c r="AG3" s="65"/>
-      <c r="AH3" s="65"/>
-      <c r="AI3" s="65"/>
-      <c r="AJ3" s="65"/>
-      <c r="AK3" s="65"/>
-      <c r="AL3" s="66"/>
-      <c r="AM3" s="66"/>
-      <c r="AN3" s="66"/>
-      <c r="AO3" s="66"/>
-      <c r="AP3" s="66"/>
-      <c r="AQ3" s="65"/>
-      <c r="AR3" s="65"/>
-      <c r="AS3" s="65"/>
-      <c r="AT3" s="65"/>
-      <c r="AU3" s="65"/>
-      <c r="AV3" s="65"/>
-      <c r="AW3" s="65"/>
-      <c r="AX3" s="65"/>
-      <c r="AY3" s="65"/>
-      <c r="AZ3" s="65"/>
-      <c r="BA3" s="64"/>
-    </row>
-    <row r="4" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="63" t="s">
-        <v>114</v>
-      </c>
-      <c r="B4" s="65"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
-      <c r="H4" s="65"/>
-      <c r="I4" s="65"/>
-      <c r="J4" s="65"/>
-      <c r="K4" s="65"/>
-      <c r="L4" s="65"/>
-      <c r="M4" s="65"/>
-      <c r="N4" s="65"/>
-      <c r="O4" s="65"/>
-      <c r="P4" s="65"/>
-      <c r="Q4" s="65"/>
-      <c r="R4" s="65"/>
-      <c r="S4" s="64"/>
+    <row r="3" spans="1:65" x14ac:dyDescent="0.35">
+      <c r="A3" s="64" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="63" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" s="63" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63" t="s">
+        <v>143</v>
+      </c>
+      <c r="I3" s="63" t="s">
+        <v>144</v>
+      </c>
+      <c r="J3" s="63" t="s">
+        <v>145</v>
+      </c>
+      <c r="K3" s="63" t="s">
+        <v>146</v>
+      </c>
+      <c r="L3" s="63" t="s">
+        <v>139</v>
+      </c>
+      <c r="M3" s="63" t="s">
+        <v>140</v>
+      </c>
+      <c r="N3" s="63" t="s">
+        <v>150</v>
+      </c>
+      <c r="O3" s="63" t="s">
+        <v>141</v>
+      </c>
+      <c r="P3" s="63" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q3" s="63" t="s">
+        <v>139</v>
+      </c>
+      <c r="R3" s="63" t="s">
+        <v>141</v>
+      </c>
+      <c r="S3" s="63" t="s">
+        <v>152</v>
+      </c>
+      <c r="T3" s="63" t="s">
+        <v>153</v>
+      </c>
+      <c r="U3" s="63" t="s">
+        <v>154</v>
+      </c>
+      <c r="V3" s="63" t="s">
+        <v>123</v>
+      </c>
+      <c r="W3" s="63" t="s">
+        <v>79</v>
+      </c>
+      <c r="X3" s="63" t="s">
+        <v>124</v>
+      </c>
+      <c r="Y3" s="63" t="s">
+        <v>125</v>
+      </c>
+      <c r="Z3" s="63"/>
+      <c r="AA3" s="63"/>
+      <c r="AB3" s="63" t="s">
+        <v>155</v>
+      </c>
+      <c r="AC3" s="63"/>
+      <c r="AD3" s="63" t="s">
+        <v>156</v>
+      </c>
+      <c r="AE3" s="63"/>
+      <c r="AF3" s="63"/>
+      <c r="AG3" s="63"/>
+      <c r="AH3" s="63"/>
+      <c r="AI3" s="63"/>
+      <c r="AJ3" s="63"/>
+      <c r="AK3" s="63"/>
+      <c r="AL3" s="63"/>
+      <c r="AM3" s="63" t="s">
+        <v>157</v>
+      </c>
+      <c r="AN3" s="63" t="s">
+        <v>158</v>
+      </c>
+      <c r="AO3" s="63" t="s">
+        <v>62</v>
+      </c>
+      <c r="AP3" s="63" t="s">
+        <v>134</v>
+      </c>
+      <c r="AQ3" s="63"/>
+      <c r="AR3" s="63" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS3" s="63"/>
+      <c r="AT3" s="63" t="s">
+        <v>101</v>
+      </c>
+      <c r="AU3" s="63"/>
+      <c r="AV3" s="63" t="s">
+        <v>159</v>
+      </c>
+      <c r="AW3" s="63" t="s">
+        <v>160</v>
+      </c>
+      <c r="AX3" s="63" t="s">
+        <v>105</v>
+      </c>
+      <c r="AY3" s="63" t="s">
+        <v>106</v>
+      </c>
+      <c r="AZ3" s="63" t="s">
+        <v>161</v>
+      </c>
+      <c r="BA3" s="65"/>
+      <c r="BB3" t="s">
+        <v>162</v>
+      </c>
+      <c r="BC3" t="s">
+        <v>158</v>
+      </c>
+      <c r="BD3" t="s">
+        <v>62</v>
+      </c>
+      <c r="BE3" t="s">
+        <v>105</v>
+      </c>
+      <c r="BF3" t="s">
+        <v>106</v>
+      </c>
+      <c r="BG3" t="s">
+        <v>161</v>
+      </c>
+      <c r="BI3" t="s">
+        <v>136</v>
+      </c>
+      <c r="BJ3" t="s">
+        <v>105</v>
+      </c>
+      <c r="BK3" t="s">
+        <v>106</v>
+      </c>
+      <c r="BL3" t="s">
+        <v>163</v>
+      </c>
+      <c r="BM3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:65" x14ac:dyDescent="0.35">
+      <c r="A4" s="64" t="s">
+        <v>164</v>
+      </c>
+      <c r="B4" s="63"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="63" t="s">
+        <v>165</v>
+      </c>
+      <c r="E4" s="63" t="s">
+        <v>166</v>
+      </c>
+      <c r="F4" s="63" t="s">
+        <v>167</v>
+      </c>
+      <c r="G4" s="63" t="s">
+        <v>168</v>
+      </c>
+      <c r="H4" s="63"/>
+      <c r="I4" s="63"/>
+      <c r="J4" s="63"/>
+      <c r="K4" s="63"/>
+      <c r="L4" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="M4" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="N4" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="O4" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="P4" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q4" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="R4" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="S4" s="63" t="s">
+        <v>80</v>
+      </c>
       <c r="T4" s="63" t="s">
-        <v>115</v>
-      </c>
-      <c r="U4" s="65"/>
-      <c r="V4" s="65"/>
-      <c r="W4" s="65"/>
-      <c r="X4" s="65"/>
-      <c r="Y4" s="65"/>
-      <c r="Z4" s="65"/>
-      <c r="AA4" s="65"/>
-      <c r="AB4" s="65"/>
-      <c r="AC4" s="65"/>
-      <c r="AD4" s="65"/>
-      <c r="AE4" s="65"/>
-      <c r="AF4" s="65"/>
-      <c r="AG4" s="65"/>
-      <c r="AH4" s="65"/>
-      <c r="AI4" s="65"/>
-      <c r="AJ4" s="65"/>
-      <c r="AK4" s="64"/>
-      <c r="AL4" s="63" t="s">
-        <v>116</v>
-      </c>
-      <c r="AM4" s="66"/>
-      <c r="AN4" s="66"/>
-      <c r="AO4" s="66"/>
-      <c r="AP4" s="67"/>
+        <v>169</v>
+      </c>
+      <c r="U4" s="63"/>
+      <c r="V4" s="63" t="s">
+        <v>147</v>
+      </c>
+      <c r="W4" s="63"/>
+      <c r="X4" s="63"/>
+      <c r="Y4" s="63" t="s">
+        <v>148</v>
+      </c>
+      <c r="Z4" s="63" t="s">
+        <v>149</v>
+      </c>
+      <c r="AA4" s="63" t="s">
+        <v>142</v>
+      </c>
+      <c r="AB4" s="63" t="s">
+        <v>170</v>
+      </c>
+      <c r="AC4" s="63" t="s">
+        <v>171</v>
+      </c>
+      <c r="AD4" s="63" t="s">
+        <v>172</v>
+      </c>
+      <c r="AE4" s="63" t="s">
+        <v>173</v>
+      </c>
+      <c r="AF4" s="63" t="s">
+        <v>174</v>
+      </c>
+      <c r="AG4" s="63" t="s">
+        <v>175</v>
+      </c>
+      <c r="AH4" s="63" t="s">
+        <v>176</v>
+      </c>
+      <c r="AI4" s="63" t="s">
+        <v>177</v>
+      </c>
+      <c r="AJ4" s="63" t="s">
+        <v>178</v>
+      </c>
+      <c r="AK4" s="63" t="s">
+        <v>132</v>
+      </c>
+      <c r="AL4" s="63"/>
+      <c r="AM4" s="63"/>
+      <c r="AN4" s="63"/>
+      <c r="AO4" s="63"/>
+      <c r="AP4" s="63" t="s">
+        <v>105</v>
+      </c>
       <c r="AQ4" s="63" t="s">
-        <v>2</v>
-      </c>
-      <c r="AR4" s="65"/>
-      <c r="AS4" s="65"/>
-      <c r="AT4" s="64"/>
-      <c r="AU4" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="AV4" s="63" t="s">
-        <v>118</v>
-      </c>
-      <c r="AW4" s="65"/>
-      <c r="AX4" s="65"/>
-      <c r="AY4" s="65"/>
-      <c r="AZ4" s="64"/>
-      <c r="BA4" s="27" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="5" spans="1:53" ht="58.5" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>120</v>
-      </c>
-      <c r="C5" s="31" t="s">
-        <v>78</v>
-      </c>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="68" t="s">
-        <v>82</v>
-      </c>
-      <c r="H5" s="69"/>
-      <c r="I5" s="69"/>
-      <c r="J5" s="70"/>
-      <c r="K5" s="68" t="s">
-        <v>121</v>
-      </c>
-      <c r="L5" s="69"/>
-      <c r="M5" s="69"/>
-      <c r="N5" s="70"/>
-      <c r="O5" s="71" t="s">
-        <v>122</v>
-      </c>
-      <c r="P5" s="65"/>
-      <c r="Q5" s="65"/>
-      <c r="R5" s="64"/>
-      <c r="S5" s="51" t="s">
-        <v>123</v>
-      </c>
-      <c r="T5" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="U5" s="31" t="s">
-        <v>124</v>
-      </c>
-      <c r="V5" s="63" t="s">
-        <v>125</v>
-      </c>
-      <c r="W5" s="65"/>
-      <c r="X5" s="64"/>
-      <c r="Y5" s="52" t="s">
-        <v>126</v>
-      </c>
-      <c r="Z5" s="52" t="s">
-        <v>127</v>
-      </c>
-      <c r="AA5" s="52" t="s">
-        <v>128</v>
-      </c>
-      <c r="AB5" s="52" t="s">
-        <v>129</v>
-      </c>
-      <c r="AC5" s="52" t="s">
-        <v>130</v>
-      </c>
-      <c r="AD5" s="52" t="s">
-        <v>131</v>
-      </c>
-      <c r="AE5" s="53" t="s">
-        <v>132</v>
-      </c>
-      <c r="AF5" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="AG5" s="72" t="s">
-        <v>134</v>
-      </c>
-      <c r="AH5" s="64"/>
-      <c r="AI5" s="63" t="s">
-        <v>135</v>
-      </c>
-      <c r="AJ5" s="64"/>
-      <c r="AK5" s="27" t="s">
-        <v>101</v>
-      </c>
-      <c r="AL5" s="27" t="s">
-        <v>136</v>
-      </c>
-      <c r="AM5" s="27" t="s">
-        <v>137</v>
-      </c>
-      <c r="AN5" s="54" t="s">
+        <v>106</v>
+      </c>
+      <c r="AR4" s="63" t="s">
         <v>105</v>
       </c>
-      <c r="AO5" s="54" t="s">
-        <v>106</v>
-      </c>
-      <c r="AP5" s="27" t="s">
-        <v>101</v>
-      </c>
-      <c r="AQ5" s="27" t="s">
-        <v>136</v>
-      </c>
-      <c r="AR5" s="54" t="s">
-        <v>105</v>
-      </c>
-      <c r="AS5" s="54" t="s">
-        <v>106</v>
-      </c>
-      <c r="AT5" s="27" t="s">
-        <v>101</v>
-      </c>
-      <c r="AU5" s="53"/>
-      <c r="AV5" s="27" t="s">
-        <v>136</v>
-      </c>
-      <c r="AW5" s="54" t="s">
-        <v>105</v>
-      </c>
-      <c r="AX5" s="54" t="s">
-        <v>106</v>
-      </c>
-      <c r="AY5" s="55" t="s">
-        <v>138</v>
-      </c>
-      <c r="AZ5" s="27" t="s">
-        <v>101</v>
-      </c>
-      <c r="BA5" s="53"/>
-    </row>
-    <row r="6" spans="1:53" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="31"/>
-      <c r="B6" s="31"/>
-      <c r="C6" s="31"/>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="56" t="s">
-        <v>139</v>
-      </c>
-      <c r="H6" s="31" t="s">
-        <v>140</v>
-      </c>
-      <c r="I6" s="31" t="s">
-        <v>141</v>
-      </c>
-      <c r="J6" s="57" t="s">
-        <v>142</v>
-      </c>
-      <c r="K6" s="56" t="s">
-        <v>139</v>
-      </c>
-      <c r="L6" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="M6" s="31" t="s">
-        <v>141</v>
-      </c>
-      <c r="N6" s="57" t="s">
-        <v>142</v>
-      </c>
-      <c r="O6" s="54" t="s">
-        <v>143</v>
-      </c>
-      <c r="P6" s="54" t="s">
-        <v>144</v>
-      </c>
-      <c r="Q6" s="54" t="s">
-        <v>145</v>
-      </c>
-      <c r="R6" s="54" t="s">
-        <v>146</v>
-      </c>
-      <c r="S6" s="58" t="s">
-        <v>147</v>
-      </c>
-      <c r="T6" s="36"/>
-      <c r="U6" s="27"/>
-      <c r="V6" s="27" t="s">
-        <v>148</v>
-      </c>
-      <c r="W6" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="X6" s="27" t="s">
-        <v>142</v>
-      </c>
-      <c r="Y6" s="53"/>
-      <c r="Z6" s="53"/>
-      <c r="AA6" s="53"/>
-      <c r="AB6" s="53"/>
-      <c r="AC6" s="53"/>
-      <c r="AD6" s="53"/>
-      <c r="AE6" s="36"/>
-      <c r="AF6" s="36"/>
-      <c r="AG6" s="54" t="s">
-        <v>105</v>
-      </c>
-      <c r="AH6" s="54" t="s">
-        <v>106</v>
-      </c>
-      <c r="AI6" s="54" t="s">
-        <v>105</v>
-      </c>
-      <c r="AJ6" s="54" t="s">
-        <v>106</v>
-      </c>
-      <c r="AK6" s="36"/>
-      <c r="AL6" s="36"/>
-      <c r="AM6" s="36"/>
-      <c r="AN6" s="54"/>
-      <c r="AO6" s="54"/>
-      <c r="AP6" s="36"/>
-      <c r="AQ6" s="36"/>
-      <c r="AR6" s="54"/>
-      <c r="AS6" s="54"/>
-      <c r="AT6" s="36"/>
-      <c r="AU6" s="36"/>
-      <c r="AV6" s="36"/>
-      <c r="AW6" s="54"/>
-      <c r="AX6" s="54"/>
-      <c r="AY6" s="59"/>
-      <c r="AZ6" s="36"/>
-      <c r="BA6" s="36"/>
-    </row>
-    <row r="9" spans="1:53" x14ac:dyDescent="0.35">
+      <c r="AS4" s="63">
+        <v>9</v>
+      </c>
+      <c r="AT4" s="63"/>
+      <c r="AU4" s="63"/>
+      <c r="AV4" s="63"/>
+      <c r="AW4" s="63"/>
+      <c r="AX4" s="63"/>
+      <c r="AY4" s="63"/>
+      <c r="AZ4" s="63"/>
+      <c r="BA4" s="65"/>
+    </row>
+    <row r="6" spans="1:65" x14ac:dyDescent="0.35">
+      <c r="A6" s="64"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
+      <c r="G6" s="63"/>
+      <c r="H6" s="63"/>
+      <c r="I6" s="63"/>
+      <c r="J6" s="63"/>
+      <c r="K6" s="63"/>
+      <c r="L6" s="63"/>
+      <c r="M6" s="63"/>
+      <c r="N6" s="63"/>
+      <c r="O6" s="63"/>
+      <c r="P6" s="63"/>
+      <c r="Q6" s="63"/>
+      <c r="R6" s="63"/>
+      <c r="S6" s="63"/>
+      <c r="T6" s="63"/>
+      <c r="U6" s="63"/>
+      <c r="V6" s="63"/>
+      <c r="W6" s="63"/>
+      <c r="X6" s="63"/>
+      <c r="Y6" s="63"/>
+      <c r="Z6" s="63"/>
+      <c r="AA6" s="63"/>
+      <c r="AB6" s="63"/>
+      <c r="AC6" s="63"/>
+      <c r="AD6" s="63"/>
+      <c r="AE6" s="63"/>
+      <c r="AF6" s="63"/>
+      <c r="AG6" s="63"/>
+      <c r="AH6" s="63"/>
+      <c r="AI6" s="63"/>
+      <c r="AJ6" s="63"/>
+      <c r="AK6" s="63"/>
+      <c r="AL6" s="63"/>
+      <c r="AM6" s="63"/>
+      <c r="AN6" s="63"/>
+      <c r="AO6" s="63"/>
+      <c r="AP6" s="63"/>
+      <c r="AQ6" s="63"/>
+      <c r="AR6" s="63"/>
+      <c r="AS6" s="63"/>
+      <c r="AT6" s="63"/>
+      <c r="AU6" s="63"/>
+      <c r="AV6" s="63"/>
+      <c r="AW6" s="63"/>
+      <c r="AX6" s="63"/>
+      <c r="AY6" s="63"/>
+      <c r="AZ6" s="63"/>
+      <c r="BA6" s="65"/>
+    </row>
+    <row r="9" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="10" spans="1:53" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:65" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="6" t="s">
         <v>63</v>
       </c>
@@ -3252,42 +3384,29 @@
       <c r="D10" s="6"/>
       <c r="H10" s="61"/>
       <c r="I10" s="61"/>
-      <c r="J10" s="6" t="s">
-        <v>82</v>
-      </c>
       <c r="M10" s="6"/>
       <c r="N10" s="17"/>
       <c r="O10" s="60"/>
-      <c r="P10" s="61"/>
+      <c r="P10" s="6" t="s">
+        <v>82</v>
+      </c>
       <c r="Q10" s="62"/>
-      <c r="AQ10" s="60" t="s">
+      <c r="BB10" s="60" t="s">
         <v>55</v>
       </c>
-      <c r="AR10" s="6" t="s">
+      <c r="BE10" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="AS10" s="6" t="s">
+      <c r="BF10" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="AT10" s="6" t="s">
+      <c r="BG10" s="6" t="s">
         <v>35</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="AI5:AJ5"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:BA1"/>
-    <mergeCell ref="A3:BA3"/>
-    <mergeCell ref="A4:S4"/>
-    <mergeCell ref="T4:AK4"/>
-    <mergeCell ref="AL4:AP4"/>
-    <mergeCell ref="AQ4:AT4"/>
-    <mergeCell ref="AV4:AZ4"/>
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="O5:R5"/>
-    <mergeCell ref="V5:X5"/>
-    <mergeCell ref="AG5:AH5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3307,351 +3426,409 @@
       </c>
     </row>
     <row r="3" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A3" s="63" t="str">
-        <f>+[1]Summary!A5</f>
-        <v>Progress of 220kV Line</v>
-      </c>
-      <c r="B3" s="65"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="65"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="65"/>
-      <c r="I3" s="65"/>
-      <c r="J3" s="65"/>
-      <c r="K3" s="65"/>
-      <c r="L3" s="65"/>
-      <c r="M3" s="65"/>
-      <c r="N3" s="65"/>
-      <c r="O3" s="65"/>
-      <c r="P3" s="65"/>
-      <c r="Q3" s="65"/>
-      <c r="R3" s="65"/>
-      <c r="S3" s="65"/>
-      <c r="T3" s="65"/>
-      <c r="U3" s="65"/>
-      <c r="V3" s="65"/>
-      <c r="W3" s="65"/>
-      <c r="X3" s="65"/>
-      <c r="Y3" s="65"/>
-      <c r="Z3" s="65"/>
-      <c r="AA3" s="65"/>
-      <c r="AB3" s="65"/>
-      <c r="AC3" s="65"/>
-      <c r="AD3" s="65"/>
-      <c r="AE3" s="65"/>
-      <c r="AF3" s="65"/>
-      <c r="AG3" s="65"/>
-      <c r="AH3" s="65"/>
-      <c r="AI3" s="65"/>
-      <c r="AJ3" s="65"/>
-      <c r="AK3" s="65"/>
-      <c r="AL3" s="66"/>
-      <c r="AM3" s="66"/>
-      <c r="AN3" s="66"/>
-      <c r="AO3" s="66"/>
-      <c r="AP3" s="66"/>
-      <c r="AQ3" s="65"/>
-      <c r="AR3" s="65"/>
-      <c r="AS3" s="65"/>
-      <c r="AT3" s="65"/>
-      <c r="AU3" s="65"/>
-      <c r="AV3" s="65"/>
-      <c r="AW3" s="65"/>
-      <c r="AX3" s="65"/>
-      <c r="AY3" s="65"/>
-      <c r="AZ3" s="65"/>
-      <c r="BA3" s="64"/>
-    </row>
-    <row r="4" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="63" t="s">
+      <c r="A3" s="66" t="str">
+        <f>+[2]Summary!A4</f>
+        <v>Office:  Neemuch</v>
+      </c>
+      <c r="B3" s="67"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
+      <c r="L3" s="67"/>
+      <c r="M3" s="67"/>
+      <c r="N3" s="67"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="67"/>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="67"/>
+      <c r="W3" s="67"/>
+      <c r="X3" s="67"/>
+      <c r="Y3" s="67"/>
+      <c r="Z3" s="67"/>
+      <c r="AA3" s="67"/>
+      <c r="AB3" s="67"/>
+      <c r="AC3" s="67"/>
+      <c r="AD3" s="67"/>
+      <c r="AE3" s="67"/>
+      <c r="AF3" s="67"/>
+      <c r="AG3" s="67"/>
+      <c r="AH3" s="67"/>
+      <c r="AI3" s="67"/>
+      <c r="AJ3" s="67"/>
+      <c r="AK3" s="67"/>
+      <c r="AL3" s="68"/>
+      <c r="AM3" s="68"/>
+      <c r="AN3" s="68"/>
+      <c r="AO3" s="68"/>
+      <c r="AP3" s="68"/>
+      <c r="AQ3" s="67"/>
+      <c r="AR3" s="67"/>
+      <c r="AS3" s="67"/>
+      <c r="AT3" s="67"/>
+      <c r="AU3" s="67"/>
+      <c r="AV3" s="67"/>
+      <c r="AW3" s="67"/>
+      <c r="AX3" s="67"/>
+      <c r="AY3" s="67"/>
+      <c r="AZ3" s="67"/>
+      <c r="BA3" s="69"/>
+    </row>
+    <row r="4" spans="1:53" x14ac:dyDescent="0.35">
+      <c r="A4" s="66">
+        <f>+[2]Summary!A7</f>
+        <v>0</v>
+      </c>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="67"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
+      <c r="I4" s="67"/>
+      <c r="J4" s="67"/>
+      <c r="K4" s="67"/>
+      <c r="L4" s="67"/>
+      <c r="M4" s="67"/>
+      <c r="N4" s="67"/>
+      <c r="O4" s="67"/>
+      <c r="P4" s="67"/>
+      <c r="Q4" s="67"/>
+      <c r="R4" s="67"/>
+      <c r="S4" s="67"/>
+      <c r="T4" s="67"/>
+      <c r="U4" s="67"/>
+      <c r="V4" s="67"/>
+      <c r="W4" s="67"/>
+      <c r="X4" s="67"/>
+      <c r="Y4" s="67"/>
+      <c r="Z4" s="67"/>
+      <c r="AA4" s="67"/>
+      <c r="AB4" s="67"/>
+      <c r="AC4" s="67"/>
+      <c r="AD4" s="67"/>
+      <c r="AE4" s="67"/>
+      <c r="AF4" s="67"/>
+      <c r="AG4" s="67"/>
+      <c r="AH4" s="67"/>
+      <c r="AI4" s="67"/>
+      <c r="AJ4" s="67"/>
+      <c r="AK4" s="67"/>
+      <c r="AL4" s="68"/>
+      <c r="AM4" s="68"/>
+      <c r="AN4" s="68"/>
+      <c r="AO4" s="68"/>
+      <c r="AP4" s="68"/>
+      <c r="AQ4" s="67"/>
+      <c r="AR4" s="67"/>
+      <c r="AS4" s="67"/>
+      <c r="AT4" s="67"/>
+      <c r="AU4" s="67"/>
+      <c r="AV4" s="67"/>
+      <c r="AW4" s="67"/>
+      <c r="AX4" s="67"/>
+      <c r="AY4" s="67"/>
+      <c r="AZ4" s="67"/>
+      <c r="BA4" s="69"/>
+    </row>
+    <row r="5" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="66" t="s">
         <v>114</v>
       </c>
-      <c r="B4" s="65"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
-      <c r="H4" s="65"/>
-      <c r="I4" s="65"/>
-      <c r="J4" s="65"/>
-      <c r="K4" s="65"/>
-      <c r="L4" s="65"/>
-      <c r="M4" s="65"/>
-      <c r="N4" s="65"/>
-      <c r="O4" s="65"/>
-      <c r="P4" s="65"/>
-      <c r="Q4" s="65"/>
-      <c r="R4" s="65"/>
-      <c r="S4" s="64"/>
-      <c r="T4" s="63" t="s">
+      <c r="B5" s="67"/>
+      <c r="C5" s="67"/>
+      <c r="D5" s="67"/>
+      <c r="E5" s="67"/>
+      <c r="F5" s="67"/>
+      <c r="G5" s="67"/>
+      <c r="H5" s="67"/>
+      <c r="I5" s="67"/>
+      <c r="J5" s="67"/>
+      <c r="K5" s="67"/>
+      <c r="L5" s="67"/>
+      <c r="M5" s="67"/>
+      <c r="N5" s="67"/>
+      <c r="O5" s="67"/>
+      <c r="P5" s="67"/>
+      <c r="Q5" s="67"/>
+      <c r="R5" s="67"/>
+      <c r="S5" s="69"/>
+      <c r="T5" s="66" t="s">
         <v>115</v>
       </c>
-      <c r="U4" s="65"/>
-      <c r="V4" s="65"/>
-      <c r="W4" s="65"/>
-      <c r="X4" s="65"/>
-      <c r="Y4" s="65"/>
-      <c r="Z4" s="65"/>
-      <c r="AA4" s="65"/>
-      <c r="AB4" s="65"/>
-      <c r="AC4" s="65"/>
-      <c r="AD4" s="65"/>
-      <c r="AE4" s="65"/>
-      <c r="AF4" s="65"/>
-      <c r="AG4" s="65"/>
-      <c r="AH4" s="65"/>
-      <c r="AI4" s="65"/>
-      <c r="AJ4" s="65"/>
-      <c r="AK4" s="64"/>
-      <c r="AL4" s="63" t="s">
+      <c r="U5" s="67"/>
+      <c r="V5" s="67"/>
+      <c r="W5" s="67"/>
+      <c r="X5" s="67"/>
+      <c r="Y5" s="67"/>
+      <c r="Z5" s="67"/>
+      <c r="AA5" s="67"/>
+      <c r="AB5" s="67"/>
+      <c r="AC5" s="67"/>
+      <c r="AD5" s="67"/>
+      <c r="AE5" s="67"/>
+      <c r="AF5" s="67"/>
+      <c r="AG5" s="67"/>
+      <c r="AH5" s="67"/>
+      <c r="AI5" s="67"/>
+      <c r="AJ5" s="67"/>
+      <c r="AK5" s="69"/>
+      <c r="AL5" s="66" t="s">
         <v>116</v>
       </c>
-      <c r="AM4" s="66"/>
-      <c r="AN4" s="66"/>
-      <c r="AO4" s="66"/>
-      <c r="AP4" s="67"/>
-      <c r="AQ4" s="63" t="s">
+      <c r="AM5" s="68"/>
+      <c r="AN5" s="68"/>
+      <c r="AO5" s="68"/>
+      <c r="AP5" s="71"/>
+      <c r="AQ5" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="AR4" s="65"/>
-      <c r="AS4" s="65"/>
-      <c r="AT4" s="64"/>
-      <c r="AU4" s="27" t="s">
+      <c r="AR5" s="67"/>
+      <c r="AS5" s="67"/>
+      <c r="AT5" s="69"/>
+      <c r="AU5" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="AV4" s="63" t="s">
+      <c r="AV5" s="66" t="s">
         <v>118</v>
       </c>
-      <c r="AW4" s="65"/>
-      <c r="AX4" s="65"/>
-      <c r="AY4" s="65"/>
-      <c r="AZ4" s="64"/>
-      <c r="BA4" s="27" t="s">
+      <c r="AW5" s="67"/>
+      <c r="AX5" s="67"/>
+      <c r="AY5" s="67"/>
+      <c r="AZ5" s="69"/>
+      <c r="BA5" s="27" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="5" spans="1:53" ht="58.5" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="31" t="s">
+    <row r="6" spans="1:53" ht="58.5" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="31" t="s">
         <v>93</v>
       </c>
-      <c r="B5" s="31" t="s">
+      <c r="B6" s="31" t="s">
         <v>120</v>
       </c>
-      <c r="C5" s="31" t="s">
+      <c r="C6" s="31" t="s">
         <v>78</v>
       </c>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="68" t="s">
+      <c r="D6" s="50"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="50"/>
+      <c r="G6" s="74" t="s">
         <v>82</v>
       </c>
-      <c r="H5" s="69"/>
-      <c r="I5" s="69"/>
-      <c r="J5" s="70"/>
-      <c r="K5" s="68" t="s">
+      <c r="H6" s="75"/>
+      <c r="I6" s="75"/>
+      <c r="J6" s="76"/>
+      <c r="K6" s="74" t="s">
         <v>121</v>
       </c>
-      <c r="L5" s="69"/>
-      <c r="M5" s="69"/>
-      <c r="N5" s="70"/>
-      <c r="O5" s="71" t="s">
+      <c r="L6" s="75"/>
+      <c r="M6" s="75"/>
+      <c r="N6" s="76"/>
+      <c r="O6" s="77" t="s">
         <v>122</v>
       </c>
-      <c r="P5" s="65"/>
-      <c r="Q5" s="65"/>
-      <c r="R5" s="64"/>
-      <c r="S5" s="51" t="s">
+      <c r="P6" s="67"/>
+      <c r="Q6" s="67"/>
+      <c r="R6" s="69"/>
+      <c r="S6" s="51" t="s">
         <v>123</v>
       </c>
-      <c r="T5" s="27" t="s">
+      <c r="T6" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="U5" s="31" t="s">
+      <c r="U6" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="V5" s="63" t="s">
+      <c r="V6" s="66" t="s">
         <v>125</v>
       </c>
-      <c r="W5" s="65"/>
-      <c r="X5" s="64"/>
-      <c r="Y5" s="52" t="s">
+      <c r="W6" s="67"/>
+      <c r="X6" s="69"/>
+      <c r="Y6" s="52" t="s">
         <v>126</v>
       </c>
-      <c r="Z5" s="52" t="s">
+      <c r="Z6" s="52" t="s">
         <v>127</v>
       </c>
-      <c r="AA5" s="52" t="s">
+      <c r="AA6" s="52" t="s">
         <v>128</v>
       </c>
-      <c r="AB5" s="52" t="s">
+      <c r="AB6" s="52" t="s">
         <v>129</v>
       </c>
-      <c r="AC5" s="52" t="s">
+      <c r="AC6" s="52" t="s">
         <v>130</v>
       </c>
-      <c r="AD5" s="52" t="s">
+      <c r="AD6" s="52" t="s">
         <v>131</v>
       </c>
-      <c r="AE5" s="53" t="s">
+      <c r="AE6" s="53" t="s">
         <v>132</v>
       </c>
-      <c r="AF5" s="27" t="s">
+      <c r="AF6" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="AG5" s="72" t="s">
+      <c r="AG6" s="78" t="s">
         <v>134</v>
       </c>
-      <c r="AH5" s="64"/>
-      <c r="AI5" s="63" t="s">
+      <c r="AH6" s="69"/>
+      <c r="AI6" s="66" t="s">
         <v>135</v>
       </c>
-      <c r="AJ5" s="64"/>
-      <c r="AK5" s="27" t="s">
+      <c r="AJ6" s="69"/>
+      <c r="AK6" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="AL5" s="27" t="s">
+      <c r="AL6" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="AM5" s="27" t="s">
+      <c r="AM6" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="AN5" s="54" t="s">
+      <c r="AN6" s="54" t="s">
         <v>105</v>
       </c>
-      <c r="AO5" s="54" t="s">
+      <c r="AO6" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AP5" s="27" t="s">
+      <c r="AP6" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="AQ5" s="27" t="s">
+      <c r="AQ6" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="AR5" s="54" t="s">
+      <c r="AR6" s="54" t="s">
         <v>105</v>
       </c>
-      <c r="AS5" s="54" t="s">
+      <c r="AS6" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AT5" s="27" t="s">
+      <c r="AT6" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="AU5" s="53"/>
-      <c r="AV5" s="27" t="s">
+      <c r="AU6" s="53"/>
+      <c r="AV6" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="AW5" s="54" t="s">
+      <c r="AW6" s="54" t="s">
         <v>105</v>
       </c>
-      <c r="AX5" s="54" t="s">
+      <c r="AX6" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AY5" s="55" t="s">
+      <c r="AY6" s="55" t="s">
         <v>138</v>
       </c>
-      <c r="AZ5" s="27" t="s">
+      <c r="AZ6" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="BA5" s="53"/>
-    </row>
-    <row r="6" spans="1:53" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="31"/>
-      <c r="B6" s="31"/>
-      <c r="C6" s="31"/>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="56" t="s">
+      <c r="BA6" s="53"/>
+    </row>
+    <row r="7" spans="1:53" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="31"/>
+      <c r="B7" s="31"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="56" t="s">
         <v>139</v>
       </c>
-      <c r="H6" s="31" t="s">
+      <c r="H7" s="31" t="s">
         <v>140</v>
       </c>
-      <c r="I6" s="31" t="s">
+      <c r="I7" s="31" t="s">
         <v>141</v>
       </c>
-      <c r="J6" s="57" t="s">
+      <c r="J7" s="57" t="s">
         <v>142</v>
       </c>
-      <c r="K6" s="56" t="s">
+      <c r="K7" s="56" t="s">
         <v>139</v>
       </c>
-      <c r="L6" s="29" t="s">
+      <c r="L7" s="29" t="s">
         <v>140</v>
       </c>
-      <c r="M6" s="31" t="s">
+      <c r="M7" s="31" t="s">
         <v>141</v>
       </c>
-      <c r="N6" s="57" t="s">
+      <c r="N7" s="57" t="s">
         <v>142</v>
       </c>
-      <c r="O6" s="54" t="s">
+      <c r="O7" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="P6" s="54" t="s">
+      <c r="P7" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="Q6" s="54" t="s">
+      <c r="Q7" s="54" t="s">
         <v>145</v>
       </c>
-      <c r="R6" s="54" t="s">
+      <c r="R7" s="54" t="s">
         <v>146</v>
       </c>
-      <c r="S6" s="58" t="s">
+      <c r="S7" s="58" t="s">
         <v>147</v>
       </c>
-      <c r="T6" s="36"/>
-      <c r="U6" s="27"/>
-      <c r="V6" s="27" t="s">
+      <c r="T7" s="36"/>
+      <c r="U7" s="27"/>
+      <c r="V7" s="27" t="s">
         <v>148</v>
       </c>
-      <c r="W6" s="27" t="s">
+      <c r="W7" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="X6" s="27" t="s">
+      <c r="X7" s="27" t="s">
         <v>142</v>
       </c>
-      <c r="Y6" s="53"/>
-      <c r="Z6" s="53"/>
-      <c r="AA6" s="53"/>
-      <c r="AB6" s="53"/>
-      <c r="AC6" s="53"/>
-      <c r="AD6" s="53"/>
-      <c r="AE6" s="36"/>
-      <c r="AF6" s="36"/>
-      <c r="AG6" s="54" t="s">
+      <c r="Y7" s="53"/>
+      <c r="Z7" s="53"/>
+      <c r="AA7" s="53"/>
+      <c r="AB7" s="53"/>
+      <c r="AC7" s="53"/>
+      <c r="AD7" s="53"/>
+      <c r="AE7" s="36"/>
+      <c r="AF7" s="36"/>
+      <c r="AG7" s="54" t="s">
         <v>105</v>
       </c>
-      <c r="AH6" s="54" t="s">
+      <c r="AH7" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AI6" s="54" t="s">
+      <c r="AI7" s="54" t="s">
         <v>105</v>
       </c>
-      <c r="AJ6" s="54" t="s">
+      <c r="AJ7" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="AK6" s="36"/>
-      <c r="AL6" s="36"/>
-      <c r="AM6" s="36"/>
-      <c r="AN6" s="54"/>
-      <c r="AO6" s="54"/>
-      <c r="AP6" s="36"/>
-      <c r="AQ6" s="36"/>
-      <c r="AR6" s="54"/>
-      <c r="AS6" s="54"/>
-      <c r="AT6" s="36"/>
-      <c r="AU6" s="36"/>
-      <c r="AV6" s="36"/>
-      <c r="AW6" s="54"/>
-      <c r="AX6" s="54"/>
-      <c r="AY6" s="59"/>
-      <c r="AZ6" s="36"/>
-      <c r="BA6" s="36"/>
+      <c r="AK7" s="36"/>
+      <c r="AL7" s="36"/>
+      <c r="AM7" s="36"/>
+      <c r="AN7" s="54"/>
+      <c r="AO7" s="54"/>
+      <c r="AP7" s="36"/>
+      <c r="AQ7" s="36"/>
+      <c r="AR7" s="54"/>
+      <c r="AS7" s="54"/>
+      <c r="AT7" s="36"/>
+      <c r="AU7" s="36"/>
+      <c r="AV7" s="36"/>
+      <c r="AW7" s="54"/>
+      <c r="AX7" s="54"/>
+      <c r="AY7" s="59"/>
+      <c r="AZ7" s="36"/>
+      <c r="BA7" s="36"/>
     </row>
     <row r="9" spans="1:53" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -3693,19 +3870,20 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="AI5:AJ5"/>
+  <mergeCells count="13">
+    <mergeCell ref="AL5:AP5"/>
+    <mergeCell ref="AQ5:AT5"/>
+    <mergeCell ref="AV5:AZ5"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="O6:R6"/>
+    <mergeCell ref="V6:X6"/>
+    <mergeCell ref="AG6:AH6"/>
+    <mergeCell ref="AI6:AJ6"/>
     <mergeCell ref="A3:BA3"/>
-    <mergeCell ref="A4:S4"/>
-    <mergeCell ref="T4:AK4"/>
-    <mergeCell ref="AL4:AP4"/>
-    <mergeCell ref="AQ4:AT4"/>
-    <mergeCell ref="AV4:AZ4"/>
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="O5:R5"/>
-    <mergeCell ref="V5:X5"/>
-    <mergeCell ref="AG5:AH5"/>
+    <mergeCell ref="A4:BA4"/>
+    <mergeCell ref="A5:S5"/>
+    <mergeCell ref="T5:AK5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3722,35 +3900,35 @@
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="78" t="s">
+      <c r="A3" s="81" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="79" t="s">
+      <c r="B3" s="82" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="66"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="79" t="s">
+      <c r="C3" s="68"/>
+      <c r="D3" s="71"/>
+      <c r="E3" s="82" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="66"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="79" t="s">
+      <c r="F3" s="68"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="82" t="s">
         <v>38</v>
       </c>
-      <c r="I3" s="66"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="78" t="s">
+      <c r="I3" s="68"/>
+      <c r="J3" s="71"/>
+      <c r="K3" s="81" t="s">
         <v>75</v>
       </c>
-      <c r="L3" s="76" t="s">
+      <c r="L3" s="79" t="s">
         <v>43</v>
       </c>
       <c r="M3" s="8"/>
       <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="31" x14ac:dyDescent="0.35">
-      <c r="A4" s="77"/>
+      <c r="A4" s="80"/>
       <c r="B4" s="12" t="s">
         <v>39</v>
       </c>
@@ -3778,8 +3956,8 @@
       <c r="J4" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="K4" s="77"/>
-      <c r="L4" s="77"/>
+      <c r="K4" s="80"/>
+      <c r="L4" s="80"/>
       <c r="M4" s="10"/>
       <c r="N4" s="11"/>
     </row>
@@ -3858,46 +4036,46 @@
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A3" s="83" t="s">
+      <c r="A3" s="86" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="83" t="s">
+      <c r="B3" s="86" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83" t="s">
+      <c r="C3" s="86"/>
+      <c r="D3" s="86" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="83" t="s">
+      <c r="E3" s="86" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="83" t="s">
+      <c r="F3" s="86" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="84" t="s">
+      <c r="G3" s="87" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="84"/>
-      <c r="I3" s="84"/>
-      <c r="J3" s="80" t="s">
+      <c r="H3" s="87"/>
+      <c r="I3" s="87"/>
+      <c r="J3" s="83" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="81"/>
-      <c r="L3" s="81"/>
-      <c r="M3" s="81"/>
-      <c r="N3" s="82"/>
+      <c r="K3" s="84"/>
+      <c r="L3" s="84"/>
+      <c r="M3" s="84"/>
+      <c r="N3" s="85"/>
     </row>
     <row r="4" spans="1:23" ht="26" x14ac:dyDescent="0.35">
-      <c r="A4" s="83"/>
+      <c r="A4" s="86"/>
       <c r="B4" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="83"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="83"/>
+      <c r="D4" s="86"/>
+      <c r="E4" s="86"/>
+      <c r="F4" s="86"/>
       <c r="G4" s="1" t="s">
         <v>36</v>
       </c>
@@ -4028,14 +4206,14 @@
       <c r="C3" s="7"/>
       <c r="D3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="85"/>
-      <c r="H3" s="86"/>
-      <c r="I3" s="86"/>
-      <c r="J3" s="87"/>
+      <c r="G3" s="88"/>
+      <c r="H3" s="89"/>
+      <c r="I3" s="89"/>
+      <c r="J3" s="90"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="85"/>
-      <c r="O3" s="86"/>
-      <c r="P3" s="87"/>
+      <c r="N3" s="88"/>
+      <c r="O3" s="89"/>
+      <c r="P3" s="90"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -4117,14 +4295,14 @@
       <c r="C3" s="7"/>
       <c r="D3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="85"/>
-      <c r="H3" s="86"/>
-      <c r="I3" s="86"/>
-      <c r="J3" s="87"/>
+      <c r="G3" s="88"/>
+      <c r="H3" s="89"/>
+      <c r="I3" s="89"/>
+      <c r="J3" s="90"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="85"/>
-      <c r="O3" s="86"/>
-      <c r="P3" s="87"/>
+      <c r="N3" s="88"/>
+      <c r="O3" s="89"/>
+      <c r="P3" s="90"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">

</xml_diff>

<commit_message>
Auto pipeline update 2026-04-02 16:08:12
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3742A297-9DD6-461F-BF71-EB403A6381F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A66FAB75-312A-4960-A195-5DB0FF064ABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" activeTab="4" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet Names Check" sheetId="1" r:id="rId1"/>
@@ -1403,37 +1403,37 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1602,11 +1602,6 @@
       <sheetData sheetId="2" refreshError="1"/>
       <sheetData sheetId="3" refreshError="1"/>
       <sheetData sheetId="4">
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>Name of the Line: 220KV DC AL59 line from Neemuch - Chanderiya + 132KV DC ACSS Line from Chanderiya to Hindustan Zinc</v>
-          </cell>
-        </row>
         <row r="4">
           <cell r="A4" t="str">
             <v>Office:  Neemuch</v>
@@ -1650,26 +1645,31 @@
       <sheetName val="Mail Body"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
       <sheetData sheetId="4">
+        <row r="2">
+          <cell r="A2" t="str">
+            <v>Name of the Line: 220KV DC AL59 line from Neemuch - Chanderiya + 132KV DC ACSS Line from Chanderiya to Hindustan Zinc</v>
+          </cell>
+        </row>
         <row r="4">
           <cell r="A4" t="str">
             <v>Office:  Neemuch</v>
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2289,79 +2289,79 @@
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="70" t="str">
-        <f>+[1]Summary!A4</f>
+      <c r="A3" s="78" t="str">
+        <f>+[2]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="68"/>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="68"/>
-      <c r="K3" s="68"/>
-      <c r="L3" s="68"/>
-      <c r="M3" s="68"/>
-      <c r="N3" s="68"/>
-      <c r="O3" s="68"/>
-      <c r="P3" s="68"/>
-      <c r="Q3" s="68"/>
-      <c r="R3" s="68"/>
-      <c r="S3" s="68"/>
-      <c r="T3" s="68"/>
-      <c r="U3" s="68"/>
-      <c r="V3" s="68"/>
-      <c r="W3" s="68"/>
-      <c r="X3" s="68"/>
-      <c r="Y3" s="68"/>
-      <c r="Z3" s="71"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
+      <c r="L3" s="67"/>
+      <c r="M3" s="67"/>
+      <c r="N3" s="67"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="67"/>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="67"/>
+      <c r="W3" s="67"/>
+      <c r="X3" s="67"/>
+      <c r="Y3" s="67"/>
+      <c r="Z3" s="68"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="70">
-        <f>+[1]Summary!A7</f>
+      <c r="A4" s="78">
+        <f>+[2]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="71"/>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="68"/>
       <c r="E4" s="18"/>
-      <c r="F4" s="70" t="s">
+      <c r="F4" s="78" t="s">
         <v>90</v>
       </c>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
-      <c r="N4" s="68"/>
-      <c r="O4" s="68"/>
-      <c r="P4" s="68"/>
-      <c r="Q4" s="68"/>
-      <c r="R4" s="71"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
+      <c r="I4" s="67"/>
+      <c r="J4" s="67"/>
+      <c r="K4" s="67"/>
+      <c r="L4" s="67"/>
+      <c r="M4" s="67"/>
+      <c r="N4" s="67"/>
+      <c r="O4" s="67"/>
+      <c r="P4" s="67"/>
+      <c r="Q4" s="67"/>
+      <c r="R4" s="68"/>
       <c r="S4" s="19"/>
-      <c r="T4" s="70" t="s">
+      <c r="T4" s="78" t="s">
         <v>91</v>
       </c>
-      <c r="U4" s="68"/>
-      <c r="V4" s="68"/>
-      <c r="W4" s="68"/>
-      <c r="X4" s="68"/>
-      <c r="Y4" s="68"/>
-      <c r="Z4" s="71"/>
+      <c r="U4" s="67"/>
+      <c r="V4" s="67"/>
+      <c r="W4" s="67"/>
+      <c r="X4" s="67"/>
+      <c r="Y4" s="67"/>
+      <c r="Z4" s="68"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="70" t="s">
+      <c r="A5" s="78" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="68"/>
-      <c r="C5" s="71"/>
+      <c r="B5" s="67"/>
+      <c r="C5" s="68"/>
       <c r="D5" s="20">
-        <f>[1]Summary!R7</f>
+        <f>[2]Summary!R7</f>
         <v>0</v>
       </c>
       <c r="E5" s="21">
@@ -2418,10 +2418,10 @@
       <c r="A6" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="B6" s="72" t="s">
+      <c r="B6" s="76" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="71"/>
+      <c r="C6" s="68"/>
       <c r="D6" s="25" t="s">
         <v>94</v>
       </c>
@@ -2431,16 +2431,16 @@
       <c r="F6" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="73" t="s">
+      <c r="G6" s="77" t="s">
         <v>97</v>
       </c>
-      <c r="H6" s="68"/>
-      <c r="I6" s="71"/>
-      <c r="J6" s="73" t="s">
+      <c r="H6" s="67"/>
+      <c r="I6" s="68"/>
+      <c r="J6" s="77" t="s">
         <v>38</v>
       </c>
-      <c r="K6" s="68"/>
-      <c r="L6" s="71"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="68"/>
       <c r="M6" s="28" t="s">
         <v>98</v>
       </c>
@@ -2463,13 +2463,13 @@
       <c r="T6" s="66" t="s">
         <v>103</v>
       </c>
-      <c r="U6" s="68"/>
-      <c r="V6" s="71"/>
+      <c r="U6" s="67"/>
+      <c r="V6" s="68"/>
       <c r="W6" s="66" t="s">
         <v>104</v>
       </c>
-      <c r="X6" s="68"/>
-      <c r="Y6" s="71"/>
+      <c r="X6" s="67"/>
+      <c r="Y6" s="68"/>
       <c r="Z6" s="31" t="s">
         <v>101</v>
       </c>
@@ -2617,16 +2617,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A3:Z3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="F4:R4"/>
+    <mergeCell ref="T4:Z4"/>
+    <mergeCell ref="A5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="G6:I6"/>
     <mergeCell ref="J6:L6"/>
     <mergeCell ref="T6:V6"/>
     <mergeCell ref="W6:Y6"/>
-    <mergeCell ref="A3:Z3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="F4:R4"/>
-    <mergeCell ref="T4:Z4"/>
-    <mergeCell ref="A5:C5"/>
   </mergeCells>
   <conditionalFormatting sqref="B11">
     <cfRule type="duplicateValues" dxfId="7" priority="2"/>
@@ -2649,79 +2649,79 @@
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="70" t="str">
-        <f>+[1]Summary!A4</f>
+      <c r="A3" s="78" t="str">
+        <f>+[2]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="68"/>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="68"/>
-      <c r="K3" s="68"/>
-      <c r="L3" s="68"/>
-      <c r="M3" s="68"/>
-      <c r="N3" s="68"/>
-      <c r="O3" s="68"/>
-      <c r="P3" s="68"/>
-      <c r="Q3" s="68"/>
-      <c r="R3" s="68"/>
-      <c r="S3" s="68"/>
-      <c r="T3" s="68"/>
-      <c r="U3" s="68"/>
-      <c r="V3" s="68"/>
-      <c r="W3" s="68"/>
-      <c r="X3" s="68"/>
-      <c r="Y3" s="68"/>
-      <c r="Z3" s="71"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
+      <c r="L3" s="67"/>
+      <c r="M3" s="67"/>
+      <c r="N3" s="67"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="67"/>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="67"/>
+      <c r="W3" s="67"/>
+      <c r="X3" s="67"/>
+      <c r="Y3" s="67"/>
+      <c r="Z3" s="68"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="70">
-        <f>+[1]Summary!A7</f>
+      <c r="A4" s="78">
+        <f>+[2]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="71"/>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="68"/>
       <c r="E4" s="18"/>
-      <c r="F4" s="70" t="s">
+      <c r="F4" s="78" t="s">
         <v>90</v>
       </c>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
-      <c r="N4" s="68"/>
-      <c r="O4" s="68"/>
-      <c r="P4" s="68"/>
-      <c r="Q4" s="68"/>
-      <c r="R4" s="71"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
+      <c r="I4" s="67"/>
+      <c r="J4" s="67"/>
+      <c r="K4" s="67"/>
+      <c r="L4" s="67"/>
+      <c r="M4" s="67"/>
+      <c r="N4" s="67"/>
+      <c r="O4" s="67"/>
+      <c r="P4" s="67"/>
+      <c r="Q4" s="67"/>
+      <c r="R4" s="68"/>
       <c r="S4" s="19"/>
-      <c r="T4" s="70" t="s">
+      <c r="T4" s="78" t="s">
         <v>91</v>
       </c>
-      <c r="U4" s="68"/>
-      <c r="V4" s="68"/>
-      <c r="W4" s="68"/>
-      <c r="X4" s="68"/>
-      <c r="Y4" s="68"/>
-      <c r="Z4" s="71"/>
+      <c r="U4" s="67"/>
+      <c r="V4" s="67"/>
+      <c r="W4" s="67"/>
+      <c r="X4" s="67"/>
+      <c r="Y4" s="67"/>
+      <c r="Z4" s="68"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="70" t="s">
+      <c r="A5" s="78" t="s">
         <v>92</v>
       </c>
-      <c r="B5" s="68"/>
-      <c r="C5" s="71"/>
+      <c r="B5" s="67"/>
+      <c r="C5" s="68"/>
       <c r="D5" s="20">
-        <f>[1]Summary!R7</f>
+        <f>[2]Summary!R7</f>
         <v>0</v>
       </c>
       <c r="E5" s="21">
@@ -2778,10 +2778,10 @@
       <c r="A6" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="B6" s="72" t="s">
+      <c r="B6" s="76" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="71"/>
+      <c r="C6" s="68"/>
       <c r="D6" s="25" t="s">
         <v>94</v>
       </c>
@@ -2791,16 +2791,16 @@
       <c r="F6" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="73" t="s">
+      <c r="G6" s="77" t="s">
         <v>97</v>
       </c>
-      <c r="H6" s="68"/>
-      <c r="I6" s="71"/>
-      <c r="J6" s="73" t="s">
+      <c r="H6" s="67"/>
+      <c r="I6" s="68"/>
+      <c r="J6" s="77" t="s">
         <v>38</v>
       </c>
-      <c r="K6" s="68"/>
-      <c r="L6" s="71"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="68"/>
       <c r="M6" s="28" t="s">
         <v>98</v>
       </c>
@@ -2823,13 +2823,13 @@
       <c r="T6" s="66" t="s">
         <v>103</v>
       </c>
-      <c r="U6" s="68"/>
-      <c r="V6" s="71"/>
+      <c r="U6" s="67"/>
+      <c r="V6" s="68"/>
       <c r="W6" s="66" t="s">
         <v>104</v>
       </c>
-      <c r="X6" s="68"/>
-      <c r="Y6" s="71"/>
+      <c r="X6" s="67"/>
+      <c r="Y6" s="68"/>
       <c r="Z6" s="31" t="s">
         <v>101</v>
       </c>
@@ -2950,16 +2950,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A3:Z3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="F4:R4"/>
+    <mergeCell ref="T4:Z4"/>
+    <mergeCell ref="A5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="G6:I6"/>
     <mergeCell ref="J6:L6"/>
     <mergeCell ref="T6:V6"/>
     <mergeCell ref="W6:Y6"/>
-    <mergeCell ref="A3:Z3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="F4:R4"/>
-    <mergeCell ref="T4:Z4"/>
-    <mergeCell ref="A5:C5"/>
   </mergeCells>
   <conditionalFormatting sqref="B11">
     <cfRule type="duplicateValues" dxfId="5" priority="2"/>
@@ -2978,58 +2978,58 @@
   <sheetData>
     <row r="1" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A1" s="66"/>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
-      <c r="AD1" s="67"/>
-      <c r="AE1" s="67"/>
-      <c r="AF1" s="67"/>
-      <c r="AG1" s="67"/>
-      <c r="AH1" s="67"/>
-      <c r="AI1" s="67"/>
-      <c r="AJ1" s="67"/>
-      <c r="AK1" s="67"/>
-      <c r="AL1" s="68"/>
-      <c r="AM1" s="68"/>
-      <c r="AN1" s="68"/>
-      <c r="AO1" s="68"/>
-      <c r="AP1" s="68"/>
-      <c r="AQ1" s="67"/>
-      <c r="AR1" s="67"/>
-      <c r="AS1" s="67"/>
-      <c r="AT1" s="67"/>
-      <c r="AU1" s="67"/>
-      <c r="AV1" s="67"/>
-      <c r="AW1" s="67"/>
-      <c r="AX1" s="67"/>
-      <c r="AY1" s="67"/>
-      <c r="AZ1" s="67"/>
-      <c r="BA1" s="69"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
+      <c r="AD1" s="69"/>
+      <c r="AE1" s="69"/>
+      <c r="AF1" s="69"/>
+      <c r="AG1" s="69"/>
+      <c r="AH1" s="69"/>
+      <c r="AI1" s="69"/>
+      <c r="AJ1" s="69"/>
+      <c r="AK1" s="69"/>
+      <c r="AL1" s="67"/>
+      <c r="AM1" s="67"/>
+      <c r="AN1" s="67"/>
+      <c r="AO1" s="67"/>
+      <c r="AP1" s="67"/>
+      <c r="AQ1" s="69"/>
+      <c r="AR1" s="69"/>
+      <c r="AS1" s="69"/>
+      <c r="AT1" s="69"/>
+      <c r="AU1" s="69"/>
+      <c r="AV1" s="69"/>
+      <c r="AW1" s="69"/>
+      <c r="AX1" s="69"/>
+      <c r="AY1" s="69"/>
+      <c r="AZ1" s="69"/>
+      <c r="BA1" s="70"/>
     </row>
     <row r="2" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -3427,185 +3427,185 @@
     </row>
     <row r="3" spans="1:53" x14ac:dyDescent="0.35">
       <c r="A3" s="66" t="str">
-        <f>+[2]Summary!A4</f>
+        <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="67"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
-      <c r="L3" s="67"/>
-      <c r="M3" s="67"/>
-      <c r="N3" s="67"/>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="67"/>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-      <c r="V3" s="67"/>
-      <c r="W3" s="67"/>
-      <c r="X3" s="67"/>
-      <c r="Y3" s="67"/>
-      <c r="Z3" s="67"/>
-      <c r="AA3" s="67"/>
-      <c r="AB3" s="67"/>
-      <c r="AC3" s="67"/>
-      <c r="AD3" s="67"/>
-      <c r="AE3" s="67"/>
-      <c r="AF3" s="67"/>
-      <c r="AG3" s="67"/>
-      <c r="AH3" s="67"/>
-      <c r="AI3" s="67"/>
-      <c r="AJ3" s="67"/>
-      <c r="AK3" s="67"/>
-      <c r="AL3" s="68"/>
-      <c r="AM3" s="68"/>
-      <c r="AN3" s="68"/>
-      <c r="AO3" s="68"/>
-      <c r="AP3" s="68"/>
-      <c r="AQ3" s="67"/>
-      <c r="AR3" s="67"/>
-      <c r="AS3" s="67"/>
-      <c r="AT3" s="67"/>
-      <c r="AU3" s="67"/>
-      <c r="AV3" s="67"/>
-      <c r="AW3" s="67"/>
-      <c r="AX3" s="67"/>
-      <c r="AY3" s="67"/>
-      <c r="AZ3" s="67"/>
-      <c r="BA3" s="69"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="69"/>
+      <c r="I3" s="69"/>
+      <c r="J3" s="69"/>
+      <c r="K3" s="69"/>
+      <c r="L3" s="69"/>
+      <c r="M3" s="69"/>
+      <c r="N3" s="69"/>
+      <c r="O3" s="69"/>
+      <c r="P3" s="69"/>
+      <c r="Q3" s="69"/>
+      <c r="R3" s="69"/>
+      <c r="S3" s="69"/>
+      <c r="T3" s="69"/>
+      <c r="U3" s="69"/>
+      <c r="V3" s="69"/>
+      <c r="W3" s="69"/>
+      <c r="X3" s="69"/>
+      <c r="Y3" s="69"/>
+      <c r="Z3" s="69"/>
+      <c r="AA3" s="69"/>
+      <c r="AB3" s="69"/>
+      <c r="AC3" s="69"/>
+      <c r="AD3" s="69"/>
+      <c r="AE3" s="69"/>
+      <c r="AF3" s="69"/>
+      <c r="AG3" s="69"/>
+      <c r="AH3" s="69"/>
+      <c r="AI3" s="69"/>
+      <c r="AJ3" s="69"/>
+      <c r="AK3" s="69"/>
+      <c r="AL3" s="67"/>
+      <c r="AM3" s="67"/>
+      <c r="AN3" s="67"/>
+      <c r="AO3" s="67"/>
+      <c r="AP3" s="67"/>
+      <c r="AQ3" s="69"/>
+      <c r="AR3" s="69"/>
+      <c r="AS3" s="69"/>
+      <c r="AT3" s="69"/>
+      <c r="AU3" s="69"/>
+      <c r="AV3" s="69"/>
+      <c r="AW3" s="69"/>
+      <c r="AX3" s="69"/>
+      <c r="AY3" s="69"/>
+      <c r="AZ3" s="69"/>
+      <c r="BA3" s="70"/>
     </row>
     <row r="4" spans="1:53" x14ac:dyDescent="0.35">
       <c r="A4" s="66">
-        <f>+[2]Summary!A7</f>
+        <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="67"/>
-      <c r="C4" s="67"/>
-      <c r="D4" s="67"/>
-      <c r="E4" s="67"/>
-      <c r="F4" s="67"/>
-      <c r="G4" s="67"/>
-      <c r="H4" s="67"/>
-      <c r="I4" s="67"/>
-      <c r="J4" s="67"/>
-      <c r="K4" s="67"/>
-      <c r="L4" s="67"/>
-      <c r="M4" s="67"/>
-      <c r="N4" s="67"/>
-      <c r="O4" s="67"/>
-      <c r="P4" s="67"/>
-      <c r="Q4" s="67"/>
-      <c r="R4" s="67"/>
-      <c r="S4" s="67"/>
-      <c r="T4" s="67"/>
-      <c r="U4" s="67"/>
-      <c r="V4" s="67"/>
-      <c r="W4" s="67"/>
-      <c r="X4" s="67"/>
-      <c r="Y4" s="67"/>
-      <c r="Z4" s="67"/>
-      <c r="AA4" s="67"/>
-      <c r="AB4" s="67"/>
-      <c r="AC4" s="67"/>
-      <c r="AD4" s="67"/>
-      <c r="AE4" s="67"/>
-      <c r="AF4" s="67"/>
-      <c r="AG4" s="67"/>
-      <c r="AH4" s="67"/>
-      <c r="AI4" s="67"/>
-      <c r="AJ4" s="67"/>
-      <c r="AK4" s="67"/>
-      <c r="AL4" s="68"/>
-      <c r="AM4" s="68"/>
-      <c r="AN4" s="68"/>
-      <c r="AO4" s="68"/>
-      <c r="AP4" s="68"/>
-      <c r="AQ4" s="67"/>
-      <c r="AR4" s="67"/>
-      <c r="AS4" s="67"/>
-      <c r="AT4" s="67"/>
-      <c r="AU4" s="67"/>
-      <c r="AV4" s="67"/>
-      <c r="AW4" s="67"/>
-      <c r="AX4" s="67"/>
-      <c r="AY4" s="67"/>
-      <c r="AZ4" s="67"/>
-      <c r="BA4" s="69"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="69"/>
+      <c r="D4" s="69"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="69"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="69"/>
+      <c r="J4" s="69"/>
+      <c r="K4" s="69"/>
+      <c r="L4" s="69"/>
+      <c r="M4" s="69"/>
+      <c r="N4" s="69"/>
+      <c r="O4" s="69"/>
+      <c r="P4" s="69"/>
+      <c r="Q4" s="69"/>
+      <c r="R4" s="69"/>
+      <c r="S4" s="69"/>
+      <c r="T4" s="69"/>
+      <c r="U4" s="69"/>
+      <c r="V4" s="69"/>
+      <c r="W4" s="69"/>
+      <c r="X4" s="69"/>
+      <c r="Y4" s="69"/>
+      <c r="Z4" s="69"/>
+      <c r="AA4" s="69"/>
+      <c r="AB4" s="69"/>
+      <c r="AC4" s="69"/>
+      <c r="AD4" s="69"/>
+      <c r="AE4" s="69"/>
+      <c r="AF4" s="69"/>
+      <c r="AG4" s="69"/>
+      <c r="AH4" s="69"/>
+      <c r="AI4" s="69"/>
+      <c r="AJ4" s="69"/>
+      <c r="AK4" s="69"/>
+      <c r="AL4" s="67"/>
+      <c r="AM4" s="67"/>
+      <c r="AN4" s="67"/>
+      <c r="AO4" s="67"/>
+      <c r="AP4" s="67"/>
+      <c r="AQ4" s="69"/>
+      <c r="AR4" s="69"/>
+      <c r="AS4" s="69"/>
+      <c r="AT4" s="69"/>
+      <c r="AU4" s="69"/>
+      <c r="AV4" s="69"/>
+      <c r="AW4" s="69"/>
+      <c r="AX4" s="69"/>
+      <c r="AY4" s="69"/>
+      <c r="AZ4" s="69"/>
+      <c r="BA4" s="70"/>
     </row>
     <row r="5" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="66" t="s">
         <v>114</v>
       </c>
-      <c r="B5" s="67"/>
-      <c r="C5" s="67"/>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="67"/>
-      <c r="H5" s="67"/>
-      <c r="I5" s="67"/>
-      <c r="J5" s="67"/>
-      <c r="K5" s="67"/>
-      <c r="L5" s="67"/>
-      <c r="M5" s="67"/>
-      <c r="N5" s="67"/>
-      <c r="O5" s="67"/>
-      <c r="P5" s="67"/>
-      <c r="Q5" s="67"/>
-      <c r="R5" s="67"/>
-      <c r="S5" s="69"/>
+      <c r="B5" s="69"/>
+      <c r="C5" s="69"/>
+      <c r="D5" s="69"/>
+      <c r="E5" s="69"/>
+      <c r="F5" s="69"/>
+      <c r="G5" s="69"/>
+      <c r="H5" s="69"/>
+      <c r="I5" s="69"/>
+      <c r="J5" s="69"/>
+      <c r="K5" s="69"/>
+      <c r="L5" s="69"/>
+      <c r="M5" s="69"/>
+      <c r="N5" s="69"/>
+      <c r="O5" s="69"/>
+      <c r="P5" s="69"/>
+      <c r="Q5" s="69"/>
+      <c r="R5" s="69"/>
+      <c r="S5" s="70"/>
       <c r="T5" s="66" t="s">
         <v>115</v>
       </c>
-      <c r="U5" s="67"/>
-      <c r="V5" s="67"/>
-      <c r="W5" s="67"/>
-      <c r="X5" s="67"/>
-      <c r="Y5" s="67"/>
-      <c r="Z5" s="67"/>
-      <c r="AA5" s="67"/>
-      <c r="AB5" s="67"/>
-      <c r="AC5" s="67"/>
-      <c r="AD5" s="67"/>
-      <c r="AE5" s="67"/>
-      <c r="AF5" s="67"/>
-      <c r="AG5" s="67"/>
-      <c r="AH5" s="67"/>
-      <c r="AI5" s="67"/>
-      <c r="AJ5" s="67"/>
-      <c r="AK5" s="69"/>
+      <c r="U5" s="69"/>
+      <c r="V5" s="69"/>
+      <c r="W5" s="69"/>
+      <c r="X5" s="69"/>
+      <c r="Y5" s="69"/>
+      <c r="Z5" s="69"/>
+      <c r="AA5" s="69"/>
+      <c r="AB5" s="69"/>
+      <c r="AC5" s="69"/>
+      <c r="AD5" s="69"/>
+      <c r="AE5" s="69"/>
+      <c r="AF5" s="69"/>
+      <c r="AG5" s="69"/>
+      <c r="AH5" s="69"/>
+      <c r="AI5" s="69"/>
+      <c r="AJ5" s="69"/>
+      <c r="AK5" s="70"/>
       <c r="AL5" s="66" t="s">
         <v>116</v>
       </c>
-      <c r="AM5" s="68"/>
-      <c r="AN5" s="68"/>
-      <c r="AO5" s="68"/>
-      <c r="AP5" s="71"/>
+      <c r="AM5" s="67"/>
+      <c r="AN5" s="67"/>
+      <c r="AO5" s="67"/>
+      <c r="AP5" s="68"/>
       <c r="AQ5" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="AR5" s="67"/>
-      <c r="AS5" s="67"/>
-      <c r="AT5" s="69"/>
+      <c r="AR5" s="69"/>
+      <c r="AS5" s="69"/>
+      <c r="AT5" s="70"/>
       <c r="AU5" s="27" t="s">
         <v>117</v>
       </c>
       <c r="AV5" s="66" t="s">
         <v>118</v>
       </c>
-      <c r="AW5" s="67"/>
-      <c r="AX5" s="67"/>
-      <c r="AY5" s="67"/>
-      <c r="AZ5" s="69"/>
+      <c r="AW5" s="69"/>
+      <c r="AX5" s="69"/>
+      <c r="AY5" s="69"/>
+      <c r="AZ5" s="70"/>
       <c r="BA5" s="27" t="s">
         <v>119</v>
       </c>
@@ -3623,24 +3623,24 @@
       <c r="D6" s="50"/>
       <c r="E6" s="50"/>
       <c r="F6" s="50"/>
-      <c r="G6" s="74" t="s">
+      <c r="G6" s="71" t="s">
         <v>82</v>
       </c>
-      <c r="H6" s="75"/>
-      <c r="I6" s="75"/>
-      <c r="J6" s="76"/>
-      <c r="K6" s="74" t="s">
+      <c r="H6" s="72"/>
+      <c r="I6" s="72"/>
+      <c r="J6" s="73"/>
+      <c r="K6" s="71" t="s">
         <v>121</v>
       </c>
-      <c r="L6" s="75"/>
-      <c r="M6" s="75"/>
-      <c r="N6" s="76"/>
-      <c r="O6" s="77" t="s">
+      <c r="L6" s="72"/>
+      <c r="M6" s="72"/>
+      <c r="N6" s="73"/>
+      <c r="O6" s="74" t="s">
         <v>122</v>
       </c>
-      <c r="P6" s="67"/>
-      <c r="Q6" s="67"/>
-      <c r="R6" s="69"/>
+      <c r="P6" s="69"/>
+      <c r="Q6" s="69"/>
+      <c r="R6" s="70"/>
       <c r="S6" s="51" t="s">
         <v>123</v>
       </c>
@@ -3653,8 +3653,8 @@
       <c r="V6" s="66" t="s">
         <v>125</v>
       </c>
-      <c r="W6" s="67"/>
-      <c r="X6" s="69"/>
+      <c r="W6" s="69"/>
+      <c r="X6" s="70"/>
       <c r="Y6" s="52" t="s">
         <v>126</v>
       </c>
@@ -3679,14 +3679,14 @@
       <c r="AF6" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="AG6" s="78" t="s">
+      <c r="AG6" s="75" t="s">
         <v>134</v>
       </c>
-      <c r="AH6" s="69"/>
+      <c r="AH6" s="70"/>
       <c r="AI6" s="66" t="s">
         <v>135</v>
       </c>
-      <c r="AJ6" s="69"/>
+      <c r="AJ6" s="70"/>
       <c r="AK6" s="27" t="s">
         <v>101</v>
       </c>
@@ -3871,6 +3871,10 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A3:BA3"/>
+    <mergeCell ref="A4:BA4"/>
+    <mergeCell ref="A5:S5"/>
+    <mergeCell ref="T5:AK5"/>
     <mergeCell ref="AL5:AP5"/>
     <mergeCell ref="AQ5:AT5"/>
     <mergeCell ref="AV5:AZ5"/>
@@ -3880,10 +3884,6 @@
     <mergeCell ref="V6:X6"/>
     <mergeCell ref="AG6:AH6"/>
     <mergeCell ref="AI6:AJ6"/>
-    <mergeCell ref="A3:BA3"/>
-    <mergeCell ref="A4:BA4"/>
-    <mergeCell ref="A5:S5"/>
-    <mergeCell ref="T5:AK5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3906,18 +3906,18 @@
       <c r="B3" s="82" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="68"/>
-      <c r="D3" s="71"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="68"/>
       <c r="E3" s="82" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="68"/>
-      <c r="G3" s="71"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="68"/>
       <c r="H3" s="82" t="s">
         <v>38</v>
       </c>
-      <c r="I3" s="68"/>
-      <c r="J3" s="71"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="68"/>
       <c r="K3" s="81" t="s">
         <v>75</v>
       </c>

</xml_diff>

<commit_message>
Auto pipeline update 2026-04-15 12:12:08
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -8,26 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A66FAB75-312A-4960-A195-5DB0FF064ABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FFF31B4-0A06-4209-B1D6-13BB5BF991C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" firstSheet="2" activeTab="7" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet Names Check" sheetId="1" r:id="rId1"/>
-    <sheet name="TB 501 132kV Stringing" sheetId="11" r:id="rId2"/>
+    <sheet name="TA 601 Stringing" sheetId="12" r:id="rId2"/>
     <sheet name="TB 501 220kV Stringing" sheetId="10" r:id="rId3"/>
-    <sheet name="TB 501 220kV Erection" sheetId="9" r:id="rId4"/>
-    <sheet name="TB 501 132kV Erection" sheetId="8" r:id="rId5"/>
-    <sheet name="TB 401 Stringing" sheetId="6" r:id="rId6"/>
-    <sheet name="TB 408 Stringing" sheetId="2" r:id="rId7"/>
-    <sheet name="TA 509 Erection" sheetId="3" r:id="rId8"/>
-    <sheet name="TA 601 Erection" sheetId="7" r:id="rId9"/>
+    <sheet name="TB 501 132kV Stringing" sheetId="11" r:id="rId4"/>
+    <sheet name="TB 501 220kV Erection" sheetId="9" r:id="rId5"/>
+    <sheet name="TB 501 132kV Erection" sheetId="8" r:id="rId6"/>
+    <sheet name="TB 401 Stringing" sheetId="6" r:id="rId7"/>
+    <sheet name="TB 408 Stringing" sheetId="2" r:id="rId8"/>
+    <sheet name="TA 509 Erection" sheetId="3" r:id="rId9"/>
+    <sheet name="TA 601 Erection" sheetId="7" r:id="rId10"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId10"/>
     <externalReference r:id="rId11"/>
+    <externalReference r:id="rId12"/>
   </externalReferences>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="179">
   <si>
     <t>Project Code</t>
   </si>
@@ -105,9 +106,6 @@
   </si>
   <si>
     <t>TA 421</t>
-  </si>
-  <si>
-    <t>Stringing compliled</t>
   </si>
   <si>
     <t xml:space="preserve">Erection Compiled </t>
@@ -591,6 +589,9 @@
   </si>
   <si>
     <t>Total Steel (Kgs)</t>
+  </si>
+  <si>
+    <t>Stringing compiled</t>
   </si>
 </sst>
 </file>
@@ -603,7 +604,7 @@
     <numFmt numFmtId="166" formatCode="[$-4009]0.00"/>
     <numFmt numFmtId="167" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -688,6 +689,12 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="11">
@@ -1199,7 +1206,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="8">
+  <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -1208,8 +1215,9 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1400,11 +1408,68 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="23" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="26" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1426,15 +1491,6 @@
     <xf numFmtId="166" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1470,7 +1526,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="8">
+  <cellStyles count="9">
     <cellStyle name="Comma 2" xfId="5" xr:uid="{1517F127-7F55-42AF-952C-D923BD4ECBE3}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 15" xfId="1" xr:uid="{34FE60CE-A1DA-4616-AA23-0BBDDF9DD7D6}"/>
@@ -1478,6 +1534,7 @@
     <cellStyle name="Normal 3" xfId="6" xr:uid="{02E4DB69-C37B-458C-97B6-3E554FA1E55A}"/>
     <cellStyle name="Normal 4" xfId="7" xr:uid="{91588BA5-8ED7-4728-AC43-559C5A5DAACB}"/>
     <cellStyle name="Normal 5" xfId="3" xr:uid="{72642DE1-8DD2-444D-8A81-E2A5D7BD22B8}"/>
+    <cellStyle name="Normal 6" xfId="8" xr:uid="{E2AC1BB0-A24A-450A-B605-14A01490AC0E}"/>
     <cellStyle name="Normal 8 2" xfId="2" xr:uid="{E356B690-246D-43B2-86AF-A6FE97B16461}"/>
   </cellStyles>
   <dxfs count="8">
@@ -1602,6 +1659,11 @@
       <sheetData sheetId="2" refreshError="1"/>
       <sheetData sheetId="3" refreshError="1"/>
       <sheetData sheetId="4">
+        <row r="2">
+          <cell r="A2" t="str">
+            <v>Name of the Line: 220KV DC AL59 line from Neemuch - Chanderiya + 132KV DC ACSS Line from Chanderiya to Hindustan Zinc</v>
+          </cell>
+        </row>
         <row r="4">
           <cell r="A4" t="str">
             <v>Office:  Neemuch</v>
@@ -1650,11 +1712,6 @@
       <sheetData sheetId="2" refreshError="1"/>
       <sheetData sheetId="3" refreshError="1"/>
       <sheetData sheetId="4">
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>Name of the Line: 220KV DC AL59 line from Neemuch - Chanderiya + 132KV DC ACSS Line from Chanderiya to Hindustan Zinc</v>
-          </cell>
-        </row>
         <row r="4">
           <cell r="A4" t="str">
             <v>Office:  Neemuch</v>
@@ -1677,7 +1734,6 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DBDF0E1F-C881-4514-9437-5BEB0B253989}" name="Table1" displayName="Table1" ref="A1:G22" totalsRowShown="0">
-  <autoFilter ref="A1:G22" xr:uid="{DBDF0E1F-C881-4514-9437-5BEB0B253989}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{1C0814EE-AA83-4802-806C-8F58A35BCB7F}" name="Project Code"/>
     <tableColumn id="2" xr3:uid="{648AD748-C4AF-4406-94C1-AD47F69D9A33}" name="Erection Sheet Names"/>
@@ -2013,7 +2069,7 @@
   <cols>
     <col min="1" max="1" width="10.453125" customWidth="1"/>
     <col min="2" max="2" width="28.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.453125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.7265625" bestFit="1" customWidth="1"/>
   </cols>
@@ -2029,16 +2085,16 @@
         <v>5</v>
       </c>
       <c r="D1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E1" t="s">
         <v>70</v>
       </c>
-      <c r="E1" t="s">
-        <v>71</v>
-      </c>
       <c r="F1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -2049,7 +2105,7 @@
         <v>3</v>
       </c>
       <c r="F2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -2150,18 +2206,18 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>19</v>
+        <v>178</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
         <v>6</v>
@@ -2172,7 +2228,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14" t="s">
         <v>6</v>
@@ -2181,26 +2237,26 @@
         <v>11</v>
       </c>
       <c r="E14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
         <v>6</v>
       </c>
       <c r="C15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" t="s">
         <v>25</v>
-      </c>
-      <c r="B16" t="s">
-        <v>26</v>
       </c>
       <c r="C16" t="s">
         <v>9</v>
@@ -2208,18 +2264,18 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B17" t="s">
         <v>2</v>
       </c>
       <c r="D17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B18" t="s">
         <v>6</v>
@@ -2228,43 +2284,43 @@
         <v>9</v>
       </c>
       <c r="D18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F19" t="s">
+        <v>86</v>
+      </c>
+      <c r="G19" t="s">
         <v>87</v>
-      </c>
-      <c r="G19" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B21" t="s">
         <v>6</v>
@@ -2278,90 +2334,464 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46CC22E7-0431-4564-825A-DCAC81041178}">
+  <dimension ref="A1:P5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="26" x14ac:dyDescent="0.35">
+      <c r="A2" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="G2" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C3" s="7"/>
+      <c r="D3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="106"/>
+      <c r="H3" s="107"/>
+      <c r="I3" s="107"/>
+      <c r="J3" s="108"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="106"/>
+      <c r="O3" s="107"/>
+      <c r="P3" s="108"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="N3:P3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAEF05BD-52B1-49ED-A017-76486C00039F}">
-  <dimension ref="A2:Z16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7C2946C-A784-4830-B129-5E94E117C5CC}">
+  <dimension ref="A2:Z11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="2" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="76" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="77" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="77" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="77" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="78" t="s">
+        <v>107</v>
+      </c>
+      <c r="G3" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="H3" s="44" t="s">
+        <v>95</v>
+      </c>
+      <c r="I3" s="79" t="s">
+        <v>48</v>
+      </c>
+      <c r="J3" s="78" t="s">
+        <v>49</v>
+      </c>
+      <c r="K3" s="77" t="s">
+        <v>50</v>
+      </c>
+      <c r="L3" s="78" t="s">
+        <v>51</v>
+      </c>
+      <c r="M3" s="80" t="s">
+        <v>52</v>
+      </c>
+      <c r="N3" s="76" t="s">
+        <v>109</v>
+      </c>
+      <c r="O3" s="81" t="s">
+        <v>110</v>
+      </c>
+      <c r="P3" s="82" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q3" s="83" t="s">
+        <v>53</v>
+      </c>
+      <c r="R3" s="77" t="s">
+        <v>54</v>
+      </c>
+      <c r="S3" s="77" t="s">
+        <v>34</v>
+      </c>
+      <c r="T3" s="77" t="s">
+        <v>80</v>
+      </c>
+      <c r="U3" s="77" t="s">
+        <v>111</v>
+      </c>
+      <c r="V3" s="77" t="s">
+        <v>112</v>
+      </c>
+      <c r="W3" s="82" t="s">
+        <v>42</v>
+      </c>
+      <c r="X3" s="74"/>
+      <c r="Y3" s="74"/>
+      <c r="Z3" s="74"/>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A4" s="69"/>
+      <c r="B4" s="74"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="74"/>
+      <c r="H4" s="74"/>
+      <c r="I4" s="74"/>
+      <c r="J4" s="74"/>
+      <c r="K4" s="74"/>
+      <c r="L4" s="74"/>
+      <c r="M4" s="74"/>
+      <c r="N4" s="74"/>
+      <c r="O4" s="74"/>
+      <c r="P4" s="74"/>
+      <c r="Q4" s="74"/>
+      <c r="R4" s="74"/>
+      <c r="S4" s="66"/>
+      <c r="T4" s="69"/>
+      <c r="U4" s="74"/>
+      <c r="V4" s="74"/>
+      <c r="W4" s="74"/>
+      <c r="X4" s="74"/>
+      <c r="Y4" s="74"/>
+      <c r="Z4" s="74"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A5" s="69"/>
+      <c r="B5" s="74"/>
+      <c r="C5" s="74"/>
+      <c r="D5" s="67"/>
+      <c r="E5" s="68"/>
+      <c r="F5" s="69"/>
+      <c r="G5" s="69"/>
+      <c r="H5" s="68"/>
+      <c r="I5" s="68"/>
+      <c r="J5" s="69"/>
+      <c r="K5" s="68"/>
+      <c r="L5" s="68"/>
+      <c r="M5" s="69"/>
+      <c r="N5" s="69"/>
+      <c r="O5" s="69"/>
+      <c r="P5" s="69"/>
+      <c r="Q5" s="69"/>
+      <c r="R5" s="69"/>
+      <c r="S5" s="69"/>
+      <c r="T5" s="69"/>
+      <c r="U5" s="68"/>
+      <c r="V5" s="68"/>
+      <c r="W5" s="68"/>
+      <c r="X5" s="68"/>
+      <c r="Y5" s="68"/>
+      <c r="Z5" s="69"/>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A6" s="70"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="70"/>
+      <c r="E6" s="70"/>
+      <c r="F6" s="70"/>
+      <c r="G6" s="75"/>
+      <c r="H6" s="74"/>
+      <c r="I6" s="74"/>
+      <c r="J6" s="75"/>
+      <c r="K6" s="74"/>
+      <c r="L6" s="74"/>
+      <c r="M6" s="71"/>
+      <c r="N6" s="70"/>
+      <c r="O6" s="72"/>
+      <c r="P6" s="70"/>
+      <c r="Q6" s="71"/>
+      <c r="R6" s="70"/>
+      <c r="S6" s="70"/>
+      <c r="T6" s="63"/>
+      <c r="U6" s="74"/>
+      <c r="V6" s="74"/>
+      <c r="W6" s="63"/>
+      <c r="X6" s="74"/>
+      <c r="Y6" s="74"/>
+      <c r="Z6" s="70"/>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A7" s="70"/>
+      <c r="B7" s="73"/>
+      <c r="C7" s="73"/>
+      <c r="D7" s="70"/>
+      <c r="E7" s="70"/>
+      <c r="F7" s="70"/>
+      <c r="G7" s="72"/>
+      <c r="H7" s="73"/>
+      <c r="I7" s="72"/>
+      <c r="J7" s="72"/>
+      <c r="K7" s="72"/>
+      <c r="L7" s="72"/>
+      <c r="M7" s="72"/>
+      <c r="N7" s="72"/>
+      <c r="O7" s="72"/>
+      <c r="P7" s="70"/>
+      <c r="Q7" s="71"/>
+      <c r="R7" s="70"/>
+      <c r="S7" s="70"/>
+      <c r="T7" s="72"/>
+      <c r="U7" s="72"/>
+      <c r="V7" s="72"/>
+      <c r="W7" s="72"/>
+      <c r="X7" s="72"/>
+      <c r="Y7" s="72"/>
+      <c r="Z7" s="70"/>
+    </row>
+    <row r="9" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="10" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>68</v>
+      </c>
+      <c r="N10" s="40"/>
+    </row>
+    <row r="11" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="76" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="77" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="77" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="77" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="78" t="s">
+        <v>107</v>
+      </c>
+      <c r="G11" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="H11" s="44" t="s">
+        <v>95</v>
+      </c>
+      <c r="I11" s="79" t="s">
+        <v>48</v>
+      </c>
+      <c r="J11" s="78" t="s">
+        <v>49</v>
+      </c>
+      <c r="K11" s="77" t="s">
+        <v>50</v>
+      </c>
+      <c r="L11" s="78" t="s">
+        <v>51</v>
+      </c>
+      <c r="M11" s="80" t="s">
+        <v>52</v>
+      </c>
+      <c r="N11" s="76" t="s">
+        <v>109</v>
+      </c>
+      <c r="O11" s="81" t="s">
+        <v>110</v>
+      </c>
+      <c r="P11" s="82" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q11" s="83" t="s">
+        <v>53</v>
+      </c>
+      <c r="R11" s="77" t="s">
+        <v>54</v>
+      </c>
+      <c r="S11" s="77" t="s">
+        <v>34</v>
+      </c>
+      <c r="T11" s="77" t="s">
+        <v>80</v>
+      </c>
+      <c r="U11" s="77" t="s">
+        <v>111</v>
+      </c>
+      <c r="V11" s="77" t="s">
+        <v>112</v>
+      </c>
+      <c r="W11" s="82" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9301C2D9-B641-4509-82EB-A6381EB78A1E}">
+  <dimension ref="A2:Z11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="78" t="str">
-        <f>+[2]Summary!A4</f>
+      <c r="A3" s="89" t="str">
+        <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="67"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
-      <c r="L3" s="67"/>
-      <c r="M3" s="67"/>
-      <c r="N3" s="67"/>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="67"/>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-      <c r="V3" s="67"/>
-      <c r="W3" s="67"/>
-      <c r="X3" s="67"/>
-      <c r="Y3" s="67"/>
-      <c r="Z3" s="68"/>
+      <c r="B3" s="87"/>
+      <c r="C3" s="87"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
+      <c r="G3" s="87"/>
+      <c r="H3" s="87"/>
+      <c r="I3" s="87"/>
+      <c r="J3" s="87"/>
+      <c r="K3" s="87"/>
+      <c r="L3" s="87"/>
+      <c r="M3" s="87"/>
+      <c r="N3" s="87"/>
+      <c r="O3" s="87"/>
+      <c r="P3" s="87"/>
+      <c r="Q3" s="87"/>
+      <c r="R3" s="87"/>
+      <c r="S3" s="87"/>
+      <c r="T3" s="87"/>
+      <c r="U3" s="87"/>
+      <c r="V3" s="87"/>
+      <c r="W3" s="87"/>
+      <c r="X3" s="87"/>
+      <c r="Y3" s="87"/>
+      <c r="Z3" s="85"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="78">
-        <f>+[2]Summary!A7</f>
+      <c r="A4" s="89">
+        <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="67"/>
-      <c r="C4" s="67"/>
-      <c r="D4" s="68"/>
+      <c r="B4" s="87"/>
+      <c r="C4" s="87"/>
+      <c r="D4" s="85"/>
       <c r="E4" s="18"/>
-      <c r="F4" s="78" t="s">
+      <c r="F4" s="89" t="s">
+        <v>89</v>
+      </c>
+      <c r="G4" s="87"/>
+      <c r="H4" s="87"/>
+      <c r="I4" s="87"/>
+      <c r="J4" s="87"/>
+      <c r="K4" s="87"/>
+      <c r="L4" s="87"/>
+      <c r="M4" s="87"/>
+      <c r="N4" s="87"/>
+      <c r="O4" s="87"/>
+      <c r="P4" s="87"/>
+      <c r="Q4" s="87"/>
+      <c r="R4" s="85"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="G4" s="67"/>
-      <c r="H4" s="67"/>
-      <c r="I4" s="67"/>
-      <c r="J4" s="67"/>
-      <c r="K4" s="67"/>
-      <c r="L4" s="67"/>
-      <c r="M4" s="67"/>
-      <c r="N4" s="67"/>
-      <c r="O4" s="67"/>
-      <c r="P4" s="67"/>
-      <c r="Q4" s="67"/>
-      <c r="R4" s="68"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="78" t="s">
+      <c r="U4" s="87"/>
+      <c r="V4" s="87"/>
+      <c r="W4" s="87"/>
+      <c r="X4" s="87"/>
+      <c r="Y4" s="87"/>
+      <c r="Z4" s="85"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A5" s="89" t="s">
         <v>91</v>
       </c>
-      <c r="U4" s="67"/>
-      <c r="V4" s="67"/>
-      <c r="W4" s="67"/>
-      <c r="X4" s="67"/>
-      <c r="Y4" s="67"/>
-      <c r="Z4" s="68"/>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="78" t="s">
-        <v>92</v>
-      </c>
-      <c r="B5" s="67"/>
-      <c r="C5" s="68"/>
+      <c r="B5" s="87"/>
+      <c r="C5" s="85"/>
       <c r="D5" s="20">
-        <f>[2]Summary!R7</f>
+        <f>[1]Summary!R7</f>
         <v>0</v>
       </c>
       <c r="E5" s="21">
@@ -2416,203 +2846,176 @@
     </row>
     <row r="6" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="B6" s="84" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="85"/>
+      <c r="D6" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="B6" s="76" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="68"/>
-      <c r="D6" s="25" t="s">
+      <c r="E6" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="E6" s="26" t="s">
+      <c r="F6" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="G6" s="86" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="77" t="s">
+      <c r="H6" s="87"/>
+      <c r="I6" s="85"/>
+      <c r="J6" s="86" t="s">
+        <v>37</v>
+      </c>
+      <c r="K6" s="87"/>
+      <c r="L6" s="85"/>
+      <c r="M6" s="28" t="s">
         <v>97</v>
       </c>
-      <c r="H6" s="67"/>
-      <c r="I6" s="68"/>
-      <c r="J6" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="K6" s="67"/>
-      <c r="L6" s="68"/>
-      <c r="M6" s="28" t="s">
+      <c r="N6" s="29" t="s">
         <v>98</v>
       </c>
-      <c r="N6" s="29" t="s">
+      <c r="O6" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="O6" s="30" t="s">
+      <c r="P6" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="P6" s="31" t="s">
+      <c r="Q6" s="32" t="s">
         <v>101</v>
       </c>
-      <c r="Q6" s="32" t="s">
+      <c r="R6" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="S6" s="33"/>
+      <c r="T6" s="88" t="s">
         <v>102</v>
       </c>
-      <c r="R6" s="27" t="s">
-        <v>43</v>
-      </c>
-      <c r="S6" s="33"/>
-      <c r="T6" s="66" t="s">
+      <c r="U6" s="87"/>
+      <c r="V6" s="85"/>
+      <c r="W6" s="88" t="s">
         <v>103</v>
       </c>
-      <c r="U6" s="67"/>
-      <c r="V6" s="68"/>
-      <c r="W6" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="X6" s="67"/>
-      <c r="Y6" s="68"/>
+      <c r="X6" s="87"/>
+      <c r="Y6" s="85"/>
       <c r="Z6" s="31" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A7" s="25"/>
       <c r="B7" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="34" t="s">
         <v>39</v>
-      </c>
-      <c r="C7" s="34" t="s">
-        <v>40</v>
       </c>
       <c r="D7" s="25"/>
       <c r="E7" s="35"/>
       <c r="F7" s="36"/>
       <c r="G7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H7" s="37" t="s">
+        <v>104</v>
+      </c>
+      <c r="I7" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="I7" s="30" t="s">
-        <v>106</v>
-      </c>
       <c r="J7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K7" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="L7" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="L7" s="30" t="s">
-        <v>106</v>
-      </c>
       <c r="M7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="N7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="P7" s="31"/>
       <c r="Q7" s="38"/>
       <c r="R7" s="36"/>
       <c r="S7" s="39"/>
       <c r="T7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="U7" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="V7" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="V7" s="30" t="s">
-        <v>106</v>
-      </c>
       <c r="W7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="X7" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="Y7" s="30" t="s">
         <v>105</v>
-      </c>
-      <c r="Y7" s="30" t="s">
-        <v>106</v>
       </c>
       <c r="Z7" s="31"/>
     </row>
     <row r="10" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="40" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="41" t="s">
+      <c r="C11" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="41" t="s">
+      <c r="D11" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="E11" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="F11" s="44" t="s">
+        <v>95</v>
+      </c>
+      <c r="H11" s="45" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="43" t="s">
+      <c r="I11" s="42" t="s">
+        <v>49</v>
+      </c>
+      <c r="K11" s="42" t="s">
+        <v>51</v>
+      </c>
+      <c r="L11" s="46" t="s">
+        <v>52</v>
+      </c>
+      <c r="M11" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="N11" s="47" t="s">
+        <v>110</v>
+      </c>
+      <c r="O11" s="40" t="s">
         <v>109</v>
       </c>
-      <c r="F11" s="44" t="s">
-        <v>96</v>
-      </c>
-      <c r="H11" s="45" t="s">
-        <v>49</v>
-      </c>
-      <c r="I11" s="42" t="s">
-        <v>50</v>
-      </c>
-      <c r="K11" s="42" t="s">
-        <v>52</v>
-      </c>
-      <c r="L11" s="46" t="s">
-        <v>53</v>
-      </c>
-      <c r="M11" s="48" t="s">
-        <v>98</v>
-      </c>
-      <c r="N11" s="47" t="s">
-        <v>111</v>
-      </c>
-      <c r="O11" s="40" t="s">
-        <v>110</v>
-      </c>
       <c r="P11" s="41" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="R11" s="48" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="16" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="41" t="s">
-        <v>107</v>
-      </c>
-      <c r="F16" s="42" t="s">
-        <v>108</v>
-      </c>
-      <c r="K16" s="41" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q16" s="49" t="s">
-        <v>54</v>
-      </c>
-      <c r="R16" s="41" t="s">
-        <v>55</v>
-      </c>
-      <c r="T16" s="41" t="s">
-        <v>81</v>
-      </c>
-      <c r="U16" s="41" t="s">
-        <v>112</v>
-      </c>
-      <c r="V16" s="41" t="s">
-        <v>113</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -2638,90 +3041,90 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9301C2D9-B641-4509-82EB-A6381EB78A1E}">
-  <dimension ref="A2:Z11"/>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAEF05BD-52B1-49ED-A017-76486C00039F}">
+  <dimension ref="A2:Z16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="78" t="str">
-        <f>+[2]Summary!A4</f>
+      <c r="A3" s="89" t="str">
+        <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="67"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
-      <c r="L3" s="67"/>
-      <c r="M3" s="67"/>
-      <c r="N3" s="67"/>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="67"/>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-      <c r="V3" s="67"/>
-      <c r="W3" s="67"/>
-      <c r="X3" s="67"/>
-      <c r="Y3" s="67"/>
-      <c r="Z3" s="68"/>
+      <c r="B3" s="87"/>
+      <c r="C3" s="87"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
+      <c r="G3" s="87"/>
+      <c r="H3" s="87"/>
+      <c r="I3" s="87"/>
+      <c r="J3" s="87"/>
+      <c r="K3" s="87"/>
+      <c r="L3" s="87"/>
+      <c r="M3" s="87"/>
+      <c r="N3" s="87"/>
+      <c r="O3" s="87"/>
+      <c r="P3" s="87"/>
+      <c r="Q3" s="87"/>
+      <c r="R3" s="87"/>
+      <c r="S3" s="87"/>
+      <c r="T3" s="87"/>
+      <c r="U3" s="87"/>
+      <c r="V3" s="87"/>
+      <c r="W3" s="87"/>
+      <c r="X3" s="87"/>
+      <c r="Y3" s="87"/>
+      <c r="Z3" s="85"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="78">
-        <f>+[2]Summary!A7</f>
+      <c r="A4" s="89">
+        <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="67"/>
-      <c r="C4" s="67"/>
-      <c r="D4" s="68"/>
+      <c r="B4" s="87"/>
+      <c r="C4" s="87"/>
+      <c r="D4" s="85"/>
       <c r="E4" s="18"/>
-      <c r="F4" s="78" t="s">
+      <c r="F4" s="89" t="s">
+        <v>89</v>
+      </c>
+      <c r="G4" s="87"/>
+      <c r="H4" s="87"/>
+      <c r="I4" s="87"/>
+      <c r="J4" s="87"/>
+      <c r="K4" s="87"/>
+      <c r="L4" s="87"/>
+      <c r="M4" s="87"/>
+      <c r="N4" s="87"/>
+      <c r="O4" s="87"/>
+      <c r="P4" s="87"/>
+      <c r="Q4" s="87"/>
+      <c r="R4" s="85"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="G4" s="67"/>
-      <c r="H4" s="67"/>
-      <c r="I4" s="67"/>
-      <c r="J4" s="67"/>
-      <c r="K4" s="67"/>
-      <c r="L4" s="67"/>
-      <c r="M4" s="67"/>
-      <c r="N4" s="67"/>
-      <c r="O4" s="67"/>
-      <c r="P4" s="67"/>
-      <c r="Q4" s="67"/>
-      <c r="R4" s="68"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="78" t="s">
+      <c r="U4" s="87"/>
+      <c r="V4" s="87"/>
+      <c r="W4" s="87"/>
+      <c r="X4" s="87"/>
+      <c r="Y4" s="87"/>
+      <c r="Z4" s="85"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A5" s="89" t="s">
         <v>91</v>
       </c>
-      <c r="U4" s="67"/>
-      <c r="V4" s="67"/>
-      <c r="W4" s="67"/>
-      <c r="X4" s="67"/>
-      <c r="Y4" s="67"/>
-      <c r="Z4" s="68"/>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="78" t="s">
-        <v>92</v>
-      </c>
-      <c r="B5" s="67"/>
-      <c r="C5" s="68"/>
+      <c r="B5" s="87"/>
+      <c r="C5" s="85"/>
       <c r="D5" s="20">
-        <f>[2]Summary!R7</f>
+        <f>[1]Summary!R7</f>
         <v>0</v>
       </c>
       <c r="E5" s="21">
@@ -2776,176 +3179,203 @@
     </row>
     <row r="6" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="B6" s="84" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="85"/>
+      <c r="D6" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="B6" s="76" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="68"/>
-      <c r="D6" s="25" t="s">
+      <c r="E6" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="E6" s="26" t="s">
+      <c r="F6" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="G6" s="86" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="77" t="s">
+      <c r="H6" s="87"/>
+      <c r="I6" s="85"/>
+      <c r="J6" s="86" t="s">
+        <v>37</v>
+      </c>
+      <c r="K6" s="87"/>
+      <c r="L6" s="85"/>
+      <c r="M6" s="28" t="s">
         <v>97</v>
       </c>
-      <c r="H6" s="67"/>
-      <c r="I6" s="68"/>
-      <c r="J6" s="77" t="s">
-        <v>38</v>
-      </c>
-      <c r="K6" s="67"/>
-      <c r="L6" s="68"/>
-      <c r="M6" s="28" t="s">
+      <c r="N6" s="29" t="s">
         <v>98</v>
       </c>
-      <c r="N6" s="29" t="s">
+      <c r="O6" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="O6" s="30" t="s">
+      <c r="P6" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="P6" s="31" t="s">
+      <c r="Q6" s="32" t="s">
         <v>101</v>
       </c>
-      <c r="Q6" s="32" t="s">
+      <c r="R6" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="S6" s="33"/>
+      <c r="T6" s="88" t="s">
         <v>102</v>
       </c>
-      <c r="R6" s="27" t="s">
-        <v>43</v>
-      </c>
-      <c r="S6" s="33"/>
-      <c r="T6" s="66" t="s">
+      <c r="U6" s="87"/>
+      <c r="V6" s="85"/>
+      <c r="W6" s="88" t="s">
         <v>103</v>
       </c>
-      <c r="U6" s="67"/>
-      <c r="V6" s="68"/>
-      <c r="W6" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="X6" s="67"/>
-      <c r="Y6" s="68"/>
+      <c r="X6" s="87"/>
+      <c r="Y6" s="85"/>
       <c r="Z6" s="31" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A7" s="25"/>
       <c r="B7" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="34" t="s">
         <v>39</v>
-      </c>
-      <c r="C7" s="34" t="s">
-        <v>40</v>
       </c>
       <c r="D7" s="25"/>
       <c r="E7" s="35"/>
       <c r="F7" s="36"/>
       <c r="G7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H7" s="37" t="s">
+        <v>104</v>
+      </c>
+      <c r="I7" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="I7" s="30" t="s">
-        <v>106</v>
-      </c>
       <c r="J7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K7" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="L7" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="L7" s="30" t="s">
-        <v>106</v>
-      </c>
       <c r="M7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="N7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="P7" s="31"/>
       <c r="Q7" s="38"/>
       <c r="R7" s="36"/>
       <c r="S7" s="39"/>
       <c r="T7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="U7" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="V7" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="V7" s="30" t="s">
-        <v>106</v>
-      </c>
       <c r="W7" s="30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="X7" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="Y7" s="30" t="s">
         <v>105</v>
-      </c>
-      <c r="Y7" s="30" t="s">
-        <v>106</v>
       </c>
       <c r="Z7" s="31"/>
     </row>
     <row r="10" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="40" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="41" t="s">
+      <c r="C11" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="41" t="s">
+      <c r="D11" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="E11" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="F11" s="44" t="s">
+        <v>95</v>
+      </c>
+      <c r="H11" s="45" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="43" t="s">
+      <c r="I11" s="42" t="s">
+        <v>49</v>
+      </c>
+      <c r="K11" s="42" t="s">
+        <v>51</v>
+      </c>
+      <c r="L11" s="46" t="s">
+        <v>52</v>
+      </c>
+      <c r="M11" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="N11" s="47" t="s">
+        <v>110</v>
+      </c>
+      <c r="O11" s="40" t="s">
         <v>109</v>
       </c>
-      <c r="F11" s="44" t="s">
-        <v>96</v>
-      </c>
-      <c r="H11" s="45" t="s">
-        <v>49</v>
-      </c>
-      <c r="I11" s="42" t="s">
+      <c r="P11" s="41" t="s">
+        <v>34</v>
+      </c>
+      <c r="R11" s="48" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="16" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B16" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="F16" s="42" t="s">
+        <v>107</v>
+      </c>
+      <c r="K16" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="K11" s="42" t="s">
-        <v>52</v>
-      </c>
-      <c r="L11" s="46" t="s">
+      <c r="Q16" s="49" t="s">
         <v>53</v>
       </c>
-      <c r="M11" s="48" t="s">
-        <v>98</v>
-      </c>
-      <c r="N11" s="47" t="s">
+      <c r="R16" s="41" t="s">
+        <v>54</v>
+      </c>
+      <c r="T16" s="41" t="s">
+        <v>80</v>
+      </c>
+      <c r="U16" s="41" t="s">
         <v>111</v>
       </c>
-      <c r="O11" s="40" t="s">
-        <v>110</v>
-      </c>
-      <c r="P11" s="41" t="s">
-        <v>35</v>
-      </c>
-      <c r="R11" s="48" t="s">
-        <v>43</v>
+      <c r="V16" s="41" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -2971,147 +3401,147 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B501B5B8-47AF-4D49-A01B-A8E1BEE40158}">
   <dimension ref="A1:BM10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:65" x14ac:dyDescent="0.35">
-      <c r="A1" s="66"/>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
-      <c r="Q1" s="69"/>
-      <c r="R1" s="69"/>
-      <c r="S1" s="69"/>
-      <c r="T1" s="69"/>
-      <c r="U1" s="69"/>
-      <c r="V1" s="69"/>
-      <c r="W1" s="69"/>
-      <c r="X1" s="69"/>
-      <c r="Y1" s="69"/>
-      <c r="Z1" s="69"/>
-      <c r="AA1" s="69"/>
-      <c r="AB1" s="69"/>
-      <c r="AC1" s="69"/>
-      <c r="AD1" s="69"/>
-      <c r="AE1" s="69"/>
-      <c r="AF1" s="69"/>
-      <c r="AG1" s="69"/>
-      <c r="AH1" s="69"/>
-      <c r="AI1" s="69"/>
-      <c r="AJ1" s="69"/>
-      <c r="AK1" s="69"/>
-      <c r="AL1" s="67"/>
-      <c r="AM1" s="67"/>
-      <c r="AN1" s="67"/>
-      <c r="AO1" s="67"/>
-      <c r="AP1" s="67"/>
-      <c r="AQ1" s="69"/>
-      <c r="AR1" s="69"/>
-      <c r="AS1" s="69"/>
-      <c r="AT1" s="69"/>
-      <c r="AU1" s="69"/>
-      <c r="AV1" s="69"/>
-      <c r="AW1" s="69"/>
-      <c r="AX1" s="69"/>
-      <c r="AY1" s="69"/>
-      <c r="AZ1" s="69"/>
-      <c r="BA1" s="70"/>
+      <c r="A1" s="88"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="90"/>
+      <c r="N1" s="90"/>
+      <c r="O1" s="90"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="90"/>
+      <c r="R1" s="90"/>
+      <c r="S1" s="90"/>
+      <c r="T1" s="90"/>
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="90"/>
+      <c r="Z1" s="90"/>
+      <c r="AA1" s="90"/>
+      <c r="AB1" s="90"/>
+      <c r="AC1" s="90"/>
+      <c r="AD1" s="90"/>
+      <c r="AE1" s="90"/>
+      <c r="AF1" s="90"/>
+      <c r="AG1" s="90"/>
+      <c r="AH1" s="90"/>
+      <c r="AI1" s="90"/>
+      <c r="AJ1" s="90"/>
+      <c r="AK1" s="90"/>
+      <c r="AL1" s="87"/>
+      <c r="AM1" s="87"/>
+      <c r="AN1" s="87"/>
+      <c r="AO1" s="87"/>
+      <c r="AP1" s="87"/>
+      <c r="AQ1" s="90"/>
+      <c r="AR1" s="90"/>
+      <c r="AS1" s="90"/>
+      <c r="AT1" s="90"/>
+      <c r="AU1" s="90"/>
+      <c r="AV1" s="90"/>
+      <c r="AW1" s="90"/>
+      <c r="AX1" s="90"/>
+      <c r="AY1" s="90"/>
+      <c r="AZ1" s="90"/>
+      <c r="BA1" s="91"/>
     </row>
     <row r="2" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A3" s="64" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B3" s="63" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C3" s="63" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D3" s="63"/>
       <c r="E3" s="63"/>
       <c r="F3" s="63"/>
       <c r="G3" s="63"/>
       <c r="H3" s="63" t="s">
+        <v>142</v>
+      </c>
+      <c r="I3" s="63" t="s">
         <v>143</v>
       </c>
-      <c r="I3" s="63" t="s">
+      <c r="J3" s="63" t="s">
         <v>144</v>
       </c>
-      <c r="J3" s="63" t="s">
+      <c r="K3" s="63" t="s">
         <v>145</v>
       </c>
-      <c r="K3" s="63" t="s">
-        <v>146</v>
-      </c>
       <c r="L3" s="63" t="s">
+        <v>138</v>
+      </c>
+      <c r="M3" s="63" t="s">
         <v>139</v>
       </c>
-      <c r="M3" s="63" t="s">
+      <c r="N3" s="63" t="s">
+        <v>149</v>
+      </c>
+      <c r="O3" s="63" t="s">
         <v>140</v>
       </c>
-      <c r="N3" s="63" t="s">
+      <c r="P3" s="63" t="s">
         <v>150</v>
       </c>
-      <c r="O3" s="63" t="s">
-        <v>141</v>
-      </c>
-      <c r="P3" s="63" t="s">
+      <c r="Q3" s="63" t="s">
+        <v>138</v>
+      </c>
+      <c r="R3" s="63" t="s">
+        <v>140</v>
+      </c>
+      <c r="S3" s="63" t="s">
         <v>151</v>
       </c>
-      <c r="Q3" s="63" t="s">
-        <v>139</v>
-      </c>
-      <c r="R3" s="63" t="s">
-        <v>141</v>
-      </c>
-      <c r="S3" s="63" t="s">
+      <c r="T3" s="63" t="s">
         <v>152</v>
       </c>
-      <c r="T3" s="63" t="s">
+      <c r="U3" s="63" t="s">
         <v>153</v>
       </c>
-      <c r="U3" s="63" t="s">
-        <v>154</v>
-      </c>
       <c r="V3" s="63" t="s">
+        <v>122</v>
+      </c>
+      <c r="W3" s="63" t="s">
+        <v>78</v>
+      </c>
+      <c r="X3" s="63" t="s">
         <v>123</v>
       </c>
-      <c r="W3" s="63" t="s">
-        <v>79</v>
-      </c>
-      <c r="X3" s="63" t="s">
+      <c r="Y3" s="63" t="s">
         <v>124</v>
-      </c>
-      <c r="Y3" s="63" t="s">
-        <v>125</v>
       </c>
       <c r="Z3" s="63"/>
       <c r="AA3" s="63"/>
       <c r="AB3" s="63" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AC3" s="63"/>
       <c r="AD3" s="63" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="AE3" s="63"/>
       <c r="AF3" s="63"/>
@@ -3122,182 +3552,182 @@
       <c r="AK3" s="63"/>
       <c r="AL3" s="63"/>
       <c r="AM3" s="63" t="s">
+        <v>156</v>
+      </c>
+      <c r="AN3" s="63" t="s">
         <v>157</v>
       </c>
-      <c r="AN3" s="63" t="s">
-        <v>158</v>
-      </c>
       <c r="AO3" s="63" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AP3" s="63" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AQ3" s="63"/>
       <c r="AR3" s="63" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AS3" s="63"/>
       <c r="AT3" s="63" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AU3" s="63"/>
       <c r="AV3" s="63" t="s">
+        <v>158</v>
+      </c>
+      <c r="AW3" s="63" t="s">
         <v>159</v>
       </c>
-      <c r="AW3" s="63" t="s">
+      <c r="AX3" s="63" t="s">
+        <v>104</v>
+      </c>
+      <c r="AY3" s="63" t="s">
+        <v>105</v>
+      </c>
+      <c r="AZ3" s="63" t="s">
         <v>160</v>
-      </c>
-      <c r="AX3" s="63" t="s">
-        <v>105</v>
-      </c>
-      <c r="AY3" s="63" t="s">
-        <v>106</v>
-      </c>
-      <c r="AZ3" s="63" t="s">
-        <v>161</v>
       </c>
       <c r="BA3" s="65"/>
       <c r="BB3" t="s">
+        <v>161</v>
+      </c>
+      <c r="BC3" t="s">
+        <v>157</v>
+      </c>
+      <c r="BD3" t="s">
+        <v>61</v>
+      </c>
+      <c r="BE3" t="s">
+        <v>104</v>
+      </c>
+      <c r="BF3" t="s">
+        <v>105</v>
+      </c>
+      <c r="BG3" t="s">
+        <v>160</v>
+      </c>
+      <c r="BI3" t="s">
+        <v>135</v>
+      </c>
+      <c r="BJ3" t="s">
+        <v>104</v>
+      </c>
+      <c r="BK3" t="s">
+        <v>105</v>
+      </c>
+      <c r="BL3" t="s">
         <v>162</v>
       </c>
-      <c r="BC3" t="s">
-        <v>158</v>
-      </c>
-      <c r="BD3" t="s">
-        <v>62</v>
-      </c>
-      <c r="BE3" t="s">
-        <v>105</v>
-      </c>
-      <c r="BF3" t="s">
-        <v>106</v>
-      </c>
-      <c r="BG3" t="s">
-        <v>161</v>
-      </c>
-      <c r="BI3" t="s">
-        <v>136</v>
-      </c>
-      <c r="BJ3" t="s">
-        <v>105</v>
-      </c>
-      <c r="BK3" t="s">
-        <v>106</v>
-      </c>
-      <c r="BL3" t="s">
-        <v>163</v>
-      </c>
       <c r="BM3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A4" s="64" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B4" s="63"/>
       <c r="C4" s="63"/>
       <c r="D4" s="63" t="s">
+        <v>164</v>
+      </c>
+      <c r="E4" s="63" t="s">
         <v>165</v>
       </c>
-      <c r="E4" s="63" t="s">
+      <c r="F4" s="63" t="s">
         <v>166</v>
       </c>
-      <c r="F4" s="63" t="s">
+      <c r="G4" s="63" t="s">
         <v>167</v>
-      </c>
-      <c r="G4" s="63" t="s">
-        <v>168</v>
       </c>
       <c r="H4" s="63"/>
       <c r="I4" s="63"/>
       <c r="J4" s="63"/>
       <c r="K4" s="63"/>
       <c r="L4" s="63" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="M4" s="63" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N4" s="63" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O4" s="63" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="P4" s="63" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="Q4" s="63" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="R4" s="63" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="S4" s="63" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="T4" s="63" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="U4" s="63"/>
       <c r="V4" s="63" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="W4" s="63"/>
       <c r="X4" s="63"/>
       <c r="Y4" s="63" t="s">
+        <v>147</v>
+      </c>
+      <c r="Z4" s="63" t="s">
         <v>148</v>
       </c>
-      <c r="Z4" s="63" t="s">
-        <v>149</v>
-      </c>
       <c r="AA4" s="63" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AB4" s="63" t="s">
+        <v>169</v>
+      </c>
+      <c r="AC4" s="63" t="s">
         <v>170</v>
       </c>
-      <c r="AC4" s="63" t="s">
+      <c r="AD4" s="63" t="s">
         <v>171</v>
       </c>
-      <c r="AD4" s="63" t="s">
+      <c r="AE4" s="63" t="s">
         <v>172</v>
       </c>
-      <c r="AE4" s="63" t="s">
+      <c r="AF4" s="63" t="s">
         <v>173</v>
       </c>
-      <c r="AF4" s="63" t="s">
+      <c r="AG4" s="63" t="s">
         <v>174</v>
       </c>
-      <c r="AG4" s="63" t="s">
+      <c r="AH4" s="63" t="s">
         <v>175</v>
       </c>
-      <c r="AH4" s="63" t="s">
+      <c r="AI4" s="63" t="s">
         <v>176</v>
       </c>
-      <c r="AI4" s="63" t="s">
+      <c r="AJ4" s="63" t="s">
         <v>177</v>
       </c>
-      <c r="AJ4" s="63" t="s">
-        <v>178</v>
-      </c>
       <c r="AK4" s="63" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AL4" s="63"/>
       <c r="AM4" s="63"/>
       <c r="AN4" s="63"/>
       <c r="AO4" s="63"/>
       <c r="AP4" s="63" t="s">
+        <v>104</v>
+      </c>
+      <c r="AQ4" s="63" t="s">
         <v>105</v>
       </c>
-      <c r="AQ4" s="63" t="s">
-        <v>106</v>
-      </c>
       <c r="AR4" s="63" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AS4" s="63">
         <v>9</v>
@@ -3368,18 +3798,18 @@
     </row>
     <row r="9" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:65" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>64</v>
-      </c>
       <c r="C10" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D10" s="6"/>
       <c r="H10" s="61"/>
@@ -3388,20 +3818,20 @@
       <c r="N10" s="17"/>
       <c r="O10" s="60"/>
       <c r="P10" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="Q10" s="62"/>
       <c r="BB10" s="60" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="BE10" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="BF10" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="BF10" s="6" t="s">
-        <v>66</v>
-      </c>
       <c r="BG10" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -3412,7 +3842,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECB08AFA-BF49-47F5-B095-34C6A355FE30}">
   <dimension ref="A2:BA10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3422,316 +3852,316 @@
   <sheetData>
     <row r="2" spans="1:53" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A3" s="66" t="str">
-        <f>+[1]Summary!A4</f>
+      <c r="A3" s="88" t="str">
+        <f>+[2]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="69"/>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="69"/>
-      <c r="I3" s="69"/>
-      <c r="J3" s="69"/>
-      <c r="K3" s="69"/>
-      <c r="L3" s="69"/>
-      <c r="M3" s="69"/>
-      <c r="N3" s="69"/>
-      <c r="O3" s="69"/>
-      <c r="P3" s="69"/>
-      <c r="Q3" s="69"/>
-      <c r="R3" s="69"/>
-      <c r="S3" s="69"/>
-      <c r="T3" s="69"/>
-      <c r="U3" s="69"/>
-      <c r="V3" s="69"/>
-      <c r="W3" s="69"/>
-      <c r="X3" s="69"/>
-      <c r="Y3" s="69"/>
-      <c r="Z3" s="69"/>
-      <c r="AA3" s="69"/>
-      <c r="AB3" s="69"/>
-      <c r="AC3" s="69"/>
-      <c r="AD3" s="69"/>
-      <c r="AE3" s="69"/>
-      <c r="AF3" s="69"/>
-      <c r="AG3" s="69"/>
-      <c r="AH3" s="69"/>
-      <c r="AI3" s="69"/>
-      <c r="AJ3" s="69"/>
-      <c r="AK3" s="69"/>
-      <c r="AL3" s="67"/>
-      <c r="AM3" s="67"/>
-      <c r="AN3" s="67"/>
-      <c r="AO3" s="67"/>
-      <c r="AP3" s="67"/>
-      <c r="AQ3" s="69"/>
-      <c r="AR3" s="69"/>
-      <c r="AS3" s="69"/>
-      <c r="AT3" s="69"/>
-      <c r="AU3" s="69"/>
-      <c r="AV3" s="69"/>
-      <c r="AW3" s="69"/>
-      <c r="AX3" s="69"/>
-      <c r="AY3" s="69"/>
-      <c r="AZ3" s="69"/>
-      <c r="BA3" s="70"/>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="90"/>
+      <c r="L3" s="90"/>
+      <c r="M3" s="90"/>
+      <c r="N3" s="90"/>
+      <c r="O3" s="90"/>
+      <c r="P3" s="90"/>
+      <c r="Q3" s="90"/>
+      <c r="R3" s="90"/>
+      <c r="S3" s="90"/>
+      <c r="T3" s="90"/>
+      <c r="U3" s="90"/>
+      <c r="V3" s="90"/>
+      <c r="W3" s="90"/>
+      <c r="X3" s="90"/>
+      <c r="Y3" s="90"/>
+      <c r="Z3" s="90"/>
+      <c r="AA3" s="90"/>
+      <c r="AB3" s="90"/>
+      <c r="AC3" s="90"/>
+      <c r="AD3" s="90"/>
+      <c r="AE3" s="90"/>
+      <c r="AF3" s="90"/>
+      <c r="AG3" s="90"/>
+      <c r="AH3" s="90"/>
+      <c r="AI3" s="90"/>
+      <c r="AJ3" s="90"/>
+      <c r="AK3" s="90"/>
+      <c r="AL3" s="87"/>
+      <c r="AM3" s="87"/>
+      <c r="AN3" s="87"/>
+      <c r="AO3" s="87"/>
+      <c r="AP3" s="87"/>
+      <c r="AQ3" s="90"/>
+      <c r="AR3" s="90"/>
+      <c r="AS3" s="90"/>
+      <c r="AT3" s="90"/>
+      <c r="AU3" s="90"/>
+      <c r="AV3" s="90"/>
+      <c r="AW3" s="90"/>
+      <c r="AX3" s="90"/>
+      <c r="AY3" s="90"/>
+      <c r="AZ3" s="90"/>
+      <c r="BA3" s="91"/>
     </row>
     <row r="4" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A4" s="66">
-        <f>+[1]Summary!A7</f>
+      <c r="A4" s="88">
+        <f>+[2]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
-      <c r="D4" s="69"/>
-      <c r="E4" s="69"/>
-      <c r="F4" s="69"/>
-      <c r="G4" s="69"/>
-      <c r="H4" s="69"/>
-      <c r="I4" s="69"/>
-      <c r="J4" s="69"/>
-      <c r="K4" s="69"/>
-      <c r="L4" s="69"/>
-      <c r="M4" s="69"/>
-      <c r="N4" s="69"/>
-      <c r="O4" s="69"/>
-      <c r="P4" s="69"/>
-      <c r="Q4" s="69"/>
-      <c r="R4" s="69"/>
-      <c r="S4" s="69"/>
-      <c r="T4" s="69"/>
-      <c r="U4" s="69"/>
-      <c r="V4" s="69"/>
-      <c r="W4" s="69"/>
-      <c r="X4" s="69"/>
-      <c r="Y4" s="69"/>
-      <c r="Z4" s="69"/>
-      <c r="AA4" s="69"/>
-      <c r="AB4" s="69"/>
-      <c r="AC4" s="69"/>
-      <c r="AD4" s="69"/>
-      <c r="AE4" s="69"/>
-      <c r="AF4" s="69"/>
-      <c r="AG4" s="69"/>
-      <c r="AH4" s="69"/>
-      <c r="AI4" s="69"/>
-      <c r="AJ4" s="69"/>
-      <c r="AK4" s="69"/>
-      <c r="AL4" s="67"/>
-      <c r="AM4" s="67"/>
-      <c r="AN4" s="67"/>
-      <c r="AO4" s="67"/>
-      <c r="AP4" s="67"/>
-      <c r="AQ4" s="69"/>
-      <c r="AR4" s="69"/>
-      <c r="AS4" s="69"/>
-      <c r="AT4" s="69"/>
-      <c r="AU4" s="69"/>
-      <c r="AV4" s="69"/>
-      <c r="AW4" s="69"/>
-      <c r="AX4" s="69"/>
-      <c r="AY4" s="69"/>
-      <c r="AZ4" s="69"/>
-      <c r="BA4" s="70"/>
+      <c r="B4" s="90"/>
+      <c r="C4" s="90"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="90"/>
+      <c r="F4" s="90"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="90"/>
+      <c r="L4" s="90"/>
+      <c r="M4" s="90"/>
+      <c r="N4" s="90"/>
+      <c r="O4" s="90"/>
+      <c r="P4" s="90"/>
+      <c r="Q4" s="90"/>
+      <c r="R4" s="90"/>
+      <c r="S4" s="90"/>
+      <c r="T4" s="90"/>
+      <c r="U4" s="90"/>
+      <c r="V4" s="90"/>
+      <c r="W4" s="90"/>
+      <c r="X4" s="90"/>
+      <c r="Y4" s="90"/>
+      <c r="Z4" s="90"/>
+      <c r="AA4" s="90"/>
+      <c r="AB4" s="90"/>
+      <c r="AC4" s="90"/>
+      <c r="AD4" s="90"/>
+      <c r="AE4" s="90"/>
+      <c r="AF4" s="90"/>
+      <c r="AG4" s="90"/>
+      <c r="AH4" s="90"/>
+      <c r="AI4" s="90"/>
+      <c r="AJ4" s="90"/>
+      <c r="AK4" s="90"/>
+      <c r="AL4" s="87"/>
+      <c r="AM4" s="87"/>
+      <c r="AN4" s="87"/>
+      <c r="AO4" s="87"/>
+      <c r="AP4" s="87"/>
+      <c r="AQ4" s="90"/>
+      <c r="AR4" s="90"/>
+      <c r="AS4" s="90"/>
+      <c r="AT4" s="90"/>
+      <c r="AU4" s="90"/>
+      <c r="AV4" s="90"/>
+      <c r="AW4" s="90"/>
+      <c r="AX4" s="90"/>
+      <c r="AY4" s="90"/>
+      <c r="AZ4" s="90"/>
+      <c r="BA4" s="91"/>
     </row>
     <row r="5" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="66" t="s">
+      <c r="A5" s="88" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="90"/>
+      <c r="C5" s="90"/>
+      <c r="D5" s="90"/>
+      <c r="E5" s="90"/>
+      <c r="F5" s="90"/>
+      <c r="G5" s="90"/>
+      <c r="H5" s="90"/>
+      <c r="I5" s="90"/>
+      <c r="J5" s="90"/>
+      <c r="K5" s="90"/>
+      <c r="L5" s="90"/>
+      <c r="M5" s="90"/>
+      <c r="N5" s="90"/>
+      <c r="O5" s="90"/>
+      <c r="P5" s="90"/>
+      <c r="Q5" s="90"/>
+      <c r="R5" s="90"/>
+      <c r="S5" s="91"/>
+      <c r="T5" s="88" t="s">
         <v>114</v>
       </c>
-      <c r="B5" s="69"/>
-      <c r="C5" s="69"/>
-      <c r="D5" s="69"/>
-      <c r="E5" s="69"/>
-      <c r="F5" s="69"/>
-      <c r="G5" s="69"/>
-      <c r="H5" s="69"/>
-      <c r="I5" s="69"/>
-      <c r="J5" s="69"/>
-      <c r="K5" s="69"/>
-      <c r="L5" s="69"/>
-      <c r="M5" s="69"/>
-      <c r="N5" s="69"/>
-      <c r="O5" s="69"/>
-      <c r="P5" s="69"/>
-      <c r="Q5" s="69"/>
-      <c r="R5" s="69"/>
-      <c r="S5" s="70"/>
-      <c r="T5" s="66" t="s">
+      <c r="U5" s="90"/>
+      <c r="V5" s="90"/>
+      <c r="W5" s="90"/>
+      <c r="X5" s="90"/>
+      <c r="Y5" s="90"/>
+      <c r="Z5" s="90"/>
+      <c r="AA5" s="90"/>
+      <c r="AB5" s="90"/>
+      <c r="AC5" s="90"/>
+      <c r="AD5" s="90"/>
+      <c r="AE5" s="90"/>
+      <c r="AF5" s="90"/>
+      <c r="AG5" s="90"/>
+      <c r="AH5" s="90"/>
+      <c r="AI5" s="90"/>
+      <c r="AJ5" s="90"/>
+      <c r="AK5" s="91"/>
+      <c r="AL5" s="88" t="s">
         <v>115</v>
       </c>
-      <c r="U5" s="69"/>
-      <c r="V5" s="69"/>
-      <c r="W5" s="69"/>
-      <c r="X5" s="69"/>
-      <c r="Y5" s="69"/>
-      <c r="Z5" s="69"/>
-      <c r="AA5" s="69"/>
-      <c r="AB5" s="69"/>
-      <c r="AC5" s="69"/>
-      <c r="AD5" s="69"/>
-      <c r="AE5" s="69"/>
-      <c r="AF5" s="69"/>
-      <c r="AG5" s="69"/>
-      <c r="AH5" s="69"/>
-      <c r="AI5" s="69"/>
-      <c r="AJ5" s="69"/>
-      <c r="AK5" s="70"/>
-      <c r="AL5" s="66" t="s">
+      <c r="AM5" s="87"/>
+      <c r="AN5" s="87"/>
+      <c r="AO5" s="87"/>
+      <c r="AP5" s="85"/>
+      <c r="AQ5" s="88" t="s">
+        <v>2</v>
+      </c>
+      <c r="AR5" s="90"/>
+      <c r="AS5" s="90"/>
+      <c r="AT5" s="91"/>
+      <c r="AU5" s="27" t="s">
         <v>116</v>
       </c>
-      <c r="AM5" s="67"/>
-      <c r="AN5" s="67"/>
-      <c r="AO5" s="67"/>
-      <c r="AP5" s="68"/>
-      <c r="AQ5" s="66" t="s">
-        <v>2</v>
-      </c>
-      <c r="AR5" s="69"/>
-      <c r="AS5" s="69"/>
-      <c r="AT5" s="70"/>
-      <c r="AU5" s="27" t="s">
+      <c r="AV5" s="88" t="s">
         <v>117</v>
       </c>
-      <c r="AV5" s="66" t="s">
+      <c r="AW5" s="90"/>
+      <c r="AX5" s="90"/>
+      <c r="AY5" s="90"/>
+      <c r="AZ5" s="91"/>
+      <c r="BA5" s="27" t="s">
         <v>118</v>
-      </c>
-      <c r="AW5" s="69"/>
-      <c r="AX5" s="69"/>
-      <c r="AY5" s="69"/>
-      <c r="AZ5" s="70"/>
-      <c r="BA5" s="27" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:53" ht="58.5" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A6" s="31" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D6" s="50"/>
       <c r="E6" s="50"/>
       <c r="F6" s="50"/>
-      <c r="G6" s="71" t="s">
-        <v>82</v>
-      </c>
-      <c r="H6" s="72"/>
-      <c r="I6" s="72"/>
-      <c r="J6" s="73"/>
-      <c r="K6" s="71" t="s">
+      <c r="G6" s="92" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" s="93"/>
+      <c r="I6" s="93"/>
+      <c r="J6" s="94"/>
+      <c r="K6" s="92" t="s">
+        <v>120</v>
+      </c>
+      <c r="L6" s="93"/>
+      <c r="M6" s="93"/>
+      <c r="N6" s="94"/>
+      <c r="O6" s="95" t="s">
         <v>121</v>
       </c>
-      <c r="L6" s="72"/>
-      <c r="M6" s="72"/>
-      <c r="N6" s="73"/>
-      <c r="O6" s="74" t="s">
+      <c r="P6" s="90"/>
+      <c r="Q6" s="90"/>
+      <c r="R6" s="91"/>
+      <c r="S6" s="51" t="s">
         <v>122</v>
       </c>
-      <c r="P6" s="69"/>
-      <c r="Q6" s="69"/>
-      <c r="R6" s="70"/>
-      <c r="S6" s="51" t="s">
+      <c r="T6" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="U6" s="31" t="s">
         <v>123</v>
       </c>
-      <c r="T6" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="U6" s="31" t="s">
+      <c r="V6" s="88" t="s">
         <v>124</v>
       </c>
-      <c r="V6" s="66" t="s">
+      <c r="W6" s="90"/>
+      <c r="X6" s="91"/>
+      <c r="Y6" s="52" t="s">
         <v>125</v>
       </c>
-      <c r="W6" s="69"/>
-      <c r="X6" s="70"/>
-      <c r="Y6" s="52" t="s">
+      <c r="Z6" s="52" t="s">
         <v>126</v>
       </c>
-      <c r="Z6" s="52" t="s">
+      <c r="AA6" s="52" t="s">
         <v>127</v>
       </c>
-      <c r="AA6" s="52" t="s">
+      <c r="AB6" s="52" t="s">
         <v>128</v>
       </c>
-      <c r="AB6" s="52" t="s">
+      <c r="AC6" s="52" t="s">
         <v>129</v>
       </c>
-      <c r="AC6" s="52" t="s">
+      <c r="AD6" s="52" t="s">
         <v>130</v>
       </c>
-      <c r="AD6" s="52" t="s">
+      <c r="AE6" s="53" t="s">
         <v>131</v>
       </c>
-      <c r="AE6" s="53" t="s">
+      <c r="AF6" s="27" t="s">
         <v>132</v>
       </c>
-      <c r="AF6" s="27" t="s">
+      <c r="AG6" s="96" t="s">
         <v>133</v>
       </c>
-      <c r="AG6" s="75" t="s">
+      <c r="AH6" s="91"/>
+      <c r="AI6" s="88" t="s">
         <v>134</v>
       </c>
-      <c r="AH6" s="70"/>
-      <c r="AI6" s="66" t="s">
+      <c r="AJ6" s="91"/>
+      <c r="AK6" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="AL6" s="27" t="s">
         <v>135</v>
       </c>
-      <c r="AJ6" s="70"/>
-      <c r="AK6" s="27" t="s">
-        <v>101</v>
-      </c>
-      <c r="AL6" s="27" t="s">
+      <c r="AM6" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="AM6" s="27" t="s">
-        <v>137</v>
-      </c>
       <c r="AN6" s="54" t="s">
+        <v>104</v>
+      </c>
+      <c r="AO6" s="54" t="s">
         <v>105</v>
       </c>
-      <c r="AO6" s="54" t="s">
-        <v>106</v>
-      </c>
       <c r="AP6" s="27" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AQ6" s="27" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AR6" s="54" t="s">
+        <v>104</v>
+      </c>
+      <c r="AS6" s="54" t="s">
         <v>105</v>
       </c>
-      <c r="AS6" s="54" t="s">
-        <v>106</v>
-      </c>
       <c r="AT6" s="27" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AU6" s="53"/>
       <c r="AV6" s="27" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AW6" s="54" t="s">
+        <v>104</v>
+      </c>
+      <c r="AX6" s="54" t="s">
         <v>105</v>
       </c>
-      <c r="AX6" s="54" t="s">
-        <v>106</v>
-      </c>
       <c r="AY6" s="55" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AZ6" s="27" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="BA6" s="53"/>
     </row>
@@ -3743,54 +4173,54 @@
       <c r="E7" s="29"/>
       <c r="F7" s="29"/>
       <c r="G7" s="56" t="s">
+        <v>138</v>
+      </c>
+      <c r="H7" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H7" s="31" t="s">
+      <c r="I7" s="31" t="s">
         <v>140</v>
       </c>
-      <c r="I7" s="31" t="s">
+      <c r="J7" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="J7" s="57" t="s">
+      <c r="K7" s="56" t="s">
+        <v>138</v>
+      </c>
+      <c r="L7" s="29" t="s">
+        <v>139</v>
+      </c>
+      <c r="M7" s="31" t="s">
+        <v>140</v>
+      </c>
+      <c r="N7" s="57" t="s">
+        <v>141</v>
+      </c>
+      <c r="O7" s="54" t="s">
         <v>142</v>
       </c>
-      <c r="K7" s="56" t="s">
-        <v>139</v>
-      </c>
-      <c r="L7" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="M7" s="31" t="s">
-        <v>141</v>
-      </c>
-      <c r="N7" s="57" t="s">
-        <v>142</v>
-      </c>
-      <c r="O7" s="54" t="s">
+      <c r="P7" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="P7" s="54" t="s">
+      <c r="Q7" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="Q7" s="54" t="s">
+      <c r="R7" s="54" t="s">
         <v>145</v>
       </c>
-      <c r="R7" s="54" t="s">
+      <c r="S7" s="58" t="s">
         <v>146</v>
-      </c>
-      <c r="S7" s="58" t="s">
-        <v>147</v>
       </c>
       <c r="T7" s="36"/>
       <c r="U7" s="27"/>
       <c r="V7" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="W7" s="27" t="s">
         <v>148</v>
       </c>
-      <c r="W7" s="27" t="s">
-        <v>149</v>
-      </c>
       <c r="X7" s="27" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="Y7" s="53"/>
       <c r="Z7" s="53"/>
@@ -3801,16 +4231,16 @@
       <c r="AE7" s="36"/>
       <c r="AF7" s="36"/>
       <c r="AG7" s="54" t="s">
+        <v>104</v>
+      </c>
+      <c r="AH7" s="54" t="s">
         <v>105</v>
       </c>
-      <c r="AH7" s="54" t="s">
-        <v>106</v>
-      </c>
       <c r="AI7" s="54" t="s">
+        <v>104</v>
+      </c>
+      <c r="AJ7" s="54" t="s">
         <v>105</v>
-      </c>
-      <c r="AJ7" s="54" t="s">
-        <v>106</v>
       </c>
       <c r="AK7" s="36"/>
       <c r="AL7" s="36"/>
@@ -3832,24 +4262,24 @@
     </row>
     <row r="9" spans="1:53" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:53" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>64</v>
-      </c>
       <c r="C10" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D10" s="6"/>
       <c r="H10" s="61"/>
       <c r="I10" s="61"/>
       <c r="J10" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="M10" s="6"/>
       <c r="N10" s="17"/>
@@ -3857,16 +4287,16 @@
       <c r="P10" s="61"/>
       <c r="Q10" s="62"/>
       <c r="AQ10" s="60" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AR10" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="AS10" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="AS10" s="6" t="s">
-        <v>66</v>
-      </c>
       <c r="AT10" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -3878,123 +4308,123 @@
     <mergeCell ref="AL5:AP5"/>
     <mergeCell ref="AQ5:AT5"/>
     <mergeCell ref="AV5:AZ5"/>
+    <mergeCell ref="AI6:AJ6"/>
     <mergeCell ref="G6:J6"/>
     <mergeCell ref="K6:N6"/>
     <mergeCell ref="O6:R6"/>
     <mergeCell ref="V6:X6"/>
     <mergeCell ref="AG6:AH6"/>
-    <mergeCell ref="AI6:AJ6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0CAA689-52FE-4282-BFA7-7FA3F37BB8D4}">
   <dimension ref="A2:W7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="81" t="s">
+      <c r="A3" s="99" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="100" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="87"/>
+      <c r="D3" s="85"/>
+      <c r="E3" s="100" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="82" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" s="67"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="82" t="s">
+      <c r="F3" s="87"/>
+      <c r="G3" s="85"/>
+      <c r="H3" s="100" t="s">
+        <v>37</v>
+      </c>
+      <c r="I3" s="87"/>
+      <c r="J3" s="85"/>
+      <c r="K3" s="99" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="67"/>
-      <c r="G3" s="68"/>
-      <c r="H3" s="82" t="s">
-        <v>38</v>
-      </c>
-      <c r="I3" s="67"/>
-      <c r="J3" s="68"/>
-      <c r="K3" s="81" t="s">
-        <v>75</v>
-      </c>
-      <c r="L3" s="79" t="s">
-        <v>43</v>
+      <c r="L3" s="97" t="s">
+        <v>42</v>
       </c>
       <c r="M3" s="8"/>
       <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="31" x14ac:dyDescent="0.35">
-      <c r="A4" s="80"/>
+      <c r="A4" s="98"/>
       <c r="B4" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="D4" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>41</v>
-      </c>
       <c r="F4" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="G4" s="12" t="s">
-        <v>77</v>
-      </c>
       <c r="H4" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I4" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="J4" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="J4" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="K4" s="80"/>
-      <c r="L4" s="80"/>
+      <c r="K4" s="98"/>
+      <c r="L4" s="98"/>
       <c r="M4" s="10"/>
       <c r="N4" s="11"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>50</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L7" s="4"/>
       <c r="N7" s="3"/>
@@ -4025,120 +4455,123 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B225AA6-68BC-47EB-9948-84B6B216E727}">
   <dimension ref="A2:W7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A3" s="86" t="s">
+      <c r="A3" s="104" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="104" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="86" t="s">
+      <c r="C3" s="104"/>
+      <c r="D3" s="104" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="86"/>
-      <c r="D3" s="86" t="s">
+      <c r="E3" s="104" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="86" t="s">
+      <c r="F3" s="104" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="86" t="s">
+      <c r="G3" s="105" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="87" t="s">
+      <c r="H3" s="105"/>
+      <c r="I3" s="105"/>
+      <c r="J3" s="101" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="87"/>
-      <c r="I3" s="87"/>
-      <c r="J3" s="83" t="s">
+      <c r="K3" s="102"/>
+      <c r="L3" s="102"/>
+      <c r="M3" s="102"/>
+      <c r="N3" s="103"/>
+    </row>
+    <row r="4" spans="1:23" ht="26" x14ac:dyDescent="0.35">
+      <c r="A4" s="104"/>
+      <c r="B4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="84"/>
-      <c r="L3" s="84"/>
-      <c r="M3" s="84"/>
-      <c r="N3" s="85"/>
-    </row>
-    <row r="4" spans="1:23" ht="26" x14ac:dyDescent="0.35">
-      <c r="A4" s="86"/>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="104"/>
+      <c r="E4" s="104"/>
+      <c r="F4" s="104"/>
+      <c r="G4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="86"/>
-      <c r="E4" s="86"/>
-      <c r="F4" s="86"/>
-      <c r="G4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="M4" s="1" t="s">
+      <c r="N4" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="I7" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="K7" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="H7" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="K7" s="4" t="s">
+      <c r="L7" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="N7" s="3"/>
       <c r="O7" s="3"/>
@@ -4169,170 +4602,75 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBFB976A-1B92-4632-9799-0237B459A61D}">
   <dimension ref="A1:P5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>61</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C3" s="7"/>
       <c r="D3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="88"/>
-      <c r="H3" s="89"/>
-      <c r="I3" s="89"/>
-      <c r="J3" s="90"/>
+      <c r="G3" s="106"/>
+      <c r="H3" s="107"/>
+      <c r="I3" s="107"/>
+      <c r="J3" s="108"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="88"/>
-      <c r="O3" s="89"/>
-      <c r="P3" s="90"/>
+      <c r="N3" s="106"/>
+      <c r="O3" s="107"/>
+      <c r="P3" s="108"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>64</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="N3:P3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46CC22E7-0431-4564-825A-DCAC81041178}">
-  <dimension ref="A1:P5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" ht="26" x14ac:dyDescent="0.35">
-      <c r="A2" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="B2" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="G2" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="H2" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="I2" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="J2" s="15" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C3" s="7"/>
-      <c r="D3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="88"/>
-      <c r="H3" s="89"/>
-      <c r="I3" s="89"/>
-      <c r="J3" s="90"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="88"/>
-      <c r="O3" s="89"/>
-      <c r="P3" s="90"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>78</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="F5" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>35</v>
+      <c r="F5" s="6" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto pipeline update 2026-04-15 16:15:03
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -8,25 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FFF31B4-0A06-4209-B1D6-13BB5BF991C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{267EDEAC-9010-47DB-82E9-1AAF7FC2FDED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" firstSheet="2" activeTab="7" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" activeTab="2" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet Names Check" sheetId="1" r:id="rId1"/>
-    <sheet name="TA 601 Stringing" sheetId="12" r:id="rId2"/>
-    <sheet name="TB 501 220kV Stringing" sheetId="10" r:id="rId3"/>
-    <sheet name="TB 501 132kV Stringing" sheetId="11" r:id="rId4"/>
-    <sheet name="TB 501 220kV Erection" sheetId="9" r:id="rId5"/>
-    <sheet name="TB 501 132kV Erection" sheetId="8" r:id="rId6"/>
-    <sheet name="TB 401 Stringing" sheetId="6" r:id="rId7"/>
-    <sheet name="TB 408 Stringing" sheetId="2" r:id="rId8"/>
-    <sheet name="TA 509 Erection" sheetId="3" r:id="rId9"/>
-    <sheet name="TA 601 Erection" sheetId="7" r:id="rId10"/>
+    <sheet name="TA 413 Erection" sheetId="14" r:id="rId2"/>
+    <sheet name="TA 413 Stringing" sheetId="13" r:id="rId3"/>
+    <sheet name="TA 601 Stringing" sheetId="12" r:id="rId4"/>
+    <sheet name="TB 501 220kV Stringing" sheetId="10" r:id="rId5"/>
+    <sheet name="TB 501 132kV Stringing" sheetId="11" r:id="rId6"/>
+    <sheet name="TB 501 220kV Erection" sheetId="9" r:id="rId7"/>
+    <sheet name="TB 501 132kV Erection" sheetId="8" r:id="rId8"/>
+    <sheet name="TB 401 Stringing" sheetId="6" r:id="rId9"/>
+    <sheet name="TB 408 Stringing" sheetId="2" r:id="rId10"/>
+    <sheet name="TA 509 Erection" sheetId="3" r:id="rId11"/>
+    <sheet name="TA 601 Erection" sheetId="7" r:id="rId12"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId11"/>
-    <externalReference r:id="rId12"/>
+    <externalReference r:id="rId13"/>
+    <externalReference r:id="rId14"/>
   </externalReferences>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -49,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="205">
   <si>
     <t>Project Code</t>
   </si>
@@ -592,17 +594,96 @@
   </si>
   <si>
     <t>Stringing compiled</t>
+  </si>
+  <si>
+    <t>CUMM. SR.NO</t>
+  </si>
+  <si>
+    <t>MONTH SR.NO.</t>
+  </si>
+  <si>
+    <t>Loc. No.</t>
+  </si>
+  <si>
+    <t>Type of Tower</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>Gang name</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of Supervisor </t>
+  </si>
+  <si>
+    <t xml:space="preserve">JMC Status </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prop. Name </t>
+  </si>
+  <si>
+    <t>Length in Km's</t>
+  </si>
+  <si>
+    <t>Cum. Length in Km's</t>
+  </si>
+  <si>
+    <t>TSE/Manual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insulator hoisting Start </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insulator Hoisting Complete </t>
+  </si>
+  <si>
+    <t>Paying Out Start</t>
+  </si>
+  <si>
+    <t>Paying Out Completed</t>
+  </si>
+  <si>
+    <t>Final sag start</t>
+  </si>
+  <si>
+    <t>Final sag complete</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Earthwire Final Sag </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jumpuring </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clipping </t>
+  </si>
+  <si>
+    <t>JMC Status</t>
+  </si>
+  <si>
+    <t>Name of the Contractor</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="166" formatCode="[$-4009]0.00"/>
     <numFmt numFmtId="167" formatCode="#,##0.000"/>
+    <numFmt numFmtId="168" formatCode="[$-409]d\-mmm\-yy;@"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
@@ -697,7 +778,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -758,8 +839,14 @@
         <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="37">
+  <borders count="40">
     <border>
       <left/>
       <right/>
@@ -1205,6 +1292,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1217,7 +1347,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1456,19 +1586,64 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="25" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="11" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="11" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1537,7 +1712,17 @@
     <cellStyle name="Normal 6" xfId="8" xr:uid="{E2AC1BB0-A24A-450A-B605-14A01490AC0E}"/>
     <cellStyle name="Normal 8 2" xfId="2" xr:uid="{E356B690-246D-43B2-86AF-A6FE97B16461}"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2165,10 +2350,10 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -2335,6 +2520,233 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B225AA6-68BC-47EB-9948-84B6B216E727}">
+  <dimension ref="A2:W7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A3" s="119" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="119" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="119"/>
+      <c r="D3" s="119" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="119" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" s="119" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" s="120" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="120"/>
+      <c r="I3" s="120"/>
+      <c r="J3" s="116" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" s="117"/>
+      <c r="L3" s="117"/>
+      <c r="M3" s="117"/>
+      <c r="N3" s="118"/>
+    </row>
+    <row r="4" spans="1:23" ht="26" x14ac:dyDescent="0.35">
+      <c r="A4" s="119"/>
+      <c r="B4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="119"/>
+      <c r="E4" s="119"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="4"/>
+      <c r="R7" s="3"/>
+      <c r="T7" s="3"/>
+      <c r="U7" s="3"/>
+      <c r="V7" s="3"/>
+      <c r="W7" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="J3:N3"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:I3"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B7">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C7">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBFB976A-1B92-4632-9799-0237B459A61D}">
+  <dimension ref="A1:P5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C3" s="7"/>
+      <c r="D3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="121"/>
+      <c r="H3" s="122"/>
+      <c r="I3" s="122"/>
+      <c r="J3" s="123"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="121"/>
+      <c r="O3" s="122"/>
+      <c r="P3" s="123"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="N3:P3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46CC22E7-0431-4564-825A-DCAC81041178}">
   <dimension ref="A1:P5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2380,14 +2792,14 @@
       <c r="C3" s="7"/>
       <c r="D3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="106"/>
-      <c r="H3" s="107"/>
-      <c r="I3" s="107"/>
-      <c r="J3" s="108"/>
+      <c r="G3" s="121"/>
+      <c r="H3" s="122"/>
+      <c r="I3" s="122"/>
+      <c r="J3" s="123"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="106"/>
-      <c r="O3" s="107"/>
-      <c r="P3" s="108"/>
+      <c r="N3" s="121"/>
+      <c r="O3" s="122"/>
+      <c r="P3" s="123"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -2430,7 +2842,104 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7C2946C-A784-4830-B129-5E94E117C5CC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B2BFD82-3A51-4FB3-99B3-97ACBD8E712D}">
+  <dimension ref="A1:P5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="87" t="s">
+        <v>179</v>
+      </c>
+      <c r="B2" s="87" t="s">
+        <v>180</v>
+      </c>
+      <c r="C2" s="88" t="s">
+        <v>181</v>
+      </c>
+      <c r="D2" s="88" t="s">
+        <v>182</v>
+      </c>
+      <c r="E2" s="89" t="s">
+        <v>183</v>
+      </c>
+      <c r="F2" s="90" t="s">
+        <v>184</v>
+      </c>
+      <c r="G2" s="91" t="s">
+        <v>185</v>
+      </c>
+      <c r="H2" s="91" t="s">
+        <v>186</v>
+      </c>
+      <c r="I2" s="92" t="s">
+        <v>187</v>
+      </c>
+      <c r="J2" s="87" t="s">
+        <v>188</v>
+      </c>
+      <c r="K2" s="87" t="s">
+        <v>42</v>
+      </c>
+      <c r="L2" s="87" t="s">
+        <v>189</v>
+      </c>
+      <c r="M2" s="93" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="C3" s="84"/>
+      <c r="D3" s="85"/>
+      <c r="F3" s="85"/>
+      <c r="G3" s="86"/>
+      <c r="H3" s="86"/>
+      <c r="I3" s="86"/>
+      <c r="J3" s="86"/>
+      <c r="M3" s="85"/>
+      <c r="N3" s="86"/>
+      <c r="O3" s="86"/>
+      <c r="P3" s="86"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C2">
+    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F761DC74-F86C-401C-9968-F9738A14EF54}">
   <dimension ref="A2:Z11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -2439,79 +2948,70 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:26" s="98" customFormat="1" ht="53.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="76" t="s">
-        <v>44</v>
+        <v>179</v>
       </c>
       <c r="B3" s="77" t="s">
-        <v>106</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="D3" s="77" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="F3" s="78" t="s">
-        <v>107</v>
-      </c>
-      <c r="G3" s="43" t="s">
-        <v>108</v>
-      </c>
-      <c r="H3" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="I3" s="79" t="s">
-        <v>48</v>
-      </c>
-      <c r="J3" s="78" t="s">
-        <v>49</v>
-      </c>
-      <c r="K3" s="77" t="s">
-        <v>50</v>
-      </c>
-      <c r="L3" s="78" t="s">
-        <v>51</v>
-      </c>
-      <c r="M3" s="80" t="s">
-        <v>52</v>
-      </c>
-      <c r="N3" s="76" t="s">
-        <v>109</v>
-      </c>
-      <c r="O3" s="81" t="s">
+        <v>180</v>
+      </c>
+      <c r="C3" s="94" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="95" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="94" t="s">
+        <v>191</v>
+      </c>
+      <c r="F3" s="94" t="s">
+        <v>192</v>
+      </c>
+      <c r="G3" s="94" t="s">
+        <v>193</v>
+      </c>
+      <c r="H3" s="94" t="s">
+        <v>194</v>
+      </c>
+      <c r="I3" s="94" t="s">
+        <v>195</v>
+      </c>
+      <c r="J3" s="94" t="s">
+        <v>196</v>
+      </c>
+      <c r="K3" s="94" t="s">
+        <v>197</v>
+      </c>
+      <c r="L3" s="94" t="s">
+        <v>198</v>
+      </c>
+      <c r="M3" s="94" t="s">
+        <v>199</v>
+      </c>
+      <c r="N3" s="94" t="s">
+        <v>200</v>
+      </c>
+      <c r="O3" s="94" t="s">
+        <v>201</v>
+      </c>
+      <c r="P3" s="94" t="s">
         <v>110</v>
       </c>
-      <c r="P3" s="82" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q3" s="83" t="s">
-        <v>53</v>
-      </c>
-      <c r="R3" s="77" t="s">
-        <v>54</v>
-      </c>
-      <c r="S3" s="77" t="s">
-        <v>34</v>
-      </c>
-      <c r="T3" s="77" t="s">
-        <v>80</v>
-      </c>
-      <c r="U3" s="77" t="s">
-        <v>111</v>
-      </c>
-      <c r="V3" s="77" t="s">
-        <v>112</v>
-      </c>
-      <c r="W3" s="82" t="s">
+      <c r="Q3" s="94" t="s">
+        <v>202</v>
+      </c>
+      <c r="R3" s="94" t="s">
+        <v>187</v>
+      </c>
+      <c r="S3" s="94" t="s">
+        <v>203</v>
+      </c>
+      <c r="T3" s="96" t="s">
+        <v>204</v>
+      </c>
+      <c r="U3" s="97" t="s">
         <v>42</v>
       </c>
-      <c r="X3" s="74"/>
-      <c r="Y3" s="74"/>
-      <c r="Z3" s="74"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A4" s="69"/>
@@ -2648,23 +3148,17 @@
       <c r="E11" s="77" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="78" t="s">
+      <c r="G11" s="78" t="s">
         <v>107</v>
-      </c>
-      <c r="G11" s="43" t="s">
-        <v>108</v>
       </c>
       <c r="H11" s="44" t="s">
         <v>95</v>
       </c>
-      <c r="I11" s="79" t="s">
+      <c r="J11" s="79" t="s">
         <v>48</v>
       </c>
-      <c r="J11" s="78" t="s">
+      <c r="K11" s="78" t="s">
         <v>49</v>
-      </c>
-      <c r="K11" s="77" t="s">
-        <v>50</v>
       </c>
       <c r="L11" s="78" t="s">
         <v>51</v>
@@ -2672,43 +3166,314 @@
       <c r="M11" s="80" t="s">
         <v>52</v>
       </c>
-      <c r="N11" s="76" t="s">
+      <c r="O11" s="76" t="s">
         <v>109</v>
       </c>
-      <c r="O11" s="81" t="s">
+      <c r="P11" s="81" t="s">
         <v>110</v>
       </c>
-      <c r="P11" s="82" t="s">
+      <c r="Q11" s="82" t="s">
         <v>97</v>
       </c>
-      <c r="Q11" s="83" t="s">
+      <c r="R11" s="83" t="s">
         <v>53</v>
       </c>
-      <c r="R11" s="77" t="s">
-        <v>54</v>
-      </c>
-      <c r="S11" s="77" t="s">
+      <c r="S11" s="77"/>
+      <c r="T11" s="77" t="s">
         <v>34</v>
       </c>
-      <c r="T11" s="77" t="s">
-        <v>80</v>
-      </c>
-      <c r="U11" s="77" t="s">
-        <v>111</v>
-      </c>
-      <c r="V11" s="77" t="s">
-        <v>112</v>
-      </c>
-      <c r="W11" s="82" t="s">
+      <c r="U11" s="82" t="s">
         <v>42</v>
       </c>
+      <c r="V11" s="77"/>
+      <c r="W11" s="77"/>
+      <c r="X11" s="82"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7C2946C-A784-4830-B129-5E94E117C5CC}">
+  <dimension ref="A2:Z11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="2" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="76" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="77" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="77" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="77" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="78" t="s">
+        <v>107</v>
+      </c>
+      <c r="G3" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="H3" s="44" t="s">
+        <v>95</v>
+      </c>
+      <c r="I3" s="79" t="s">
+        <v>48</v>
+      </c>
+      <c r="J3" s="78" t="s">
+        <v>49</v>
+      </c>
+      <c r="K3" s="77" t="s">
+        <v>50</v>
+      </c>
+      <c r="L3" s="78" t="s">
+        <v>51</v>
+      </c>
+      <c r="M3" s="80" t="s">
+        <v>52</v>
+      </c>
+      <c r="N3" s="76" t="s">
+        <v>109</v>
+      </c>
+      <c r="O3" s="81" t="s">
+        <v>110</v>
+      </c>
+      <c r="P3" s="82" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q3" s="83" t="s">
+        <v>53</v>
+      </c>
+      <c r="R3" s="77" t="s">
+        <v>54</v>
+      </c>
+      <c r="S3" s="77" t="s">
+        <v>34</v>
+      </c>
+      <c r="T3" s="77" t="s">
+        <v>80</v>
+      </c>
+      <c r="U3" s="77" t="s">
+        <v>111</v>
+      </c>
+      <c r="V3" s="77" t="s">
+        <v>112</v>
+      </c>
+      <c r="W3" s="82" t="s">
+        <v>42</v>
+      </c>
+      <c r="X3" s="74"/>
+      <c r="Y3" s="74"/>
+      <c r="Z3" s="74"/>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A4" s="69"/>
+      <c r="B4" s="74"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="69"/>
+      <c r="G4" s="74"/>
+      <c r="H4" s="74"/>
+      <c r="I4" s="74"/>
+      <c r="J4" s="74"/>
+      <c r="K4" s="74"/>
+      <c r="L4" s="74"/>
+      <c r="M4" s="74"/>
+      <c r="N4" s="74"/>
+      <c r="O4" s="74"/>
+      <c r="P4" s="74"/>
+      <c r="Q4" s="74"/>
+      <c r="R4" s="74"/>
+      <c r="S4" s="66"/>
+      <c r="T4" s="69"/>
+      <c r="U4" s="74"/>
+      <c r="V4" s="74"/>
+      <c r="W4" s="74"/>
+      <c r="X4" s="74"/>
+      <c r="Y4" s="74"/>
+      <c r="Z4" s="74"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A5" s="69"/>
+      <c r="B5" s="74"/>
+      <c r="C5" s="74"/>
+      <c r="D5" s="67"/>
+      <c r="E5" s="68"/>
+      <c r="F5" s="69"/>
+      <c r="G5" s="69"/>
+      <c r="H5" s="68"/>
+      <c r="I5" s="68"/>
+      <c r="J5" s="69"/>
+      <c r="K5" s="68"/>
+      <c r="L5" s="68"/>
+      <c r="M5" s="69"/>
+      <c r="N5" s="69"/>
+      <c r="O5" s="69"/>
+      <c r="P5" s="69"/>
+      <c r="Q5" s="69"/>
+      <c r="R5" s="69"/>
+      <c r="S5" s="69"/>
+      <c r="T5" s="69"/>
+      <c r="U5" s="68"/>
+      <c r="V5" s="68"/>
+      <c r="W5" s="68"/>
+      <c r="X5" s="68"/>
+      <c r="Y5" s="68"/>
+      <c r="Z5" s="69"/>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A6" s="70"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="70"/>
+      <c r="E6" s="70"/>
+      <c r="F6" s="70"/>
+      <c r="G6" s="75"/>
+      <c r="H6" s="74"/>
+      <c r="I6" s="74"/>
+      <c r="J6" s="75"/>
+      <c r="K6" s="74"/>
+      <c r="L6" s="74"/>
+      <c r="M6" s="71"/>
+      <c r="N6" s="70"/>
+      <c r="O6" s="72"/>
+      <c r="P6" s="70"/>
+      <c r="Q6" s="71"/>
+      <c r="R6" s="70"/>
+      <c r="S6" s="70"/>
+      <c r="T6" s="63"/>
+      <c r="U6" s="74"/>
+      <c r="V6" s="74"/>
+      <c r="W6" s="63"/>
+      <c r="X6" s="74"/>
+      <c r="Y6" s="74"/>
+      <c r="Z6" s="70"/>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A7" s="70"/>
+      <c r="B7" s="73"/>
+      <c r="C7" s="73"/>
+      <c r="D7" s="70"/>
+      <c r="E7" s="70"/>
+      <c r="F7" s="70"/>
+      <c r="G7" s="72"/>
+      <c r="H7" s="73"/>
+      <c r="I7" s="72"/>
+      <c r="J7" s="72"/>
+      <c r="K7" s="72"/>
+      <c r="L7" s="72"/>
+      <c r="M7" s="72"/>
+      <c r="N7" s="72"/>
+      <c r="O7" s="72"/>
+      <c r="P7" s="70"/>
+      <c r="Q7" s="71"/>
+      <c r="R7" s="70"/>
+      <c r="S7" s="70"/>
+      <c r="T7" s="72"/>
+      <c r="U7" s="72"/>
+      <c r="V7" s="72"/>
+      <c r="W7" s="72"/>
+      <c r="X7" s="72"/>
+      <c r="Y7" s="72"/>
+      <c r="Z7" s="70"/>
+    </row>
+    <row r="9" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="10" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>68</v>
+      </c>
+      <c r="N10" s="40"/>
+    </row>
+    <row r="11" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="76" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="77" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" s="77" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="77" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="77" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="78" t="s">
+        <v>107</v>
+      </c>
+      <c r="G11" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="H11" s="44" t="s">
+        <v>95</v>
+      </c>
+      <c r="I11" s="79" t="s">
+        <v>48</v>
+      </c>
+      <c r="J11" s="78" t="s">
+        <v>49</v>
+      </c>
+      <c r="K11" s="77" t="s">
+        <v>50</v>
+      </c>
+      <c r="L11" s="78" t="s">
+        <v>51</v>
+      </c>
+      <c r="M11" s="80" t="s">
+        <v>52</v>
+      </c>
+      <c r="N11" s="76" t="s">
+        <v>109</v>
+      </c>
+      <c r="O11" s="81" t="s">
+        <v>110</v>
+      </c>
+      <c r="P11" s="82" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q11" s="83" t="s">
+        <v>53</v>
+      </c>
+      <c r="R11" s="77" t="s">
+        <v>54</v>
+      </c>
+      <c r="S11" s="77" t="s">
+        <v>34</v>
+      </c>
+      <c r="T11" s="77" t="s">
+        <v>80</v>
+      </c>
+      <c r="U11" s="77" t="s">
+        <v>111</v>
+      </c>
+      <c r="V11" s="77" t="s">
+        <v>112</v>
+      </c>
+      <c r="W11" s="82" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9301C2D9-B641-4509-82EB-A6381EB78A1E}">
   <dimension ref="A2:Z11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2719,77 +3484,77 @@
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="89" t="str">
+      <c r="A3" s="99" t="str">
         <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="87"/>
-      <c r="C3" s="87"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="87"/>
-      <c r="G3" s="87"/>
-      <c r="H3" s="87"/>
-      <c r="I3" s="87"/>
-      <c r="J3" s="87"/>
-      <c r="K3" s="87"/>
-      <c r="L3" s="87"/>
-      <c r="M3" s="87"/>
-      <c r="N3" s="87"/>
-      <c r="O3" s="87"/>
-      <c r="P3" s="87"/>
-      <c r="Q3" s="87"/>
-      <c r="R3" s="87"/>
-      <c r="S3" s="87"/>
-      <c r="T3" s="87"/>
-      <c r="U3" s="87"/>
-      <c r="V3" s="87"/>
-      <c r="W3" s="87"/>
-      <c r="X3" s="87"/>
-      <c r="Y3" s="87"/>
-      <c r="Z3" s="85"/>
+      <c r="B3" s="100"/>
+      <c r="C3" s="100"/>
+      <c r="D3" s="100"/>
+      <c r="E3" s="100"/>
+      <c r="F3" s="100"/>
+      <c r="G3" s="100"/>
+      <c r="H3" s="100"/>
+      <c r="I3" s="100"/>
+      <c r="J3" s="100"/>
+      <c r="K3" s="100"/>
+      <c r="L3" s="100"/>
+      <c r="M3" s="100"/>
+      <c r="N3" s="100"/>
+      <c r="O3" s="100"/>
+      <c r="P3" s="100"/>
+      <c r="Q3" s="100"/>
+      <c r="R3" s="100"/>
+      <c r="S3" s="100"/>
+      <c r="T3" s="100"/>
+      <c r="U3" s="100"/>
+      <c r="V3" s="100"/>
+      <c r="W3" s="100"/>
+      <c r="X3" s="100"/>
+      <c r="Y3" s="100"/>
+      <c r="Z3" s="101"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="89">
+      <c r="A4" s="99">
         <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="87"/>
-      <c r="C4" s="87"/>
-      <c r="D4" s="85"/>
+      <c r="B4" s="100"/>
+      <c r="C4" s="100"/>
+      <c r="D4" s="101"/>
       <c r="E4" s="18"/>
-      <c r="F4" s="89" t="s">
+      <c r="F4" s="99" t="s">
         <v>89</v>
       </c>
-      <c r="G4" s="87"/>
-      <c r="H4" s="87"/>
-      <c r="I4" s="87"/>
-      <c r="J4" s="87"/>
-      <c r="K4" s="87"/>
-      <c r="L4" s="87"/>
-      <c r="M4" s="87"/>
-      <c r="N4" s="87"/>
-      <c r="O4" s="87"/>
-      <c r="P4" s="87"/>
-      <c r="Q4" s="87"/>
-      <c r="R4" s="85"/>
+      <c r="G4" s="100"/>
+      <c r="H4" s="100"/>
+      <c r="I4" s="100"/>
+      <c r="J4" s="100"/>
+      <c r="K4" s="100"/>
+      <c r="L4" s="100"/>
+      <c r="M4" s="100"/>
+      <c r="N4" s="100"/>
+      <c r="O4" s="100"/>
+      <c r="P4" s="100"/>
+      <c r="Q4" s="100"/>
+      <c r="R4" s="101"/>
       <c r="S4" s="19"/>
-      <c r="T4" s="89" t="s">
+      <c r="T4" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="U4" s="87"/>
-      <c r="V4" s="87"/>
-      <c r="W4" s="87"/>
-      <c r="X4" s="87"/>
-      <c r="Y4" s="87"/>
-      <c r="Z4" s="85"/>
+      <c r="U4" s="100"/>
+      <c r="V4" s="100"/>
+      <c r="W4" s="100"/>
+      <c r="X4" s="100"/>
+      <c r="Y4" s="100"/>
+      <c r="Z4" s="101"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="89" t="s">
+      <c r="A5" s="99" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="87"/>
-      <c r="C5" s="85"/>
+      <c r="B5" s="100"/>
+      <c r="C5" s="101"/>
       <c r="D5" s="20">
         <f>[1]Summary!R7</f>
         <v>0</v>
@@ -2848,10 +3613,10 @@
       <c r="A6" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="84" t="s">
+      <c r="B6" s="102" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="85"/>
+      <c r="C6" s="101"/>
       <c r="D6" s="25" t="s">
         <v>93</v>
       </c>
@@ -2861,16 +3626,16 @@
       <c r="F6" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="G6" s="86" t="s">
+      <c r="G6" s="103" t="s">
         <v>96</v>
       </c>
-      <c r="H6" s="87"/>
-      <c r="I6" s="85"/>
-      <c r="J6" s="86" t="s">
+      <c r="H6" s="100"/>
+      <c r="I6" s="101"/>
+      <c r="J6" s="103" t="s">
         <v>37</v>
       </c>
-      <c r="K6" s="87"/>
-      <c r="L6" s="85"/>
+      <c r="K6" s="100"/>
+      <c r="L6" s="101"/>
       <c r="M6" s="28" t="s">
         <v>97</v>
       </c>
@@ -2890,16 +3655,16 @@
         <v>42</v>
       </c>
       <c r="S6" s="33"/>
-      <c r="T6" s="88" t="s">
+      <c r="T6" s="104" t="s">
         <v>102</v>
       </c>
-      <c r="U6" s="87"/>
-      <c r="V6" s="85"/>
-      <c r="W6" s="88" t="s">
+      <c r="U6" s="100"/>
+      <c r="V6" s="101"/>
+      <c r="W6" s="104" t="s">
         <v>103</v>
       </c>
-      <c r="X6" s="87"/>
-      <c r="Y6" s="85"/>
+      <c r="X6" s="100"/>
+      <c r="Y6" s="101"/>
       <c r="Z6" s="31" t="s">
         <v>100</v>
       </c>
@@ -3020,16 +3785,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="W6:Y6"/>
     <mergeCell ref="A3:Z3"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:R4"/>
     <mergeCell ref="T4:Z4"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="W6:Y6"/>
   </mergeCells>
   <conditionalFormatting sqref="B11">
     <cfRule type="duplicateValues" dxfId="7" priority="2"/>
@@ -3041,7 +3806,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAEF05BD-52B1-49ED-A017-76486C00039F}">
   <dimension ref="A2:Z16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3052,77 +3817,77 @@
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="89" t="str">
+      <c r="A3" s="99" t="str">
         <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="87"/>
-      <c r="C3" s="87"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="87"/>
-      <c r="G3" s="87"/>
-      <c r="H3" s="87"/>
-      <c r="I3" s="87"/>
-      <c r="J3" s="87"/>
-      <c r="K3" s="87"/>
-      <c r="L3" s="87"/>
-      <c r="M3" s="87"/>
-      <c r="N3" s="87"/>
-      <c r="O3" s="87"/>
-      <c r="P3" s="87"/>
-      <c r="Q3" s="87"/>
-      <c r="R3" s="87"/>
-      <c r="S3" s="87"/>
-      <c r="T3" s="87"/>
-      <c r="U3" s="87"/>
-      <c r="V3" s="87"/>
-      <c r="W3" s="87"/>
-      <c r="X3" s="87"/>
-      <c r="Y3" s="87"/>
-      <c r="Z3" s="85"/>
+      <c r="B3" s="100"/>
+      <c r="C3" s="100"/>
+      <c r="D3" s="100"/>
+      <c r="E3" s="100"/>
+      <c r="F3" s="100"/>
+      <c r="G3" s="100"/>
+      <c r="H3" s="100"/>
+      <c r="I3" s="100"/>
+      <c r="J3" s="100"/>
+      <c r="K3" s="100"/>
+      <c r="L3" s="100"/>
+      <c r="M3" s="100"/>
+      <c r="N3" s="100"/>
+      <c r="O3" s="100"/>
+      <c r="P3" s="100"/>
+      <c r="Q3" s="100"/>
+      <c r="R3" s="100"/>
+      <c r="S3" s="100"/>
+      <c r="T3" s="100"/>
+      <c r="U3" s="100"/>
+      <c r="V3" s="100"/>
+      <c r="W3" s="100"/>
+      <c r="X3" s="100"/>
+      <c r="Y3" s="100"/>
+      <c r="Z3" s="101"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="89">
+      <c r="A4" s="99">
         <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="87"/>
-      <c r="C4" s="87"/>
-      <c r="D4" s="85"/>
+      <c r="B4" s="100"/>
+      <c r="C4" s="100"/>
+      <c r="D4" s="101"/>
       <c r="E4" s="18"/>
-      <c r="F4" s="89" t="s">
+      <c r="F4" s="99" t="s">
         <v>89</v>
       </c>
-      <c r="G4" s="87"/>
-      <c r="H4" s="87"/>
-      <c r="I4" s="87"/>
-      <c r="J4" s="87"/>
-      <c r="K4" s="87"/>
-      <c r="L4" s="87"/>
-      <c r="M4" s="87"/>
-      <c r="N4" s="87"/>
-      <c r="O4" s="87"/>
-      <c r="P4" s="87"/>
-      <c r="Q4" s="87"/>
-      <c r="R4" s="85"/>
+      <c r="G4" s="100"/>
+      <c r="H4" s="100"/>
+      <c r="I4" s="100"/>
+      <c r="J4" s="100"/>
+      <c r="K4" s="100"/>
+      <c r="L4" s="100"/>
+      <c r="M4" s="100"/>
+      <c r="N4" s="100"/>
+      <c r="O4" s="100"/>
+      <c r="P4" s="100"/>
+      <c r="Q4" s="100"/>
+      <c r="R4" s="101"/>
       <c r="S4" s="19"/>
-      <c r="T4" s="89" t="s">
+      <c r="T4" s="99" t="s">
         <v>90</v>
       </c>
-      <c r="U4" s="87"/>
-      <c r="V4" s="87"/>
-      <c r="W4" s="87"/>
-      <c r="X4" s="87"/>
-      <c r="Y4" s="87"/>
-      <c r="Z4" s="85"/>
+      <c r="U4" s="100"/>
+      <c r="V4" s="100"/>
+      <c r="W4" s="100"/>
+      <c r="X4" s="100"/>
+      <c r="Y4" s="100"/>
+      <c r="Z4" s="101"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="89" t="s">
+      <c r="A5" s="99" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="87"/>
-      <c r="C5" s="85"/>
+      <c r="B5" s="100"/>
+      <c r="C5" s="101"/>
       <c r="D5" s="20">
         <f>[1]Summary!R7</f>
         <v>0</v>
@@ -3181,10 +3946,10 @@
       <c r="A6" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="84" t="s">
+      <c r="B6" s="102" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="85"/>
+      <c r="C6" s="101"/>
       <c r="D6" s="25" t="s">
         <v>93</v>
       </c>
@@ -3194,16 +3959,16 @@
       <c r="F6" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="G6" s="86" t="s">
+      <c r="G6" s="103" t="s">
         <v>96</v>
       </c>
-      <c r="H6" s="87"/>
-      <c r="I6" s="85"/>
-      <c r="J6" s="86" t="s">
+      <c r="H6" s="100"/>
+      <c r="I6" s="101"/>
+      <c r="J6" s="103" t="s">
         <v>37</v>
       </c>
-      <c r="K6" s="87"/>
-      <c r="L6" s="85"/>
+      <c r="K6" s="100"/>
+      <c r="L6" s="101"/>
       <c r="M6" s="28" t="s">
         <v>97</v>
       </c>
@@ -3223,16 +3988,16 @@
         <v>42</v>
       </c>
       <c r="S6" s="33"/>
-      <c r="T6" s="88" t="s">
+      <c r="T6" s="104" t="s">
         <v>102</v>
       </c>
-      <c r="U6" s="87"/>
-      <c r="V6" s="85"/>
-      <c r="W6" s="88" t="s">
+      <c r="U6" s="100"/>
+      <c r="V6" s="101"/>
+      <c r="W6" s="104" t="s">
         <v>103</v>
       </c>
-      <c r="X6" s="87"/>
-      <c r="Y6" s="85"/>
+      <c r="X6" s="100"/>
+      <c r="Y6" s="101"/>
       <c r="Z6" s="31" t="s">
         <v>100</v>
       </c>
@@ -3380,16 +4145,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="W6:Y6"/>
     <mergeCell ref="A3:Z3"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="F4:R4"/>
     <mergeCell ref="T4:Z4"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="W6:Y6"/>
   </mergeCells>
   <conditionalFormatting sqref="B11">
     <cfRule type="duplicateValues" dxfId="5" priority="2"/>
@@ -3401,65 +4166,65 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B501B5B8-47AF-4D49-A01B-A8E1BEE40158}">
   <dimension ref="A1:BM10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:65" x14ac:dyDescent="0.35">
-      <c r="A1" s="88"/>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
-      <c r="N1" s="90"/>
-      <c r="O1" s="90"/>
-      <c r="P1" s="90"/>
-      <c r="Q1" s="90"/>
-      <c r="R1" s="90"/>
-      <c r="S1" s="90"/>
-      <c r="T1" s="90"/>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="90"/>
-      <c r="Z1" s="90"/>
-      <c r="AA1" s="90"/>
-      <c r="AB1" s="90"/>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="90"/>
-      <c r="AE1" s="90"/>
-      <c r="AF1" s="90"/>
-      <c r="AG1" s="90"/>
-      <c r="AH1" s="90"/>
-      <c r="AI1" s="90"/>
-      <c r="AJ1" s="90"/>
-      <c r="AK1" s="90"/>
-      <c r="AL1" s="87"/>
-      <c r="AM1" s="87"/>
-      <c r="AN1" s="87"/>
-      <c r="AO1" s="87"/>
-      <c r="AP1" s="87"/>
-      <c r="AQ1" s="90"/>
-      <c r="AR1" s="90"/>
-      <c r="AS1" s="90"/>
-      <c r="AT1" s="90"/>
-      <c r="AU1" s="90"/>
-      <c r="AV1" s="90"/>
-      <c r="AW1" s="90"/>
-      <c r="AX1" s="90"/>
-      <c r="AY1" s="90"/>
-      <c r="AZ1" s="90"/>
-      <c r="BA1" s="91"/>
+      <c r="A1" s="104"/>
+      <c r="B1" s="105"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="105"/>
+      <c r="F1" s="105"/>
+      <c r="G1" s="105"/>
+      <c r="H1" s="105"/>
+      <c r="I1" s="105"/>
+      <c r="J1" s="105"/>
+      <c r="K1" s="105"/>
+      <c r="L1" s="105"/>
+      <c r="M1" s="105"/>
+      <c r="N1" s="105"/>
+      <c r="O1" s="105"/>
+      <c r="P1" s="105"/>
+      <c r="Q1" s="105"/>
+      <c r="R1" s="105"/>
+      <c r="S1" s="105"/>
+      <c r="T1" s="105"/>
+      <c r="U1" s="105"/>
+      <c r="V1" s="105"/>
+      <c r="W1" s="105"/>
+      <c r="X1" s="105"/>
+      <c r="Y1" s="105"/>
+      <c r="Z1" s="105"/>
+      <c r="AA1" s="105"/>
+      <c r="AB1" s="105"/>
+      <c r="AC1" s="105"/>
+      <c r="AD1" s="105"/>
+      <c r="AE1" s="105"/>
+      <c r="AF1" s="105"/>
+      <c r="AG1" s="105"/>
+      <c r="AH1" s="105"/>
+      <c r="AI1" s="105"/>
+      <c r="AJ1" s="105"/>
+      <c r="AK1" s="105"/>
+      <c r="AL1" s="100"/>
+      <c r="AM1" s="100"/>
+      <c r="AN1" s="100"/>
+      <c r="AO1" s="100"/>
+      <c r="AP1" s="100"/>
+      <c r="AQ1" s="105"/>
+      <c r="AR1" s="105"/>
+      <c r="AS1" s="105"/>
+      <c r="AT1" s="105"/>
+      <c r="AU1" s="105"/>
+      <c r="AV1" s="105"/>
+      <c r="AW1" s="105"/>
+      <c r="AX1" s="105"/>
+      <c r="AY1" s="105"/>
+      <c r="AZ1" s="105"/>
+      <c r="BA1" s="106"/>
     </row>
     <row r="2" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -3842,7 +4607,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECB08AFA-BF49-47F5-B095-34C6A355FE30}">
   <dimension ref="A2:BA10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3856,186 +4621,186 @@
       </c>
     </row>
     <row r="3" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A3" s="88" t="str">
+      <c r="A3" s="104" t="str">
         <f>+[2]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="90"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
-      <c r="J3" s="90"/>
-      <c r="K3" s="90"/>
-      <c r="L3" s="90"/>
-      <c r="M3" s="90"/>
-      <c r="N3" s="90"/>
-      <c r="O3" s="90"/>
-      <c r="P3" s="90"/>
-      <c r="Q3" s="90"/>
-      <c r="R3" s="90"/>
-      <c r="S3" s="90"/>
-      <c r="T3" s="90"/>
-      <c r="U3" s="90"/>
-      <c r="V3" s="90"/>
-      <c r="W3" s="90"/>
-      <c r="X3" s="90"/>
-      <c r="Y3" s="90"/>
-      <c r="Z3" s="90"/>
-      <c r="AA3" s="90"/>
-      <c r="AB3" s="90"/>
-      <c r="AC3" s="90"/>
-      <c r="AD3" s="90"/>
-      <c r="AE3" s="90"/>
-      <c r="AF3" s="90"/>
-      <c r="AG3" s="90"/>
-      <c r="AH3" s="90"/>
-      <c r="AI3" s="90"/>
-      <c r="AJ3" s="90"/>
-      <c r="AK3" s="90"/>
-      <c r="AL3" s="87"/>
-      <c r="AM3" s="87"/>
-      <c r="AN3" s="87"/>
-      <c r="AO3" s="87"/>
-      <c r="AP3" s="87"/>
-      <c r="AQ3" s="90"/>
-      <c r="AR3" s="90"/>
-      <c r="AS3" s="90"/>
-      <c r="AT3" s="90"/>
-      <c r="AU3" s="90"/>
-      <c r="AV3" s="90"/>
-      <c r="AW3" s="90"/>
-      <c r="AX3" s="90"/>
-      <c r="AY3" s="90"/>
-      <c r="AZ3" s="90"/>
-      <c r="BA3" s="91"/>
+      <c r="B3" s="105"/>
+      <c r="C3" s="105"/>
+      <c r="D3" s="105"/>
+      <c r="E3" s="105"/>
+      <c r="F3" s="105"/>
+      <c r="G3" s="105"/>
+      <c r="H3" s="105"/>
+      <c r="I3" s="105"/>
+      <c r="J3" s="105"/>
+      <c r="K3" s="105"/>
+      <c r="L3" s="105"/>
+      <c r="M3" s="105"/>
+      <c r="N3" s="105"/>
+      <c r="O3" s="105"/>
+      <c r="P3" s="105"/>
+      <c r="Q3" s="105"/>
+      <c r="R3" s="105"/>
+      <c r="S3" s="105"/>
+      <c r="T3" s="105"/>
+      <c r="U3" s="105"/>
+      <c r="V3" s="105"/>
+      <c r="W3" s="105"/>
+      <c r="X3" s="105"/>
+      <c r="Y3" s="105"/>
+      <c r="Z3" s="105"/>
+      <c r="AA3" s="105"/>
+      <c r="AB3" s="105"/>
+      <c r="AC3" s="105"/>
+      <c r="AD3" s="105"/>
+      <c r="AE3" s="105"/>
+      <c r="AF3" s="105"/>
+      <c r="AG3" s="105"/>
+      <c r="AH3" s="105"/>
+      <c r="AI3" s="105"/>
+      <c r="AJ3" s="105"/>
+      <c r="AK3" s="105"/>
+      <c r="AL3" s="100"/>
+      <c r="AM3" s="100"/>
+      <c r="AN3" s="100"/>
+      <c r="AO3" s="100"/>
+      <c r="AP3" s="100"/>
+      <c r="AQ3" s="105"/>
+      <c r="AR3" s="105"/>
+      <c r="AS3" s="105"/>
+      <c r="AT3" s="105"/>
+      <c r="AU3" s="105"/>
+      <c r="AV3" s="105"/>
+      <c r="AW3" s="105"/>
+      <c r="AX3" s="105"/>
+      <c r="AY3" s="105"/>
+      <c r="AZ3" s="105"/>
+      <c r="BA3" s="106"/>
     </row>
     <row r="4" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A4" s="88">
+      <c r="A4" s="104">
         <f>+[2]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="90"/>
-      <c r="C4" s="90"/>
-      <c r="D4" s="90"/>
-      <c r="E4" s="90"/>
-      <c r="F4" s="90"/>
-      <c r="G4" s="90"/>
-      <c r="H4" s="90"/>
-      <c r="I4" s="90"/>
-      <c r="J4" s="90"/>
-      <c r="K4" s="90"/>
-      <c r="L4" s="90"/>
-      <c r="M4" s="90"/>
-      <c r="N4" s="90"/>
-      <c r="O4" s="90"/>
-      <c r="P4" s="90"/>
-      <c r="Q4" s="90"/>
-      <c r="R4" s="90"/>
-      <c r="S4" s="90"/>
-      <c r="T4" s="90"/>
-      <c r="U4" s="90"/>
-      <c r="V4" s="90"/>
-      <c r="W4" s="90"/>
-      <c r="X4" s="90"/>
-      <c r="Y4" s="90"/>
-      <c r="Z4" s="90"/>
-      <c r="AA4" s="90"/>
-      <c r="AB4" s="90"/>
-      <c r="AC4" s="90"/>
-      <c r="AD4" s="90"/>
-      <c r="AE4" s="90"/>
-      <c r="AF4" s="90"/>
-      <c r="AG4" s="90"/>
-      <c r="AH4" s="90"/>
-      <c r="AI4" s="90"/>
-      <c r="AJ4" s="90"/>
-      <c r="AK4" s="90"/>
-      <c r="AL4" s="87"/>
-      <c r="AM4" s="87"/>
-      <c r="AN4" s="87"/>
-      <c r="AO4" s="87"/>
-      <c r="AP4" s="87"/>
-      <c r="AQ4" s="90"/>
-      <c r="AR4" s="90"/>
-      <c r="AS4" s="90"/>
-      <c r="AT4" s="90"/>
-      <c r="AU4" s="90"/>
-      <c r="AV4" s="90"/>
-      <c r="AW4" s="90"/>
-      <c r="AX4" s="90"/>
-      <c r="AY4" s="90"/>
-      <c r="AZ4" s="90"/>
-      <c r="BA4" s="91"/>
+      <c r="B4" s="105"/>
+      <c r="C4" s="105"/>
+      <c r="D4" s="105"/>
+      <c r="E4" s="105"/>
+      <c r="F4" s="105"/>
+      <c r="G4" s="105"/>
+      <c r="H4" s="105"/>
+      <c r="I4" s="105"/>
+      <c r="J4" s="105"/>
+      <c r="K4" s="105"/>
+      <c r="L4" s="105"/>
+      <c r="M4" s="105"/>
+      <c r="N4" s="105"/>
+      <c r="O4" s="105"/>
+      <c r="P4" s="105"/>
+      <c r="Q4" s="105"/>
+      <c r="R4" s="105"/>
+      <c r="S4" s="105"/>
+      <c r="T4" s="105"/>
+      <c r="U4" s="105"/>
+      <c r="V4" s="105"/>
+      <c r="W4" s="105"/>
+      <c r="X4" s="105"/>
+      <c r="Y4" s="105"/>
+      <c r="Z4" s="105"/>
+      <c r="AA4" s="105"/>
+      <c r="AB4" s="105"/>
+      <c r="AC4" s="105"/>
+      <c r="AD4" s="105"/>
+      <c r="AE4" s="105"/>
+      <c r="AF4" s="105"/>
+      <c r="AG4" s="105"/>
+      <c r="AH4" s="105"/>
+      <c r="AI4" s="105"/>
+      <c r="AJ4" s="105"/>
+      <c r="AK4" s="105"/>
+      <c r="AL4" s="100"/>
+      <c r="AM4" s="100"/>
+      <c r="AN4" s="100"/>
+      <c r="AO4" s="100"/>
+      <c r="AP4" s="100"/>
+      <c r="AQ4" s="105"/>
+      <c r="AR4" s="105"/>
+      <c r="AS4" s="105"/>
+      <c r="AT4" s="105"/>
+      <c r="AU4" s="105"/>
+      <c r="AV4" s="105"/>
+      <c r="AW4" s="105"/>
+      <c r="AX4" s="105"/>
+      <c r="AY4" s="105"/>
+      <c r="AZ4" s="105"/>
+      <c r="BA4" s="106"/>
     </row>
     <row r="5" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="88" t="s">
+      <c r="A5" s="104" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="90"/>
-      <c r="C5" s="90"/>
-      <c r="D5" s="90"/>
-      <c r="E5" s="90"/>
-      <c r="F5" s="90"/>
-      <c r="G5" s="90"/>
-      <c r="H5" s="90"/>
-      <c r="I5" s="90"/>
-      <c r="J5" s="90"/>
-      <c r="K5" s="90"/>
-      <c r="L5" s="90"/>
-      <c r="M5" s="90"/>
-      <c r="N5" s="90"/>
-      <c r="O5" s="90"/>
-      <c r="P5" s="90"/>
-      <c r="Q5" s="90"/>
-      <c r="R5" s="90"/>
-      <c r="S5" s="91"/>
-      <c r="T5" s="88" t="s">
+      <c r="B5" s="105"/>
+      <c r="C5" s="105"/>
+      <c r="D5" s="105"/>
+      <c r="E5" s="105"/>
+      <c r="F5" s="105"/>
+      <c r="G5" s="105"/>
+      <c r="H5" s="105"/>
+      <c r="I5" s="105"/>
+      <c r="J5" s="105"/>
+      <c r="K5" s="105"/>
+      <c r="L5" s="105"/>
+      <c r="M5" s="105"/>
+      <c r="N5" s="105"/>
+      <c r="O5" s="105"/>
+      <c r="P5" s="105"/>
+      <c r="Q5" s="105"/>
+      <c r="R5" s="105"/>
+      <c r="S5" s="106"/>
+      <c r="T5" s="104" t="s">
         <v>114</v>
       </c>
-      <c r="U5" s="90"/>
-      <c r="V5" s="90"/>
-      <c r="W5" s="90"/>
-      <c r="X5" s="90"/>
-      <c r="Y5" s="90"/>
-      <c r="Z5" s="90"/>
-      <c r="AA5" s="90"/>
-      <c r="AB5" s="90"/>
-      <c r="AC5" s="90"/>
-      <c r="AD5" s="90"/>
-      <c r="AE5" s="90"/>
-      <c r="AF5" s="90"/>
-      <c r="AG5" s="90"/>
-      <c r="AH5" s="90"/>
-      <c r="AI5" s="90"/>
-      <c r="AJ5" s="90"/>
-      <c r="AK5" s="91"/>
-      <c r="AL5" s="88" t="s">
+      <c r="U5" s="105"/>
+      <c r="V5" s="105"/>
+      <c r="W5" s="105"/>
+      <c r="X5" s="105"/>
+      <c r="Y5" s="105"/>
+      <c r="Z5" s="105"/>
+      <c r="AA5" s="105"/>
+      <c r="AB5" s="105"/>
+      <c r="AC5" s="105"/>
+      <c r="AD5" s="105"/>
+      <c r="AE5" s="105"/>
+      <c r="AF5" s="105"/>
+      <c r="AG5" s="105"/>
+      <c r="AH5" s="105"/>
+      <c r="AI5" s="105"/>
+      <c r="AJ5" s="105"/>
+      <c r="AK5" s="106"/>
+      <c r="AL5" s="104" t="s">
         <v>115</v>
       </c>
-      <c r="AM5" s="87"/>
-      <c r="AN5" s="87"/>
-      <c r="AO5" s="87"/>
-      <c r="AP5" s="85"/>
-      <c r="AQ5" s="88" t="s">
+      <c r="AM5" s="100"/>
+      <c r="AN5" s="100"/>
+      <c r="AO5" s="100"/>
+      <c r="AP5" s="101"/>
+      <c r="AQ5" s="104" t="s">
         <v>2</v>
       </c>
-      <c r="AR5" s="90"/>
-      <c r="AS5" s="90"/>
-      <c r="AT5" s="91"/>
+      <c r="AR5" s="105"/>
+      <c r="AS5" s="105"/>
+      <c r="AT5" s="106"/>
       <c r="AU5" s="27" t="s">
         <v>116</v>
       </c>
-      <c r="AV5" s="88" t="s">
+      <c r="AV5" s="104" t="s">
         <v>117</v>
       </c>
-      <c r="AW5" s="90"/>
-      <c r="AX5" s="90"/>
-      <c r="AY5" s="90"/>
-      <c r="AZ5" s="91"/>
+      <c r="AW5" s="105"/>
+      <c r="AX5" s="105"/>
+      <c r="AY5" s="105"/>
+      <c r="AZ5" s="106"/>
       <c r="BA5" s="27" t="s">
         <v>118</v>
       </c>
@@ -4053,24 +4818,24 @@
       <c r="D6" s="50"/>
       <c r="E6" s="50"/>
       <c r="F6" s="50"/>
-      <c r="G6" s="92" t="s">
+      <c r="G6" s="107" t="s">
         <v>81</v>
       </c>
-      <c r="H6" s="93"/>
-      <c r="I6" s="93"/>
-      <c r="J6" s="94"/>
-      <c r="K6" s="92" t="s">
+      <c r="H6" s="108"/>
+      <c r="I6" s="108"/>
+      <c r="J6" s="109"/>
+      <c r="K6" s="107" t="s">
         <v>120</v>
       </c>
-      <c r="L6" s="93"/>
-      <c r="M6" s="93"/>
-      <c r="N6" s="94"/>
-      <c r="O6" s="95" t="s">
+      <c r="L6" s="108"/>
+      <c r="M6" s="108"/>
+      <c r="N6" s="109"/>
+      <c r="O6" s="110" t="s">
         <v>121</v>
       </c>
-      <c r="P6" s="90"/>
-      <c r="Q6" s="90"/>
-      <c r="R6" s="91"/>
+      <c r="P6" s="105"/>
+      <c r="Q6" s="105"/>
+      <c r="R6" s="106"/>
       <c r="S6" s="51" t="s">
         <v>122</v>
       </c>
@@ -4080,11 +4845,11 @@
       <c r="U6" s="31" t="s">
         <v>123</v>
       </c>
-      <c r="V6" s="88" t="s">
+      <c r="V6" s="104" t="s">
         <v>124</v>
       </c>
-      <c r="W6" s="90"/>
-      <c r="X6" s="91"/>
+      <c r="W6" s="105"/>
+      <c r="X6" s="106"/>
       <c r="Y6" s="52" t="s">
         <v>125</v>
       </c>
@@ -4109,14 +4874,14 @@
       <c r="AF6" s="27" t="s">
         <v>132</v>
       </c>
-      <c r="AG6" s="96" t="s">
+      <c r="AG6" s="111" t="s">
         <v>133</v>
       </c>
-      <c r="AH6" s="91"/>
-      <c r="AI6" s="88" t="s">
+      <c r="AH6" s="106"/>
+      <c r="AI6" s="104" t="s">
         <v>134</v>
       </c>
-      <c r="AJ6" s="91"/>
+      <c r="AJ6" s="106"/>
       <c r="AK6" s="27" t="s">
         <v>100</v>
       </c>
@@ -4301,6 +5066,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="O6:R6"/>
+    <mergeCell ref="V6:X6"/>
+    <mergeCell ref="AG6:AH6"/>
     <mergeCell ref="A3:BA3"/>
     <mergeCell ref="A4:BA4"/>
     <mergeCell ref="A5:S5"/>
@@ -4308,18 +5079,12 @@
     <mergeCell ref="AL5:AP5"/>
     <mergeCell ref="AQ5:AT5"/>
     <mergeCell ref="AV5:AZ5"/>
-    <mergeCell ref="AI6:AJ6"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="K6:N6"/>
-    <mergeCell ref="O6:R6"/>
-    <mergeCell ref="V6:X6"/>
-    <mergeCell ref="AG6:AH6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0CAA689-52FE-4282-BFA7-7FA3F37BB8D4}">
   <dimension ref="A2:W7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -4330,35 +5095,35 @@
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="99" t="s">
+      <c r="A3" s="114" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="100" t="s">
+      <c r="B3" s="115" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="87"/>
-      <c r="D3" s="85"/>
-      <c r="E3" s="100" t="s">
+      <c r="C3" s="100"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="115" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="87"/>
-      <c r="G3" s="85"/>
-      <c r="H3" s="100" t="s">
+      <c r="F3" s="100"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="115" t="s">
         <v>37</v>
       </c>
-      <c r="I3" s="87"/>
-      <c r="J3" s="85"/>
-      <c r="K3" s="99" t="s">
+      <c r="I3" s="100"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="114" t="s">
         <v>74</v>
       </c>
-      <c r="L3" s="97" t="s">
+      <c r="L3" s="112" t="s">
         <v>42</v>
       </c>
       <c r="M3" s="8"/>
       <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="31" x14ac:dyDescent="0.35">
-      <c r="A4" s="98"/>
+      <c r="A4" s="113"/>
       <c r="B4" s="12" t="s">
         <v>38</v>
       </c>
@@ -4386,8 +5151,8 @@
       <c r="J4" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="K4" s="98"/>
-      <c r="L4" s="98"/>
+      <c r="K4" s="113"/>
+      <c r="L4" s="113"/>
       <c r="M4" s="10"/>
       <c r="N4" s="11"/>
     </row>
@@ -4453,231 +5218,4 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B225AA6-68BC-47EB-9948-84B6B216E727}">
-  <dimension ref="A2:W7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A3" s="104" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="104" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="104"/>
-      <c r="D3" s="104" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="104" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" s="104" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="105" t="s">
-        <v>36</v>
-      </c>
-      <c r="H3" s="105"/>
-      <c r="I3" s="105"/>
-      <c r="J3" s="101" t="s">
-        <v>37</v>
-      </c>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="103"/>
-    </row>
-    <row r="4" spans="1:23" ht="26" x14ac:dyDescent="0.35">
-      <c r="A4" s="104"/>
-      <c r="B4" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="104"/>
-      <c r="E4" s="104"/>
-      <c r="F4" s="104"/>
-      <c r="G4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D7" t="s">
-        <v>107</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="4"/>
-      <c r="R7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="3"/>
-      <c r="V7" s="3"/>
-      <c r="W7" s="4"/>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="J3:N3"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:I3"/>
-  </mergeCells>
-  <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C7">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBFB976A-1B92-4632-9799-0237B459A61D}">
-  <dimension ref="A1:P5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C3" s="7"/>
-      <c r="D3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="106"/>
-      <c r="H3" s="107"/>
-      <c r="I3" s="107"/>
-      <c r="J3" s="108"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="106"/>
-      <c r="O3" s="107"/>
-      <c r="P3" s="108"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="N3:P3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Auto pipeline update 2026-04-21 16:09:52
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{267EDEAC-9010-47DB-82E9-1AAF7FC2FDED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{175B78F5-822C-49FB-BA36-5C186F7038E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="962" activeTab="2" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="899" firstSheet="2" activeTab="4" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet Names Check" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
     <externalReference r:id="rId13"/>
     <externalReference r:id="rId14"/>
   </externalReferences>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="205">
   <si>
     <t>Project Code</t>
   </si>
@@ -1631,19 +1631,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3475,7 +3475,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9301C2D9-B641-4509-82EB-A6381EB78A1E}">
-  <dimension ref="A2:Z11"/>
+  <dimension ref="A2:Z7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
@@ -3483,323 +3483,213 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="99" t="str">
-        <f>+[1]Summary!A4</f>
-        <v>Office:  Neemuch</v>
-      </c>
-      <c r="B3" s="100"/>
+    <row r="3" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" s="99" t="s">
+        <v>32</v>
+      </c>
       <c r="C3" s="100"/>
-      <c r="D3" s="100"/>
-      <c r="E3" s="100"/>
-      <c r="F3" s="100"/>
-      <c r="G3" s="100"/>
-      <c r="H3" s="100"/>
+      <c r="D3" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="E3" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="F3" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="G3" s="101" t="s">
+        <v>96</v>
+      </c>
+      <c r="H3" s="102"/>
       <c r="I3" s="100"/>
-      <c r="J3" s="100"/>
-      <c r="K3" s="100"/>
+      <c r="J3" s="101" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" s="102"/>
       <c r="L3" s="100"/>
-      <c r="M3" s="100"/>
-      <c r="N3" s="100"/>
-      <c r="O3" s="100"/>
-      <c r="P3" s="100"/>
-      <c r="Q3" s="100"/>
-      <c r="R3" s="100"/>
-      <c r="S3" s="100"/>
-      <c r="T3" s="100"/>
+      <c r="M3" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="N3" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="O3" s="31" t="s">
+        <v>100</v>
+      </c>
+      <c r="P3" s="32" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q3" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="R3" s="33"/>
+      <c r="S3" s="103" t="s">
+        <v>102</v>
+      </c>
+      <c r="T3" s="102"/>
       <c r="U3" s="100"/>
-      <c r="V3" s="100"/>
-      <c r="W3" s="100"/>
+      <c r="V3" s="103" t="s">
+        <v>103</v>
+      </c>
+      <c r="W3" s="102"/>
       <c r="X3" s="100"/>
-      <c r="Y3" s="100"/>
-      <c r="Z3" s="101"/>
+      <c r="Y3" s="31" t="s">
+        <v>100</v>
+      </c>
+      <c r="Z3" s="74"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="99">
-        <f>+[1]Summary!A7</f>
-        <v>0</v>
-      </c>
-      <c r="B4" s="100"/>
-      <c r="C4" s="100"/>
-      <c r="D4" s="101"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="99" t="s">
-        <v>89</v>
-      </c>
-      <c r="G4" s="100"/>
-      <c r="H4" s="100"/>
-      <c r="I4" s="100"/>
-      <c r="J4" s="100"/>
-      <c r="K4" s="100"/>
-      <c r="L4" s="100"/>
-      <c r="M4" s="100"/>
-      <c r="N4" s="100"/>
-      <c r="O4" s="100"/>
-      <c r="P4" s="100"/>
-      <c r="Q4" s="100"/>
-      <c r="R4" s="101"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="99" t="s">
-        <v>90</v>
-      </c>
-      <c r="U4" s="100"/>
-      <c r="V4" s="100"/>
-      <c r="W4" s="100"/>
-      <c r="X4" s="100"/>
-      <c r="Y4" s="100"/>
-      <c r="Z4" s="101"/>
+      <c r="A4" s="25"/>
+      <c r="B4" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="25"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="H4" s="37" t="s">
+        <v>104</v>
+      </c>
+      <c r="I4" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="J4" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="K4" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="L4" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="M4" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="N4" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="O4" s="31"/>
+      <c r="P4" s="38"/>
+      <c r="Q4" s="36"/>
+      <c r="R4" s="39"/>
+      <c r="S4" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="T4" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="U4" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="V4" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="W4" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="X4" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="Y4" s="31"/>
+      <c r="Z4" s="74"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="99" t="s">
-        <v>91</v>
-      </c>
-      <c r="B5" s="100"/>
-      <c r="C5" s="101"/>
-      <c r="D5" s="20">
-        <f>[1]Summary!R7</f>
-        <v>0</v>
-      </c>
-      <c r="E5" s="21">
-        <f>SUMIF(E8:E215,"C",$D$6:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="23">
-        <f>SUMIF(G9:G215,"WIP",$D$7:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="I5" s="21">
-        <f>SUMIF(G8:G215,"C",$D$6:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="J5" s="22"/>
-      <c r="K5" s="23">
-        <f>SUMIF(J9:J215,"WIP",$D$7:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L5" s="21">
-        <f>SUMIF(J8:J215,"C",$D$6:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="22"/>
-      <c r="R5" s="22"/>
-      <c r="S5" s="24"/>
-      <c r="T5" s="22"/>
-      <c r="U5" s="23">
-        <f>SUMIF(T9:T215,"WIP",$D$7:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="V5" s="23">
-        <f>SUMIF(T9:T215,"C",$D$7:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="W5" s="23"/>
-      <c r="X5" s="23">
-        <f>SUMIF(W9:W215,"WIP",$D$7:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="Y5" s="23">
-        <f>SUMIF(W9:W215,"C",$D$7:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="Z5" s="22"/>
-    </row>
-    <row r="6" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="B6" s="102" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="101"/>
-      <c r="D6" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="E6" s="26" t="s">
-        <v>94</v>
-      </c>
-      <c r="F6" s="27" t="s">
+      <c r="A5" s="69"/>
+      <c r="B5" s="74"/>
+      <c r="C5" s="74"/>
+      <c r="D5" s="67"/>
+      <c r="E5" s="68"/>
+      <c r="F5" s="69"/>
+      <c r="G5" s="69"/>
+      <c r="H5" s="68"/>
+      <c r="I5" s="68"/>
+      <c r="J5" s="69"/>
+      <c r="K5" s="68"/>
+      <c r="L5" s="68"/>
+      <c r="M5" s="69"/>
+      <c r="N5" s="69"/>
+      <c r="O5" s="69"/>
+      <c r="P5" s="69"/>
+      <c r="Q5" s="69"/>
+      <c r="R5" s="69"/>
+      <c r="S5" s="69"/>
+      <c r="T5" s="69"/>
+      <c r="U5" s="68"/>
+      <c r="V5" s="68"/>
+      <c r="W5" s="68"/>
+      <c r="X5" s="68"/>
+      <c r="Y5" s="68"/>
+      <c r="Z5" s="69"/>
+    </row>
+    <row r="6" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="40" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="41" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="41" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="F7" s="44" t="s">
         <v>95</v>
       </c>
-      <c r="G6" s="103" t="s">
-        <v>96</v>
-      </c>
-      <c r="H6" s="100"/>
-      <c r="I6" s="101"/>
-      <c r="J6" s="103" t="s">
-        <v>37</v>
-      </c>
-      <c r="K6" s="100"/>
-      <c r="L6" s="101"/>
-      <c r="M6" s="28" t="s">
+      <c r="H7" s="45" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" s="42" t="s">
+        <v>49</v>
+      </c>
+      <c r="K7" s="42" t="s">
+        <v>51</v>
+      </c>
+      <c r="L7" s="46" t="s">
+        <v>52</v>
+      </c>
+      <c r="M7" s="48" t="s">
         <v>97</v>
       </c>
-      <c r="N6" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="O6" s="30" t="s">
-        <v>99</v>
-      </c>
-      <c r="P6" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q6" s="32" t="s">
-        <v>101</v>
-      </c>
-      <c r="R6" s="27" t="s">
+      <c r="N7" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="O7" s="41" t="s">
+        <v>34</v>
+      </c>
+      <c r="R7" s="48" t="s">
         <v>42</v>
       </c>
-      <c r="S6" s="33"/>
-      <c r="T6" s="104" t="s">
-        <v>102</v>
-      </c>
-      <c r="U6" s="100"/>
-      <c r="V6" s="101"/>
-      <c r="W6" s="104" t="s">
-        <v>103</v>
-      </c>
-      <c r="X6" s="100"/>
-      <c r="Y6" s="101"/>
-      <c r="Z6" s="31" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A7" s="25"/>
-      <c r="B7" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="25"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="H7" s="37" t="s">
-        <v>104</v>
-      </c>
-      <c r="I7" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="J7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="K7" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="L7" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="M7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="N7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="O7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="P7" s="31"/>
-      <c r="Q7" s="38"/>
-      <c r="R7" s="36"/>
-      <c r="S7" s="39"/>
-      <c r="T7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="U7" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="V7" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="W7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="X7" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="Y7" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="Z7" s="31"/>
-    </row>
-    <row r="10" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="40" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" s="41" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="41" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" s="41" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" s="43" t="s">
-        <v>108</v>
-      </c>
-      <c r="F11" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="H11" s="45" t="s">
-        <v>48</v>
-      </c>
-      <c r="I11" s="42" t="s">
-        <v>49</v>
-      </c>
-      <c r="K11" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="L11" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="M11" s="48" t="s">
-        <v>97</v>
-      </c>
-      <c r="N11" s="47" t="s">
-        <v>110</v>
-      </c>
-      <c r="O11" s="40" t="s">
-        <v>109</v>
-      </c>
-      <c r="P11" s="41" t="s">
-        <v>34</v>
-      </c>
-      <c r="R11" s="48" t="s">
-        <v>42</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="W6:Y6"/>
-    <mergeCell ref="A3:Z3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="F4:R4"/>
-    <mergeCell ref="T4:Z4"/>
-    <mergeCell ref="A5:C5"/>
+  <mergeCells count="5">
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="J3:L3"/>
+    <mergeCell ref="S3:U3"/>
+    <mergeCell ref="V3:X3"/>
   </mergeCells>
-  <conditionalFormatting sqref="B11">
+  <conditionalFormatting sqref="B7">
     <cfRule type="duplicateValues" dxfId="7" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C11">
+  <conditionalFormatting sqref="C7">
     <cfRule type="duplicateValues" dxfId="6" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3817,77 +3707,77 @@
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="99" t="str">
+      <c r="A3" s="104" t="str">
         <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="100"/>
-      <c r="C3" s="100"/>
-      <c r="D3" s="100"/>
-      <c r="E3" s="100"/>
-      <c r="F3" s="100"/>
-      <c r="G3" s="100"/>
-      <c r="H3" s="100"/>
-      <c r="I3" s="100"/>
-      <c r="J3" s="100"/>
-      <c r="K3" s="100"/>
-      <c r="L3" s="100"/>
-      <c r="M3" s="100"/>
-      <c r="N3" s="100"/>
-      <c r="O3" s="100"/>
-      <c r="P3" s="100"/>
-      <c r="Q3" s="100"/>
-      <c r="R3" s="100"/>
-      <c r="S3" s="100"/>
-      <c r="T3" s="100"/>
-      <c r="U3" s="100"/>
-      <c r="V3" s="100"/>
-      <c r="W3" s="100"/>
-      <c r="X3" s="100"/>
-      <c r="Y3" s="100"/>
-      <c r="Z3" s="101"/>
+      <c r="B3" s="102"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="102"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="102"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="102"/>
+      <c r="K3" s="102"/>
+      <c r="L3" s="102"/>
+      <c r="M3" s="102"/>
+      <c r="N3" s="102"/>
+      <c r="O3" s="102"/>
+      <c r="P3" s="102"/>
+      <c r="Q3" s="102"/>
+      <c r="R3" s="102"/>
+      <c r="S3" s="102"/>
+      <c r="T3" s="102"/>
+      <c r="U3" s="102"/>
+      <c r="V3" s="102"/>
+      <c r="W3" s="102"/>
+      <c r="X3" s="102"/>
+      <c r="Y3" s="102"/>
+      <c r="Z3" s="100"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="99">
+      <c r="A4" s="104">
         <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="100"/>
-      <c r="C4" s="100"/>
-      <c r="D4" s="101"/>
+      <c r="B4" s="102"/>
+      <c r="C4" s="102"/>
+      <c r="D4" s="100"/>
       <c r="E4" s="18"/>
-      <c r="F4" s="99" t="s">
+      <c r="F4" s="104" t="s">
         <v>89</v>
       </c>
-      <c r="G4" s="100"/>
-      <c r="H4" s="100"/>
-      <c r="I4" s="100"/>
-      <c r="J4" s="100"/>
-      <c r="K4" s="100"/>
-      <c r="L4" s="100"/>
-      <c r="M4" s="100"/>
-      <c r="N4" s="100"/>
-      <c r="O4" s="100"/>
-      <c r="P4" s="100"/>
-      <c r="Q4" s="100"/>
-      <c r="R4" s="101"/>
+      <c r="G4" s="102"/>
+      <c r="H4" s="102"/>
+      <c r="I4" s="102"/>
+      <c r="J4" s="102"/>
+      <c r="K4" s="102"/>
+      <c r="L4" s="102"/>
+      <c r="M4" s="102"/>
+      <c r="N4" s="102"/>
+      <c r="O4" s="102"/>
+      <c r="P4" s="102"/>
+      <c r="Q4" s="102"/>
+      <c r="R4" s="100"/>
       <c r="S4" s="19"/>
-      <c r="T4" s="99" t="s">
+      <c r="T4" s="104" t="s">
         <v>90</v>
       </c>
-      <c r="U4" s="100"/>
-      <c r="V4" s="100"/>
-      <c r="W4" s="100"/>
-      <c r="X4" s="100"/>
-      <c r="Y4" s="100"/>
-      <c r="Z4" s="101"/>
+      <c r="U4" s="102"/>
+      <c r="V4" s="102"/>
+      <c r="W4" s="102"/>
+      <c r="X4" s="102"/>
+      <c r="Y4" s="102"/>
+      <c r="Z4" s="100"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="99" t="s">
+      <c r="A5" s="104" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="100"/>
-      <c r="C5" s="101"/>
+      <c r="B5" s="102"/>
+      <c r="C5" s="100"/>
       <c r="D5" s="20">
         <f>[1]Summary!R7</f>
         <v>0</v>
@@ -3946,10 +3836,10 @@
       <c r="A6" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="102" t="s">
+      <c r="B6" s="99" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="101"/>
+      <c r="C6" s="100"/>
       <c r="D6" s="25" t="s">
         <v>93</v>
       </c>
@@ -3959,16 +3849,16 @@
       <c r="F6" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="G6" s="103" t="s">
+      <c r="G6" s="101" t="s">
         <v>96</v>
       </c>
-      <c r="H6" s="100"/>
-      <c r="I6" s="101"/>
-      <c r="J6" s="103" t="s">
+      <c r="H6" s="102"/>
+      <c r="I6" s="100"/>
+      <c r="J6" s="101" t="s">
         <v>37</v>
       </c>
-      <c r="K6" s="100"/>
-      <c r="L6" s="101"/>
+      <c r="K6" s="102"/>
+      <c r="L6" s="100"/>
       <c r="M6" s="28" t="s">
         <v>97</v>
       </c>
@@ -3988,16 +3878,16 @@
         <v>42</v>
       </c>
       <c r="S6" s="33"/>
-      <c r="T6" s="104" t="s">
+      <c r="T6" s="103" t="s">
         <v>102</v>
       </c>
-      <c r="U6" s="100"/>
-      <c r="V6" s="101"/>
-      <c r="W6" s="104" t="s">
+      <c r="U6" s="102"/>
+      <c r="V6" s="100"/>
+      <c r="W6" s="103" t="s">
         <v>103</v>
       </c>
-      <c r="X6" s="100"/>
-      <c r="Y6" s="101"/>
+      <c r="X6" s="102"/>
+      <c r="Y6" s="100"/>
       <c r="Z6" s="31" t="s">
         <v>100</v>
       </c>
@@ -4172,7 +4062,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:65" x14ac:dyDescent="0.35">
-      <c r="A1" s="104"/>
+      <c r="A1" s="103"/>
       <c r="B1" s="105"/>
       <c r="C1" s="105"/>
       <c r="D1" s="105"/>
@@ -4209,11 +4099,11 @@
       <c r="AI1" s="105"/>
       <c r="AJ1" s="105"/>
       <c r="AK1" s="105"/>
-      <c r="AL1" s="100"/>
-      <c r="AM1" s="100"/>
-      <c r="AN1" s="100"/>
-      <c r="AO1" s="100"/>
-      <c r="AP1" s="100"/>
+      <c r="AL1" s="102"/>
+      <c r="AM1" s="102"/>
+      <c r="AN1" s="102"/>
+      <c r="AO1" s="102"/>
+      <c r="AP1" s="102"/>
       <c r="AQ1" s="105"/>
       <c r="AR1" s="105"/>
       <c r="AS1" s="105"/>
@@ -4621,7 +4511,7 @@
       </c>
     </row>
     <row r="3" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A3" s="104" t="str">
+      <c r="A3" s="103" t="str">
         <f>+[2]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
@@ -4661,11 +4551,11 @@
       <c r="AI3" s="105"/>
       <c r="AJ3" s="105"/>
       <c r="AK3" s="105"/>
-      <c r="AL3" s="100"/>
-      <c r="AM3" s="100"/>
-      <c r="AN3" s="100"/>
-      <c r="AO3" s="100"/>
-      <c r="AP3" s="100"/>
+      <c r="AL3" s="102"/>
+      <c r="AM3" s="102"/>
+      <c r="AN3" s="102"/>
+      <c r="AO3" s="102"/>
+      <c r="AP3" s="102"/>
       <c r="AQ3" s="105"/>
       <c r="AR3" s="105"/>
       <c r="AS3" s="105"/>
@@ -4679,7 +4569,7 @@
       <c r="BA3" s="106"/>
     </row>
     <row r="4" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A4" s="104">
+      <c r="A4" s="103">
         <f>+[2]Summary!A7</f>
         <v>0</v>
       </c>
@@ -4719,11 +4609,11 @@
       <c r="AI4" s="105"/>
       <c r="AJ4" s="105"/>
       <c r="AK4" s="105"/>
-      <c r="AL4" s="100"/>
-      <c r="AM4" s="100"/>
-      <c r="AN4" s="100"/>
-      <c r="AO4" s="100"/>
-      <c r="AP4" s="100"/>
+      <c r="AL4" s="102"/>
+      <c r="AM4" s="102"/>
+      <c r="AN4" s="102"/>
+      <c r="AO4" s="102"/>
+      <c r="AP4" s="102"/>
       <c r="AQ4" s="105"/>
       <c r="AR4" s="105"/>
       <c r="AS4" s="105"/>
@@ -4737,7 +4627,7 @@
       <c r="BA4" s="106"/>
     </row>
     <row r="5" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="104" t="s">
+      <c r="A5" s="103" t="s">
         <v>113</v>
       </c>
       <c r="B5" s="105"/>
@@ -4758,7 +4648,7 @@
       <c r="Q5" s="105"/>
       <c r="R5" s="105"/>
       <c r="S5" s="106"/>
-      <c r="T5" s="104" t="s">
+      <c r="T5" s="103" t="s">
         <v>114</v>
       </c>
       <c r="U5" s="105"/>
@@ -4778,14 +4668,14 @@
       <c r="AI5" s="105"/>
       <c r="AJ5" s="105"/>
       <c r="AK5" s="106"/>
-      <c r="AL5" s="104" t="s">
+      <c r="AL5" s="103" t="s">
         <v>115</v>
       </c>
-      <c r="AM5" s="100"/>
-      <c r="AN5" s="100"/>
-      <c r="AO5" s="100"/>
-      <c r="AP5" s="101"/>
-      <c r="AQ5" s="104" t="s">
+      <c r="AM5" s="102"/>
+      <c r="AN5" s="102"/>
+      <c r="AO5" s="102"/>
+      <c r="AP5" s="100"/>
+      <c r="AQ5" s="103" t="s">
         <v>2</v>
       </c>
       <c r="AR5" s="105"/>
@@ -4794,7 +4684,7 @@
       <c r="AU5" s="27" t="s">
         <v>116</v>
       </c>
-      <c r="AV5" s="104" t="s">
+      <c r="AV5" s="103" t="s">
         <v>117</v>
       </c>
       <c r="AW5" s="105"/>
@@ -4845,7 +4735,7 @@
       <c r="U6" s="31" t="s">
         <v>123</v>
       </c>
-      <c r="V6" s="104" t="s">
+      <c r="V6" s="103" t="s">
         <v>124</v>
       </c>
       <c r="W6" s="105"/>
@@ -4878,7 +4768,7 @@
         <v>133</v>
       </c>
       <c r="AH6" s="106"/>
-      <c r="AI6" s="104" t="s">
+      <c r="AI6" s="103" t="s">
         <v>134</v>
       </c>
       <c r="AJ6" s="106"/>
@@ -5101,18 +4991,18 @@
       <c r="B3" s="115" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="100"/>
-      <c r="D3" s="101"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="100"/>
       <c r="E3" s="115" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="100"/>
-      <c r="G3" s="101"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="100"/>
       <c r="H3" s="115" t="s">
         <v>37</v>
       </c>
-      <c r="I3" s="100"/>
-      <c r="J3" s="101"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="100"/>
       <c r="K3" s="114" t="s">
         <v>74</v>
       </c>

</xml_diff>

<commit_message>
Auto pipeline update 2026-04-22 11:36:13
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{175B78F5-822C-49FB-BA36-5C186F7038E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{838680F7-B0E9-487F-B0FE-307E9A22D9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="899" firstSheet="2" activeTab="4" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
   </bookViews>
@@ -28,7 +28,6 @@
   </sheets>
   <externalReferences>
     <externalReference r:id="rId13"/>
-    <externalReference r:id="rId14"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="202">
   <si>
     <t>Project Code</t>
   </si>
@@ -318,15 +317,6 @@
   </si>
   <si>
     <t>Stringing-132KV; Stringing-220kV</t>
-  </si>
-  <si>
-    <t>Stringing Progress (Conductor &amp; Earthwire)</t>
-  </si>
-  <si>
-    <t>OPGW Progress</t>
-  </si>
-  <si>
-    <t>Stringing Section</t>
   </si>
   <si>
     <t>Sl. No.</t>
@@ -778,7 +768,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -825,12 +815,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFAEABAB"/>
         <bgColor rgb="FFAEABAB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -1347,7 +1331,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="124">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1400,25 +1384,10 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="9" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="10" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1442,10 +1411,10 @@
     <xf numFmtId="0" fontId="10" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1604,10 +1573,10 @@
     <xf numFmtId="168" fontId="2" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="11" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="2" fillId="10" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="11" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="2" fillId="10" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="168" fontId="2" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1631,7 +1600,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1642,9 +1611,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1699,6 +1665,33 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -1817,59 +1810,6 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Detail Survey-220kV"/>
-      <sheetName val="Check Survey-220kV"/>
-      <sheetName val="Detail Survey-132kV"/>
-      <sheetName val="Check Survey-132kV"/>
-      <sheetName val="Summary"/>
-      <sheetName val="Statutory"/>
-      <sheetName val="Progress-132kV"/>
-      <sheetName val="Progress-220kV"/>
-      <sheetName val="Stringing-220kV"/>
-      <sheetName val="Stringing-132KV"/>
-      <sheetName val="VC-220kV"/>
-      <sheetName val="VC-132kV"/>
-      <sheetName val="Supply"/>
-      <sheetName val="Mail Body"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4">
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>Name of the Line: 220KV DC AL59 line from Neemuch - Chanderiya + 132KV DC ACSS Line from Chanderiya to Hindustan Zinc</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>Office:  Neemuch</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
@@ -2397,7 +2337,7 @@
         <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -2530,46 +2470,46 @@
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A3" s="119" t="s">
+      <c r="A3" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="119" t="s">
+      <c r="B3" s="111" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="119"/>
-      <c r="D3" s="119" t="s">
+      <c r="C3" s="111"/>
+      <c r="D3" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="119" t="s">
+      <c r="E3" s="111" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="119" t="s">
+      <c r="F3" s="111" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="120" t="s">
+      <c r="G3" s="112" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="120"/>
-      <c r="I3" s="120"/>
-      <c r="J3" s="116" t="s">
+      <c r="H3" s="112"/>
+      <c r="I3" s="112"/>
+      <c r="J3" s="108" t="s">
         <v>37</v>
       </c>
-      <c r="K3" s="117"/>
-      <c r="L3" s="117"/>
-      <c r="M3" s="117"/>
-      <c r="N3" s="118"/>
+      <c r="K3" s="109"/>
+      <c r="L3" s="109"/>
+      <c r="M3" s="109"/>
+      <c r="N3" s="110"/>
     </row>
     <row r="4" spans="1:23" ht="26" x14ac:dyDescent="0.35">
-      <c r="A4" s="119"/>
+      <c r="A4" s="111"/>
       <c r="B4" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="119"/>
-      <c r="E4" s="119"/>
-      <c r="F4" s="119"/>
+      <c r="D4" s="111"/>
+      <c r="E4" s="111"/>
+      <c r="F4" s="111"/>
       <c r="G4" s="1" t="s">
         <v>35</v>
       </c>
@@ -2611,7 +2551,7 @@
         <v>46</v>
       </c>
       <c r="D7" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>34</v>
@@ -2703,14 +2643,14 @@
       <c r="C3" s="7"/>
       <c r="D3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="121"/>
-      <c r="H3" s="122"/>
-      <c r="I3" s="122"/>
-      <c r="J3" s="123"/>
+      <c r="G3" s="113"/>
+      <c r="H3" s="114"/>
+      <c r="I3" s="114"/>
+      <c r="J3" s="115"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="121"/>
-      <c r="O3" s="122"/>
-      <c r="P3" s="123"/>
+      <c r="N3" s="113"/>
+      <c r="O3" s="114"/>
+      <c r="P3" s="115"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -2792,14 +2732,14 @@
       <c r="C3" s="7"/>
       <c r="D3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="121"/>
-      <c r="H3" s="122"/>
-      <c r="I3" s="122"/>
-      <c r="J3" s="123"/>
+      <c r="G3" s="113"/>
+      <c r="H3" s="114"/>
+      <c r="I3" s="114"/>
+      <c r="J3" s="115"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="121"/>
-      <c r="O3" s="122"/>
-      <c r="P3" s="123"/>
+      <c r="N3" s="113"/>
+      <c r="O3" s="114"/>
+      <c r="P3" s="115"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -2852,58 +2792,58 @@
       </c>
     </row>
     <row r="2" spans="1:16" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="87" t="s">
+      <c r="A2" s="80" t="s">
+        <v>176</v>
+      </c>
+      <c r="B2" s="80" t="s">
+        <v>177</v>
+      </c>
+      <c r="C2" s="81" t="s">
+        <v>178</v>
+      </c>
+      <c r="D2" s="81" t="s">
         <v>179</v>
       </c>
-      <c r="B2" s="87" t="s">
+      <c r="E2" s="82" t="s">
         <v>180</v>
       </c>
-      <c r="C2" s="88" t="s">
+      <c r="F2" s="83" t="s">
         <v>181</v>
       </c>
-      <c r="D2" s="88" t="s">
+      <c r="G2" s="84" t="s">
         <v>182</v>
       </c>
-      <c r="E2" s="89" t="s">
+      <c r="H2" s="84" t="s">
         <v>183</v>
       </c>
-      <c r="F2" s="90" t="s">
+      <c r="I2" s="85" t="s">
         <v>184</v>
       </c>
-      <c r="G2" s="91" t="s">
+      <c r="J2" s="80" t="s">
         <v>185</v>
       </c>
-      <c r="H2" s="91" t="s">
+      <c r="K2" s="80" t="s">
+        <v>42</v>
+      </c>
+      <c r="L2" s="80" t="s">
         <v>186</v>
       </c>
-      <c r="I2" s="92" t="s">
+      <c r="M2" s="86" t="s">
         <v>187</v>
       </c>
-      <c r="J2" s="87" t="s">
-        <v>188</v>
-      </c>
-      <c r="K2" s="87" t="s">
-        <v>42</v>
-      </c>
-      <c r="L2" s="87" t="s">
-        <v>189</v>
-      </c>
-      <c r="M2" s="93" t="s">
-        <v>190</v>
-      </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="C3" s="84"/>
-      <c r="D3" s="85"/>
-      <c r="F3" s="85"/>
-      <c r="G3" s="86"/>
-      <c r="H3" s="86"/>
-      <c r="I3" s="86"/>
-      <c r="J3" s="86"/>
-      <c r="M3" s="85"/>
-      <c r="N3" s="86"/>
-      <c r="O3" s="86"/>
-      <c r="P3" s="86"/>
+      <c r="C3" s="77"/>
+      <c r="D3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="79"/>
+      <c r="H3" s="79"/>
+      <c r="I3" s="79"/>
+      <c r="J3" s="79"/>
+      <c r="M3" s="78"/>
+      <c r="N3" s="79"/>
+      <c r="O3" s="79"/>
+      <c r="P3" s="79"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -2948,246 +2888,246 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:26" s="98" customFormat="1" ht="53.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="76" t="s">
-        <v>179</v>
-      </c>
-      <c r="B3" s="77" t="s">
-        <v>180</v>
-      </c>
-      <c r="C3" s="94" t="s">
+    <row r="3" spans="1:26" s="91" customFormat="1" ht="53.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="69" t="s">
+        <v>176</v>
+      </c>
+      <c r="B3" s="70" t="s">
+        <v>177</v>
+      </c>
+      <c r="C3" s="87" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="95" t="s">
+      <c r="D3" s="88" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="94" t="s">
+      <c r="E3" s="87" t="s">
+        <v>188</v>
+      </c>
+      <c r="F3" s="87" t="s">
+        <v>189</v>
+      </c>
+      <c r="G3" s="87" t="s">
+        <v>190</v>
+      </c>
+      <c r="H3" s="87" t="s">
         <v>191</v>
       </c>
-      <c r="F3" s="94" t="s">
+      <c r="I3" s="87" t="s">
         <v>192</v>
       </c>
-      <c r="G3" s="94" t="s">
+      <c r="J3" s="87" t="s">
         <v>193</v>
       </c>
-      <c r="H3" s="94" t="s">
+      <c r="K3" s="87" t="s">
         <v>194</v>
       </c>
-      <c r="I3" s="94" t="s">
+      <c r="L3" s="87" t="s">
         <v>195</v>
       </c>
-      <c r="J3" s="94" t="s">
+      <c r="M3" s="87" t="s">
         <v>196</v>
       </c>
-      <c r="K3" s="94" t="s">
+      <c r="N3" s="87" t="s">
         <v>197</v>
       </c>
-      <c r="L3" s="94" t="s">
+      <c r="O3" s="87" t="s">
         <v>198</v>
       </c>
-      <c r="M3" s="94" t="s">
+      <c r="P3" s="87" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q3" s="87" t="s">
         <v>199</v>
       </c>
-      <c r="N3" s="94" t="s">
+      <c r="R3" s="87" t="s">
+        <v>184</v>
+      </c>
+      <c r="S3" s="87" t="s">
         <v>200</v>
       </c>
-      <c r="O3" s="94" t="s">
+      <c r="T3" s="89" t="s">
         <v>201</v>
       </c>
-      <c r="P3" s="94" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q3" s="94" t="s">
-        <v>202</v>
-      </c>
-      <c r="R3" s="94" t="s">
-        <v>187</v>
-      </c>
-      <c r="S3" s="94" t="s">
-        <v>203</v>
-      </c>
-      <c r="T3" s="96" t="s">
-        <v>204</v>
-      </c>
-      <c r="U3" s="97" t="s">
+      <c r="U3" s="90" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="69"/>
-      <c r="B4" s="74"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="66"/>
-      <c r="F4" s="69"/>
-      <c r="G4" s="74"/>
-      <c r="H4" s="74"/>
-      <c r="I4" s="74"/>
-      <c r="J4" s="74"/>
-      <c r="K4" s="74"/>
-      <c r="L4" s="74"/>
-      <c r="M4" s="74"/>
-      <c r="N4" s="74"/>
-      <c r="O4" s="74"/>
-      <c r="P4" s="74"/>
-      <c r="Q4" s="74"/>
-      <c r="R4" s="74"/>
-      <c r="S4" s="66"/>
-      <c r="T4" s="69"/>
-      <c r="U4" s="74"/>
-      <c r="V4" s="74"/>
-      <c r="W4" s="74"/>
-      <c r="X4" s="74"/>
-      <c r="Y4" s="74"/>
-      <c r="Z4" s="74"/>
+      <c r="A4" s="62"/>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
+      <c r="I4" s="67"/>
+      <c r="J4" s="67"/>
+      <c r="K4" s="67"/>
+      <c r="L4" s="67"/>
+      <c r="M4" s="67"/>
+      <c r="N4" s="67"/>
+      <c r="O4" s="67"/>
+      <c r="P4" s="67"/>
+      <c r="Q4" s="67"/>
+      <c r="R4" s="67"/>
+      <c r="S4" s="59"/>
+      <c r="T4" s="62"/>
+      <c r="U4" s="67"/>
+      <c r="V4" s="67"/>
+      <c r="W4" s="67"/>
+      <c r="X4" s="67"/>
+      <c r="Y4" s="67"/>
+      <c r="Z4" s="67"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="69"/>
-      <c r="B5" s="74"/>
-      <c r="C5" s="74"/>
-      <c r="D5" s="67"/>
-      <c r="E5" s="68"/>
-      <c r="F5" s="69"/>
-      <c r="G5" s="69"/>
-      <c r="H5" s="68"/>
-      <c r="I5" s="68"/>
-      <c r="J5" s="69"/>
-      <c r="K5" s="68"/>
-      <c r="L5" s="68"/>
-      <c r="M5" s="69"/>
-      <c r="N5" s="69"/>
-      <c r="O5" s="69"/>
-      <c r="P5" s="69"/>
-      <c r="Q5" s="69"/>
-      <c r="R5" s="69"/>
-      <c r="S5" s="69"/>
-      <c r="T5" s="69"/>
-      <c r="U5" s="68"/>
-      <c r="V5" s="68"/>
-      <c r="W5" s="68"/>
-      <c r="X5" s="68"/>
-      <c r="Y5" s="68"/>
-      <c r="Z5" s="69"/>
+      <c r="A5" s="62"/>
+      <c r="B5" s="67"/>
+      <c r="C5" s="67"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="61"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
+      <c r="H5" s="61"/>
+      <c r="I5" s="61"/>
+      <c r="J5" s="62"/>
+      <c r="K5" s="61"/>
+      <c r="L5" s="61"/>
+      <c r="M5" s="62"/>
+      <c r="N5" s="62"/>
+      <c r="O5" s="62"/>
+      <c r="P5" s="62"/>
+      <c r="Q5" s="62"/>
+      <c r="R5" s="62"/>
+      <c r="S5" s="62"/>
+      <c r="T5" s="62"/>
+      <c r="U5" s="61"/>
+      <c r="V5" s="61"/>
+      <c r="W5" s="61"/>
+      <c r="X5" s="61"/>
+      <c r="Y5" s="61"/>
+      <c r="Z5" s="62"/>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A6" s="70"/>
-      <c r="B6" s="63"/>
-      <c r="C6" s="74"/>
-      <c r="D6" s="70"/>
-      <c r="E6" s="70"/>
-      <c r="F6" s="70"/>
-      <c r="G6" s="75"/>
-      <c r="H6" s="74"/>
-      <c r="I6" s="74"/>
-      <c r="J6" s="75"/>
-      <c r="K6" s="74"/>
-      <c r="L6" s="74"/>
-      <c r="M6" s="71"/>
-      <c r="N6" s="70"/>
-      <c r="O6" s="72"/>
-      <c r="P6" s="70"/>
-      <c r="Q6" s="71"/>
-      <c r="R6" s="70"/>
-      <c r="S6" s="70"/>
-      <c r="T6" s="63"/>
-      <c r="U6" s="74"/>
-      <c r="V6" s="74"/>
-      <c r="W6" s="63"/>
-      <c r="X6" s="74"/>
-      <c r="Y6" s="74"/>
-      <c r="Z6" s="70"/>
+      <c r="A6" s="63"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="67"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="67"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="68"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="67"/>
+      <c r="M6" s="64"/>
+      <c r="N6" s="63"/>
+      <c r="O6" s="65"/>
+      <c r="P6" s="63"/>
+      <c r="Q6" s="64"/>
+      <c r="R6" s="63"/>
+      <c r="S6" s="63"/>
+      <c r="T6" s="56"/>
+      <c r="U6" s="67"/>
+      <c r="V6" s="67"/>
+      <c r="W6" s="56"/>
+      <c r="X6" s="67"/>
+      <c r="Y6" s="67"/>
+      <c r="Z6" s="63"/>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A7" s="70"/>
-      <c r="B7" s="73"/>
-      <c r="C7" s="73"/>
-      <c r="D7" s="70"/>
-      <c r="E7" s="70"/>
-      <c r="F7" s="70"/>
-      <c r="G7" s="72"/>
-      <c r="H7" s="73"/>
-      <c r="I7" s="72"/>
-      <c r="J7" s="72"/>
-      <c r="K7" s="72"/>
-      <c r="L7" s="72"/>
-      <c r="M7" s="72"/>
-      <c r="N7" s="72"/>
-      <c r="O7" s="72"/>
-      <c r="P7" s="70"/>
-      <c r="Q7" s="71"/>
-      <c r="R7" s="70"/>
-      <c r="S7" s="70"/>
-      <c r="T7" s="72"/>
-      <c r="U7" s="72"/>
-      <c r="V7" s="72"/>
-      <c r="W7" s="72"/>
-      <c r="X7" s="72"/>
-      <c r="Y7" s="72"/>
-      <c r="Z7" s="70"/>
+      <c r="A7" s="63"/>
+      <c r="B7" s="66"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="63"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="63"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="66"/>
+      <c r="I7" s="65"/>
+      <c r="J7" s="65"/>
+      <c r="K7" s="65"/>
+      <c r="L7" s="65"/>
+      <c r="M7" s="65"/>
+      <c r="N7" s="65"/>
+      <c r="O7" s="65"/>
+      <c r="P7" s="63"/>
+      <c r="Q7" s="64"/>
+      <c r="R7" s="63"/>
+      <c r="S7" s="63"/>
+      <c r="T7" s="65"/>
+      <c r="U7" s="65"/>
+      <c r="V7" s="65"/>
+      <c r="W7" s="65"/>
+      <c r="X7" s="65"/>
+      <c r="Y7" s="65"/>
+      <c r="Z7" s="63"/>
     </row>
     <row r="9" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="10" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>68</v>
       </c>
-      <c r="N10" s="40"/>
+      <c r="N10" s="33"/>
     </row>
     <row r="11" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="76" t="s">
+      <c r="A11" s="69" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="77" t="s">
+      <c r="B11" s="70" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11" s="70" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="70" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="70" t="s">
+        <v>47</v>
+      </c>
+      <c r="G11" s="71" t="s">
+        <v>104</v>
+      </c>
+      <c r="H11" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="J11" s="72" t="s">
+        <v>48</v>
+      </c>
+      <c r="K11" s="71" t="s">
+        <v>49</v>
+      </c>
+      <c r="L11" s="71" t="s">
+        <v>51</v>
+      </c>
+      <c r="M11" s="73" t="s">
+        <v>52</v>
+      </c>
+      <c r="O11" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="C11" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="D11" s="77" t="s">
-        <v>46</v>
-      </c>
-      <c r="E11" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="G11" s="78" t="s">
+      <c r="P11" s="74" t="s">
         <v>107</v>
       </c>
-      <c r="H11" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="J11" s="79" t="s">
-        <v>48</v>
-      </c>
-      <c r="K11" s="78" t="s">
-        <v>49</v>
-      </c>
-      <c r="L11" s="78" t="s">
-        <v>51</v>
-      </c>
-      <c r="M11" s="80" t="s">
-        <v>52</v>
-      </c>
-      <c r="O11" s="76" t="s">
-        <v>109</v>
-      </c>
-      <c r="P11" s="81" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q11" s="82" t="s">
-        <v>97</v>
-      </c>
-      <c r="R11" s="83" t="s">
+      <c r="Q11" s="75" t="s">
+        <v>94</v>
+      </c>
+      <c r="R11" s="76" t="s">
         <v>53</v>
       </c>
-      <c r="S11" s="77"/>
-      <c r="T11" s="77" t="s">
+      <c r="S11" s="70"/>
+      <c r="T11" s="70" t="s">
         <v>34</v>
       </c>
-      <c r="U11" s="82" t="s">
+      <c r="U11" s="75" t="s">
         <v>42</v>
       </c>
-      <c r="V11" s="77"/>
-      <c r="W11" s="77"/>
-      <c r="X11" s="82"/>
+      <c r="V11" s="70"/>
+      <c r="W11" s="70"/>
+      <c r="X11" s="75"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3205,266 +3145,266 @@
       </c>
     </row>
     <row r="3" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="76" t="s">
+      <c r="A3" s="69" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="77" t="s">
+      <c r="B3" s="70" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="70" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="70" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="70" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="71" t="s">
+        <v>104</v>
+      </c>
+      <c r="G3" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="H3" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="I3" s="72" t="s">
+        <v>48</v>
+      </c>
+      <c r="J3" s="71" t="s">
+        <v>49</v>
+      </c>
+      <c r="K3" s="70" t="s">
+        <v>50</v>
+      </c>
+      <c r="L3" s="71" t="s">
+        <v>51</v>
+      </c>
+      <c r="M3" s="73" t="s">
+        <v>52</v>
+      </c>
+      <c r="N3" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="D3" s="77" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="F3" s="78" t="s">
+      <c r="O3" s="74" t="s">
         <v>107</v>
       </c>
-      <c r="G3" s="43" t="s">
+      <c r="P3" s="75" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q3" s="76" t="s">
+        <v>53</v>
+      </c>
+      <c r="R3" s="70" t="s">
+        <v>54</v>
+      </c>
+      <c r="S3" s="70" t="s">
+        <v>34</v>
+      </c>
+      <c r="T3" s="70" t="s">
+        <v>80</v>
+      </c>
+      <c r="U3" s="70" t="s">
         <v>108</v>
       </c>
-      <c r="H3" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="I3" s="79" t="s">
-        <v>48</v>
-      </c>
-      <c r="J3" s="78" t="s">
-        <v>49</v>
-      </c>
-      <c r="K3" s="77" t="s">
-        <v>50</v>
-      </c>
-      <c r="L3" s="78" t="s">
-        <v>51</v>
-      </c>
-      <c r="M3" s="80" t="s">
-        <v>52</v>
-      </c>
-      <c r="N3" s="76" t="s">
+      <c r="V3" s="70" t="s">
         <v>109</v>
       </c>
-      <c r="O3" s="81" t="s">
-        <v>110</v>
-      </c>
-      <c r="P3" s="82" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q3" s="83" t="s">
-        <v>53</v>
-      </c>
-      <c r="R3" s="77" t="s">
-        <v>54</v>
-      </c>
-      <c r="S3" s="77" t="s">
-        <v>34</v>
-      </c>
-      <c r="T3" s="77" t="s">
-        <v>80</v>
-      </c>
-      <c r="U3" s="77" t="s">
-        <v>111</v>
-      </c>
-      <c r="V3" s="77" t="s">
-        <v>112</v>
-      </c>
-      <c r="W3" s="82" t="s">
+      <c r="W3" s="75" t="s">
         <v>42</v>
       </c>
-      <c r="X3" s="74"/>
-      <c r="Y3" s="74"/>
-      <c r="Z3" s="74"/>
+      <c r="X3" s="67"/>
+      <c r="Y3" s="67"/>
+      <c r="Z3" s="67"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="69"/>
-      <c r="B4" s="74"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="66"/>
-      <c r="F4" s="69"/>
-      <c r="G4" s="74"/>
-      <c r="H4" s="74"/>
-      <c r="I4" s="74"/>
-      <c r="J4" s="74"/>
-      <c r="K4" s="74"/>
-      <c r="L4" s="74"/>
-      <c r="M4" s="74"/>
-      <c r="N4" s="74"/>
-      <c r="O4" s="74"/>
-      <c r="P4" s="74"/>
-      <c r="Q4" s="74"/>
-      <c r="R4" s="74"/>
-      <c r="S4" s="66"/>
-      <c r="T4" s="69"/>
-      <c r="U4" s="74"/>
-      <c r="V4" s="74"/>
-      <c r="W4" s="74"/>
-      <c r="X4" s="74"/>
-      <c r="Y4" s="74"/>
-      <c r="Z4" s="74"/>
+      <c r="A4" s="62"/>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
+      <c r="I4" s="67"/>
+      <c r="J4" s="67"/>
+      <c r="K4" s="67"/>
+      <c r="L4" s="67"/>
+      <c r="M4" s="67"/>
+      <c r="N4" s="67"/>
+      <c r="O4" s="67"/>
+      <c r="P4" s="67"/>
+      <c r="Q4" s="67"/>
+      <c r="R4" s="67"/>
+      <c r="S4" s="59"/>
+      <c r="T4" s="62"/>
+      <c r="U4" s="67"/>
+      <c r="V4" s="67"/>
+      <c r="W4" s="67"/>
+      <c r="X4" s="67"/>
+      <c r="Y4" s="67"/>
+      <c r="Z4" s="67"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="69"/>
-      <c r="B5" s="74"/>
-      <c r="C5" s="74"/>
-      <c r="D5" s="67"/>
-      <c r="E5" s="68"/>
-      <c r="F5" s="69"/>
-      <c r="G5" s="69"/>
-      <c r="H5" s="68"/>
-      <c r="I5" s="68"/>
-      <c r="J5" s="69"/>
-      <c r="K5" s="68"/>
-      <c r="L5" s="68"/>
-      <c r="M5" s="69"/>
-      <c r="N5" s="69"/>
-      <c r="O5" s="69"/>
-      <c r="P5" s="69"/>
-      <c r="Q5" s="69"/>
-      <c r="R5" s="69"/>
-      <c r="S5" s="69"/>
-      <c r="T5" s="69"/>
-      <c r="U5" s="68"/>
-      <c r="V5" s="68"/>
-      <c r="W5" s="68"/>
-      <c r="X5" s="68"/>
-      <c r="Y5" s="68"/>
-      <c r="Z5" s="69"/>
+      <c r="A5" s="62"/>
+      <c r="B5" s="67"/>
+      <c r="C5" s="67"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="61"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
+      <c r="H5" s="61"/>
+      <c r="I5" s="61"/>
+      <c r="J5" s="62"/>
+      <c r="K5" s="61"/>
+      <c r="L5" s="61"/>
+      <c r="M5" s="62"/>
+      <c r="N5" s="62"/>
+      <c r="O5" s="62"/>
+      <c r="P5" s="62"/>
+      <c r="Q5" s="62"/>
+      <c r="R5" s="62"/>
+      <c r="S5" s="62"/>
+      <c r="T5" s="62"/>
+      <c r="U5" s="61"/>
+      <c r="V5" s="61"/>
+      <c r="W5" s="61"/>
+      <c r="X5" s="61"/>
+      <c r="Y5" s="61"/>
+      <c r="Z5" s="62"/>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A6" s="70"/>
-      <c r="B6" s="63"/>
-      <c r="C6" s="74"/>
-      <c r="D6" s="70"/>
-      <c r="E6" s="70"/>
-      <c r="F6" s="70"/>
-      <c r="G6" s="75"/>
-      <c r="H6" s="74"/>
-      <c r="I6" s="74"/>
-      <c r="J6" s="75"/>
-      <c r="K6" s="74"/>
-      <c r="L6" s="74"/>
-      <c r="M6" s="71"/>
-      <c r="N6" s="70"/>
-      <c r="O6" s="72"/>
-      <c r="P6" s="70"/>
-      <c r="Q6" s="71"/>
-      <c r="R6" s="70"/>
-      <c r="S6" s="70"/>
-      <c r="T6" s="63"/>
-      <c r="U6" s="74"/>
-      <c r="V6" s="74"/>
-      <c r="W6" s="63"/>
-      <c r="X6" s="74"/>
-      <c r="Y6" s="74"/>
-      <c r="Z6" s="70"/>
+      <c r="A6" s="63"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="67"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="67"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="68"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="67"/>
+      <c r="M6" s="64"/>
+      <c r="N6" s="63"/>
+      <c r="O6" s="65"/>
+      <c r="P6" s="63"/>
+      <c r="Q6" s="64"/>
+      <c r="R6" s="63"/>
+      <c r="S6" s="63"/>
+      <c r="T6" s="56"/>
+      <c r="U6" s="67"/>
+      <c r="V6" s="67"/>
+      <c r="W6" s="56"/>
+      <c r="X6" s="67"/>
+      <c r="Y6" s="67"/>
+      <c r="Z6" s="63"/>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A7" s="70"/>
-      <c r="B7" s="73"/>
-      <c r="C7" s="73"/>
-      <c r="D7" s="70"/>
-      <c r="E7" s="70"/>
-      <c r="F7" s="70"/>
-      <c r="G7" s="72"/>
-      <c r="H7" s="73"/>
-      <c r="I7" s="72"/>
-      <c r="J7" s="72"/>
-      <c r="K7" s="72"/>
-      <c r="L7" s="72"/>
-      <c r="M7" s="72"/>
-      <c r="N7" s="72"/>
-      <c r="O7" s="72"/>
-      <c r="P7" s="70"/>
-      <c r="Q7" s="71"/>
-      <c r="R7" s="70"/>
-      <c r="S7" s="70"/>
-      <c r="T7" s="72"/>
-      <c r="U7" s="72"/>
-      <c r="V7" s="72"/>
-      <c r="W7" s="72"/>
-      <c r="X7" s="72"/>
-      <c r="Y7" s="72"/>
-      <c r="Z7" s="70"/>
+      <c r="A7" s="63"/>
+      <c r="B7" s="66"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="63"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="63"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="66"/>
+      <c r="I7" s="65"/>
+      <c r="J7" s="65"/>
+      <c r="K7" s="65"/>
+      <c r="L7" s="65"/>
+      <c r="M7" s="65"/>
+      <c r="N7" s="65"/>
+      <c r="O7" s="65"/>
+      <c r="P7" s="63"/>
+      <c r="Q7" s="64"/>
+      <c r="R7" s="63"/>
+      <c r="S7" s="63"/>
+      <c r="T7" s="65"/>
+      <c r="U7" s="65"/>
+      <c r="V7" s="65"/>
+      <c r="W7" s="65"/>
+      <c r="X7" s="65"/>
+      <c r="Y7" s="65"/>
+      <c r="Z7" s="63"/>
     </row>
     <row r="9" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="10" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>68</v>
       </c>
-      <c r="N10" s="40"/>
+      <c r="N10" s="33"/>
     </row>
     <row r="11" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="76" t="s">
+      <c r="A11" s="69" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="77" t="s">
+      <c r="B11" s="70" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11" s="70" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="70" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="70" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="71" t="s">
+        <v>104</v>
+      </c>
+      <c r="G11" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="H11" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="I11" s="72" t="s">
+        <v>48</v>
+      </c>
+      <c r="J11" s="71" t="s">
+        <v>49</v>
+      </c>
+      <c r="K11" s="70" t="s">
+        <v>50</v>
+      </c>
+      <c r="L11" s="71" t="s">
+        <v>51</v>
+      </c>
+      <c r="M11" s="73" t="s">
+        <v>52</v>
+      </c>
+      <c r="N11" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="C11" s="77" t="s">
-        <v>45</v>
-      </c>
-      <c r="D11" s="77" t="s">
-        <v>46</v>
-      </c>
-      <c r="E11" s="77" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" s="78" t="s">
+      <c r="O11" s="74" t="s">
         <v>107</v>
       </c>
-      <c r="G11" s="43" t="s">
+      <c r="P11" s="75" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q11" s="76" t="s">
+        <v>53</v>
+      </c>
+      <c r="R11" s="70" t="s">
+        <v>54</v>
+      </c>
+      <c r="S11" s="70" t="s">
+        <v>34</v>
+      </c>
+      <c r="T11" s="70" t="s">
+        <v>80</v>
+      </c>
+      <c r="U11" s="70" t="s">
         <v>108</v>
       </c>
-      <c r="H11" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="I11" s="79" t="s">
-        <v>48</v>
-      </c>
-      <c r="J11" s="78" t="s">
-        <v>49</v>
-      </c>
-      <c r="K11" s="77" t="s">
-        <v>50</v>
-      </c>
-      <c r="L11" s="78" t="s">
-        <v>51</v>
-      </c>
-      <c r="M11" s="80" t="s">
-        <v>52</v>
-      </c>
-      <c r="N11" s="76" t="s">
+      <c r="V11" s="70" t="s">
         <v>109</v>
       </c>
-      <c r="O11" s="81" t="s">
-        <v>110</v>
-      </c>
-      <c r="P11" s="82" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q11" s="83" t="s">
-        <v>53</v>
-      </c>
-      <c r="R11" s="77" t="s">
-        <v>54</v>
-      </c>
-      <c r="S11" s="77" t="s">
-        <v>34</v>
-      </c>
-      <c r="T11" s="77" t="s">
-        <v>80</v>
-      </c>
-      <c r="U11" s="77" t="s">
-        <v>111</v>
-      </c>
-      <c r="V11" s="77" t="s">
-        <v>112</v>
-      </c>
-      <c r="W11" s="82" t="s">
+      <c r="W11" s="75" t="s">
         <v>42</v>
       </c>
     </row>
@@ -3484,150 +3424,150 @@
       </c>
     </row>
     <row r="3" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="92" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="93"/>
+      <c r="D3" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="F3" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="B3" s="99" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="100"/>
-      <c r="D3" s="25" t="s">
+      <c r="G3" s="94" t="s">
         <v>93</v>
       </c>
-      <c r="E3" s="26" t="s">
+      <c r="H3" s="95"/>
+      <c r="I3" s="93"/>
+      <c r="J3" s="94" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" s="95"/>
+      <c r="L3" s="93"/>
+      <c r="M3" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="F3" s="27" t="s">
-        <v>95</v>
-      </c>
-      <c r="G3" s="101" t="s">
+      <c r="N3" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="H3" s="102"/>
-      <c r="I3" s="100"/>
-      <c r="J3" s="101" t="s">
-        <v>37</v>
-      </c>
-      <c r="K3" s="102"/>
-      <c r="L3" s="100"/>
-      <c r="M3" s="28" t="s">
+      <c r="O3" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="N3" s="30" t="s">
+      <c r="P3" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q3" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="R3" s="26"/>
+      <c r="S3" s="96" t="s">
         <v>99</v>
       </c>
-      <c r="O3" s="31" t="s">
+      <c r="T3" s="95"/>
+      <c r="U3" s="93"/>
+      <c r="V3" s="96" t="s">
         <v>100</v>
       </c>
-      <c r="P3" s="32" t="s">
+      <c r="W3" s="95"/>
+      <c r="X3" s="93"/>
+      <c r="Y3" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="Z3" s="67"/>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="A4" s="18"/>
+      <c r="B4" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="18"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="H4" s="30" t="s">
         <v>101</v>
       </c>
-      <c r="Q3" s="27" t="s">
-        <v>42</v>
-      </c>
-      <c r="R3" s="33"/>
-      <c r="S3" s="103" t="s">
+      <c r="I4" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="T3" s="102"/>
-      <c r="U3" s="100"/>
-      <c r="V3" s="103" t="s">
-        <v>103</v>
-      </c>
-      <c r="W3" s="102"/>
-      <c r="X3" s="100"/>
-      <c r="Y3" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="Z3" s="74"/>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="25"/>
-      <c r="B4" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="25"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="30" t="s">
+      <c r="J4" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="H4" s="37" t="s">
-        <v>104</v>
-      </c>
-      <c r="I4" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="J4" s="30" t="s">
+      <c r="K4" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="L4" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="M4" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="K4" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="L4" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="M4" s="30" t="s">
+      <c r="N4" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="N4" s="30" t="s">
+      <c r="O4" s="24"/>
+      <c r="P4" s="31"/>
+      <c r="Q4" s="29"/>
+      <c r="R4" s="32"/>
+      <c r="S4" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="O4" s="31"/>
-      <c r="P4" s="38"/>
-      <c r="Q4" s="36"/>
-      <c r="R4" s="39"/>
-      <c r="S4" s="30" t="s">
+      <c r="T4" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="U4" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="V4" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="T4" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="U4" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="V4" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="W4" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="X4" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="Y4" s="31"/>
-      <c r="Z4" s="74"/>
+      <c r="W4" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="X4" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="Y4" s="24"/>
+      <c r="Z4" s="67"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="69"/>
-      <c r="B5" s="74"/>
-      <c r="C5" s="74"/>
-      <c r="D5" s="67"/>
-      <c r="E5" s="68"/>
-      <c r="F5" s="69"/>
-      <c r="G5" s="69"/>
-      <c r="H5" s="68"/>
-      <c r="I5" s="68"/>
-      <c r="J5" s="69"/>
-      <c r="K5" s="68"/>
-      <c r="L5" s="68"/>
-      <c r="M5" s="69"/>
-      <c r="N5" s="69"/>
-      <c r="O5" s="69"/>
-      <c r="P5" s="69"/>
-      <c r="Q5" s="69"/>
-      <c r="R5" s="69"/>
-      <c r="S5" s="69"/>
-      <c r="T5" s="69"/>
-      <c r="U5" s="68"/>
-      <c r="V5" s="68"/>
-      <c r="W5" s="68"/>
-      <c r="X5" s="68"/>
-      <c r="Y5" s="68"/>
-      <c r="Z5" s="69"/>
+      <c r="A5" s="62"/>
+      <c r="B5" s="67"/>
+      <c r="C5" s="67"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="61"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
+      <c r="H5" s="61"/>
+      <c r="I5" s="61"/>
+      <c r="J5" s="62"/>
+      <c r="K5" s="61"/>
+      <c r="L5" s="61"/>
+      <c r="M5" s="62"/>
+      <c r="N5" s="62"/>
+      <c r="O5" s="62"/>
+      <c r="P5" s="62"/>
+      <c r="Q5" s="62"/>
+      <c r="R5" s="62"/>
+      <c r="S5" s="62"/>
+      <c r="T5" s="62"/>
+      <c r="U5" s="61"/>
+      <c r="V5" s="61"/>
+      <c r="W5" s="61"/>
+      <c r="X5" s="61"/>
+      <c r="Y5" s="61"/>
+      <c r="Z5" s="62"/>
     </row>
     <row r="6" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
@@ -3635,46 +3575,46 @@
       </c>
     </row>
     <row r="7" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="40" t="s">
+      <c r="A7" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="41" t="s">
+      <c r="B7" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="41" t="s">
+      <c r="C7" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="D7" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="E7" s="43" t="s">
-        <v>108</v>
-      </c>
-      <c r="F7" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="H7" s="45" t="s">
+      <c r="E7" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="F7" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="H7" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="42" t="s">
+      <c r="I7" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="K7" s="42" t="s">
+      <c r="K7" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="L7" s="46" t="s">
+      <c r="L7" s="39" t="s">
         <v>52</v>
       </c>
-      <c r="M7" s="48" t="s">
-        <v>97</v>
-      </c>
-      <c r="N7" s="40" t="s">
-        <v>109</v>
-      </c>
-      <c r="O7" s="41" t="s">
+      <c r="M7" s="41" t="s">
+        <v>94</v>
+      </c>
+      <c r="N7" s="33" t="s">
+        <v>106</v>
+      </c>
+      <c r="O7" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="R7" s="48" t="s">
+      <c r="R7" s="41" t="s">
         <v>42</v>
       </c>
     </row>
@@ -3698,7 +3638,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAEF05BD-52B1-49ED-A017-76486C00039F}">
-  <dimension ref="A2:Z16"/>
+  <dimension ref="A2:Z13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
@@ -3706,350 +3646,203 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A3" s="104" t="str">
-        <f>+[1]Summary!A4</f>
-        <v>Office:  Neemuch</v>
-      </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102"/>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="102"/>
-      <c r="O3" s="102"/>
-      <c r="P3" s="102"/>
-      <c r="Q3" s="102"/>
-      <c r="R3" s="102"/>
-      <c r="S3" s="102"/>
-      <c r="T3" s="102"/>
-      <c r="U3" s="102"/>
-      <c r="V3" s="102"/>
-      <c r="W3" s="102"/>
-      <c r="X3" s="102"/>
-      <c r="Y3" s="102"/>
-      <c r="Z3" s="100"/>
+    <row r="3" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="116" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="117" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="118"/>
+      <c r="D3" s="116" t="s">
+        <v>90</v>
+      </c>
+      <c r="E3" s="116" t="s">
+        <v>91</v>
+      </c>
+      <c r="F3" s="119" t="s">
+        <v>92</v>
+      </c>
+      <c r="G3" s="120" t="s">
+        <v>93</v>
+      </c>
+      <c r="H3" s="118"/>
+      <c r="I3" s="118"/>
+      <c r="J3" s="120" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" s="118"/>
+      <c r="L3" s="118"/>
+      <c r="M3" s="119" t="s">
+        <v>94</v>
+      </c>
+      <c r="N3" s="119" t="s">
+        <v>95</v>
+      </c>
+      <c r="O3" s="121" t="s">
+        <v>96</v>
+      </c>
+      <c r="P3" s="119" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q3" s="119" t="s">
+        <v>98</v>
+      </c>
+      <c r="R3" s="119" t="s">
+        <v>42</v>
+      </c>
+      <c r="S3" s="122"/>
+      <c r="T3" s="123" t="s">
+        <v>99</v>
+      </c>
+      <c r="U3" s="118"/>
+      <c r="V3" s="118"/>
+      <c r="W3" s="123" t="s">
+        <v>100</v>
+      </c>
+      <c r="X3" s="118"/>
+      <c r="Y3" s="118"/>
+      <c r="Z3" s="119" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="104">
-        <f>+[1]Summary!A7</f>
-        <v>0</v>
-      </c>
-      <c r="B4" s="102"/>
-      <c r="C4" s="102"/>
-      <c r="D4" s="100"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="104" t="s">
-        <v>89</v>
-      </c>
-      <c r="G4" s="102"/>
-      <c r="H4" s="102"/>
-      <c r="I4" s="102"/>
-      <c r="J4" s="102"/>
-      <c r="K4" s="102"/>
-      <c r="L4" s="102"/>
-      <c r="M4" s="102"/>
-      <c r="N4" s="102"/>
-      <c r="O4" s="102"/>
-      <c r="P4" s="102"/>
-      <c r="Q4" s="102"/>
-      <c r="R4" s="100"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="104" t="s">
-        <v>90</v>
-      </c>
-      <c r="U4" s="102"/>
-      <c r="V4" s="102"/>
-      <c r="W4" s="102"/>
-      <c r="X4" s="102"/>
-      <c r="Y4" s="102"/>
-      <c r="Z4" s="100"/>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A5" s="104" t="s">
-        <v>91</v>
-      </c>
-      <c r="B5" s="102"/>
-      <c r="C5" s="100"/>
-      <c r="D5" s="20">
-        <f>[1]Summary!R7</f>
-        <v>0</v>
-      </c>
-      <c r="E5" s="21">
-        <f>SUMIF(E8:E215,"C",$D$6:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="23">
-        <f>SUMIF(G9:G215,"WIP",$D$7:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="I5" s="21">
-        <f>SUMIF(G8:G215,"C",$D$6:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="J5" s="22"/>
-      <c r="K5" s="23">
-        <f>SUMIF(J9:J215,"WIP",$D$7:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L5" s="21">
-        <f>SUMIF(J8:J215,"C",$D$6:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="22"/>
-      <c r="R5" s="22"/>
-      <c r="S5" s="24"/>
-      <c r="T5" s="22"/>
-      <c r="U5" s="23">
-        <f>SUMIF(T9:T215,"WIP",$D$7:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="V5" s="23">
-        <f>SUMIF(T9:T215,"C",$D$7:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="W5" s="23"/>
-      <c r="X5" s="23">
-        <f>SUMIF(W9:W215,"WIP",$D$7:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="Y5" s="23">
-        <f>SUMIF(W9:W215,"C",$D$7:$D$213)/1000</f>
-        <v>0</v>
-      </c>
-      <c r="Z5" s="22"/>
-    </row>
-    <row r="6" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="25" t="s">
+      <c r="A4" s="116"/>
+      <c r="B4" s="124" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="124" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="116"/>
+      <c r="E4" s="116"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="121" t="s">
+        <v>54</v>
+      </c>
+      <c r="H4" s="121" t="s">
+        <v>101</v>
+      </c>
+      <c r="I4" s="121" t="s">
+        <v>102</v>
+      </c>
+      <c r="J4" s="121" t="s">
+        <v>54</v>
+      </c>
+      <c r="K4" s="121" t="s">
+        <v>101</v>
+      </c>
+      <c r="L4" s="121" t="s">
+        <v>102</v>
+      </c>
+      <c r="M4" s="121" t="s">
+        <v>54</v>
+      </c>
+      <c r="N4" s="121" t="s">
+        <v>54</v>
+      </c>
+      <c r="O4" s="121" t="s">
+        <v>54</v>
+      </c>
+      <c r="P4" s="119"/>
+      <c r="Q4" s="119"/>
+      <c r="R4" s="119"/>
+      <c r="S4" s="122"/>
+      <c r="T4" s="121" t="s">
+        <v>54</v>
+      </c>
+      <c r="U4" s="121" t="s">
+        <v>101</v>
+      </c>
+      <c r="V4" s="121" t="s">
+        <v>102</v>
+      </c>
+      <c r="W4" s="121" t="s">
+        <v>54</v>
+      </c>
+      <c r="X4" s="121" t="s">
+        <v>101</v>
+      </c>
+      <c r="Y4" s="121" t="s">
+        <v>102</v>
+      </c>
+      <c r="Z4" s="119"/>
+    </row>
+    <row r="7" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="34" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="F8" s="37" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="99" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="100"/>
-      <c r="D6" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="E6" s="26" t="s">
+      <c r="H8" s="38" t="s">
+        <v>48</v>
+      </c>
+      <c r="I8" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K8" s="35" t="s">
+        <v>51</v>
+      </c>
+      <c r="L8" s="39" t="s">
+        <v>52</v>
+      </c>
+      <c r="M8" s="41" t="s">
         <v>94</v>
       </c>
-      <c r="F6" s="27" t="s">
-        <v>95</v>
-      </c>
-      <c r="G6" s="101" t="s">
-        <v>96</v>
-      </c>
-      <c r="H6" s="102"/>
-      <c r="I6" s="100"/>
-      <c r="J6" s="101" t="s">
-        <v>37</v>
-      </c>
-      <c r="K6" s="102"/>
-      <c r="L6" s="100"/>
-      <c r="M6" s="28" t="s">
-        <v>97</v>
-      </c>
-      <c r="N6" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="O6" s="30" t="s">
-        <v>99</v>
-      </c>
-      <c r="P6" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q6" s="32" t="s">
-        <v>101</v>
-      </c>
-      <c r="R6" s="27" t="s">
+      <c r="N8" s="40" t="s">
+        <v>107</v>
+      </c>
+      <c r="O8" s="33" t="s">
+        <v>106</v>
+      </c>
+      <c r="P8" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="R8" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="S6" s="33"/>
-      <c r="T6" s="103" t="s">
-        <v>102</v>
-      </c>
-      <c r="U6" s="102"/>
-      <c r="V6" s="100"/>
-      <c r="W6" s="103" t="s">
-        <v>103</v>
-      </c>
-      <c r="X6" s="102"/>
-      <c r="Y6" s="100"/>
-      <c r="Z6" s="31" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A7" s="25"/>
-      <c r="B7" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="25"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="H7" s="37" t="s">
-        <v>104</v>
-      </c>
-      <c r="I7" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="J7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="K7" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="L7" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="M7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="N7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="O7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="P7" s="31"/>
-      <c r="Q7" s="38"/>
-      <c r="R7" s="36"/>
-      <c r="S7" s="39"/>
-      <c r="T7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="U7" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="V7" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="W7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="X7" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="Y7" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="Z7" s="31"/>
-    </row>
-    <row r="10" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="40" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" s="41" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="41" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" s="41" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" s="43" t="s">
-        <v>108</v>
-      </c>
-      <c r="F11" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="H11" s="45" t="s">
-        <v>48</v>
-      </c>
-      <c r="I11" s="42" t="s">
-        <v>49</v>
-      </c>
-      <c r="K11" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="L11" s="46" t="s">
-        <v>52</v>
-      </c>
-      <c r="M11" s="48" t="s">
-        <v>97</v>
-      </c>
-      <c r="N11" s="47" t="s">
-        <v>110</v>
-      </c>
-      <c r="O11" s="40" t="s">
-        <v>109</v>
-      </c>
-      <c r="P11" s="41" t="s">
-        <v>34</v>
-      </c>
-      <c r="R11" s="48" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="16" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="41" t="s">
-        <v>106</v>
-      </c>
-      <c r="F16" s="42" t="s">
-        <v>107</v>
-      </c>
-      <c r="K16" s="41" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q16" s="49" t="s">
-        <v>53</v>
-      </c>
-      <c r="R16" s="41" t="s">
-        <v>54</v>
-      </c>
-      <c r="T16" s="41" t="s">
-        <v>80</v>
-      </c>
-      <c r="U16" s="41" t="s">
-        <v>111</v>
-      </c>
-      <c r="V16" s="41" t="s">
-        <v>112</v>
-      </c>
+    </row>
+    <row r="12" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="13" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B13" s="34"/>
+      <c r="F13" s="35"/>
+      <c r="K13" s="34"/>
+      <c r="Q13" s="42"/>
+      <c r="R13" s="34"/>
+      <c r="T13" s="34"/>
+      <c r="U13" s="34"/>
+      <c r="V13" s="34"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="W6:Y6"/>
-    <mergeCell ref="A3:Z3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="F4:R4"/>
-    <mergeCell ref="T4:Z4"/>
-    <mergeCell ref="A5:C5"/>
+  <mergeCells count="5">
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="J3:L3"/>
+    <mergeCell ref="T3:V3"/>
+    <mergeCell ref="W3:Y3"/>
   </mergeCells>
-  <conditionalFormatting sqref="B11">
+  <conditionalFormatting sqref="B8">
     <cfRule type="duplicateValues" dxfId="5" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C11">
+  <conditionalFormatting sqref="C8">
     <cfRule type="duplicateValues" dxfId="4" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4062,59 +3855,59 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:65" x14ac:dyDescent="0.35">
-      <c r="A1" s="103"/>
-      <c r="B1" s="105"/>
-      <c r="C1" s="105"/>
-      <c r="D1" s="105"/>
-      <c r="E1" s="105"/>
-      <c r="F1" s="105"/>
-      <c r="G1" s="105"/>
-      <c r="H1" s="105"/>
-      <c r="I1" s="105"/>
-      <c r="J1" s="105"/>
-      <c r="K1" s="105"/>
-      <c r="L1" s="105"/>
-      <c r="M1" s="105"/>
-      <c r="N1" s="105"/>
-      <c r="O1" s="105"/>
-      <c r="P1" s="105"/>
-      <c r="Q1" s="105"/>
-      <c r="R1" s="105"/>
-      <c r="S1" s="105"/>
-      <c r="T1" s="105"/>
-      <c r="U1" s="105"/>
-      <c r="V1" s="105"/>
-      <c r="W1" s="105"/>
-      <c r="X1" s="105"/>
-      <c r="Y1" s="105"/>
-      <c r="Z1" s="105"/>
-      <c r="AA1" s="105"/>
-      <c r="AB1" s="105"/>
-      <c r="AC1" s="105"/>
-      <c r="AD1" s="105"/>
-      <c r="AE1" s="105"/>
-      <c r="AF1" s="105"/>
-      <c r="AG1" s="105"/>
-      <c r="AH1" s="105"/>
-      <c r="AI1" s="105"/>
-      <c r="AJ1" s="105"/>
-      <c r="AK1" s="105"/>
-      <c r="AL1" s="102"/>
-      <c r="AM1" s="102"/>
-      <c r="AN1" s="102"/>
-      <c r="AO1" s="102"/>
-      <c r="AP1" s="102"/>
-      <c r="AQ1" s="105"/>
-      <c r="AR1" s="105"/>
-      <c r="AS1" s="105"/>
-      <c r="AT1" s="105"/>
-      <c r="AU1" s="105"/>
-      <c r="AV1" s="105"/>
-      <c r="AW1" s="105"/>
-      <c r="AX1" s="105"/>
-      <c r="AY1" s="105"/>
-      <c r="AZ1" s="105"/>
-      <c r="BA1" s="106"/>
+      <c r="A1" s="96"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="97"/>
+      <c r="R1" s="97"/>
+      <c r="S1" s="97"/>
+      <c r="T1" s="97"/>
+      <c r="U1" s="97"/>
+      <c r="V1" s="97"/>
+      <c r="W1" s="97"/>
+      <c r="X1" s="97"/>
+      <c r="Y1" s="97"/>
+      <c r="Z1" s="97"/>
+      <c r="AA1" s="97"/>
+      <c r="AB1" s="97"/>
+      <c r="AC1" s="97"/>
+      <c r="AD1" s="97"/>
+      <c r="AE1" s="97"/>
+      <c r="AF1" s="97"/>
+      <c r="AG1" s="97"/>
+      <c r="AH1" s="97"/>
+      <c r="AI1" s="97"/>
+      <c r="AJ1" s="97"/>
+      <c r="AK1" s="97"/>
+      <c r="AL1" s="95"/>
+      <c r="AM1" s="95"/>
+      <c r="AN1" s="95"/>
+      <c r="AO1" s="95"/>
+      <c r="AP1" s="95"/>
+      <c r="AQ1" s="97"/>
+      <c r="AR1" s="97"/>
+      <c r="AS1" s="97"/>
+      <c r="AT1" s="97"/>
+      <c r="AU1" s="97"/>
+      <c r="AV1" s="97"/>
+      <c r="AW1" s="97"/>
+      <c r="AX1" s="97"/>
+      <c r="AY1" s="97"/>
+      <c r="AZ1" s="97"/>
+      <c r="BA1" s="98"/>
     </row>
     <row r="2" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -4122,334 +3915,334 @@
       </c>
     </row>
     <row r="3" spans="1:65" x14ac:dyDescent="0.35">
-      <c r="A3" s="64" t="s">
-        <v>92</v>
-      </c>
-      <c r="B3" s="63" t="s">
+      <c r="A3" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="56" t="s">
+        <v>116</v>
+      </c>
+      <c r="C3" s="56" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
+      <c r="G3" s="56"/>
+      <c r="H3" s="56" t="s">
+        <v>139</v>
+      </c>
+      <c r="I3" s="56" t="s">
+        <v>140</v>
+      </c>
+      <c r="J3" s="56" t="s">
+        <v>141</v>
+      </c>
+      <c r="K3" s="56" t="s">
+        <v>142</v>
+      </c>
+      <c r="L3" s="56" t="s">
+        <v>135</v>
+      </c>
+      <c r="M3" s="56" t="s">
+        <v>136</v>
+      </c>
+      <c r="N3" s="56" t="s">
+        <v>146</v>
+      </c>
+      <c r="O3" s="56" t="s">
+        <v>137</v>
+      </c>
+      <c r="P3" s="56" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q3" s="56" t="s">
+        <v>135</v>
+      </c>
+      <c r="R3" s="56" t="s">
+        <v>137</v>
+      </c>
+      <c r="S3" s="56" t="s">
+        <v>148</v>
+      </c>
+      <c r="T3" s="56" t="s">
+        <v>149</v>
+      </c>
+      <c r="U3" s="56" t="s">
+        <v>150</v>
+      </c>
+      <c r="V3" s="56" t="s">
         <v>119</v>
       </c>
-      <c r="C3" s="63" t="s">
-        <v>77</v>
-      </c>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63" t="s">
-        <v>142</v>
-      </c>
-      <c r="I3" s="63" t="s">
-        <v>143</v>
-      </c>
-      <c r="J3" s="63" t="s">
-        <v>144</v>
-      </c>
-      <c r="K3" s="63" t="s">
-        <v>145</v>
-      </c>
-      <c r="L3" s="63" t="s">
-        <v>138</v>
-      </c>
-      <c r="M3" s="63" t="s">
-        <v>139</v>
-      </c>
-      <c r="N3" s="63" t="s">
-        <v>149</v>
-      </c>
-      <c r="O3" s="63" t="s">
-        <v>140</v>
-      </c>
-      <c r="P3" s="63" t="s">
-        <v>150</v>
-      </c>
-      <c r="Q3" s="63" t="s">
-        <v>138</v>
-      </c>
-      <c r="R3" s="63" t="s">
-        <v>140</v>
-      </c>
-      <c r="S3" s="63" t="s">
+      <c r="W3" s="56" t="s">
+        <v>78</v>
+      </c>
+      <c r="X3" s="56" t="s">
+        <v>120</v>
+      </c>
+      <c r="Y3" s="56" t="s">
+        <v>121</v>
+      </c>
+      <c r="Z3" s="56"/>
+      <c r="AA3" s="56"/>
+      <c r="AB3" s="56" t="s">
         <v>151</v>
       </c>
-      <c r="T3" s="63" t="s">
+      <c r="AC3" s="56"/>
+      <c r="AD3" s="56" t="s">
         <v>152</v>
       </c>
-      <c r="U3" s="63" t="s">
+      <c r="AE3" s="56"/>
+      <c r="AF3" s="56"/>
+      <c r="AG3" s="56"/>
+      <c r="AH3" s="56"/>
+      <c r="AI3" s="56"/>
+      <c r="AJ3" s="56"/>
+      <c r="AK3" s="56"/>
+      <c r="AL3" s="56"/>
+      <c r="AM3" s="56" t="s">
         <v>153</v>
       </c>
-      <c r="V3" s="63" t="s">
-        <v>122</v>
-      </c>
-      <c r="W3" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="X3" s="63" t="s">
-        <v>123</v>
-      </c>
-      <c r="Y3" s="63" t="s">
-        <v>124</v>
-      </c>
-      <c r="Z3" s="63"/>
-      <c r="AA3" s="63"/>
-      <c r="AB3" s="63" t="s">
+      <c r="AN3" s="56" t="s">
         <v>154</v>
       </c>
-      <c r="AC3" s="63"/>
-      <c r="AD3" s="63" t="s">
+      <c r="AO3" s="56" t="s">
+        <v>61</v>
+      </c>
+      <c r="AP3" s="56" t="s">
+        <v>130</v>
+      </c>
+      <c r="AQ3" s="56"/>
+      <c r="AR3" s="56" t="s">
+        <v>131</v>
+      </c>
+      <c r="AS3" s="56"/>
+      <c r="AT3" s="56" t="s">
+        <v>97</v>
+      </c>
+      <c r="AU3" s="56"/>
+      <c r="AV3" s="56" t="s">
         <v>155</v>
       </c>
-      <c r="AE3" s="63"/>
-      <c r="AF3" s="63"/>
-      <c r="AG3" s="63"/>
-      <c r="AH3" s="63"/>
-      <c r="AI3" s="63"/>
-      <c r="AJ3" s="63"/>
-      <c r="AK3" s="63"/>
-      <c r="AL3" s="63"/>
-      <c r="AM3" s="63" t="s">
+      <c r="AW3" s="56" t="s">
         <v>156</v>
       </c>
-      <c r="AN3" s="63" t="s">
+      <c r="AX3" s="56" t="s">
+        <v>101</v>
+      </c>
+      <c r="AY3" s="56" t="s">
+        <v>102</v>
+      </c>
+      <c r="AZ3" s="56" t="s">
         <v>157</v>
       </c>
-      <c r="AO3" s="63" t="s">
-        <v>61</v>
-      </c>
-      <c r="AP3" s="63" t="s">
-        <v>133</v>
-      </c>
-      <c r="AQ3" s="63"/>
-      <c r="AR3" s="63" t="s">
-        <v>134</v>
-      </c>
-      <c r="AS3" s="63"/>
-      <c r="AT3" s="63" t="s">
-        <v>100</v>
-      </c>
-      <c r="AU3" s="63"/>
-      <c r="AV3" s="63" t="s">
+      <c r="BA3" s="58"/>
+      <c r="BB3" t="s">
         <v>158</v>
       </c>
-      <c r="AW3" s="63" t="s">
-        <v>159</v>
-      </c>
-      <c r="AX3" s="63" t="s">
-        <v>104</v>
-      </c>
-      <c r="AY3" s="63" t="s">
-        <v>105</v>
-      </c>
-      <c r="AZ3" s="63" t="s">
-        <v>160</v>
-      </c>
-      <c r="BA3" s="65"/>
-      <c r="BB3" t="s">
-        <v>161</v>
-      </c>
       <c r="BC3" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="BD3" t="s">
         <v>61</v>
       </c>
       <c r="BE3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="BF3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="BG3" t="s">
+        <v>157</v>
+      </c>
+      <c r="BI3" t="s">
+        <v>132</v>
+      </c>
+      <c r="BJ3" t="s">
+        <v>101</v>
+      </c>
+      <c r="BK3" t="s">
+        <v>102</v>
+      </c>
+      <c r="BL3" t="s">
+        <v>159</v>
+      </c>
+      <c r="BM3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:65" x14ac:dyDescent="0.35">
+      <c r="A4" s="57" t="s">
         <v>160</v>
       </c>
-      <c r="BI3" t="s">
-        <v>135</v>
-      </c>
-      <c r="BJ3" t="s">
-        <v>104</v>
-      </c>
-      <c r="BK3" t="s">
-        <v>105</v>
-      </c>
-      <c r="BL3" t="s">
+      <c r="B4" s="56"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="56" t="s">
+        <v>161</v>
+      </c>
+      <c r="E4" s="56" t="s">
         <v>162</v>
       </c>
-      <c r="BM3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:65" x14ac:dyDescent="0.35">
-      <c r="A4" s="64" t="s">
+      <c r="F4" s="56" t="s">
         <v>163</v>
       </c>
-      <c r="B4" s="63"/>
-      <c r="C4" s="63"/>
-      <c r="D4" s="63" t="s">
+      <c r="G4" s="56" t="s">
         <v>164</v>
       </c>
-      <c r="E4" s="63" t="s">
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
+      <c r="K4" s="56"/>
+      <c r="L4" s="56" t="s">
+        <v>79</v>
+      </c>
+      <c r="M4" s="56" t="s">
+        <v>79</v>
+      </c>
+      <c r="N4" s="56" t="s">
+        <v>79</v>
+      </c>
+      <c r="O4" s="56" t="s">
+        <v>79</v>
+      </c>
+      <c r="P4" s="56" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q4" s="56" t="s">
+        <v>79</v>
+      </c>
+      <c r="R4" s="56" t="s">
+        <v>79</v>
+      </c>
+      <c r="S4" s="56" t="s">
+        <v>79</v>
+      </c>
+      <c r="T4" s="56" t="s">
         <v>165</v>
       </c>
-      <c r="F4" s="63" t="s">
+      <c r="U4" s="56"/>
+      <c r="V4" s="56" t="s">
+        <v>143</v>
+      </c>
+      <c r="W4" s="56"/>
+      <c r="X4" s="56"/>
+      <c r="Y4" s="56" t="s">
+        <v>144</v>
+      </c>
+      <c r="Z4" s="56" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA4" s="56" t="s">
+        <v>138</v>
+      </c>
+      <c r="AB4" s="56" t="s">
         <v>166</v>
       </c>
-      <c r="G4" s="63" t="s">
+      <c r="AC4" s="56" t="s">
         <v>167</v>
       </c>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="63"/>
-      <c r="L4" s="63" t="s">
-        <v>79</v>
-      </c>
-      <c r="M4" s="63" t="s">
-        <v>79</v>
-      </c>
-      <c r="N4" s="63" t="s">
-        <v>79</v>
-      </c>
-      <c r="O4" s="63" t="s">
-        <v>79</v>
-      </c>
-      <c r="P4" s="63" t="s">
-        <v>79</v>
-      </c>
-      <c r="Q4" s="63" t="s">
-        <v>79</v>
-      </c>
-      <c r="R4" s="63" t="s">
-        <v>79</v>
-      </c>
-      <c r="S4" s="63" t="s">
-        <v>79</v>
-      </c>
-      <c r="T4" s="63" t="s">
+      <c r="AD4" s="56" t="s">
         <v>168</v>
       </c>
-      <c r="U4" s="63"/>
-      <c r="V4" s="63" t="s">
-        <v>146</v>
-      </c>
-      <c r="W4" s="63"/>
-      <c r="X4" s="63"/>
-      <c r="Y4" s="63" t="s">
-        <v>147</v>
-      </c>
-      <c r="Z4" s="63" t="s">
-        <v>148</v>
-      </c>
-      <c r="AA4" s="63" t="s">
-        <v>141</v>
-      </c>
-      <c r="AB4" s="63" t="s">
+      <c r="AE4" s="56" t="s">
         <v>169</v>
       </c>
-      <c r="AC4" s="63" t="s">
+      <c r="AF4" s="56" t="s">
         <v>170</v>
       </c>
-      <c r="AD4" s="63" t="s">
+      <c r="AG4" s="56" t="s">
         <v>171</v>
       </c>
-      <c r="AE4" s="63" t="s">
+      <c r="AH4" s="56" t="s">
         <v>172</v>
       </c>
-      <c r="AF4" s="63" t="s">
+      <c r="AI4" s="56" t="s">
         <v>173</v>
       </c>
-      <c r="AG4" s="63" t="s">
+      <c r="AJ4" s="56" t="s">
         <v>174</v>
       </c>
-      <c r="AH4" s="63" t="s">
-        <v>175</v>
-      </c>
-      <c r="AI4" s="63" t="s">
-        <v>176</v>
-      </c>
-      <c r="AJ4" s="63" t="s">
-        <v>177</v>
-      </c>
-      <c r="AK4" s="63" t="s">
-        <v>131</v>
-      </c>
-      <c r="AL4" s="63"/>
-      <c r="AM4" s="63"/>
-      <c r="AN4" s="63"/>
-      <c r="AO4" s="63"/>
-      <c r="AP4" s="63" t="s">
-        <v>104</v>
-      </c>
-      <c r="AQ4" s="63" t="s">
-        <v>105</v>
-      </c>
-      <c r="AR4" s="63" t="s">
-        <v>104</v>
-      </c>
-      <c r="AS4" s="63">
+      <c r="AK4" s="56" t="s">
+        <v>128</v>
+      </c>
+      <c r="AL4" s="56"/>
+      <c r="AM4" s="56"/>
+      <c r="AN4" s="56"/>
+      <c r="AO4" s="56"/>
+      <c r="AP4" s="56" t="s">
+        <v>101</v>
+      </c>
+      <c r="AQ4" s="56" t="s">
+        <v>102</v>
+      </c>
+      <c r="AR4" s="56" t="s">
+        <v>101</v>
+      </c>
+      <c r="AS4" s="56">
         <v>9</v>
       </c>
-      <c r="AT4" s="63"/>
-      <c r="AU4" s="63"/>
-      <c r="AV4" s="63"/>
-      <c r="AW4" s="63"/>
-      <c r="AX4" s="63"/>
-      <c r="AY4" s="63"/>
-      <c r="AZ4" s="63"/>
-      <c r="BA4" s="65"/>
+      <c r="AT4" s="56"/>
+      <c r="AU4" s="56"/>
+      <c r="AV4" s="56"/>
+      <c r="AW4" s="56"/>
+      <c r="AX4" s="56"/>
+      <c r="AY4" s="56"/>
+      <c r="AZ4" s="56"/>
+      <c r="BA4" s="58"/>
     </row>
     <row r="6" spans="1:65" x14ac:dyDescent="0.35">
-      <c r="A6" s="64"/>
-      <c r="B6" s="63"/>
-      <c r="C6" s="63"/>
-      <c r="D6" s="63"/>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="63"/>
-      <c r="H6" s="63"/>
-      <c r="I6" s="63"/>
-      <c r="J6" s="63"/>
-      <c r="K6" s="63"/>
-      <c r="L6" s="63"/>
-      <c r="M6" s="63"/>
-      <c r="N6" s="63"/>
-      <c r="O6" s="63"/>
-      <c r="P6" s="63"/>
-      <c r="Q6" s="63"/>
-      <c r="R6" s="63"/>
-      <c r="S6" s="63"/>
-      <c r="T6" s="63"/>
-      <c r="U6" s="63"/>
-      <c r="V6" s="63"/>
-      <c r="W6" s="63"/>
-      <c r="X6" s="63"/>
-      <c r="Y6" s="63"/>
-      <c r="Z6" s="63"/>
-      <c r="AA6" s="63"/>
-      <c r="AB6" s="63"/>
-      <c r="AC6" s="63"/>
-      <c r="AD6" s="63"/>
-      <c r="AE6" s="63"/>
-      <c r="AF6" s="63"/>
-      <c r="AG6" s="63"/>
-      <c r="AH6" s="63"/>
-      <c r="AI6" s="63"/>
-      <c r="AJ6" s="63"/>
-      <c r="AK6" s="63"/>
-      <c r="AL6" s="63"/>
-      <c r="AM6" s="63"/>
-      <c r="AN6" s="63"/>
-      <c r="AO6" s="63"/>
-      <c r="AP6" s="63"/>
-      <c r="AQ6" s="63"/>
-      <c r="AR6" s="63"/>
-      <c r="AS6" s="63"/>
-      <c r="AT6" s="63"/>
-      <c r="AU6" s="63"/>
-      <c r="AV6" s="63"/>
-      <c r="AW6" s="63"/>
-      <c r="AX6" s="63"/>
-      <c r="AY6" s="63"/>
-      <c r="AZ6" s="63"/>
-      <c r="BA6" s="65"/>
+      <c r="A6" s="57"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="56"/>
+      <c r="D6" s="56"/>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56"/>
+      <c r="G6" s="56"/>
+      <c r="H6" s="56"/>
+      <c r="I6" s="56"/>
+      <c r="J6" s="56"/>
+      <c r="K6" s="56"/>
+      <c r="L6" s="56"/>
+      <c r="M6" s="56"/>
+      <c r="N6" s="56"/>
+      <c r="O6" s="56"/>
+      <c r="P6" s="56"/>
+      <c r="Q6" s="56"/>
+      <c r="R6" s="56"/>
+      <c r="S6" s="56"/>
+      <c r="T6" s="56"/>
+      <c r="U6" s="56"/>
+      <c r="V6" s="56"/>
+      <c r="W6" s="56"/>
+      <c r="X6" s="56"/>
+      <c r="Y6" s="56"/>
+      <c r="Z6" s="56"/>
+      <c r="AA6" s="56"/>
+      <c r="AB6" s="56"/>
+      <c r="AC6" s="56"/>
+      <c r="AD6" s="56"/>
+      <c r="AE6" s="56"/>
+      <c r="AF6" s="56"/>
+      <c r="AG6" s="56"/>
+      <c r="AH6" s="56"/>
+      <c r="AI6" s="56"/>
+      <c r="AJ6" s="56"/>
+      <c r="AK6" s="56"/>
+      <c r="AL6" s="56"/>
+      <c r="AM6" s="56"/>
+      <c r="AN6" s="56"/>
+      <c r="AO6" s="56"/>
+      <c r="AP6" s="56"/>
+      <c r="AQ6" s="56"/>
+      <c r="AR6" s="56"/>
+      <c r="AS6" s="56"/>
+      <c r="AT6" s="56"/>
+      <c r="AU6" s="56"/>
+      <c r="AV6" s="56"/>
+      <c r="AW6" s="56"/>
+      <c r="AX6" s="56"/>
+      <c r="AY6" s="56"/>
+      <c r="AZ6" s="56"/>
+      <c r="BA6" s="58"/>
     </row>
     <row r="9" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -4467,16 +4260,16 @@
         <v>77</v>
       </c>
       <c r="D10" s="6"/>
-      <c r="H10" s="61"/>
-      <c r="I10" s="61"/>
+      <c r="H10" s="54"/>
+      <c r="I10" s="54"/>
       <c r="M10" s="6"/>
       <c r="N10" s="17"/>
-      <c r="O10" s="60"/>
+      <c r="O10" s="53"/>
       <c r="P10" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="Q10" s="62"/>
-      <c r="BB10" s="60" t="s">
+      <c r="Q10" s="55"/>
+      <c r="BB10" s="53" t="s">
         <v>54</v>
       </c>
       <c r="BE10" s="6" t="s">
@@ -4511,409 +4304,409 @@
       </c>
     </row>
     <row r="3" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A3" s="103" t="str">
-        <f>+[2]Summary!A4</f>
+      <c r="A3" s="96" t="str">
+        <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="105"/>
-      <c r="C3" s="105"/>
-      <c r="D3" s="105"/>
-      <c r="E3" s="105"/>
-      <c r="F3" s="105"/>
-      <c r="G3" s="105"/>
-      <c r="H3" s="105"/>
-      <c r="I3" s="105"/>
-      <c r="J3" s="105"/>
-      <c r="K3" s="105"/>
-      <c r="L3" s="105"/>
-      <c r="M3" s="105"/>
-      <c r="N3" s="105"/>
-      <c r="O3" s="105"/>
-      <c r="P3" s="105"/>
-      <c r="Q3" s="105"/>
-      <c r="R3" s="105"/>
-      <c r="S3" s="105"/>
-      <c r="T3" s="105"/>
-      <c r="U3" s="105"/>
-      <c r="V3" s="105"/>
-      <c r="W3" s="105"/>
-      <c r="X3" s="105"/>
-      <c r="Y3" s="105"/>
-      <c r="Z3" s="105"/>
-      <c r="AA3" s="105"/>
-      <c r="AB3" s="105"/>
-      <c r="AC3" s="105"/>
-      <c r="AD3" s="105"/>
-      <c r="AE3" s="105"/>
-      <c r="AF3" s="105"/>
-      <c r="AG3" s="105"/>
-      <c r="AH3" s="105"/>
-      <c r="AI3" s="105"/>
-      <c r="AJ3" s="105"/>
-      <c r="AK3" s="105"/>
-      <c r="AL3" s="102"/>
-      <c r="AM3" s="102"/>
-      <c r="AN3" s="102"/>
-      <c r="AO3" s="102"/>
-      <c r="AP3" s="102"/>
-      <c r="AQ3" s="105"/>
-      <c r="AR3" s="105"/>
-      <c r="AS3" s="105"/>
-      <c r="AT3" s="105"/>
-      <c r="AU3" s="105"/>
-      <c r="AV3" s="105"/>
-      <c r="AW3" s="105"/>
-      <c r="AX3" s="105"/>
-      <c r="AY3" s="105"/>
-      <c r="AZ3" s="105"/>
-      <c r="BA3" s="106"/>
+      <c r="B3" s="97"/>
+      <c r="C3" s="97"/>
+      <c r="D3" s="97"/>
+      <c r="E3" s="97"/>
+      <c r="F3" s="97"/>
+      <c r="G3" s="97"/>
+      <c r="H3" s="97"/>
+      <c r="I3" s="97"/>
+      <c r="J3" s="97"/>
+      <c r="K3" s="97"/>
+      <c r="L3" s="97"/>
+      <c r="M3" s="97"/>
+      <c r="N3" s="97"/>
+      <c r="O3" s="97"/>
+      <c r="P3" s="97"/>
+      <c r="Q3" s="97"/>
+      <c r="R3" s="97"/>
+      <c r="S3" s="97"/>
+      <c r="T3" s="97"/>
+      <c r="U3" s="97"/>
+      <c r="V3" s="97"/>
+      <c r="W3" s="97"/>
+      <c r="X3" s="97"/>
+      <c r="Y3" s="97"/>
+      <c r="Z3" s="97"/>
+      <c r="AA3" s="97"/>
+      <c r="AB3" s="97"/>
+      <c r="AC3" s="97"/>
+      <c r="AD3" s="97"/>
+      <c r="AE3" s="97"/>
+      <c r="AF3" s="97"/>
+      <c r="AG3" s="97"/>
+      <c r="AH3" s="97"/>
+      <c r="AI3" s="97"/>
+      <c r="AJ3" s="97"/>
+      <c r="AK3" s="97"/>
+      <c r="AL3" s="95"/>
+      <c r="AM3" s="95"/>
+      <c r="AN3" s="95"/>
+      <c r="AO3" s="95"/>
+      <c r="AP3" s="95"/>
+      <c r="AQ3" s="97"/>
+      <c r="AR3" s="97"/>
+      <c r="AS3" s="97"/>
+      <c r="AT3" s="97"/>
+      <c r="AU3" s="97"/>
+      <c r="AV3" s="97"/>
+      <c r="AW3" s="97"/>
+      <c r="AX3" s="97"/>
+      <c r="AY3" s="97"/>
+      <c r="AZ3" s="97"/>
+      <c r="BA3" s="98"/>
     </row>
     <row r="4" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A4" s="103">
-        <f>+[2]Summary!A7</f>
+      <c r="A4" s="96">
+        <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="105"/>
-      <c r="C4" s="105"/>
-      <c r="D4" s="105"/>
-      <c r="E4" s="105"/>
-      <c r="F4" s="105"/>
-      <c r="G4" s="105"/>
-      <c r="H4" s="105"/>
-      <c r="I4" s="105"/>
-      <c r="J4" s="105"/>
-      <c r="K4" s="105"/>
-      <c r="L4" s="105"/>
-      <c r="M4" s="105"/>
-      <c r="N4" s="105"/>
-      <c r="O4" s="105"/>
-      <c r="P4" s="105"/>
-      <c r="Q4" s="105"/>
-      <c r="R4" s="105"/>
-      <c r="S4" s="105"/>
-      <c r="T4" s="105"/>
-      <c r="U4" s="105"/>
-      <c r="V4" s="105"/>
-      <c r="W4" s="105"/>
-      <c r="X4" s="105"/>
-      <c r="Y4" s="105"/>
-      <c r="Z4" s="105"/>
-      <c r="AA4" s="105"/>
-      <c r="AB4" s="105"/>
-      <c r="AC4" s="105"/>
-      <c r="AD4" s="105"/>
-      <c r="AE4" s="105"/>
-      <c r="AF4" s="105"/>
-      <c r="AG4" s="105"/>
-      <c r="AH4" s="105"/>
-      <c r="AI4" s="105"/>
-      <c r="AJ4" s="105"/>
-      <c r="AK4" s="105"/>
-      <c r="AL4" s="102"/>
-      <c r="AM4" s="102"/>
-      <c r="AN4" s="102"/>
-      <c r="AO4" s="102"/>
-      <c r="AP4" s="102"/>
-      <c r="AQ4" s="105"/>
-      <c r="AR4" s="105"/>
-      <c r="AS4" s="105"/>
-      <c r="AT4" s="105"/>
-      <c r="AU4" s="105"/>
-      <c r="AV4" s="105"/>
-      <c r="AW4" s="105"/>
-      <c r="AX4" s="105"/>
-      <c r="AY4" s="105"/>
-      <c r="AZ4" s="105"/>
-      <c r="BA4" s="106"/>
+      <c r="B4" s="97"/>
+      <c r="C4" s="97"/>
+      <c r="D4" s="97"/>
+      <c r="E4" s="97"/>
+      <c r="F4" s="97"/>
+      <c r="G4" s="97"/>
+      <c r="H4" s="97"/>
+      <c r="I4" s="97"/>
+      <c r="J4" s="97"/>
+      <c r="K4" s="97"/>
+      <c r="L4" s="97"/>
+      <c r="M4" s="97"/>
+      <c r="N4" s="97"/>
+      <c r="O4" s="97"/>
+      <c r="P4" s="97"/>
+      <c r="Q4" s="97"/>
+      <c r="R4" s="97"/>
+      <c r="S4" s="97"/>
+      <c r="T4" s="97"/>
+      <c r="U4" s="97"/>
+      <c r="V4" s="97"/>
+      <c r="W4" s="97"/>
+      <c r="X4" s="97"/>
+      <c r="Y4" s="97"/>
+      <c r="Z4" s="97"/>
+      <c r="AA4" s="97"/>
+      <c r="AB4" s="97"/>
+      <c r="AC4" s="97"/>
+      <c r="AD4" s="97"/>
+      <c r="AE4" s="97"/>
+      <c r="AF4" s="97"/>
+      <c r="AG4" s="97"/>
+      <c r="AH4" s="97"/>
+      <c r="AI4" s="97"/>
+      <c r="AJ4" s="97"/>
+      <c r="AK4" s="97"/>
+      <c r="AL4" s="95"/>
+      <c r="AM4" s="95"/>
+      <c r="AN4" s="95"/>
+      <c r="AO4" s="95"/>
+      <c r="AP4" s="95"/>
+      <c r="AQ4" s="97"/>
+      <c r="AR4" s="97"/>
+      <c r="AS4" s="97"/>
+      <c r="AT4" s="97"/>
+      <c r="AU4" s="97"/>
+      <c r="AV4" s="97"/>
+      <c r="AW4" s="97"/>
+      <c r="AX4" s="97"/>
+      <c r="AY4" s="97"/>
+      <c r="AZ4" s="97"/>
+      <c r="BA4" s="98"/>
     </row>
     <row r="5" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="103" t="s">
+      <c r="A5" s="96" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="97"/>
+      <c r="C5" s="97"/>
+      <c r="D5" s="97"/>
+      <c r="E5" s="97"/>
+      <c r="F5" s="97"/>
+      <c r="G5" s="97"/>
+      <c r="H5" s="97"/>
+      <c r="I5" s="97"/>
+      <c r="J5" s="97"/>
+      <c r="K5" s="97"/>
+      <c r="L5" s="97"/>
+      <c r="M5" s="97"/>
+      <c r="N5" s="97"/>
+      <c r="O5" s="97"/>
+      <c r="P5" s="97"/>
+      <c r="Q5" s="97"/>
+      <c r="R5" s="97"/>
+      <c r="S5" s="98"/>
+      <c r="T5" s="96" t="s">
+        <v>111</v>
+      </c>
+      <c r="U5" s="97"/>
+      <c r="V5" s="97"/>
+      <c r="W5" s="97"/>
+      <c r="X5" s="97"/>
+      <c r="Y5" s="97"/>
+      <c r="Z5" s="97"/>
+      <c r="AA5" s="97"/>
+      <c r="AB5" s="97"/>
+      <c r="AC5" s="97"/>
+      <c r="AD5" s="97"/>
+      <c r="AE5" s="97"/>
+      <c r="AF5" s="97"/>
+      <c r="AG5" s="97"/>
+      <c r="AH5" s="97"/>
+      <c r="AI5" s="97"/>
+      <c r="AJ5" s="97"/>
+      <c r="AK5" s="98"/>
+      <c r="AL5" s="96" t="s">
+        <v>112</v>
+      </c>
+      <c r="AM5" s="95"/>
+      <c r="AN5" s="95"/>
+      <c r="AO5" s="95"/>
+      <c r="AP5" s="93"/>
+      <c r="AQ5" s="96" t="s">
+        <v>2</v>
+      </c>
+      <c r="AR5" s="97"/>
+      <c r="AS5" s="97"/>
+      <c r="AT5" s="98"/>
+      <c r="AU5" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="105"/>
-      <c r="C5" s="105"/>
-      <c r="D5" s="105"/>
-      <c r="E5" s="105"/>
-      <c r="F5" s="105"/>
-      <c r="G5" s="105"/>
-      <c r="H5" s="105"/>
-      <c r="I5" s="105"/>
-      <c r="J5" s="105"/>
-      <c r="K5" s="105"/>
-      <c r="L5" s="105"/>
-      <c r="M5" s="105"/>
-      <c r="N5" s="105"/>
-      <c r="O5" s="105"/>
-      <c r="P5" s="105"/>
-      <c r="Q5" s="105"/>
-      <c r="R5" s="105"/>
-      <c r="S5" s="106"/>
-      <c r="T5" s="103" t="s">
+      <c r="AV5" s="96" t="s">
         <v>114</v>
       </c>
-      <c r="U5" s="105"/>
-      <c r="V5" s="105"/>
-      <c r="W5" s="105"/>
-      <c r="X5" s="105"/>
-      <c r="Y5" s="105"/>
-      <c r="Z5" s="105"/>
-      <c r="AA5" s="105"/>
-      <c r="AB5" s="105"/>
-      <c r="AC5" s="105"/>
-      <c r="AD5" s="105"/>
-      <c r="AE5" s="105"/>
-      <c r="AF5" s="105"/>
-      <c r="AG5" s="105"/>
-      <c r="AH5" s="105"/>
-      <c r="AI5" s="105"/>
-      <c r="AJ5" s="105"/>
-      <c r="AK5" s="106"/>
-      <c r="AL5" s="103" t="s">
+      <c r="AW5" s="97"/>
+      <c r="AX5" s="97"/>
+      <c r="AY5" s="97"/>
+      <c r="AZ5" s="98"/>
+      <c r="BA5" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="AM5" s="102"/>
-      <c r="AN5" s="102"/>
-      <c r="AO5" s="102"/>
-      <c r="AP5" s="100"/>
-      <c r="AQ5" s="103" t="s">
-        <v>2</v>
-      </c>
-      <c r="AR5" s="105"/>
-      <c r="AS5" s="105"/>
-      <c r="AT5" s="106"/>
-      <c r="AU5" s="27" t="s">
+    </row>
+    <row r="6" spans="1:53" ht="58.5" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="AV5" s="103" t="s">
+      <c r="C6" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="99" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" s="100"/>
+      <c r="I6" s="100"/>
+      <c r="J6" s="101"/>
+      <c r="K6" s="99" t="s">
         <v>117</v>
       </c>
-      <c r="AW5" s="105"/>
-      <c r="AX5" s="105"/>
-      <c r="AY5" s="105"/>
-      <c r="AZ5" s="106"/>
-      <c r="BA5" s="27" t="s">
+      <c r="L6" s="100"/>
+      <c r="M6" s="100"/>
+      <c r="N6" s="101"/>
+      <c r="O6" s="102" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="6" spans="1:53" ht="58.5" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="31" t="s">
-        <v>92</v>
-      </c>
-      <c r="B6" s="31" t="s">
+      <c r="P6" s="97"/>
+      <c r="Q6" s="97"/>
+      <c r="R6" s="98"/>
+      <c r="S6" s="44" t="s">
         <v>119</v>
       </c>
-      <c r="C6" s="31" t="s">
-        <v>77</v>
-      </c>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="107" t="s">
-        <v>81</v>
-      </c>
-      <c r="H6" s="108"/>
-      <c r="I6" s="108"/>
-      <c r="J6" s="109"/>
-      <c r="K6" s="107" t="s">
+      <c r="T6" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="U6" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="L6" s="108"/>
-      <c r="M6" s="108"/>
-      <c r="N6" s="109"/>
-      <c r="O6" s="110" t="s">
+      <c r="V6" s="96" t="s">
         <v>121</v>
       </c>
-      <c r="P6" s="105"/>
-      <c r="Q6" s="105"/>
-      <c r="R6" s="106"/>
-      <c r="S6" s="51" t="s">
+      <c r="W6" s="97"/>
+      <c r="X6" s="98"/>
+      <c r="Y6" s="45" t="s">
         <v>122</v>
       </c>
-      <c r="T6" s="27" t="s">
-        <v>78</v>
-      </c>
-      <c r="U6" s="31" t="s">
+      <c r="Z6" s="45" t="s">
         <v>123</v>
       </c>
-      <c r="V6" s="103" t="s">
+      <c r="AA6" s="45" t="s">
         <v>124</v>
       </c>
-      <c r="W6" s="105"/>
-      <c r="X6" s="106"/>
-      <c r="Y6" s="52" t="s">
+      <c r="AB6" s="45" t="s">
         <v>125</v>
       </c>
-      <c r="Z6" s="52" t="s">
+      <c r="AC6" s="45" t="s">
         <v>126</v>
       </c>
-      <c r="AA6" s="52" t="s">
+      <c r="AD6" s="45" t="s">
         <v>127</v>
       </c>
-      <c r="AB6" s="52" t="s">
+      <c r="AE6" s="46" t="s">
         <v>128</v>
       </c>
-      <c r="AC6" s="52" t="s">
+      <c r="AF6" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="AD6" s="52" t="s">
+      <c r="AG6" s="103" t="s">
         <v>130</v>
       </c>
-      <c r="AE6" s="53" t="s">
+      <c r="AH6" s="98"/>
+      <c r="AI6" s="96" t="s">
         <v>131</v>
       </c>
-      <c r="AF6" s="27" t="s">
+      <c r="AJ6" s="98"/>
+      <c r="AK6" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="AL6" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="AG6" s="111" t="s">
+      <c r="AM6" s="20" t="s">
         <v>133</v>
       </c>
-      <c r="AH6" s="106"/>
-      <c r="AI6" s="103" t="s">
+      <c r="AN6" s="47" t="s">
+        <v>101</v>
+      </c>
+      <c r="AO6" s="47" t="s">
+        <v>102</v>
+      </c>
+      <c r="AP6" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="AQ6" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="AR6" s="47" t="s">
+        <v>101</v>
+      </c>
+      <c r="AS6" s="47" t="s">
+        <v>102</v>
+      </c>
+      <c r="AT6" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="AU6" s="46"/>
+      <c r="AV6" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="AW6" s="47" t="s">
+        <v>101</v>
+      </c>
+      <c r="AX6" s="47" t="s">
+        <v>102</v>
+      </c>
+      <c r="AY6" s="48" t="s">
         <v>134</v>
       </c>
-      <c r="AJ6" s="106"/>
-      <c r="AK6" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="AL6" s="27" t="s">
+      <c r="AZ6" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="BA6" s="46"/>
+    </row>
+    <row r="7" spans="1:53" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="24"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="AM6" s="27" t="s">
+      <c r="H7" s="24" t="s">
         <v>136</v>
       </c>
-      <c r="AN6" s="54" t="s">
-        <v>104</v>
-      </c>
-      <c r="AO6" s="54" t="s">
-        <v>105</v>
-      </c>
-      <c r="AP6" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="AQ6" s="27" t="s">
+      <c r="I7" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="J7" s="50" t="s">
+        <v>138</v>
+      </c>
+      <c r="K7" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="AR6" s="54" t="s">
-        <v>104</v>
-      </c>
-      <c r="AS6" s="54" t="s">
-        <v>105</v>
-      </c>
-      <c r="AT6" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="AU6" s="53"/>
-      <c r="AV6" s="27" t="s">
-        <v>135</v>
-      </c>
-      <c r="AW6" s="54" t="s">
-        <v>104</v>
-      </c>
-      <c r="AX6" s="54" t="s">
-        <v>105</v>
-      </c>
-      <c r="AY6" s="55" t="s">
+      <c r="L7" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="M7" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="AZ6" s="27" t="s">
-        <v>100</v>
-      </c>
-      <c r="BA6" s="53"/>
-    </row>
-    <row r="7" spans="1:53" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="31"/>
-      <c r="B7" s="31"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="29"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="29"/>
-      <c r="G7" s="56" t="s">
+      <c r="N7" s="50" t="s">
         <v>138</v>
       </c>
-      <c r="H7" s="31" t="s">
+      <c r="O7" s="47" t="s">
         <v>139</v>
       </c>
-      <c r="I7" s="31" t="s">
+      <c r="P7" s="47" t="s">
         <v>140</v>
       </c>
-      <c r="J7" s="57" t="s">
+      <c r="Q7" s="47" t="s">
         <v>141</v>
       </c>
-      <c r="K7" s="56" t="s">
+      <c r="R7" s="47" t="s">
+        <v>142</v>
+      </c>
+      <c r="S7" s="51" t="s">
+        <v>143</v>
+      </c>
+      <c r="T7" s="29"/>
+      <c r="U7" s="20"/>
+      <c r="V7" s="20" t="s">
+        <v>144</v>
+      </c>
+      <c r="W7" s="20" t="s">
+        <v>145</v>
+      </c>
+      <c r="X7" s="20" t="s">
         <v>138</v>
       </c>
-      <c r="L7" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="M7" s="31" t="s">
-        <v>140</v>
-      </c>
-      <c r="N7" s="57" t="s">
-        <v>141</v>
-      </c>
-      <c r="O7" s="54" t="s">
-        <v>142</v>
-      </c>
-      <c r="P7" s="54" t="s">
-        <v>143</v>
-      </c>
-      <c r="Q7" s="54" t="s">
-        <v>144</v>
-      </c>
-      <c r="R7" s="54" t="s">
-        <v>145</v>
-      </c>
-      <c r="S7" s="58" t="s">
-        <v>146</v>
-      </c>
-      <c r="T7" s="36"/>
-      <c r="U7" s="27"/>
-      <c r="V7" s="27" t="s">
-        <v>147</v>
-      </c>
-      <c r="W7" s="27" t="s">
-        <v>148</v>
-      </c>
-      <c r="X7" s="27" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y7" s="53"/>
-      <c r="Z7" s="53"/>
-      <c r="AA7" s="53"/>
-      <c r="AB7" s="53"/>
-      <c r="AC7" s="53"/>
-      <c r="AD7" s="53"/>
-      <c r="AE7" s="36"/>
-      <c r="AF7" s="36"/>
-      <c r="AG7" s="54" t="s">
-        <v>104</v>
-      </c>
-      <c r="AH7" s="54" t="s">
-        <v>105</v>
-      </c>
-      <c r="AI7" s="54" t="s">
-        <v>104</v>
-      </c>
-      <c r="AJ7" s="54" t="s">
-        <v>105</v>
-      </c>
-      <c r="AK7" s="36"/>
-      <c r="AL7" s="36"/>
-      <c r="AM7" s="36"/>
-      <c r="AN7" s="54"/>
-      <c r="AO7" s="54"/>
-      <c r="AP7" s="36"/>
-      <c r="AQ7" s="36"/>
-      <c r="AR7" s="54"/>
-      <c r="AS7" s="54"/>
-      <c r="AT7" s="36"/>
-      <c r="AU7" s="36"/>
-      <c r="AV7" s="36"/>
-      <c r="AW7" s="54"/>
-      <c r="AX7" s="54"/>
-      <c r="AY7" s="59"/>
-      <c r="AZ7" s="36"/>
-      <c r="BA7" s="36"/>
+      <c r="Y7" s="46"/>
+      <c r="Z7" s="46"/>
+      <c r="AA7" s="46"/>
+      <c r="AB7" s="46"/>
+      <c r="AC7" s="46"/>
+      <c r="AD7" s="46"/>
+      <c r="AE7" s="29"/>
+      <c r="AF7" s="29"/>
+      <c r="AG7" s="47" t="s">
+        <v>101</v>
+      </c>
+      <c r="AH7" s="47" t="s">
+        <v>102</v>
+      </c>
+      <c r="AI7" s="47" t="s">
+        <v>101</v>
+      </c>
+      <c r="AJ7" s="47" t="s">
+        <v>102</v>
+      </c>
+      <c r="AK7" s="29"/>
+      <c r="AL7" s="29"/>
+      <c r="AM7" s="29"/>
+      <c r="AN7" s="47"/>
+      <c r="AO7" s="47"/>
+      <c r="AP7" s="29"/>
+      <c r="AQ7" s="29"/>
+      <c r="AR7" s="47"/>
+      <c r="AS7" s="47"/>
+      <c r="AT7" s="29"/>
+      <c r="AU7" s="29"/>
+      <c r="AV7" s="29"/>
+      <c r="AW7" s="47"/>
+      <c r="AX7" s="47"/>
+      <c r="AY7" s="52"/>
+      <c r="AZ7" s="29"/>
+      <c r="BA7" s="29"/>
     </row>
     <row r="9" spans="1:53" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -4931,17 +4724,17 @@
         <v>77</v>
       </c>
       <c r="D10" s="6"/>
-      <c r="H10" s="61"/>
-      <c r="I10" s="61"/>
+      <c r="H10" s="54"/>
+      <c r="I10" s="54"/>
       <c r="J10" s="6" t="s">
         <v>81</v>
       </c>
       <c r="M10" s="6"/>
       <c r="N10" s="17"/>
-      <c r="O10" s="60"/>
-      <c r="P10" s="61"/>
-      <c r="Q10" s="62"/>
-      <c r="AQ10" s="60" t="s">
+      <c r="O10" s="53"/>
+      <c r="P10" s="54"/>
+      <c r="Q10" s="55"/>
+      <c r="AQ10" s="53" t="s">
         <v>54</v>
       </c>
       <c r="AR10" s="6" t="s">
@@ -4956,12 +4749,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="AI6:AJ6"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="K6:N6"/>
-    <mergeCell ref="O6:R6"/>
-    <mergeCell ref="V6:X6"/>
-    <mergeCell ref="AG6:AH6"/>
     <mergeCell ref="A3:BA3"/>
     <mergeCell ref="A4:BA4"/>
     <mergeCell ref="A5:S5"/>
@@ -4969,6 +4756,12 @@
     <mergeCell ref="AL5:AP5"/>
     <mergeCell ref="AQ5:AT5"/>
     <mergeCell ref="AV5:AZ5"/>
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="O6:R6"/>
+    <mergeCell ref="V6:X6"/>
+    <mergeCell ref="AG6:AH6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4985,35 +4778,35 @@
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="114" t="s">
+      <c r="A3" s="106" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="115" t="s">
+      <c r="B3" s="107" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="102"/>
-      <c r="D3" s="100"/>
-      <c r="E3" s="115" t="s">
+      <c r="C3" s="95"/>
+      <c r="D3" s="93"/>
+      <c r="E3" s="107" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="102"/>
-      <c r="G3" s="100"/>
-      <c r="H3" s="115" t="s">
+      <c r="F3" s="95"/>
+      <c r="G3" s="93"/>
+      <c r="H3" s="107" t="s">
         <v>37</v>
       </c>
-      <c r="I3" s="102"/>
-      <c r="J3" s="100"/>
-      <c r="K3" s="114" t="s">
+      <c r="I3" s="95"/>
+      <c r="J3" s="93"/>
+      <c r="K3" s="106" t="s">
         <v>74</v>
       </c>
-      <c r="L3" s="112" t="s">
+      <c r="L3" s="104" t="s">
         <v>42</v>
       </c>
       <c r="M3" s="8"/>
       <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="31" x14ac:dyDescent="0.35">
-      <c r="A4" s="113"/>
+      <c r="A4" s="105"/>
       <c r="B4" s="12" t="s">
         <v>38</v>
       </c>
@@ -5041,8 +4834,8 @@
       <c r="J4" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="K4" s="113"/>
-      <c r="L4" s="113"/>
+      <c r="K4" s="105"/>
+      <c r="L4" s="105"/>
       <c r="M4" s="10"/>
       <c r="N4" s="11"/>
     </row>

</xml_diff>

<commit_message>
Auto pipeline update 2026-04-23 16:09:18
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{838680F7-B0E9-487F-B0FE-307E9A22D9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A188424-14F4-4829-B899-78D14BFFE9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="899" firstSheet="2" activeTab="4" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="899" xr2:uid="{2458F121-AB3E-4F80-952F-EEA9DC2A69DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet Names Check" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="202">
   <si>
     <t>Project Code</t>
   </si>
@@ -765,6 +765,7 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1600,6 +1601,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1611,6 +1627,18 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1665,33 +1693,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -1705,7 +1706,27 @@
     <cellStyle name="Normal 6" xfId="8" xr:uid="{E2AC1BB0-A24A-450A-B605-14A01490AC0E}"/>
     <cellStyle name="Normal 8 2" xfId="2" xr:uid="{E356B690-246D-43B2-86AF-A6FE97B16461}"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="11">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2197,6 +2218,7 @@
     <col min="3" max="3" width="27.453125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -2294,6 +2316,12 @@
       </c>
       <c r="C8" t="s">
         <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -2470,46 +2498,46 @@
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A3" s="111" t="s">
+      <c r="A3" s="120" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="111" t="s">
+      <c r="B3" s="120" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="111"/>
-      <c r="D3" s="111" t="s">
+      <c r="C3" s="120"/>
+      <c r="D3" s="120" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="111" t="s">
+      <c r="E3" s="120" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="111" t="s">
+      <c r="F3" s="120" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="112" t="s">
+      <c r="G3" s="121" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="112"/>
-      <c r="I3" s="112"/>
-      <c r="J3" s="108" t="s">
+      <c r="H3" s="121"/>
+      <c r="I3" s="121"/>
+      <c r="J3" s="117" t="s">
         <v>37</v>
       </c>
-      <c r="K3" s="109"/>
-      <c r="L3" s="109"/>
-      <c r="M3" s="109"/>
-      <c r="N3" s="110"/>
+      <c r="K3" s="118"/>
+      <c r="L3" s="118"/>
+      <c r="M3" s="118"/>
+      <c r="N3" s="119"/>
     </row>
     <row r="4" spans="1:23" ht="26" x14ac:dyDescent="0.35">
-      <c r="A4" s="111"/>
+      <c r="A4" s="120"/>
       <c r="B4" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="111"/>
-      <c r="E4" s="111"/>
-      <c r="F4" s="111"/>
+      <c r="D4" s="120"/>
+      <c r="E4" s="120"/>
+      <c r="F4" s="120"/>
       <c r="G4" s="1" t="s">
         <v>35</v>
       </c>
@@ -2597,10 +2625,10 @@
     <mergeCell ref="G3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C7">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2643,14 +2671,14 @@
       <c r="C3" s="7"/>
       <c r="D3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="113"/>
-      <c r="H3" s="114"/>
-      <c r="I3" s="114"/>
-      <c r="J3" s="115"/>
+      <c r="G3" s="122"/>
+      <c r="H3" s="123"/>
+      <c r="I3" s="123"/>
+      <c r="J3" s="124"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="113"/>
-      <c r="O3" s="114"/>
-      <c r="P3" s="115"/>
+      <c r="N3" s="122"/>
+      <c r="O3" s="123"/>
+      <c r="P3" s="124"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -2732,14 +2760,14 @@
       <c r="C3" s="7"/>
       <c r="D3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="113"/>
-      <c r="H3" s="114"/>
-      <c r="I3" s="114"/>
-      <c r="J3" s="115"/>
+      <c r="G3" s="122"/>
+      <c r="H3" s="123"/>
+      <c r="I3" s="123"/>
+      <c r="J3" s="124"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="113"/>
-      <c r="O3" s="114"/>
-      <c r="P3" s="115"/>
+      <c r="N3" s="122"/>
+      <c r="O3" s="123"/>
+      <c r="P3" s="124"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -2866,13 +2894,16 @@
       <c r="G5" s="6" t="s">
         <v>34</v>
       </c>
+      <c r="H5" s="14" t="s">
+        <v>81</v>
+      </c>
       <c r="K5" s="7" t="s">
         <v>54</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2">
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3427,10 +3458,10 @@
       <c r="A3" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="92" t="s">
+      <c r="B3" s="97" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="93"/>
+      <c r="C3" s="98"/>
       <c r="D3" s="18" t="s">
         <v>90</v>
       </c>
@@ -3440,16 +3471,16 @@
       <c r="F3" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="G3" s="94" t="s">
+      <c r="G3" s="99" t="s">
         <v>93</v>
       </c>
-      <c r="H3" s="95"/>
-      <c r="I3" s="93"/>
-      <c r="J3" s="94" t="s">
+      <c r="H3" s="100"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="99" t="s">
         <v>37</v>
       </c>
-      <c r="K3" s="95"/>
-      <c r="L3" s="93"/>
+      <c r="K3" s="100"/>
+      <c r="L3" s="98"/>
       <c r="M3" s="21" t="s">
         <v>94</v>
       </c>
@@ -3466,16 +3497,16 @@
         <v>42</v>
       </c>
       <c r="R3" s="26"/>
-      <c r="S3" s="96" t="s">
+      <c r="S3" s="101" t="s">
         <v>99</v>
       </c>
-      <c r="T3" s="95"/>
-      <c r="U3" s="93"/>
-      <c r="V3" s="96" t="s">
+      <c r="T3" s="100"/>
+      <c r="U3" s="98"/>
+      <c r="V3" s="101" t="s">
         <v>100</v>
       </c>
-      <c r="W3" s="95"/>
-      <c r="X3" s="93"/>
+      <c r="W3" s="100"/>
+      <c r="X3" s="98"/>
       <c r="Y3" s="24" t="s">
         <v>97</v>
       </c>
@@ -3627,10 +3658,10 @@
     <mergeCell ref="V3:X3"/>
   </mergeCells>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C7">
-    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3647,126 +3678,126 @@
       </c>
     </row>
     <row r="3" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="116" t="s">
+      <c r="A3" s="92" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="117" t="s">
+      <c r="B3" s="102" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="118"/>
-      <c r="D3" s="116" t="s">
+      <c r="C3" s="103"/>
+      <c r="D3" s="92" t="s">
         <v>90</v>
       </c>
-      <c r="E3" s="116" t="s">
+      <c r="E3" s="92" t="s">
         <v>91</v>
       </c>
-      <c r="F3" s="119" t="s">
+      <c r="F3" s="94" t="s">
         <v>92</v>
       </c>
-      <c r="G3" s="120" t="s">
+      <c r="G3" s="104" t="s">
         <v>93</v>
       </c>
-      <c r="H3" s="118"/>
-      <c r="I3" s="118"/>
-      <c r="J3" s="120" t="s">
+      <c r="H3" s="103"/>
+      <c r="I3" s="103"/>
+      <c r="J3" s="104" t="s">
         <v>37</v>
       </c>
-      <c r="K3" s="118"/>
-      <c r="L3" s="118"/>
-      <c r="M3" s="119" t="s">
+      <c r="K3" s="103"/>
+      <c r="L3" s="103"/>
+      <c r="M3" s="94" t="s">
         <v>94</v>
       </c>
-      <c r="N3" s="119" t="s">
+      <c r="N3" s="94" t="s">
         <v>95</v>
       </c>
-      <c r="O3" s="121" t="s">
+      <c r="O3" s="95" t="s">
         <v>96</v>
       </c>
-      <c r="P3" s="119" t="s">
+      <c r="P3" s="94" t="s">
         <v>97</v>
       </c>
-      <c r="Q3" s="119" t="s">
+      <c r="Q3" s="94" t="s">
         <v>98</v>
       </c>
-      <c r="R3" s="119" t="s">
+      <c r="R3" s="94" t="s">
         <v>42</v>
       </c>
-      <c r="S3" s="122"/>
-      <c r="T3" s="123" t="s">
+      <c r="S3" s="96"/>
+      <c r="T3" s="105" t="s">
         <v>99</v>
       </c>
-      <c r="U3" s="118"/>
-      <c r="V3" s="118"/>
-      <c r="W3" s="123" t="s">
+      <c r="U3" s="103"/>
+      <c r="V3" s="103"/>
+      <c r="W3" s="105" t="s">
         <v>100</v>
       </c>
-      <c r="X3" s="118"/>
-      <c r="Y3" s="118"/>
-      <c r="Z3" s="119" t="s">
+      <c r="X3" s="103"/>
+      <c r="Y3" s="103"/>
+      <c r="Z3" s="94" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A4" s="116"/>
-      <c r="B4" s="124" t="s">
+      <c r="A4" s="92"/>
+      <c r="B4" s="93" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="124" t="s">
+      <c r="C4" s="93" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="116"/>
-      <c r="E4" s="116"/>
-      <c r="F4" s="119"/>
-      <c r="G4" s="121" t="s">
+      <c r="D4" s="92"/>
+      <c r="E4" s="92"/>
+      <c r="F4" s="94"/>
+      <c r="G4" s="95" t="s">
         <v>54</v>
       </c>
-      <c r="H4" s="121" t="s">
+      <c r="H4" s="95" t="s">
         <v>101</v>
       </c>
-      <c r="I4" s="121" t="s">
+      <c r="I4" s="95" t="s">
         <v>102</v>
       </c>
-      <c r="J4" s="121" t="s">
+      <c r="J4" s="95" t="s">
         <v>54</v>
       </c>
-      <c r="K4" s="121" t="s">
+      <c r="K4" s="95" t="s">
         <v>101</v>
       </c>
-      <c r="L4" s="121" t="s">
+      <c r="L4" s="95" t="s">
         <v>102</v>
       </c>
-      <c r="M4" s="121" t="s">
+      <c r="M4" s="95" t="s">
         <v>54</v>
       </c>
-      <c r="N4" s="121" t="s">
+      <c r="N4" s="95" t="s">
         <v>54</v>
       </c>
-      <c r="O4" s="121" t="s">
+      <c r="O4" s="95" t="s">
         <v>54</v>
       </c>
-      <c r="P4" s="119"/>
-      <c r="Q4" s="119"/>
-      <c r="R4" s="119"/>
-      <c r="S4" s="122"/>
-      <c r="T4" s="121" t="s">
+      <c r="P4" s="94"/>
+      <c r="Q4" s="94"/>
+      <c r="R4" s="94"/>
+      <c r="S4" s="96"/>
+      <c r="T4" s="95" t="s">
         <v>54</v>
       </c>
-      <c r="U4" s="121" t="s">
+      <c r="U4" s="95" t="s">
         <v>101</v>
       </c>
-      <c r="V4" s="121" t="s">
+      <c r="V4" s="95" t="s">
         <v>102</v>
       </c>
-      <c r="W4" s="121" t="s">
+      <c r="W4" s="95" t="s">
         <v>54</v>
       </c>
-      <c r="X4" s="121" t="s">
+      <c r="X4" s="95" t="s">
         <v>101</v>
       </c>
-      <c r="Y4" s="121" t="s">
+      <c r="Y4" s="95" t="s">
         <v>102</v>
       </c>
-      <c r="Z4" s="119"/>
+      <c r="Z4" s="94"/>
     </row>
     <row r="7" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
@@ -3840,10 +3871,10 @@
     <mergeCell ref="W3:Y3"/>
   </mergeCells>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C8">
-    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3855,59 +3886,59 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:65" x14ac:dyDescent="0.35">
-      <c r="A1" s="96"/>
-      <c r="B1" s="97"/>
-      <c r="C1" s="97"/>
-      <c r="D1" s="97"/>
-      <c r="E1" s="97"/>
-      <c r="F1" s="97"/>
-      <c r="G1" s="97"/>
-      <c r="H1" s="97"/>
-      <c r="I1" s="97"/>
-      <c r="J1" s="97"/>
-      <c r="K1" s="97"/>
-      <c r="L1" s="97"/>
-      <c r="M1" s="97"/>
-      <c r="N1" s="97"/>
-      <c r="O1" s="97"/>
-      <c r="P1" s="97"/>
-      <c r="Q1" s="97"/>
-      <c r="R1" s="97"/>
-      <c r="S1" s="97"/>
-      <c r="T1" s="97"/>
-      <c r="U1" s="97"/>
-      <c r="V1" s="97"/>
-      <c r="W1" s="97"/>
-      <c r="X1" s="97"/>
-      <c r="Y1" s="97"/>
-      <c r="Z1" s="97"/>
-      <c r="AA1" s="97"/>
-      <c r="AB1" s="97"/>
-      <c r="AC1" s="97"/>
-      <c r="AD1" s="97"/>
-      <c r="AE1" s="97"/>
-      <c r="AF1" s="97"/>
-      <c r="AG1" s="97"/>
-      <c r="AH1" s="97"/>
-      <c r="AI1" s="97"/>
-      <c r="AJ1" s="97"/>
-      <c r="AK1" s="97"/>
-      <c r="AL1" s="95"/>
-      <c r="AM1" s="95"/>
-      <c r="AN1" s="95"/>
-      <c r="AO1" s="95"/>
-      <c r="AP1" s="95"/>
-      <c r="AQ1" s="97"/>
-      <c r="AR1" s="97"/>
-      <c r="AS1" s="97"/>
-      <c r="AT1" s="97"/>
-      <c r="AU1" s="97"/>
-      <c r="AV1" s="97"/>
-      <c r="AW1" s="97"/>
-      <c r="AX1" s="97"/>
-      <c r="AY1" s="97"/>
-      <c r="AZ1" s="97"/>
-      <c r="BA1" s="98"/>
+      <c r="A1" s="101"/>
+      <c r="B1" s="106"/>
+      <c r="C1" s="106"/>
+      <c r="D1" s="106"/>
+      <c r="E1" s="106"/>
+      <c r="F1" s="106"/>
+      <c r="G1" s="106"/>
+      <c r="H1" s="106"/>
+      <c r="I1" s="106"/>
+      <c r="J1" s="106"/>
+      <c r="K1" s="106"/>
+      <c r="L1" s="106"/>
+      <c r="M1" s="106"/>
+      <c r="N1" s="106"/>
+      <c r="O1" s="106"/>
+      <c r="P1" s="106"/>
+      <c r="Q1" s="106"/>
+      <c r="R1" s="106"/>
+      <c r="S1" s="106"/>
+      <c r="T1" s="106"/>
+      <c r="U1" s="106"/>
+      <c r="V1" s="106"/>
+      <c r="W1" s="106"/>
+      <c r="X1" s="106"/>
+      <c r="Y1" s="106"/>
+      <c r="Z1" s="106"/>
+      <c r="AA1" s="106"/>
+      <c r="AB1" s="106"/>
+      <c r="AC1" s="106"/>
+      <c r="AD1" s="106"/>
+      <c r="AE1" s="106"/>
+      <c r="AF1" s="106"/>
+      <c r="AG1" s="106"/>
+      <c r="AH1" s="106"/>
+      <c r="AI1" s="106"/>
+      <c r="AJ1" s="106"/>
+      <c r="AK1" s="106"/>
+      <c r="AL1" s="100"/>
+      <c r="AM1" s="100"/>
+      <c r="AN1" s="100"/>
+      <c r="AO1" s="100"/>
+      <c r="AP1" s="100"/>
+      <c r="AQ1" s="106"/>
+      <c r="AR1" s="106"/>
+      <c r="AS1" s="106"/>
+      <c r="AT1" s="106"/>
+      <c r="AU1" s="106"/>
+      <c r="AV1" s="106"/>
+      <c r="AW1" s="106"/>
+      <c r="AX1" s="106"/>
+      <c r="AY1" s="106"/>
+      <c r="AZ1" s="106"/>
+      <c r="BA1" s="107"/>
     </row>
     <row r="2" spans="1:65" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -4304,186 +4335,186 @@
       </c>
     </row>
     <row r="3" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A3" s="96" t="str">
+      <c r="A3" s="101" t="str">
         <f>+[1]Summary!A4</f>
         <v>Office:  Neemuch</v>
       </c>
-      <c r="B3" s="97"/>
-      <c r="C3" s="97"/>
-      <c r="D3" s="97"/>
-      <c r="E3" s="97"/>
-      <c r="F3" s="97"/>
-      <c r="G3" s="97"/>
-      <c r="H3" s="97"/>
-      <c r="I3" s="97"/>
-      <c r="J3" s="97"/>
-      <c r="K3" s="97"/>
-      <c r="L3" s="97"/>
-      <c r="M3" s="97"/>
-      <c r="N3" s="97"/>
-      <c r="O3" s="97"/>
-      <c r="P3" s="97"/>
-      <c r="Q3" s="97"/>
-      <c r="R3" s="97"/>
-      <c r="S3" s="97"/>
-      <c r="T3" s="97"/>
-      <c r="U3" s="97"/>
-      <c r="V3" s="97"/>
-      <c r="W3" s="97"/>
-      <c r="X3" s="97"/>
-      <c r="Y3" s="97"/>
-      <c r="Z3" s="97"/>
-      <c r="AA3" s="97"/>
-      <c r="AB3" s="97"/>
-      <c r="AC3" s="97"/>
-      <c r="AD3" s="97"/>
-      <c r="AE3" s="97"/>
-      <c r="AF3" s="97"/>
-      <c r="AG3" s="97"/>
-      <c r="AH3" s="97"/>
-      <c r="AI3" s="97"/>
-      <c r="AJ3" s="97"/>
-      <c r="AK3" s="97"/>
-      <c r="AL3" s="95"/>
-      <c r="AM3" s="95"/>
-      <c r="AN3" s="95"/>
-      <c r="AO3" s="95"/>
-      <c r="AP3" s="95"/>
-      <c r="AQ3" s="97"/>
-      <c r="AR3" s="97"/>
-      <c r="AS3" s="97"/>
-      <c r="AT3" s="97"/>
-      <c r="AU3" s="97"/>
-      <c r="AV3" s="97"/>
-      <c r="AW3" s="97"/>
-      <c r="AX3" s="97"/>
-      <c r="AY3" s="97"/>
-      <c r="AZ3" s="97"/>
-      <c r="BA3" s="98"/>
+      <c r="B3" s="106"/>
+      <c r="C3" s="106"/>
+      <c r="D3" s="106"/>
+      <c r="E3" s="106"/>
+      <c r="F3" s="106"/>
+      <c r="G3" s="106"/>
+      <c r="H3" s="106"/>
+      <c r="I3" s="106"/>
+      <c r="J3" s="106"/>
+      <c r="K3" s="106"/>
+      <c r="L3" s="106"/>
+      <c r="M3" s="106"/>
+      <c r="N3" s="106"/>
+      <c r="O3" s="106"/>
+      <c r="P3" s="106"/>
+      <c r="Q3" s="106"/>
+      <c r="R3" s="106"/>
+      <c r="S3" s="106"/>
+      <c r="T3" s="106"/>
+      <c r="U3" s="106"/>
+      <c r="V3" s="106"/>
+      <c r="W3" s="106"/>
+      <c r="X3" s="106"/>
+      <c r="Y3" s="106"/>
+      <c r="Z3" s="106"/>
+      <c r="AA3" s="106"/>
+      <c r="AB3" s="106"/>
+      <c r="AC3" s="106"/>
+      <c r="AD3" s="106"/>
+      <c r="AE3" s="106"/>
+      <c r="AF3" s="106"/>
+      <c r="AG3" s="106"/>
+      <c r="AH3" s="106"/>
+      <c r="AI3" s="106"/>
+      <c r="AJ3" s="106"/>
+      <c r="AK3" s="106"/>
+      <c r="AL3" s="100"/>
+      <c r="AM3" s="100"/>
+      <c r="AN3" s="100"/>
+      <c r="AO3" s="100"/>
+      <c r="AP3" s="100"/>
+      <c r="AQ3" s="106"/>
+      <c r="AR3" s="106"/>
+      <c r="AS3" s="106"/>
+      <c r="AT3" s="106"/>
+      <c r="AU3" s="106"/>
+      <c r="AV3" s="106"/>
+      <c r="AW3" s="106"/>
+      <c r="AX3" s="106"/>
+      <c r="AY3" s="106"/>
+      <c r="AZ3" s="106"/>
+      <c r="BA3" s="107"/>
     </row>
     <row r="4" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A4" s="96">
+      <c r="A4" s="101">
         <f>+[1]Summary!A7</f>
         <v>0</v>
       </c>
-      <c r="B4" s="97"/>
-      <c r="C4" s="97"/>
-      <c r="D4" s="97"/>
-      <c r="E4" s="97"/>
-      <c r="F4" s="97"/>
-      <c r="G4" s="97"/>
-      <c r="H4" s="97"/>
-      <c r="I4" s="97"/>
-      <c r="J4" s="97"/>
-      <c r="K4" s="97"/>
-      <c r="L4" s="97"/>
-      <c r="M4" s="97"/>
-      <c r="N4" s="97"/>
-      <c r="O4" s="97"/>
-      <c r="P4" s="97"/>
-      <c r="Q4" s="97"/>
-      <c r="R4" s="97"/>
-      <c r="S4" s="97"/>
-      <c r="T4" s="97"/>
-      <c r="U4" s="97"/>
-      <c r="V4" s="97"/>
-      <c r="W4" s="97"/>
-      <c r="X4" s="97"/>
-      <c r="Y4" s="97"/>
-      <c r="Z4" s="97"/>
-      <c r="AA4" s="97"/>
-      <c r="AB4" s="97"/>
-      <c r="AC4" s="97"/>
-      <c r="AD4" s="97"/>
-      <c r="AE4" s="97"/>
-      <c r="AF4" s="97"/>
-      <c r="AG4" s="97"/>
-      <c r="AH4" s="97"/>
-      <c r="AI4" s="97"/>
-      <c r="AJ4" s="97"/>
-      <c r="AK4" s="97"/>
-      <c r="AL4" s="95"/>
-      <c r="AM4" s="95"/>
-      <c r="AN4" s="95"/>
-      <c r="AO4" s="95"/>
-      <c r="AP4" s="95"/>
-      <c r="AQ4" s="97"/>
-      <c r="AR4" s="97"/>
-      <c r="AS4" s="97"/>
-      <c r="AT4" s="97"/>
-      <c r="AU4" s="97"/>
-      <c r="AV4" s="97"/>
-      <c r="AW4" s="97"/>
-      <c r="AX4" s="97"/>
-      <c r="AY4" s="97"/>
-      <c r="AZ4" s="97"/>
-      <c r="BA4" s="98"/>
+      <c r="B4" s="106"/>
+      <c r="C4" s="106"/>
+      <c r="D4" s="106"/>
+      <c r="E4" s="106"/>
+      <c r="F4" s="106"/>
+      <c r="G4" s="106"/>
+      <c r="H4" s="106"/>
+      <c r="I4" s="106"/>
+      <c r="J4" s="106"/>
+      <c r="K4" s="106"/>
+      <c r="L4" s="106"/>
+      <c r="M4" s="106"/>
+      <c r="N4" s="106"/>
+      <c r="O4" s="106"/>
+      <c r="P4" s="106"/>
+      <c r="Q4" s="106"/>
+      <c r="R4" s="106"/>
+      <c r="S4" s="106"/>
+      <c r="T4" s="106"/>
+      <c r="U4" s="106"/>
+      <c r="V4" s="106"/>
+      <c r="W4" s="106"/>
+      <c r="X4" s="106"/>
+      <c r="Y4" s="106"/>
+      <c r="Z4" s="106"/>
+      <c r="AA4" s="106"/>
+      <c r="AB4" s="106"/>
+      <c r="AC4" s="106"/>
+      <c r="AD4" s="106"/>
+      <c r="AE4" s="106"/>
+      <c r="AF4" s="106"/>
+      <c r="AG4" s="106"/>
+      <c r="AH4" s="106"/>
+      <c r="AI4" s="106"/>
+      <c r="AJ4" s="106"/>
+      <c r="AK4" s="106"/>
+      <c r="AL4" s="100"/>
+      <c r="AM4" s="100"/>
+      <c r="AN4" s="100"/>
+      <c r="AO4" s="100"/>
+      <c r="AP4" s="100"/>
+      <c r="AQ4" s="106"/>
+      <c r="AR4" s="106"/>
+      <c r="AS4" s="106"/>
+      <c r="AT4" s="106"/>
+      <c r="AU4" s="106"/>
+      <c r="AV4" s="106"/>
+      <c r="AW4" s="106"/>
+      <c r="AX4" s="106"/>
+      <c r="AY4" s="106"/>
+      <c r="AZ4" s="106"/>
+      <c r="BA4" s="107"/>
     </row>
     <row r="5" spans="1:53" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="96" t="s">
+      <c r="A5" s="101" t="s">
         <v>110</v>
       </c>
-      <c r="B5" s="97"/>
-      <c r="C5" s="97"/>
-      <c r="D5" s="97"/>
-      <c r="E5" s="97"/>
-      <c r="F5" s="97"/>
-      <c r="G5" s="97"/>
-      <c r="H5" s="97"/>
-      <c r="I5" s="97"/>
-      <c r="J5" s="97"/>
-      <c r="K5" s="97"/>
-      <c r="L5" s="97"/>
-      <c r="M5" s="97"/>
-      <c r="N5" s="97"/>
-      <c r="O5" s="97"/>
-      <c r="P5" s="97"/>
-      <c r="Q5" s="97"/>
-      <c r="R5" s="97"/>
-      <c r="S5" s="98"/>
-      <c r="T5" s="96" t="s">
+      <c r="B5" s="106"/>
+      <c r="C5" s="106"/>
+      <c r="D5" s="106"/>
+      <c r="E5" s="106"/>
+      <c r="F5" s="106"/>
+      <c r="G5" s="106"/>
+      <c r="H5" s="106"/>
+      <c r="I5" s="106"/>
+      <c r="J5" s="106"/>
+      <c r="K5" s="106"/>
+      <c r="L5" s="106"/>
+      <c r="M5" s="106"/>
+      <c r="N5" s="106"/>
+      <c r="O5" s="106"/>
+      <c r="P5" s="106"/>
+      <c r="Q5" s="106"/>
+      <c r="R5" s="106"/>
+      <c r="S5" s="107"/>
+      <c r="T5" s="101" t="s">
         <v>111</v>
       </c>
-      <c r="U5" s="97"/>
-      <c r="V5" s="97"/>
-      <c r="W5" s="97"/>
-      <c r="X5" s="97"/>
-      <c r="Y5" s="97"/>
-      <c r="Z5" s="97"/>
-      <c r="AA5" s="97"/>
-      <c r="AB5" s="97"/>
-      <c r="AC5" s="97"/>
-      <c r="AD5" s="97"/>
-      <c r="AE5" s="97"/>
-      <c r="AF5" s="97"/>
-      <c r="AG5" s="97"/>
-      <c r="AH5" s="97"/>
-      <c r="AI5" s="97"/>
-      <c r="AJ5" s="97"/>
-      <c r="AK5" s="98"/>
-      <c r="AL5" s="96" t="s">
+      <c r="U5" s="106"/>
+      <c r="V5" s="106"/>
+      <c r="W5" s="106"/>
+      <c r="X5" s="106"/>
+      <c r="Y5" s="106"/>
+      <c r="Z5" s="106"/>
+      <c r="AA5" s="106"/>
+      <c r="AB5" s="106"/>
+      <c r="AC5" s="106"/>
+      <c r="AD5" s="106"/>
+      <c r="AE5" s="106"/>
+      <c r="AF5" s="106"/>
+      <c r="AG5" s="106"/>
+      <c r="AH5" s="106"/>
+      <c r="AI5" s="106"/>
+      <c r="AJ5" s="106"/>
+      <c r="AK5" s="107"/>
+      <c r="AL5" s="101" t="s">
         <v>112</v>
       </c>
-      <c r="AM5" s="95"/>
-      <c r="AN5" s="95"/>
-      <c r="AO5" s="95"/>
-      <c r="AP5" s="93"/>
-      <c r="AQ5" s="96" t="s">
+      <c r="AM5" s="100"/>
+      <c r="AN5" s="100"/>
+      <c r="AO5" s="100"/>
+      <c r="AP5" s="98"/>
+      <c r="AQ5" s="101" t="s">
         <v>2</v>
       </c>
-      <c r="AR5" s="97"/>
-      <c r="AS5" s="97"/>
-      <c r="AT5" s="98"/>
+      <c r="AR5" s="106"/>
+      <c r="AS5" s="106"/>
+      <c r="AT5" s="107"/>
       <c r="AU5" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="AV5" s="96" t="s">
+      <c r="AV5" s="101" t="s">
         <v>114</v>
       </c>
-      <c r="AW5" s="97"/>
-      <c r="AX5" s="97"/>
-      <c r="AY5" s="97"/>
-      <c r="AZ5" s="98"/>
+      <c r="AW5" s="106"/>
+      <c r="AX5" s="106"/>
+      <c r="AY5" s="106"/>
+      <c r="AZ5" s="107"/>
       <c r="BA5" s="20" t="s">
         <v>115</v>
       </c>
@@ -4501,24 +4532,24 @@
       <c r="D6" s="43"/>
       <c r="E6" s="43"/>
       <c r="F6" s="43"/>
-      <c r="G6" s="99" t="s">
+      <c r="G6" s="108" t="s">
         <v>81</v>
       </c>
-      <c r="H6" s="100"/>
-      <c r="I6" s="100"/>
-      <c r="J6" s="101"/>
-      <c r="K6" s="99" t="s">
+      <c r="H6" s="109"/>
+      <c r="I6" s="109"/>
+      <c r="J6" s="110"/>
+      <c r="K6" s="108" t="s">
         <v>117</v>
       </c>
-      <c r="L6" s="100"/>
-      <c r="M6" s="100"/>
-      <c r="N6" s="101"/>
-      <c r="O6" s="102" t="s">
+      <c r="L6" s="109"/>
+      <c r="M6" s="109"/>
+      <c r="N6" s="110"/>
+      <c r="O6" s="111" t="s">
         <v>118</v>
       </c>
-      <c r="P6" s="97"/>
-      <c r="Q6" s="97"/>
-      <c r="R6" s="98"/>
+      <c r="P6" s="106"/>
+      <c r="Q6" s="106"/>
+      <c r="R6" s="107"/>
       <c r="S6" s="44" t="s">
         <v>119</v>
       </c>
@@ -4528,11 +4559,11 @@
       <c r="U6" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="V6" s="96" t="s">
+      <c r="V6" s="101" t="s">
         <v>121</v>
       </c>
-      <c r="W6" s="97"/>
-      <c r="X6" s="98"/>
+      <c r="W6" s="106"/>
+      <c r="X6" s="107"/>
       <c r="Y6" s="45" t="s">
         <v>122</v>
       </c>
@@ -4557,14 +4588,14 @@
       <c r="AF6" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="AG6" s="103" t="s">
+      <c r="AG6" s="112" t="s">
         <v>130</v>
       </c>
-      <c r="AH6" s="98"/>
-      <c r="AI6" s="96" t="s">
+      <c r="AH6" s="107"/>
+      <c r="AI6" s="101" t="s">
         <v>131</v>
       </c>
-      <c r="AJ6" s="98"/>
+      <c r="AJ6" s="107"/>
       <c r="AK6" s="20" t="s">
         <v>97</v>
       </c>
@@ -4749,6 +4780,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="AI6:AJ6"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="O6:R6"/>
+    <mergeCell ref="V6:X6"/>
+    <mergeCell ref="AG6:AH6"/>
     <mergeCell ref="A3:BA3"/>
     <mergeCell ref="A4:BA4"/>
     <mergeCell ref="A5:S5"/>
@@ -4756,12 +4793,6 @@
     <mergeCell ref="AL5:AP5"/>
     <mergeCell ref="AQ5:AT5"/>
     <mergeCell ref="AV5:AZ5"/>
-    <mergeCell ref="AI6:AJ6"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="K6:N6"/>
-    <mergeCell ref="O6:R6"/>
-    <mergeCell ref="V6:X6"/>
-    <mergeCell ref="AG6:AH6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4778,35 +4809,35 @@
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="106" t="s">
+      <c r="A3" s="115" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="107" t="s">
+      <c r="B3" s="116" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="95"/>
-      <c r="D3" s="93"/>
-      <c r="E3" s="107" t="s">
+      <c r="C3" s="100"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="116" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="95"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="107" t="s">
+      <c r="F3" s="100"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="116" t="s">
         <v>37</v>
       </c>
-      <c r="I3" s="95"/>
-      <c r="J3" s="93"/>
-      <c r="K3" s="106" t="s">
+      <c r="I3" s="100"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="115" t="s">
         <v>74</v>
       </c>
-      <c r="L3" s="104" t="s">
+      <c r="L3" s="113" t="s">
         <v>42</v>
       </c>
       <c r="M3" s="8"/>
       <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="31" x14ac:dyDescent="0.35">
-      <c r="A4" s="105"/>
+      <c r="A4" s="114"/>
       <c r="B4" s="12" t="s">
         <v>38</v>
       </c>
@@ -4834,8 +4865,8 @@
       <c r="J4" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="K4" s="105"/>
-      <c r="L4" s="105"/>
+      <c r="K4" s="114"/>
+      <c r="L4" s="114"/>
       <c r="M4" s="10"/>
       <c r="N4" s="11"/>
     </row>
@@ -4894,10 +4925,10 @@
     <mergeCell ref="K3:K4"/>
   </mergeCells>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C7">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add foundation ingest pipeline and weekly export coverage
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -1,67 +1,81 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="899" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet Names Check" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TA 608 Erection" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="TA 602 Erection" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="TA 513 Ere S-P Erection" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TA 513 Ere S-F Erection" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TA 413 Erection" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="TA 413 Stringing" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="TA 601 Stringing" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="TB 501 220kV Stringing" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="TB 501 132kV Stringing" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="TB 501 220kV Erection" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="TB 501 132kV Erection" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="TB 401 Stringing" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="TB 408 Stringing" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="TA 509 Erection" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="TA 601 Erection" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="TB 408 Status" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="TA 413 Status" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="TA 414 Status" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="TA 416 Status" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="TA 418 Status" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="TA 421 Status" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="TA 419 Status" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="TA 504 Status" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="TA 505 Status" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="TA 506 Status" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="TB 507 400kV Status" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="TB 507 765kV Status" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="TB 501 Status" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="TA 413 Stretch" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="TA 418 Stretch" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="TA 419 Stretch" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="TA 421 Stretch" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="TA 504 Stretch" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="TA 505 Stretch" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="TA 506 Stretch" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="TB 507 Stretch" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="TB 605 Status" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="TA 512 Status" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="TA 601 Status" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="TB 401 Status" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="TA 325 Status" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="TA 509 Status" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="TA 310 Status" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="TA 513 Status" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="TA 601 Stretch" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="TA 512 Stretch" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="TB 401 Stretch" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="TB 408 Stretch" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="TA 421 Tack Welding Stretch" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="TA 602 Status" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="TA 608 Status" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet name="TA 510 Status" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet Names Check" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 608 Erection" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Erection" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 513 Ere S-P Erection" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 513 Ere S-F Erection" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Erection" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Stringing" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Stringing" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 220kV Stringing" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 132kV Stringing" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 220kV Erection" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 132kV Erection" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 401 Stringing" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 408 Stringing" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 509 Erection" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Erection" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 408 Status" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Status" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 414 Status" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 416 Status" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 418 Status" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 421 Status" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 419 Status" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 504 Status" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 505 Status" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 506 Status" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 400kV Status" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 765kV Status" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 Status" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Stretch" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 418 Stretch" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 419 Stretch" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 421 Stretch" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 504 Stretch" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 505 Stretch" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 506 Stretch" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 Stretch" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 Status" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 512 Status" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Status" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 401 Status" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 325 Status" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 509 Status" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 310 Status" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 513 Status" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Stretch" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 512 Stretch" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 401 Stretch" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 408 Stretch" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 421 Tack Welding Stretch" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Status" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 608 Status" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 510 Status" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Foundation" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 509 Foundation" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 132kV Foundation" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 220kV Foundation" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Foundation" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 Jammu Foundation" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 LILO Foundation" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 Punjab Foundation" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 505 Foundation" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 512 Foundation" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Foundation" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 608 Foundation" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 MAIN Foundation" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 765kV Foundation" sheetId="67" state="visible" r:id="rId67"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId54"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId68"/>
   </externalReferences>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1917,8 +1931,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook r:id="rId1">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Detail Survey-220kV"/>
       <sheetName val="Check Survey-220kV"/>
@@ -2297,7 +2311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:T25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="10.453125" customWidth="1" min="1" max="1"/>
@@ -2392,15 +2406,20 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>Foundation Template Check</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>Foundation Line Names</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Consolidation Rule</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Status File Identifier</t>
         </is>
@@ -2439,10 +2458,15 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Foundation JS-Line -Jammu; Foundation -LILO; Foundation -JS Line- Punjab</t>
+          <t>Foundation JS-Line -Jammu; LILO; Foundation -JS Line- Punjab</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>Jammu; LILO; Punjab</t>
         </is>
@@ -2642,22 +2666,27 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Foundation</t>
+          <t>Foundation; Foundation</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
           <t>MAIN; 765kV</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>split</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>[MAIN];</t>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>[MAIN] - DPR -; TB 507 - DPR -</t>
         </is>
       </c>
     </row>
@@ -2702,6 +2731,11 @@
           <t>Foundation</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2764,6 +2798,11 @@
           <t>Foundation</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3004,6 +3043,11 @@
           <t>Foundation</t>
         </is>
       </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3207,6 +3251,11 @@
           <t>FOUNDATION</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3269,6 +3318,11 @@
           <t>Progress Sheet</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3338,10 +3392,15 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
           <t>132kV; 220kV</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>split</t>
         </is>
@@ -3405,6 +3464,16 @@
           <t>Unknown</t>
         </is>
       </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>FDN S-P; FDN S-F</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>S-P; S-F</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3437,6 +3506,11 @@
           <t>FDN</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3469,6 +3543,11 @@
           <t>WIP-FDN</t>
         </is>
       </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3489,6 +3568,43 @@
       <c r="I24" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>FDN; Pile Foundation</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>FDN; Pile</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TA 515</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Erection Compiled</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>DPR</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>DPR</t>
         </is>
       </c>
     </row>
@@ -6644,11 +6760,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -7078,10 +7189,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -7629,10 +7736,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -8930,12 +9033,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -10581,12 +10678,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -10658,52 +10749,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
@@ -10780,12 +10825,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -10931,12 +10970,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -11005,6 +11038,244 @@
       <c r="M14" t="inlineStr">
         <is>
           <t>remarks</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Location No</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Foundation Completion Date</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Foundation Status</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Location No</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Foundation Status</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Foundation Completion Date</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AS2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Location No</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Foundation Status</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Foundation Completion Date</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>Foundation Completion Date Backup</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:BF2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Location No</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>Foundation Status</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>Foundation Completion Date</t>
+        </is>
+      </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>Foundation Completion Date Backup</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Location No</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Foundation Status</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Foundation Completion Date</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Location No</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Foundation Completion Date</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Foundation Status</t>
         </is>
       </c>
     </row>
@@ -11154,6 +11425,310 @@
     <cfRule type="duplicateValues" priority="1" dxfId="0"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Location No</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Foundation Completion Date</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Foundation Status</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Location No</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Foundation Completion Date</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Foundation Status</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Location No</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Foundation Starting Date</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Foundation Completion Date</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Loc. No.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Loc. No.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LOC. NO.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Completion Date</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Location Number</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Foundation Starting Date</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Foundation Completion Date</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Location Number</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Foundation Starting Date</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Foundation Completion Date</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Auto pipeline update 2026-06-10 10:45:20
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="899" firstSheet="61" activeTab="66" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="899" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet Names Check" sheetId="1" state="visible" r:id="rId1"/>
@@ -2684,12 +2684,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Erection Compiled</t>
+          <t>Erection Completed</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Stringing Compiled</t>
+          <t>Stringing Completed</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Erection Compiled</t>
+          <t>Erection</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -8863,6 +8863,12 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -8890,35 +8896,40 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>quantity_loa</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>quantity_estimated_or_total</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>cumulative_last_month</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>plan_for_month</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>progress_for_month</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
         <is>
           <t>today_progress</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>progress_for_month</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>cumulative_progress</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>balance_progress</t>
         </is>
@@ -9743,7 +9754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -9801,6 +9812,12 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -9831,35 +9848,35 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>plan_for_month</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>progress_for_month</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>today_progress</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>cumulative_progress</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>plan_for_month</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>balance_progress</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>gangs_working</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>remarks</t>
         </is>
@@ -10800,6 +10817,12 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -10835,7 +10858,7 @@
           <t>cumulative_last_month</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>plan_for_month</t>
         </is>

</xml_diff>

<commit_message>
Auto pipeline update 2026-06-16 16:16:44
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -1,81 +1,84 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="899" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet Names Check" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TB 608 Erection" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="TA 602 Erection" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="TA 513 Ere S-P Erection" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TA 513 Ere S-F Erection" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TA 413 Erection" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="TA 413 Stringing" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="TA 601 Stringing" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="TB 501 220kV Stringing" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="TB 501 132kV Stringing" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="TB 501 220kV Erection" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="TB 501 132kV Erection" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="TB 401 Stringing" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="TB 408 Stringing" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="TA 509 Erection" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="TA 601 Erection" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="TB 408 Status" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="TA 413 Status" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="TA 414 Status" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="TA 416 Status" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="TA 418 Status" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="TA 421 Status" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="TA 419 Status" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="TA 504 Status" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="TA 505 Status" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="TA 506 Status" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="TB 507 400kV Status" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="TB 507 765kV Status" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="TB 501 Status" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="TA 413 Stretch" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="TA 418 Stretch" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="TA 419 Stretch" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="TA 421 Stretch" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="TA 504 Stretch" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="TA 505 Stretch" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="TA 506 Stretch" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="TB 507 Stretch" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="TB 605 Status" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="TA 512 Status" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="TA 601 Status" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="TB 401 Status" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="TA 325 Status" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="TA 509 Status" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="TA 310 Status" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="TA 513 Status" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="TA 601 Stretch" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="TA 512 Stretch" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="TB 401 Stretch" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="TB 408 Stretch" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="TA 421 Tack Welding Stretch" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="TA 602 Status" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="TB 608 Status" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet name="TA 510 Status" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet name="TA 413 Foundation" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet name="TA 509 Foundation" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet name="TB 501 132kV Foundation" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet name="TB 501 220kV Foundation" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet name="TA 601 Foundation" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet name="TB 605 Jammu Foundation" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet name="TB 605 LILO Foundation" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet name="TB 605 Punjab Foundation" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet name="TA 505 Foundation" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet name="TA 512 Foundation" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet name="TA 602 Foundation" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet name="TB 608 Foundation" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet name="TB 507 MAIN Foundation" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet name="TB 507 765kV Foundation" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet Names Check" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 608 Erection" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Erection" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 513 Ere S-P Erection" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 513 Ere S-F Erection" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Erection" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Stringing" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Stringing" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 220kV Stringing" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 132kV Stringing" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 220kV Erection" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 132kV Erection" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 401 Stringing" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 408 Stringing" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 509 Erection" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Erection" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 408 Status" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Status" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 414 Status" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 416 Status" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 418 Status" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 421 Status" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 419 Status" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 504 Status" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 505 Status" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 506 Status" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 400kV Status" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 765kV Status" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 Status" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Stretch" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 418 Stretch" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 419 Stretch" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 421 Stretch" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 504 Stretch" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 505 Stretch" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 506 Stretch" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 Stretch" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 Status" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 512 Status" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Status" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 401 Status" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 325 Status" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 509 Status" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 310 Status" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 513 Status" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Stretch" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 512 Stretch" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 401 Stretch" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 408 Stretch" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 421 Tack Welding Stretch" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Status" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 608 Status" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 510 Status" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Foundation" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 509 Foundation" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 132kV Foundation" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 220kV Foundation" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Foundation" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 Jammu Foundation" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 LILO Foundation" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 Punjab Foundation" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 505 Foundation" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 512 Foundation" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Foundation" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 608 Foundation" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 MAIN Foundation" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 765kV Foundation" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 412 Erection Sections" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 412 Erection" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 412 WIP Erection" sheetId="70" state="visible" r:id="rId70"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId68"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId71"/>
   </externalReferences>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -93,7 +96,7 @@
     <numFmt numFmtId="169" formatCode="&quot;₹&quot;\ #,##0.00"/>
     <numFmt numFmtId="170" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -194,8 +197,11 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -266,6 +272,11 @@
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-0.09997863704336681"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -953,7 +964,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="155">
+  <cellXfs count="156">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1383,6 +1394,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1761,8 +1773,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook r:id="rId1">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Detail Survey-220kV"/>
       <sheetName val="Check Survey-220kV"/>
@@ -2141,7 +2153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T25"/>
+  <dimension ref="A1:T26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="10.453125" customWidth="1" min="1" max="1"/>
@@ -3435,6 +3447,23 @@
       <c r="P25" t="inlineStr">
         <is>
           <t>DPR</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TB 412</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Erection; WIP</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -8863,12 +8892,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -9812,12 +9835,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -10817,12 +10834,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -11577,6 +11588,377 @@
       <c r="N2" t="inlineStr">
         <is>
           <t>Foundation Completion Date</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="155" t="inlineStr">
+        <is>
+          <t>Source Sheet</t>
+        </is>
+      </c>
+      <c r="B1" s="155" t="inlineStr">
+        <is>
+          <t>Section Start Text</t>
+        </is>
+      </c>
+      <c r="C1" s="155" t="inlineStr">
+        <is>
+          <t>Section End Text</t>
+        </is>
+      </c>
+      <c r="D1" s="155" t="inlineStr">
+        <is>
+          <t>Line Name</t>
+        </is>
+      </c>
+      <c r="E1" s="155" t="inlineStr">
+        <is>
+          <t>Line Column</t>
+        </is>
+      </c>
+      <c r="F1" s="155" t="inlineStr">
+        <is>
+          <t>Line Filter Column</t>
+        </is>
+      </c>
+      <c r="G1" s="155" t="inlineStr">
+        <is>
+          <t>Line Filter Value</t>
+        </is>
+      </c>
+      <c r="H1" s="155" t="inlineStr">
+        <is>
+          <t>Template Sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Erection</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>220 KV  Chhapra(NEW) to Amnour</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>LILO of 400 KV Barh</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>220 TM Chapra-Amnour</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>TB 412 Erection</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Erection</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>LILO of 400 KV Barh</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>220 KV D/C Chapra -Gopalganj</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>400 KV LOOP IN</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>LOOP IN</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>TB 412 Erection</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Erection</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LILO of 400 KV Barh</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>220 KV D/C Chapra -Gopalganj</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>400 KV LOOP OUT</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>LOOP OUT</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>TB 412 Erection</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Erection</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>220 KV D/C Chapra -Gopalganj</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>220 SZ Chapra-Gopalganj</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>TB 412 Erection</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ERECTION</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>STRINGING</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>T/L Name</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>TB 412 WIP Erection</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="155" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="B1" s="155" t="n"/>
+      <c r="C1" s="155" t="n"/>
+      <c r="D1" s="155" t="n"/>
+      <c r="E1" s="155" t="n"/>
+      <c r="F1" s="155" t="n"/>
+      <c r="G1" s="155" t="n"/>
+      <c r="H1" s="155" t="n"/>
+      <c r="I1" s="155" t="n"/>
+      <c r="J1" s="155" t="n"/>
+      <c r="K1" s="155" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sr</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Location No.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Tower Type</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Tower Weight (MT)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Completion Date</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Agency</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Completion Month</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Cumm.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SL No.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Location No.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tower Type</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Tower Weight</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Starting Date</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Completion Date</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Gang Name</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Remarks</t>
         </is>
       </c>
     </row>
@@ -11913,6 +12295,142 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="155" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="B1" s="155" t="n"/>
+      <c r="C1" s="155" t="n"/>
+      <c r="D1" s="155" t="n"/>
+      <c r="E1" s="155" t="n"/>
+      <c r="F1" s="155" t="n"/>
+      <c r="G1" s="155" t="n"/>
+      <c r="H1" s="155" t="n"/>
+      <c r="I1" s="155" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>T/L Name</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SR.NO.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GANG</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>LOC. NO.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>T.O.T</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>D.O.S</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>D.O.C</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Line Name</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SL No.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Gang Name</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Location No.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Tower Type</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Starting Date</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Completion Date</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Auto pipeline update 2026-06-17 16:17:05
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -1,85 +1,85 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="899" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet Names Check" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 608 Erection" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 513 Ere S-P Erection" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 513 Ere S-F Erection" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Erection" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Stringing" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Stringing" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 220kV Stringing" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 132kV Stringing" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 220kV Erection" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 132kV Erection" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 401 Stringing" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 408 Stringing" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 509 Erection" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Erection" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 408 Status" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Status" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 414 Status" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 416 Status" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 418 Status" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 421 Status" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 419 Status" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 504 Status" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 505 Status" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 506 Status" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 400kV Status" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 765kV Status" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 Status" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Stretch" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 418 Stretch" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 419 Stretch" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 421 Stretch" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 504 Stretch" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 505 Stretch" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 506 Stretch" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 Stretch" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 Status" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 512 Status" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Status" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 401 Status" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 325 Status" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 509 Status" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 310 Status" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 513 Status" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Stretch" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 512 Stretch" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 401 Stretch" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 408 Stretch" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 421 Tack Welding Stretch" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 608 Status" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 510 Status" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Foundation" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 509 Foundation" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 132kV Foundation" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 220kV Foundation" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Foundation" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 Jammu Foundation" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 LILO Foundation" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 Punjab Foundation" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 505 Foundation" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 512 Foundation" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Foundation" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 608 Foundation" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 MAIN Foundation" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 765kV Foundation" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 412 Erection Sections" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 412 Erection" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 412 WIP Erection" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 412 Status" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Status" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Erection" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="Sheet Names Check" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TB 608 Erection" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TA 513 Ere S-P Erection" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TA 513 Ere S-F Erection" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TA 413 Erection" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="TA 413 Stringing" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="TA 601 Stringing" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="TB 501 220kV Stringing" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="TB 501 132kV Stringing" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="TB 501 220kV Erection" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="TB 501 132kV Erection" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="TB 401 Stringing" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="TB 408 Stringing" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="TA 509 Erection" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="TA 601 Erection" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="TB 408 Status" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="TA 413 Status" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="TA 414 Status" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="TA 416 Status" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="TA 418 Status" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="TA 421 Status" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="TA 419 Status" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="TA 504 Status" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="TA 505 Status" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="TA 506 Status" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="TB 507 400kV Status" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="TB 507 765kV Status" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="TB 501 Status" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="TA 413 Stretch" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="TA 418 Stretch" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="TA 419 Stretch" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="TA 421 Stretch" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="TA 504 Stretch" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="TA 505 Stretch" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="TA 506 Stretch" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="TB 507 Stretch" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="TB 605 Status" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="TA 512 Status" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="TA 601 Status" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="TB 401 Status" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="TA 325 Status" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="TA 509 Status" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="TA 310 Status" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="TA 513 Status" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="TA 601 Stretch" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="TA 512 Stretch" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="TB 401 Stretch" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="TB 408 Stretch" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="TA 421 Tack Welding Stretch" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="TB 608 Status" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="TA 510 Status" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="TA 413 Foundation" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="TA 509 Foundation" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="TB 501 132kV Foundation" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="TB 501 220kV Foundation" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="TA 601 Foundation" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="TB 605 Jammu Foundation" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="TB 605 LILO Foundation" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="TB 605 Punjab Foundation" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="TA 505 Foundation" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="TA 512 Foundation" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="TA 602 Foundation" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="TB 608 Foundation" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="TB 507 MAIN Foundation" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="TB 507 765kV Foundation" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="TB 412 Erection Sections" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="TB 412 Erection" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="TB 412 WIP Erection" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="TB 412 Status" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="TA 602 Status" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="TA 602 Erection" sheetId="71" state="visible" r:id="rId71"/>
   </sheets>
   <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId72"/>
+    <externalReference r:id="rId72"/>
   </externalReferences>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1774,8 +1774,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook r:id="rId1">
     <sheetNames>
       <sheetName val="Detail Survey-220kV"/>
       <sheetName val="Check Survey-220kV"/>
@@ -5145,7 +5145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -5173,37 +5173,57 @@
       </c>
       <c r="D2" s="113" t="inlineStr">
         <is>
+          <t>Comp WK</t>
+        </is>
+      </c>
+      <c r="E2" s="114" t="inlineStr">
+        <is>
+          <t>Rev</t>
+        </is>
+      </c>
+      <c r="F2" s="115" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
           <t>District wise section</t>
         </is>
       </c>
-      <c r="E2" s="114" t="inlineStr">
+      <c r="H2" s="116" t="inlineStr">
         <is>
           <t xml:space="preserve">STATUS </t>
         </is>
       </c>
-      <c r="F2" s="115" t="inlineStr">
+      <c r="I2" s="116" t="inlineStr">
         <is>
           <t>STARTING DATE</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">ENDING DATE </t>
         </is>
       </c>
-      <c r="H2" s="116" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Work starting month</t>
         </is>
       </c>
-      <c r="I2" s="116" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Work completion Month</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Sub-Contractor</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>JMC</t>
         </is>
       </c>
     </row>
@@ -5238,22 +5258,34 @@
           <t>Location No.</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Tower Type</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="152" t="inlineStr">
+        <is>
+          <t>Tower Weight</t>
+        </is>
+      </c>
+      <c r="G5" s="152" t="n"/>
+      <c r="H5" s="152" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F5" s="152" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Starting Date</t>
         </is>
       </c>
-      <c r="G5" s="152" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Completion Date</t>
         </is>
       </c>
-      <c r="H5" s="152" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Gang Name</t>
         </is>

</xml_diff>

<commit_message>
Auto pipeline update 2026-07-01 10:48:10
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -1,85 +1,85 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="899" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet Names Check" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TB 608 Erection" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="TA 513 Ere S-P Erection" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="TA 513 Ere S-F Erection" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TA 413 Erection" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TA 413 Stringing" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="TA 601 Stringing" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="TB 501 220kV Stringing" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="TB 501 132kV Stringing" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="TB 501 220kV Erection" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="TB 501 132kV Erection" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="TB 401 Stringing" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="TB 408 Stringing" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="TA 509 Erection" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="TA 601 Erection" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="TB 408 Status" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="TA 413 Status" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="TA 414 Status" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="TA 416 Status" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="TA 418 Status" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="TA 421 Status" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="TA 419 Status" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="TA 504 Status" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="TA 505 Status" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="TA 506 Status" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="TB 507 400kV Status" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="TB 507 765kV Status" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="TB 501 Status" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="TA 413 Stretch" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="TA 418 Stretch" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="TA 419 Stretch" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="TA 421 Stretch" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="TA 504 Stretch" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="TA 505 Stretch" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="TA 506 Stretch" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="TB 507 Stretch" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="TB 605 Status" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="TA 512 Status" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="TA 601 Status" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="TB 401 Status" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="TA 325 Status" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="TA 509 Status" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="TA 310 Status" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="TA 513 Status" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="TA 601 Stretch" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="TA 512 Stretch" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="TB 401 Stretch" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="TB 408 Stretch" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="TA 421 Tack Welding Stretch" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="TB 608 Status" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="TA 510 Status" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="TA 413 Foundation" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet name="TA 509 Foundation" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet name="TB 501 132kV Foundation" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet name="TB 501 220kV Foundation" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet name="TA 601 Foundation" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet name="TB 605 Jammu Foundation" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet name="TB 605 LILO Foundation" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet name="TB 605 Punjab Foundation" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet name="TA 505 Foundation" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet name="TA 512 Foundation" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet name="TA 602 Foundation" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet name="TB 608 Foundation" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet name="TB 507 MAIN Foundation" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet name="TB 507 765kV Foundation" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet name="TB 412 Erection Sections" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet name="TB 412 Erection" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet name="TB 412 WIP Erection" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet name="TB 412 Status" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="TA 602 Status" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="TA 602 Erection" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet Names Check" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 608 Erection" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 513 Ere S-P Erection" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 513 Ere S-F Erection" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Erection" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Stringing" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Stringing" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 220kV Stringing" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 132kV Stringing" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 220kV Erection" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 132kV Erection" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 401 Stringing" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 408 Stringing" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 509 Erection" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Erection" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 408 Status" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Status" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 414 Status" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 416 Status" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 418 Status" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 421 Status" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 419 Status" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 504 Status" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 505 Status" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 506 Status" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 400kV Status" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 765kV Status" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 Status" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Stretch" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 418 Stretch" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 419 Stretch" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 421 Stretch" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 504 Stretch" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 505 Stretch" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 506 Stretch" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 Stretch" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 Status" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 512 Status" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Status" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 401 Status" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 325 Status" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 509 Status" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 310 Status" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 513 Status" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Stretch" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 512 Stretch" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 401 Stretch" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 408 Stretch" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 421 Tack Welding Stretch" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 608 Status" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 510 Status" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 413 Foundation" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 509 Foundation" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 132kV Foundation" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 501 220kV Foundation" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 601 Foundation" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 Jammu Foundation" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 LILO Foundation" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 Punjab Foundation" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 505 Foundation" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 512 Foundation" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Foundation" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 608 Foundation" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 MAIN Foundation" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 507 765kV Foundation" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 412 Erection Sections" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 412 Erection" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 412 WIP Erection" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 412 Status" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Status" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Erection" sheetId="71" state="visible" r:id="rId71"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId72"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId72"/>
   </externalReferences>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1774,8 +1774,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook r:id="rId1">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Detail Survey-220kV"/>
       <sheetName val="Check Survey-220kV"/>
@@ -2365,7 +2365,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Erection compiled; Tightening</t>
+          <t>Erection compiled</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Erection compiled; Tightening</t>
+          <t>Erection compiled</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -5145,7 +5145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Auto pipeline update 2026-07-02 10:49:44
</commit_message>
<xml_diff>
--- a/Raw Data/DPR_Config.xlsx
+++ b/Raw Data/DPR_Config.xlsx
@@ -77,9 +77,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 412 Status" sheetId="69" state="visible" r:id="rId69"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Status" sheetId="70" state="visible" r:id="rId70"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 602 Erection" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TA 421 Stringing" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 412 Stringing" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TB 605 Stringing" sheetId="74" state="visible" r:id="rId74"/>
   </sheets>
   <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId72"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId75"/>
   </externalReferences>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -202,7 +205,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -278,6 +281,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -965,7 +973,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="156">
+  <cellXfs count="158">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1396,6 +1404,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2154,7 +2164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T26"/>
+  <dimension ref="A1:V26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="10.453125" customWidth="1" min="1" max="1"/>
@@ -2267,6 +2277,16 @@
           <t>Status File Identifier</t>
         </is>
       </c>
+      <c r="U1" s="156" t="inlineStr">
+        <is>
+          <t>Stringing Section Start Text</t>
+        </is>
+      </c>
+      <c r="V1" s="156" t="inlineStr">
+        <is>
+          <t>Stringing Section End Text</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2279,6 +2299,16 @@
           <t>Erection -Jammu; Erection -SK; Erection-Punjab</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Stringing JS-Jammu</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>Jammu; SK; Punjab</t>
@@ -2312,6 +2342,11 @@
       <c r="R2" t="inlineStr">
         <is>
           <t>Jammu; LILO; Punjab</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Stringing</t>
         </is>
       </c>
     </row>
@@ -2658,6 +2693,11 @@
           <t>ERECTION COMPILED</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Stringing Compiled</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>DPR_TA419</t>
@@ -2754,42 +2794,57 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t xml:space="preserve">ProGress Sheet </t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Master Sheet</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Tack Welding</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
           <t>Stringing Compiled</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Master Sheet</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Tack Welding</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Stringing Compiled</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="P11" t="inlineStr">
         <is>
           <t>ProGress Sheet</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Stringing</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>OPGW Stringing</t>
         </is>
       </c>
     </row>
@@ -3462,11 +3517,21 @@
           <t>Erection; WIP</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>TB-412 SUMMARY</t>
@@ -3475,6 +3540,11 @@
       <c r="I26" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Conductor Paying Out,Rough Sag &amp; Final Sag</t>
         </is>
       </c>
     </row>
@@ -7041,6 +7111,18 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>stringing_resolution</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>prefer_final_else_stringing</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -7171,6 +7253,18 @@
       <c r="B5" t="inlineStr">
         <is>
           <t>support required; stringing activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>stringing_resolution</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>prefer_final_else_stringing</t>
         </is>
       </c>
     </row>
@@ -8438,6 +8532,18 @@
       <c r="B5" t="inlineStr">
         <is>
           <t>line wise progress; supply status; support required</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>stringing_resolution</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>prefer_final_else_stringing</t>
         </is>
       </c>
     </row>
@@ -12728,6 +12834,460 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2">
+      <c r="A2" s="156" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="156" t="n"/>
+      <c r="B3" s="156" t="inlineStr">
+        <is>
+          <t>S.No</t>
+        </is>
+      </c>
+      <c r="C3" s="156" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="D3" s="156" t="inlineStr">
+        <is>
+          <t>Length</t>
+        </is>
+      </c>
+      <c r="E3" s="156" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F3" s="156" t="n"/>
+      <c r="G3" s="156" t="n"/>
+      <c r="H3" s="156" t="n"/>
+      <c r="I3" s="156" t="inlineStr">
+        <is>
+          <t>Gang Name</t>
+        </is>
+      </c>
+      <c r="J3" s="156" t="inlineStr">
+        <is>
+          <t>Gang Strength</t>
+        </is>
+      </c>
+      <c r="K3" s="156" t="inlineStr">
+        <is>
+          <t>RouGH SaG</t>
+        </is>
+      </c>
+      <c r="L3" s="156" t="inlineStr">
+        <is>
+          <t>F!n@L sAG</t>
+        </is>
+      </c>
+      <c r="M3" s="156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E@rthwire </t>
+        </is>
+      </c>
+      <c r="N3" s="156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Remarks </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="157" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="156" t="n"/>
+      <c r="B7" s="156" t="inlineStr">
+        <is>
+          <t>S.no</t>
+        </is>
+      </c>
+      <c r="C7" s="156" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="D7" s="156" t="inlineStr">
+        <is>
+          <t>Length</t>
+        </is>
+      </c>
+      <c r="E7" s="156" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F7" s="156" t="n"/>
+      <c r="G7" s="156" t="n"/>
+      <c r="H7" s="156" t="n"/>
+      <c r="I7" s="156" t="inlineStr">
+        <is>
+          <t>Gang Name</t>
+        </is>
+      </c>
+      <c r="J7" s="156" t="n"/>
+      <c r="K7" s="156" t="inlineStr">
+        <is>
+          <t>P/O Starting Date</t>
+        </is>
+      </c>
+      <c r="L7" s="156" t="inlineStr">
+        <is>
+          <t>F/S/ Completion Date</t>
+        </is>
+      </c>
+      <c r="M7" s="156" t="n"/>
+      <c r="N7" s="156" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2">
+      <c r="A2" s="156" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="156" t="inlineStr">
+        <is>
+          <t>T/L Name</t>
+        </is>
+      </c>
+      <c r="B3" s="156" t="inlineStr">
+        <is>
+          <t>SR.NO.</t>
+        </is>
+      </c>
+      <c r="C3" s="156" t="inlineStr">
+        <is>
+          <t>GANG</t>
+        </is>
+      </c>
+      <c r="D3" s="156" t="inlineStr">
+        <is>
+          <t>FROM</t>
+        </is>
+      </c>
+      <c r="E3" s="156" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="F3" s="156" t="inlineStr">
+        <is>
+          <t>Section  (Km)</t>
+        </is>
+      </c>
+      <c r="G3" s="156" t="inlineStr">
+        <is>
+          <t>D.O.S</t>
+        </is>
+      </c>
+      <c r="H3" s="156" t="inlineStr">
+        <is>
+          <t>D.O.S</t>
+        </is>
+      </c>
+      <c r="I3" s="156" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
+      <c r="J3" s="156" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="157" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="156" t="n"/>
+      <c r="B7" s="156" t="inlineStr">
+        <is>
+          <t>S.no</t>
+        </is>
+      </c>
+      <c r="C7" s="156" t="inlineStr">
+        <is>
+          <t>Gang Name</t>
+        </is>
+      </c>
+      <c r="D7" s="156" t="inlineStr">
+        <is>
+          <t>From AP</t>
+        </is>
+      </c>
+      <c r="E7" s="156" t="inlineStr">
+        <is>
+          <t>To AP</t>
+        </is>
+      </c>
+      <c r="F7" s="156" t="inlineStr">
+        <is>
+          <t>Length</t>
+        </is>
+      </c>
+      <c r="G7" s="156" t="inlineStr">
+        <is>
+          <t>P/O Starting Date</t>
+        </is>
+      </c>
+      <c r="H7" s="156" t="inlineStr">
+        <is>
+          <t>F/S/ Completion Date</t>
+        </is>
+      </c>
+      <c r="I7" s="156" t="n"/>
+      <c r="J7" s="156" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2">
+      <c r="A2" s="156" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="156" t="n"/>
+      <c r="B3" s="156" t="inlineStr">
+        <is>
+          <t>S.No</t>
+        </is>
+      </c>
+      <c r="C3" s="156" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="D3" s="156" t="inlineStr">
+        <is>
+          <t>Length
+Km</t>
+        </is>
+      </c>
+      <c r="E3" s="156" t="inlineStr">
+        <is>
+          <t>TSE/Manual</t>
+        </is>
+      </c>
+      <c r="F3" s="156" t="inlineStr">
+        <is>
+          <t>Insulator Hoisting</t>
+        </is>
+      </c>
+      <c r="G3" s="156" t="n"/>
+      <c r="H3" s="156" t="inlineStr">
+        <is>
+          <t>Paying Out</t>
+        </is>
+      </c>
+      <c r="I3" s="156" t="n"/>
+      <c r="J3" s="156" t="inlineStr">
+        <is>
+          <t>Rough Sag</t>
+        </is>
+      </c>
+      <c r="K3" s="156" t="n"/>
+      <c r="L3" s="156" t="inlineStr">
+        <is>
+          <t>Final Sag</t>
+        </is>
+      </c>
+      <c r="M3" s="156" t="n"/>
+      <c r="N3" s="156" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="O3" s="156" t="inlineStr">
+        <is>
+          <t>Gang</t>
+        </is>
+      </c>
+      <c r="P3" s="156" t="inlineStr">
+        <is>
+          <t>Manpower</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="157" t="inlineStr">
+        <is>
+          <t>To Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="156" t="n"/>
+      <c r="B7" s="156" t="inlineStr">
+        <is>
+          <t>S.no</t>
+        </is>
+      </c>
+      <c r="C7" s="156" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="D7" s="156" t="inlineStr">
+        <is>
+          <t>Length</t>
+        </is>
+      </c>
+      <c r="E7" s="156" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="F7" s="156" t="n"/>
+      <c r="G7" s="156" t="n"/>
+      <c r="H7" s="156" t="inlineStr">
+        <is>
+          <t>P/O Starting Date</t>
+        </is>
+      </c>
+      <c r="I7" s="156" t="inlineStr">
+        <is>
+          <t>P/O Completion Date</t>
+        </is>
+      </c>
+      <c r="J7" s="156" t="n"/>
+      <c r="K7" s="156" t="n"/>
+      <c r="L7" s="156" t="inlineStr">
+        <is>
+          <t>F/S Starting Date</t>
+        </is>
+      </c>
+      <c r="M7" s="156" t="inlineStr">
+        <is>
+          <t>F/S/ Completion Date</t>
+        </is>
+      </c>
+      <c r="N7" s="156" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="O7" s="156" t="inlineStr">
+        <is>
+          <t>Gang Name</t>
+        </is>
+      </c>
+      <c r="P7" s="156" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>